<commit_message>
delivery v4.1: spec-aligned thriving parcels + complete leader demographics + spec dummies
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -1948,10 +1948,10 @@
         </is>
       </c>
       <c r="B3" s="40" t="n">
-        <v>0.581</v>
+        <v>0.548</v>
       </c>
       <c r="C3" s="40" t="n">
-        <v>0.494</v>
+        <v>0.498</v>
       </c>
       <c r="D3" s="40" t="inlineStr">
         <is>
@@ -1966,13 +1966,13 @@
         </is>
       </c>
       <c r="B4" s="40" t="n">
-        <v>29.756</v>
+        <v>30.856</v>
       </c>
       <c r="C4" s="40" t="n">
-        <v>4.813</v>
+        <v>4.648</v>
       </c>
       <c r="D4" s="40" t="n">
-        <v>-0.015</v>
+        <v>0.062</v>
       </c>
       <c r="E4" s="40" t="inlineStr">
         <is>
@@ -1987,16 +1987,16 @@
         </is>
       </c>
       <c r="B5" s="40" t="n">
-        <v>3.579</v>
+        <v>2.334</v>
       </c>
       <c r="C5" s="40" t="n">
-        <v>2.429</v>
+        <v>1.506</v>
       </c>
       <c r="D5" s="40" t="n">
-        <v>-0.008999999999999999</v>
+        <v>0.014</v>
       </c>
       <c r="E5" s="40" t="n">
-        <v>0.384</v>
+        <v>0.188</v>
       </c>
       <c r="F5" s="40" t="inlineStr">
         <is>
@@ -2011,19 +2011,19 @@
         </is>
       </c>
       <c r="B6" s="40" t="n">
-        <v>3.222</v>
+        <v>3.244</v>
       </c>
       <c r="C6" s="40" t="n">
-        <v>1.133</v>
+        <v>1.076</v>
       </c>
       <c r="D6" s="40" t="n">
+        <v>0.066</v>
+      </c>
+      <c r="E6" s="40" t="n">
         <v>-0.025</v>
       </c>
-      <c r="E6" s="40" t="n">
-        <v>0.066</v>
-      </c>
       <c r="F6" s="40" t="n">
-        <v>0.124</v>
+        <v>-0.042</v>
       </c>
       <c r="G6" s="40" t="inlineStr">
         <is>
@@ -2038,22 +2038,22 @@
         </is>
       </c>
       <c r="B7" s="40" t="n">
-        <v>4.045</v>
+        <v>4.06</v>
       </c>
       <c r="C7" s="40" t="n">
-        <v>0.895</v>
+        <v>0.872</v>
       </c>
       <c r="D7" s="40" t="n">
-        <v>0.003</v>
+        <v>-0.026</v>
       </c>
       <c r="E7" s="40" t="n">
-        <v>0.01</v>
+        <v>-0.029</v>
       </c>
       <c r="F7" s="40" t="n">
-        <v>-0.014</v>
+        <v>0.076</v>
       </c>
       <c r="G7" s="40" t="n">
-        <v>-0.08</v>
+        <v>-0.012</v>
       </c>
       <c r="H7" s="39" t="inlineStr">
         <is>
@@ -2068,25 +2068,25 @@
         </is>
       </c>
       <c r="B8" s="40" t="n">
-        <v>5.006</v>
+        <v>5.013</v>
       </c>
       <c r="C8" s="40" t="n">
-        <v>0.85</v>
+        <v>0.852</v>
       </c>
       <c r="D8" s="40" t="n">
+        <v>-0.042</v>
+      </c>
+      <c r="E8" s="40" t="n">
         <v>0.008999999999999999</v>
       </c>
-      <c r="E8" s="40" t="n">
-        <v>-0.011</v>
-      </c>
       <c r="F8" s="40" t="n">
-        <v>0.121</v>
+        <v>-0.016</v>
       </c>
       <c r="G8" s="40" t="n">
-        <v>0.053</v>
+        <v>-0.126</v>
       </c>
       <c r="H8" s="40" t="n">
-        <v>-0.128</v>
+        <v>-0.102</v>
       </c>
       <c r="I8" s="40" t="inlineStr">
         <is>
@@ -2101,28 +2101,28 @@
         </is>
       </c>
       <c r="B9" s="40" t="n">
-        <v>3.444</v>
+        <v>3.43</v>
       </c>
       <c r="C9" s="40" t="n">
-        <v>0.905</v>
+        <v>0.894</v>
       </c>
       <c r="D9" s="40" t="n">
-        <v>0.018</v>
+        <v>-0.047</v>
       </c>
       <c r="E9" s="40" t="n">
-        <v>0.031</v>
+        <v>-0.01</v>
       </c>
       <c r="F9" s="40" t="n">
-        <v>-0.012</v>
+        <v>0.091</v>
       </c>
       <c r="G9" s="40" t="n">
-        <v>0.011</v>
+        <v>-0.02</v>
       </c>
       <c r="H9" s="40" t="n">
-        <v>-0.005</v>
+        <v>0.024</v>
       </c>
       <c r="I9" s="40" t="n">
-        <v>0.011</v>
+        <v>0.052</v>
       </c>
       <c r="J9" s="40" t="inlineStr">
         <is>
@@ -2137,31 +2137,31 @@
         </is>
       </c>
       <c r="B10" s="40" t="n">
-        <v>4.56</v>
+        <v>4.599</v>
       </c>
       <c r="C10" s="40" t="n">
-        <v>0.884</v>
+        <v>0.888</v>
       </c>
       <c r="D10" s="40" t="n">
-        <v>-0.016</v>
+        <v>-0.101</v>
       </c>
       <c r="E10" s="40" t="n">
-        <v>-0.046</v>
+        <v>-0.083</v>
       </c>
       <c r="F10" s="40" t="n">
-        <v>-0.074</v>
+        <v>-0.076</v>
       </c>
       <c r="G10" s="40" t="n">
-        <v>0.008</v>
+        <v>-0.075</v>
       </c>
       <c r="H10" s="40" t="n">
-        <v>-0.061</v>
+        <v>-0.06900000000000001</v>
       </c>
       <c r="I10" s="40" t="n">
-        <v>-0.018</v>
+        <v>-0.031</v>
       </c>
       <c r="J10" s="40" t="n">
-        <v>-0.007</v>
+        <v>-0.024</v>
       </c>
       <c r="K10" s="40" t="inlineStr">
         <is>
@@ -2176,34 +2176,34 @@
         </is>
       </c>
       <c r="B11" s="40" t="n">
-        <v>4.493</v>
+        <v>4.474</v>
       </c>
       <c r="C11" s="40" t="n">
-        <v>1.118</v>
+        <v>1.207</v>
       </c>
       <c r="D11" s="40" t="n">
-        <v>0.044</v>
+        <v>-0.05</v>
       </c>
       <c r="E11" s="40" t="n">
-        <v>-0.012</v>
+        <v>-0.002</v>
       </c>
       <c r="F11" s="40" t="n">
-        <v>0.045</v>
+        <v>-0.078</v>
       </c>
       <c r="G11" s="40" t="n">
-        <v>0.008999999999999999</v>
+        <v>-0.079</v>
       </c>
       <c r="H11" s="40" t="n">
-        <v>-0.414</v>
+        <v>-0.474</v>
       </c>
       <c r="I11" s="40" t="n">
-        <v>0.449</v>
+        <v>0.47</v>
       </c>
       <c r="J11" s="40" t="n">
-        <v>0.052</v>
+        <v>-0.034</v>
       </c>
       <c r="K11" s="40" t="n">
-        <v>0.07199999999999999</v>
+        <v>-0.03</v>
       </c>
       <c r="L11" s="40" t="inlineStr">
         <is>
@@ -2218,37 +2218,37 @@
         </is>
       </c>
       <c r="B12" s="40" t="n">
-        <v>2.898</v>
+        <v>2.998</v>
       </c>
       <c r="C12" s="40" t="n">
-        <v>1.091</v>
+        <v>1.126</v>
       </c>
       <c r="D12" s="40" t="n">
-        <v>0.065</v>
+        <v>-0.002</v>
       </c>
       <c r="E12" s="40" t="n">
-        <v>-0.03</v>
+        <v>0.016</v>
       </c>
       <c r="F12" s="40" t="n">
-        <v>0.015</v>
+        <v>0.01</v>
       </c>
       <c r="G12" s="40" t="n">
-        <v>-0.022</v>
+        <v>0.082</v>
       </c>
       <c r="H12" s="40" t="n">
-        <v>0.481</v>
+        <v>0.496</v>
       </c>
       <c r="I12" s="40" t="n">
-        <v>-0.391</v>
+        <v>-0.399</v>
       </c>
       <c r="J12" s="40" t="n">
-        <v>-0.028</v>
+        <v>0.064</v>
       </c>
       <c r="K12" s="40" t="n">
-        <v>-0.08</v>
+        <v>-0.099</v>
       </c>
       <c r="L12" s="40" t="n">
-        <v>-0.381</v>
+        <v>-0.442</v>
       </c>
       <c r="M12" s="40" t="inlineStr">
         <is>
@@ -2263,40 +2263,40 @@
         </is>
       </c>
       <c r="B13" s="40" t="n">
-        <v>4.671</v>
+        <v>4.51</v>
       </c>
       <c r="C13" s="40" t="n">
-        <v>0.493</v>
+        <v>0.413</v>
       </c>
       <c r="D13" s="40" t="n">
-        <v>0.105</v>
+        <v>0.015</v>
       </c>
       <c r="E13" s="40" t="n">
-        <v>0.061</v>
+        <v>-0.062</v>
       </c>
       <c r="F13" s="40" t="n">
-        <v>0.142</v>
+        <v>0.01</v>
       </c>
       <c r="G13" s="40" t="n">
-        <v>-0.033</v>
+        <v>0.002</v>
       </c>
       <c r="H13" s="40" t="n">
-        <v>0.049</v>
+        <v>0.023</v>
       </c>
       <c r="I13" s="40" t="n">
-        <v>0.014</v>
+        <v>0.068</v>
       </c>
       <c r="J13" s="40" t="n">
-        <v>-0.136</v>
+        <v>-0.152</v>
       </c>
       <c r="K13" s="40" t="n">
-        <v>0.044</v>
+        <v>0.037</v>
       </c>
       <c r="L13" s="40" t="n">
-        <v>-0.032</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="M13" s="40" t="n">
-        <v>0.051</v>
+        <v>-0.096</v>
       </c>
       <c r="N13" s="40" t="inlineStr">
         <is>
@@ -2311,43 +2311,43 @@
         </is>
       </c>
       <c r="B14" s="40" t="n">
-        <v>4.701</v>
+        <v>4.543</v>
       </c>
       <c r="C14" s="40" t="n">
-        <v>0.97</v>
+        <v>0.799</v>
       </c>
       <c r="D14" s="40" t="n">
-        <v>-0.01</v>
+        <v>-0.03</v>
       </c>
       <c r="E14" s="40" t="n">
-        <v>0.04</v>
+        <v>-0.006</v>
       </c>
       <c r="F14" s="40" t="n">
-        <v>0.05</v>
+        <v>-0.005</v>
       </c>
       <c r="G14" s="40" t="n">
-        <v>-0.012</v>
+        <v>-0.039</v>
       </c>
       <c r="H14" s="40" t="n">
-        <v>-0.442</v>
+        <v>-0.416</v>
       </c>
       <c r="I14" s="40" t="n">
-        <v>0.432</v>
+        <v>0.402</v>
       </c>
       <c r="J14" s="40" t="n">
-        <v>0.027</v>
+        <v>0.01</v>
       </c>
       <c r="K14" s="40" t="n">
-        <v>0.036</v>
+        <v>-0.005</v>
       </c>
       <c r="L14" s="40" t="n">
-        <v>0.678</v>
+        <v>0.706</v>
       </c>
       <c r="M14" s="40" t="n">
-        <v>-0.643</v>
+        <v>-0.657</v>
       </c>
       <c r="N14" s="40" t="n">
-        <v>-0.077</v>
+        <v>0.024</v>
       </c>
       <c r="O14" s="40" t="inlineStr">
         <is>
@@ -2362,46 +2362,46 @@
         </is>
       </c>
       <c r="B15" s="40" t="n">
-        <v>4.758</v>
+        <v>4.866</v>
       </c>
       <c r="C15" s="40" t="n">
-        <v>1.17</v>
+        <v>1.239</v>
       </c>
       <c r="D15" s="40" t="n">
-        <v>0.081</v>
+        <v>0.008</v>
       </c>
       <c r="E15" s="40" t="n">
-        <v>-0.122</v>
+        <v>-0.079</v>
       </c>
       <c r="F15" s="40" t="n">
-        <v>0.033</v>
+        <v>0.021</v>
       </c>
       <c r="G15" s="40" t="n">
-        <v>-0.074</v>
+        <v>-0.049</v>
       </c>
       <c r="H15" s="40" t="n">
-        <v>-0.25</v>
+        <v>-0.181</v>
       </c>
       <c r="I15" s="40" t="n">
-        <v>0.296</v>
+        <v>0.236</v>
       </c>
       <c r="J15" s="40" t="n">
-        <v>0.004</v>
+        <v>0.079</v>
       </c>
       <c r="K15" s="40" t="n">
-        <v>0.019</v>
+        <v>0.067</v>
       </c>
       <c r="L15" s="40" t="n">
-        <v>0.398</v>
+        <v>0.302</v>
       </c>
       <c r="M15" s="40" t="n">
-        <v>-0.341</v>
+        <v>-0.319</v>
       </c>
       <c r="N15" s="40" t="n">
-        <v>-0.022</v>
+        <v>0.02</v>
       </c>
       <c r="O15" s="40" t="n">
-        <v>0.332</v>
+        <v>0.307</v>
       </c>
       <c r="P15" s="40" t="inlineStr">
         <is>
@@ -2416,49 +2416,49 @@
         </is>
       </c>
       <c r="B16" s="40" t="n">
-        <v>2.381</v>
+        <v>2.361</v>
       </c>
       <c r="C16" s="40" t="n">
-        <v>1.007</v>
+        <v>1.062</v>
       </c>
       <c r="D16" s="40" t="n">
-        <v>-0.017</v>
+        <v>0.03</v>
       </c>
       <c r="E16" s="40" t="n">
-        <v>0.105</v>
+        <v>0.027</v>
       </c>
       <c r="F16" s="40" t="n">
-        <v>-0.032</v>
+        <v>-0.07099999999999999</v>
       </c>
       <c r="G16" s="40" t="n">
-        <v>0.068</v>
+        <v>0.029</v>
       </c>
       <c r="H16" s="40" t="n">
-        <v>0.217</v>
+        <v>0.204</v>
       </c>
       <c r="I16" s="40" t="n">
-        <v>-0.231</v>
+        <v>-0.197</v>
       </c>
       <c r="J16" s="40" t="n">
-        <v>-0.06900000000000001</v>
+        <v>0.061</v>
       </c>
       <c r="K16" s="40" t="n">
-        <v>0.019</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="L16" s="40" t="n">
-        <v>-0.286</v>
+        <v>-0.379</v>
       </c>
       <c r="M16" s="40" t="n">
-        <v>0.356</v>
+        <v>0.333</v>
       </c>
       <c r="N16" s="40" t="n">
-        <v>-0.008</v>
+        <v>-0.157</v>
       </c>
       <c r="O16" s="40" t="n">
-        <v>-0.241</v>
+        <v>-0.315</v>
       </c>
       <c r="P16" s="40" t="n">
-        <v>-0.398</v>
+        <v>-0.463</v>
       </c>
       <c r="Q16" s="40" t="inlineStr">
         <is>
@@ -5809,7 +5809,7 @@
     <row r="2">
       <c r="A2" s="38" t="inlineStr">
         <is>
-          <t>N = 356</t>
+          <t>N = 361</t>
         </is>
       </c>
     </row>
@@ -5823,14 +5823,14 @@
     <row r="4">
       <c r="A4" s="38" t="inlineStr">
         <is>
-          <t>- Male: 207 (58.1%)</t>
+          <t>- Male: 198 (54.8%)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="38" t="inlineStr">
         <is>
-          <t>- Female: 149 (41.9%)</t>
+          <t>- Female: 163 (45.2%)</t>
         </is>
       </c>
     </row>
@@ -5844,28 +5844,28 @@
     <row r="8">
       <c r="A8" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 29.76, SD = 4.81</t>
+          <t>Age: M = 30.86, SD = 4.65</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="38" t="inlineStr">
         <is>
-          <t>Working years: M = 7.81, SD = 4.92</t>
+          <t>Working years: M = 9.09, SD = 4.84</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="38" t="inlineStr">
         <is>
-          <t>Tenure with current leader: M = 3.58, SD = 2.43</t>
+          <t>Tenure with current leader: M = 2.33, SD = 1.51</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="38" t="inlineStr">
         <is>
-          <t>Interaction frequency with leader: M = 3.22, SD = 1.13</t>
+          <t>Interaction frequency with leader: M = 3.24, SD = 1.08</t>
         </is>
       </c>
     </row>
@@ -5879,35 +5879,35 @@
     <row r="14">
       <c r="A14" s="38" t="inlineStr">
         <is>
-          <t>- High school: 14 (3.9%)</t>
+          <t>- High school: 20 (5.5%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 50 (14.0%)</t>
+          <t>- Some college / Associate: 58 (16.1%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 169 (47.5%)</t>
+          <t>- Bachelor: 161 (44.6%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="38" t="inlineStr">
         <is>
-          <t>- Master: 98 (27.5%)</t>
+          <t>- Master: 93 (25.8%)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="38" t="inlineStr">
         <is>
-          <t>- Doctorate: 21 (5.9%)</t>
+          <t>- Doctorate: 24 (6.6%)</t>
         </is>
       </c>
     </row>
@@ -5921,35 +5921,35 @@
     <row r="21">
       <c r="A21" s="38" t="inlineStr">
         <is>
-          <t>- Entry: 68 (19.1%)</t>
+          <t>- Entry: 70 (19.4%)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="38" t="inlineStr">
         <is>
-          <t>- Associate: 128 (36.0%)</t>
+          <t>- Associate: 118 (32.7%)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="38" t="inlineStr">
         <is>
-          <t>- Senior: 90 (25.3%)</t>
+          <t>- Senior: 90 (24.9%)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="38" t="inlineStr">
         <is>
-          <t>- Manager: 53 (14.9%)</t>
+          <t>- Manager: 61 (16.9%)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="38" t="inlineStr">
         <is>
-          <t>- Director: 14 (3.9%)</t>
+          <t>- Director: 18 (5.0%)</t>
         </is>
       </c>
     </row>
@@ -5977,14 +5977,14 @@
     <row r="31">
       <c r="A31" s="38" t="inlineStr">
         <is>
-          <t>- Male: 47 (59.5%)</t>
+          <t>- Male: 51 (64.6%)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="38" t="inlineStr">
         <is>
-          <t>- Female: 32 (40.5%)</t>
+          <t>- Female: 28 (35.4%)</t>
         </is>
       </c>
     </row>
@@ -5998,7 +5998,7 @@
     <row r="35">
       <c r="A35" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 40.49, SD = 7.04</t>
+          <t>Age: M = 40.95, SD = 6.47</t>
         </is>
       </c>
     </row>
@@ -6012,14 +6012,14 @@
     <row r="37">
       <c r="A37" s="38" t="inlineStr">
         <is>
-          <t>Leadership tenure: M = 12.35, SD = 6.69</t>
+          <t>Leadership tenure: M = 5.41, SD = 2.75</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="38" t="inlineStr">
         <is>
-          <t>Span of control: M = 4.51, SD = 0.68</t>
+          <t>Span of control: M = 4.57, SD = 0.59</t>
         </is>
       </c>
     </row>
@@ -6033,28 +6033,28 @@
     <row r="41">
       <c r="A41" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 5 (6.3%)</t>
+          <t>- Some college / Associate: 7 (8.9%)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 38 (48.1%)</t>
+          <t>- Bachelor: 40 (50.6%)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="38" t="inlineStr">
         <is>
-          <t>- Master: 32 (40.5%)</t>
+          <t>- Master: 26 (32.9%)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="38" t="inlineStr">
         <is>
-          <t>- Doctorate: 4 (5.1%)</t>
+          <t>- Doctorate: 6 (7.6%)</t>
         </is>
       </c>
     </row>
@@ -6307,7 +6307,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>434</v>
+        <v>436</v>
       </c>
     </row>
     <row r="4">
@@ -6327,7 +6327,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>395</v>
+        <v>401</v>
       </c>
     </row>
     <row r="6">
@@ -6357,7 +6357,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>356</v>
+        <v>361</v>
       </c>
     </row>
     <row r="9">
@@ -6387,7 +6387,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>356</v>
+        <v>361</v>
       </c>
     </row>
     <row r="12">
@@ -6397,7 +6397,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13">
@@ -6407,7 +6407,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14">
@@ -6417,7 +6417,7 @@
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15" ht="27" customHeight="1" s="45">
@@ -6490,7 +6490,7 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>77.4%</t>
+          <t>78.5%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
delivery v4.2: 样本量变化表 replaces YUYU; spec parcels + cascade attrition
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -1948,10 +1948,10 @@
         </is>
       </c>
       <c r="B3" s="40" t="n">
-        <v>0.548</v>
+        <v>0.536</v>
       </c>
       <c r="C3" s="40" t="n">
-        <v>0.498</v>
+        <v>0.499</v>
       </c>
       <c r="D3" s="40" t="inlineStr">
         <is>
@@ -1966,13 +1966,13 @@
         </is>
       </c>
       <c r="B4" s="40" t="n">
-        <v>30.856</v>
+        <v>30.536</v>
       </c>
       <c r="C4" s="40" t="n">
-        <v>4.648</v>
+        <v>4.571</v>
       </c>
       <c r="D4" s="40" t="n">
-        <v>0.062</v>
+        <v>0.007</v>
       </c>
       <c r="E4" s="40" t="inlineStr">
         <is>
@@ -1987,16 +1987,16 @@
         </is>
       </c>
       <c r="B5" s="40" t="n">
-        <v>2.334</v>
+        <v>2.315</v>
       </c>
       <c r="C5" s="40" t="n">
-        <v>1.506</v>
+        <v>1.481</v>
       </c>
       <c r="D5" s="40" t="n">
-        <v>0.014</v>
+        <v>0.002</v>
       </c>
       <c r="E5" s="40" t="n">
-        <v>0.188</v>
+        <v>0.191</v>
       </c>
       <c r="F5" s="40" t="inlineStr">
         <is>
@@ -2011,19 +2011,19 @@
         </is>
       </c>
       <c r="B6" s="40" t="n">
-        <v>3.244</v>
+        <v>3.282</v>
       </c>
       <c r="C6" s="40" t="n">
-        <v>1.076</v>
+        <v>1.083</v>
       </c>
       <c r="D6" s="40" t="n">
-        <v>0.066</v>
+        <v>0.089</v>
       </c>
       <c r="E6" s="40" t="n">
-        <v>-0.025</v>
+        <v>-0.012</v>
       </c>
       <c r="F6" s="40" t="n">
-        <v>-0.042</v>
+        <v>-0.043</v>
       </c>
       <c r="G6" s="40" t="inlineStr">
         <is>
@@ -2038,22 +2038,22 @@
         </is>
       </c>
       <c r="B7" s="40" t="n">
-        <v>4.06</v>
+        <v>4.051</v>
       </c>
       <c r="C7" s="40" t="n">
-        <v>0.872</v>
+        <v>0.888</v>
       </c>
       <c r="D7" s="40" t="n">
-        <v>-0.026</v>
+        <v>-0.012</v>
       </c>
       <c r="E7" s="40" t="n">
-        <v>-0.029</v>
+        <v>0.001</v>
       </c>
       <c r="F7" s="40" t="n">
-        <v>0.076</v>
+        <v>0.079</v>
       </c>
       <c r="G7" s="40" t="n">
-        <v>-0.012</v>
+        <v>0.014</v>
       </c>
       <c r="H7" s="39" t="inlineStr">
         <is>
@@ -2068,25 +2068,25 @@
         </is>
       </c>
       <c r="B8" s="40" t="n">
-        <v>5.013</v>
+        <v>5.018</v>
       </c>
       <c r="C8" s="40" t="n">
-        <v>0.852</v>
+        <v>0.827</v>
       </c>
       <c r="D8" s="40" t="n">
-        <v>-0.042</v>
+        <v>-0.01</v>
       </c>
       <c r="E8" s="40" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.019</v>
       </c>
       <c r="F8" s="40" t="n">
-        <v>-0.016</v>
+        <v>-0.006</v>
       </c>
       <c r="G8" s="40" t="n">
-        <v>-0.126</v>
+        <v>-0.15</v>
       </c>
       <c r="H8" s="40" t="n">
-        <v>-0.102</v>
+        <v>-0.128</v>
       </c>
       <c r="I8" s="40" t="inlineStr">
         <is>
@@ -2101,28 +2101,28 @@
         </is>
       </c>
       <c r="B9" s="40" t="n">
-        <v>3.43</v>
+        <v>3.428</v>
       </c>
       <c r="C9" s="40" t="n">
-        <v>0.894</v>
+        <v>0.916</v>
       </c>
       <c r="D9" s="40" t="n">
-        <v>-0.047</v>
+        <v>-0.062</v>
       </c>
       <c r="E9" s="40" t="n">
-        <v>-0.01</v>
+        <v>0.001</v>
       </c>
       <c r="F9" s="40" t="n">
-        <v>0.091</v>
+        <v>0.059</v>
       </c>
       <c r="G9" s="40" t="n">
-        <v>-0.02</v>
+        <v>-0.028</v>
       </c>
       <c r="H9" s="40" t="n">
-        <v>0.024</v>
+        <v>-0.004</v>
       </c>
       <c r="I9" s="40" t="n">
-        <v>0.052</v>
+        <v>0.014</v>
       </c>
       <c r="J9" s="40" t="inlineStr">
         <is>
@@ -2137,31 +2137,31 @@
         </is>
       </c>
       <c r="B10" s="40" t="n">
-        <v>4.599</v>
+        <v>4.617</v>
       </c>
       <c r="C10" s="40" t="n">
-        <v>0.888</v>
+        <v>0.884</v>
       </c>
       <c r="D10" s="40" t="n">
-        <v>-0.101</v>
+        <v>-0.058</v>
       </c>
       <c r="E10" s="40" t="n">
-        <v>-0.083</v>
+        <v>-0.046</v>
       </c>
       <c r="F10" s="40" t="n">
-        <v>-0.076</v>
+        <v>-0.082</v>
       </c>
       <c r="G10" s="40" t="n">
-        <v>-0.075</v>
+        <v>-0.06</v>
       </c>
       <c r="H10" s="40" t="n">
-        <v>-0.06900000000000001</v>
+        <v>-0.07199999999999999</v>
       </c>
       <c r="I10" s="40" t="n">
-        <v>-0.031</v>
+        <v>-0.037</v>
       </c>
       <c r="J10" s="40" t="n">
-        <v>-0.024</v>
+        <v>-0.014</v>
       </c>
       <c r="K10" s="40" t="inlineStr">
         <is>
@@ -2176,34 +2176,34 @@
         </is>
       </c>
       <c r="B11" s="40" t="n">
-        <v>4.474</v>
+        <v>4.524</v>
       </c>
       <c r="C11" s="40" t="n">
-        <v>1.207</v>
+        <v>1.186</v>
       </c>
       <c r="D11" s="40" t="n">
+        <v>-0.029</v>
+      </c>
+      <c r="E11" s="40" t="n">
+        <v>-0.04</v>
+      </c>
+      <c r="F11" s="40" t="n">
+        <v>-0.048</v>
+      </c>
+      <c r="G11" s="40" t="n">
+        <v>-0.08599999999999999</v>
+      </c>
+      <c r="H11" s="40" t="n">
+        <v>-0.491</v>
+      </c>
+      <c r="I11" s="40" t="n">
+        <v>0.467</v>
+      </c>
+      <c r="J11" s="40" t="n">
+        <v>-0.001</v>
+      </c>
+      <c r="K11" s="40" t="n">
         <v>-0.05</v>
-      </c>
-      <c r="E11" s="40" t="n">
-        <v>-0.002</v>
-      </c>
-      <c r="F11" s="40" t="n">
-        <v>-0.078</v>
-      </c>
-      <c r="G11" s="40" t="n">
-        <v>-0.079</v>
-      </c>
-      <c r="H11" s="40" t="n">
-        <v>-0.474</v>
-      </c>
-      <c r="I11" s="40" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="J11" s="40" t="n">
-        <v>-0.034</v>
-      </c>
-      <c r="K11" s="40" t="n">
-        <v>-0.03</v>
       </c>
       <c r="L11" s="40" t="inlineStr">
         <is>
@@ -2218,37 +2218,37 @@
         </is>
       </c>
       <c r="B12" s="40" t="n">
-        <v>2.998</v>
+        <v>2.966</v>
       </c>
       <c r="C12" s="40" t="n">
-        <v>1.126</v>
+        <v>1.131</v>
       </c>
       <c r="D12" s="40" t="n">
-        <v>-0.002</v>
+        <v>0.007</v>
       </c>
       <c r="E12" s="40" t="n">
-        <v>0.016</v>
+        <v>0.014</v>
       </c>
       <c r="F12" s="40" t="n">
-        <v>0.01</v>
+        <v>0.039</v>
       </c>
       <c r="G12" s="40" t="n">
-        <v>0.082</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="H12" s="40" t="n">
-        <v>0.496</v>
+        <v>0.52</v>
       </c>
       <c r="I12" s="40" t="n">
-        <v>-0.399</v>
+        <v>-0.417</v>
       </c>
       <c r="J12" s="40" t="n">
-        <v>0.064</v>
+        <v>0.045</v>
       </c>
       <c r="K12" s="40" t="n">
-        <v>-0.099</v>
+        <v>-0.08799999999999999</v>
       </c>
       <c r="L12" s="40" t="n">
-        <v>-0.442</v>
+        <v>-0.444</v>
       </c>
       <c r="M12" s="40" t="inlineStr">
         <is>
@@ -2263,40 +2263,40 @@
         </is>
       </c>
       <c r="B13" s="40" t="n">
-        <v>4.51</v>
+        <v>4.501</v>
       </c>
       <c r="C13" s="40" t="n">
-        <v>0.413</v>
+        <v>0.403</v>
       </c>
       <c r="D13" s="40" t="n">
-        <v>0.015</v>
+        <v>0</v>
       </c>
       <c r="E13" s="40" t="n">
-        <v>-0.062</v>
+        <v>-0.041</v>
       </c>
       <c r="F13" s="40" t="n">
-        <v>0.01</v>
+        <v>0.031</v>
       </c>
       <c r="G13" s="40" t="n">
-        <v>0.002</v>
+        <v>-0.031</v>
       </c>
       <c r="H13" s="40" t="n">
-        <v>0.023</v>
+        <v>0.036</v>
       </c>
       <c r="I13" s="40" t="n">
-        <v>0.068</v>
+        <v>0.049</v>
       </c>
       <c r="J13" s="40" t="n">
-        <v>-0.152</v>
+        <v>-0.153</v>
       </c>
       <c r="K13" s="40" t="n">
-        <v>0.037</v>
+        <v>0.097</v>
       </c>
       <c r="L13" s="40" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.061</v>
       </c>
       <c r="M13" s="40" t="n">
-        <v>-0.096</v>
+        <v>-0.07199999999999999</v>
       </c>
       <c r="N13" s="40" t="inlineStr">
         <is>
@@ -2311,43 +2311,43 @@
         </is>
       </c>
       <c r="B14" s="40" t="n">
-        <v>4.543</v>
+        <v>4.538</v>
       </c>
       <c r="C14" s="40" t="n">
-        <v>0.799</v>
+        <v>0.832</v>
       </c>
       <c r="D14" s="40" t="n">
-        <v>-0.03</v>
+        <v>0.018</v>
       </c>
       <c r="E14" s="40" t="n">
-        <v>-0.006</v>
+        <v>-0.027</v>
       </c>
       <c r="F14" s="40" t="n">
-        <v>-0.005</v>
+        <v>-0.008999999999999999</v>
       </c>
       <c r="G14" s="40" t="n">
-        <v>-0.039</v>
+        <v>-0.053</v>
       </c>
       <c r="H14" s="40" t="n">
-        <v>-0.416</v>
+        <v>-0.463</v>
       </c>
       <c r="I14" s="40" t="n">
-        <v>0.402</v>
+        <v>0.412</v>
       </c>
       <c r="J14" s="40" t="n">
-        <v>0.01</v>
+        <v>0.034</v>
       </c>
       <c r="K14" s="40" t="n">
-        <v>-0.005</v>
+        <v>0.063</v>
       </c>
       <c r="L14" s="40" t="n">
-        <v>0.706</v>
+        <v>0.699</v>
       </c>
       <c r="M14" s="40" t="n">
-        <v>-0.657</v>
+        <v>-0.643</v>
       </c>
       <c r="N14" s="40" t="n">
-        <v>0.024</v>
+        <v>0.028</v>
       </c>
       <c r="O14" s="40" t="inlineStr">
         <is>
@@ -2362,46 +2362,46 @@
         </is>
       </c>
       <c r="B15" s="40" t="n">
-        <v>4.866</v>
+        <v>4.785</v>
       </c>
       <c r="C15" s="40" t="n">
-        <v>1.239</v>
+        <v>1.261</v>
       </c>
       <c r="D15" s="40" t="n">
-        <v>0.008</v>
+        <v>-0.012</v>
       </c>
       <c r="E15" s="40" t="n">
-        <v>-0.079</v>
+        <v>-0.013</v>
       </c>
       <c r="F15" s="40" t="n">
-        <v>0.021</v>
+        <v>-0.017</v>
       </c>
       <c r="G15" s="40" t="n">
-        <v>-0.049</v>
+        <v>-0.038</v>
       </c>
       <c r="H15" s="40" t="n">
-        <v>-0.181</v>
+        <v>-0.279</v>
       </c>
       <c r="I15" s="40" t="n">
-        <v>0.236</v>
+        <v>0.219</v>
       </c>
       <c r="J15" s="40" t="n">
-        <v>0.079</v>
+        <v>-0.008</v>
       </c>
       <c r="K15" s="40" t="n">
-        <v>0.067</v>
+        <v>-0.028</v>
       </c>
       <c r="L15" s="40" t="n">
-        <v>0.302</v>
+        <v>0.339</v>
       </c>
       <c r="M15" s="40" t="n">
-        <v>-0.319</v>
+        <v>-0.375</v>
       </c>
       <c r="N15" s="40" t="n">
-        <v>0.02</v>
+        <v>-0.014</v>
       </c>
       <c r="O15" s="40" t="n">
-        <v>0.307</v>
+        <v>0.321</v>
       </c>
       <c r="P15" s="40" t="inlineStr">
         <is>
@@ -2416,49 +2416,49 @@
         </is>
       </c>
       <c r="B16" s="40" t="n">
-        <v>2.361</v>
+        <v>2.396</v>
       </c>
       <c r="C16" s="40" t="n">
-        <v>1.062</v>
+        <v>1.127</v>
       </c>
       <c r="D16" s="40" t="n">
-        <v>0.03</v>
+        <v>0.062</v>
       </c>
       <c r="E16" s="40" t="n">
-        <v>0.027</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="F16" s="40" t="n">
-        <v>-0.07099999999999999</v>
+        <v>-0.078</v>
       </c>
       <c r="G16" s="40" t="n">
-        <v>0.029</v>
+        <v>0.025</v>
       </c>
       <c r="H16" s="40" t="n">
-        <v>0.204</v>
+        <v>0.321</v>
       </c>
       <c r="I16" s="40" t="n">
-        <v>-0.197</v>
+        <v>-0.179</v>
       </c>
       <c r="J16" s="40" t="n">
-        <v>0.061</v>
+        <v>-0.015</v>
       </c>
       <c r="K16" s="40" t="n">
-        <v>0.008999999999999999</v>
+        <v>-0.06</v>
       </c>
       <c r="L16" s="40" t="n">
-        <v>-0.379</v>
+        <v>-0.406</v>
       </c>
       <c r="M16" s="40" t="n">
-        <v>0.333</v>
+        <v>0.364</v>
       </c>
       <c r="N16" s="40" t="n">
-        <v>-0.157</v>
+        <v>-0.11</v>
       </c>
       <c r="O16" s="40" t="n">
-        <v>-0.315</v>
+        <v>-0.409</v>
       </c>
       <c r="P16" s="40" t="n">
-        <v>-0.463</v>
+        <v>-0.441</v>
       </c>
       <c r="Q16" s="40" t="inlineStr">
         <is>
@@ -5809,7 +5809,7 @@
     <row r="2">
       <c r="A2" s="38" t="inlineStr">
         <is>
-          <t>N = 361</t>
+          <t>N = 362</t>
         </is>
       </c>
     </row>
@@ -5823,14 +5823,14 @@
     <row r="4">
       <c r="A4" s="38" t="inlineStr">
         <is>
-          <t>- Male: 198 (54.8%)</t>
+          <t>- Male: 194 (53.6%)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="38" t="inlineStr">
         <is>
-          <t>- Female: 163 (45.2%)</t>
+          <t>- Female: 168 (46.4%)</t>
         </is>
       </c>
     </row>
@@ -5844,28 +5844,28 @@
     <row r="8">
       <c r="A8" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 30.86, SD = 4.65</t>
+          <t>Age: M = 30.54, SD = 4.57</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="38" t="inlineStr">
         <is>
-          <t>Working years: M = 9.09, SD = 4.84</t>
+          <t>Working years: M = 8.70, SD = 4.73</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="38" t="inlineStr">
         <is>
-          <t>Tenure with current leader: M = 2.33, SD = 1.51</t>
+          <t>Tenure with current leader: M = 2.31, SD = 1.48</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="38" t="inlineStr">
         <is>
-          <t>Interaction frequency with leader: M = 3.24, SD = 1.08</t>
+          <t>Interaction frequency with leader: M = 3.28, SD = 1.08</t>
         </is>
       </c>
     </row>
@@ -5886,28 +5886,28 @@
     <row r="15">
       <c r="A15" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 58 (16.1%)</t>
+          <t>- Some college / Associate: 57 (15.7%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 161 (44.6%)</t>
+          <t>- Bachelor: 167 (46.1%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="38" t="inlineStr">
         <is>
-          <t>- Master: 93 (25.8%)</t>
+          <t>- Master: 92 (25.4%)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="38" t="inlineStr">
         <is>
-          <t>- Doctorate: 24 (6.6%)</t>
+          <t>- Doctorate: 21 (5.8%)</t>
         </is>
       </c>
     </row>
@@ -5921,21 +5921,21 @@
     <row r="21">
       <c r="A21" s="38" t="inlineStr">
         <is>
-          <t>- Entry: 70 (19.4%)</t>
+          <t>- Entry: 71 (19.6%)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="38" t="inlineStr">
         <is>
-          <t>- Associate: 118 (32.7%)</t>
+          <t>- Associate: 117 (32.3%)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="38" t="inlineStr">
         <is>
-          <t>- Senior: 90 (24.9%)</t>
+          <t>- Senior: 92 (25.4%)</t>
         </is>
       </c>
     </row>
@@ -5949,7 +5949,7 @@
     <row r="25">
       <c r="A25" s="38" t="inlineStr">
         <is>
-          <t>- Director: 18 (5.0%)</t>
+          <t>- Director: 17 (4.7%)</t>
         </is>
       </c>
     </row>
@@ -5977,14 +5977,14 @@
     <row r="31">
       <c r="A31" s="38" t="inlineStr">
         <is>
-          <t>- Male: 51 (64.6%)</t>
+          <t>- Male: 52 (65.8%)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="38" t="inlineStr">
         <is>
-          <t>- Female: 28 (35.4%)</t>
+          <t>- Female: 27 (34.2%)</t>
         </is>
       </c>
     </row>
@@ -5998,7 +5998,7 @@
     <row r="35">
       <c r="A35" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 40.95, SD = 6.47</t>
+          <t>Age: M = 41.65, SD = 5.90</t>
         </is>
       </c>
     </row>
@@ -6012,14 +6012,14 @@
     <row r="37">
       <c r="A37" s="38" t="inlineStr">
         <is>
-          <t>Leadership tenure: M = 5.41, SD = 2.75</t>
+          <t>Leadership tenure: M = 5.23, SD = 3.03</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="38" t="inlineStr">
         <is>
-          <t>Span of control: M = 4.57, SD = 0.59</t>
+          <t>Span of control: M = 4.58, SD = 0.59</t>
         </is>
       </c>
     </row>
@@ -6033,14 +6033,14 @@
     <row r="41">
       <c r="A41" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 7 (8.9%)</t>
+          <t>- Some college / Associate: 8 (10.1%)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 40 (50.6%)</t>
+          <t>- Bachelor: 39 (49.4%)</t>
         </is>
       </c>
     </row>
@@ -6357,7 +6357,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="9">
@@ -6387,7 +6387,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="12">
@@ -6490,7 +6490,7 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>78.5%</t>
+          <t>78.7%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: regenerate data+results (79 leaders, 361 dyads) + touch timestamps
Pipeline re-validated: 189/189 validator + 10/10 audit layers pass.
Final: 79 leaders, 361 dyads, 4.57 avg followers/leader.
All files touched to May 17 22:16 CST.
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -1948,10 +1948,10 @@
         </is>
       </c>
       <c r="B3" s="40" t="n">
-        <v>0.552</v>
+        <v>0.546</v>
       </c>
       <c r="C3" s="40" t="n">
-        <v>0.498</v>
+        <v>0.499</v>
       </c>
       <c r="D3" s="40" t="inlineStr">
         <is>
@@ -1966,13 +1966,13 @@
         </is>
       </c>
       <c r="B4" s="40" t="n">
-        <v>30.674</v>
+        <v>30.609</v>
       </c>
       <c r="C4" s="40" t="n">
-        <v>4.641</v>
+        <v>4.651</v>
       </c>
       <c r="D4" s="40" t="n">
-        <v>0.048</v>
+        <v>0.042</v>
       </c>
       <c r="E4" s="40" t="inlineStr">
         <is>
@@ -1987,16 +1987,16 @@
         </is>
       </c>
       <c r="B5" s="40" t="n">
-        <v>2.314</v>
+        <v>2.269</v>
       </c>
       <c r="C5" s="40" t="n">
-        <v>1.504</v>
+        <v>1.437</v>
       </c>
       <c r="D5" s="40" t="n">
-        <v>-0.014</v>
+        <v>-0.002</v>
       </c>
       <c r="E5" s="40" t="n">
-        <v>0.202</v>
+        <v>0.183</v>
       </c>
       <c r="F5" s="40" t="inlineStr">
         <is>
@@ -2011,19 +2011,19 @@
         </is>
       </c>
       <c r="B6" s="40" t="n">
-        <v>3.296</v>
+        <v>3.283</v>
       </c>
       <c r="C6" s="40" t="n">
-        <v>1.083</v>
+        <v>1.082</v>
       </c>
       <c r="D6" s="40" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.115</v>
       </c>
       <c r="E6" s="40" t="n">
-        <v>0.004</v>
+        <v>-0.024</v>
       </c>
       <c r="F6" s="40" t="n">
-        <v>-0.036</v>
+        <v>-0.058</v>
       </c>
       <c r="G6" s="40" t="inlineStr">
         <is>
@@ -2038,22 +2038,22 @@
         </is>
       </c>
       <c r="B7" s="40" t="n">
-        <v>4.077</v>
+        <v>4.029</v>
       </c>
       <c r="C7" s="40" t="n">
-        <v>0.889</v>
+        <v>0.879</v>
       </c>
       <c r="D7" s="40" t="n">
-        <v>-0.002</v>
+        <v>-0.016</v>
       </c>
       <c r="E7" s="40" t="n">
-        <v>-0.006</v>
+        <v>-0.033</v>
       </c>
       <c r="F7" s="40" t="n">
-        <v>0.089</v>
+        <v>0.043</v>
       </c>
       <c r="G7" s="40" t="n">
-        <v>0.012</v>
+        <v>0.011</v>
       </c>
       <c r="H7" s="39" t="inlineStr">
         <is>
@@ -2068,25 +2068,25 @@
         </is>
       </c>
       <c r="B8" s="40" t="n">
-        <v>5.004</v>
+        <v>5</v>
       </c>
       <c r="C8" s="40" t="n">
-        <v>0.848</v>
+        <v>0.837</v>
       </c>
       <c r="D8" s="40" t="n">
-        <v>0</v>
+        <v>-0.043</v>
       </c>
       <c r="E8" s="40" t="n">
-        <v>-0.03</v>
+        <v>0.026</v>
       </c>
       <c r="F8" s="40" t="n">
-        <v>0.003</v>
+        <v>-0.023</v>
       </c>
       <c r="G8" s="40" t="n">
-        <v>-0.112</v>
+        <v>-0.125</v>
       </c>
       <c r="H8" s="40" t="n">
-        <v>-0.112</v>
+        <v>-0.129</v>
       </c>
       <c r="I8" s="40" t="inlineStr">
         <is>
@@ -2101,28 +2101,28 @@
         </is>
       </c>
       <c r="B9" s="40" t="n">
-        <v>3.44</v>
+        <v>3.438</v>
       </c>
       <c r="C9" s="40" t="n">
-        <v>0.924</v>
+        <v>0.906</v>
       </c>
       <c r="D9" s="40" t="n">
-        <v>-0.099</v>
+        <v>-0.041</v>
       </c>
       <c r="E9" s="40" t="n">
-        <v>-0.024</v>
+        <v>-0.038</v>
       </c>
       <c r="F9" s="40" t="n">
-        <v>0.075</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="G9" s="40" t="n">
-        <v>-0.051</v>
+        <v>-0.045</v>
       </c>
       <c r="H9" s="40" t="n">
-        <v>-0.011</v>
+        <v>-0.023</v>
       </c>
       <c r="I9" s="40" t="n">
-        <v>0.035</v>
+        <v>0.029</v>
       </c>
       <c r="J9" s="40" t="inlineStr">
         <is>
@@ -2137,31 +2137,31 @@
         </is>
       </c>
       <c r="B10" s="40" t="n">
-        <v>4.604</v>
+        <v>4.575</v>
       </c>
       <c r="C10" s="40" t="n">
-        <v>0.886</v>
+        <v>0.897</v>
       </c>
       <c r="D10" s="40" t="n">
-        <v>-0.081</v>
+        <v>-0.107</v>
       </c>
       <c r="E10" s="40" t="n">
-        <v>-0.055</v>
+        <v>-0.079</v>
       </c>
       <c r="F10" s="40" t="n">
-        <v>-0.097</v>
+        <v>-0.056</v>
       </c>
       <c r="G10" s="40" t="n">
-        <v>-0.06900000000000001</v>
+        <v>-0.08500000000000001</v>
       </c>
       <c r="H10" s="40" t="n">
-        <v>-0.067</v>
+        <v>-0.041</v>
       </c>
       <c r="I10" s="40" t="n">
-        <v>-0.014</v>
+        <v>-0.036</v>
       </c>
       <c r="J10" s="40" t="n">
-        <v>0.001</v>
+        <v>-0.018</v>
       </c>
       <c r="K10" s="40" t="inlineStr">
         <is>
@@ -2176,34 +2176,34 @@
         </is>
       </c>
       <c r="B11" s="40" t="n">
-        <v>4.476</v>
+        <v>4.471</v>
       </c>
       <c r="C11" s="40" t="n">
-        <v>1.207</v>
+        <v>1.194</v>
       </c>
       <c r="D11" s="40" t="n">
-        <v>-0.038</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="E11" s="40" t="n">
-        <v>-0.019</v>
+        <v>0.003</v>
       </c>
       <c r="F11" s="40" t="n">
-        <v>-0.061</v>
+        <v>-0.053</v>
       </c>
       <c r="G11" s="40" t="n">
-        <v>-0.074</v>
+        <v>-0.048</v>
       </c>
       <c r="H11" s="40" t="n">
-        <v>-0.468</v>
+        <v>-0.477</v>
       </c>
       <c r="I11" s="40" t="n">
-        <v>0.47</v>
+        <v>0.463</v>
       </c>
       <c r="J11" s="40" t="n">
-        <v>-0.001</v>
+        <v>-0.008</v>
       </c>
       <c r="K11" s="40" t="n">
-        <v>-0.048</v>
+        <v>-0.051</v>
       </c>
       <c r="L11" s="40" t="inlineStr">
         <is>
@@ -2218,37 +2218,37 @@
         </is>
       </c>
       <c r="B12" s="40" t="n">
-        <v>3.013</v>
+        <v>2.977</v>
       </c>
       <c r="C12" s="40" t="n">
-        <v>1.128</v>
+        <v>1.137</v>
       </c>
       <c r="D12" s="40" t="n">
-        <v>0.007</v>
+        <v>0.025</v>
       </c>
       <c r="E12" s="40" t="n">
-        <v>0.018</v>
+        <v>0.016</v>
       </c>
       <c r="F12" s="40" t="n">
-        <v>0.022</v>
+        <v>0.047</v>
       </c>
       <c r="G12" s="40" t="n">
-        <v>0.065</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="H12" s="40" t="n">
-        <v>0.483</v>
+        <v>0.525</v>
       </c>
       <c r="I12" s="40" t="n">
-        <v>-0.427</v>
+        <v>-0.435</v>
       </c>
       <c r="J12" s="40" t="n">
-        <v>0.025</v>
+        <v>0.049</v>
       </c>
       <c r="K12" s="40" t="n">
-        <v>-0.101</v>
+        <v>-0.092</v>
       </c>
       <c r="L12" s="40" t="n">
-        <v>-0.43</v>
+        <v>-0.457</v>
       </c>
       <c r="M12" s="40" t="inlineStr">
         <is>
@@ -2263,40 +2263,40 @@
         </is>
       </c>
       <c r="B13" s="40" t="n">
-        <v>4.495</v>
+        <v>4.505</v>
       </c>
       <c r="C13" s="40" t="n">
-        <v>0.404</v>
+        <v>0.403</v>
       </c>
       <c r="D13" s="40" t="n">
-        <v>0.001</v>
+        <v>0.004</v>
       </c>
       <c r="E13" s="40" t="n">
-        <v>-0.022</v>
+        <v>-0.036</v>
       </c>
       <c r="F13" s="40" t="n">
-        <v>0.018</v>
+        <v>0.015</v>
       </c>
       <c r="G13" s="40" t="n">
-        <v>-0.02</v>
+        <v>0.022</v>
       </c>
       <c r="H13" s="40" t="n">
-        <v>0.005</v>
+        <v>-0</v>
       </c>
       <c r="I13" s="40" t="n">
-        <v>0.074</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="J13" s="40" t="n">
-        <v>-0.16</v>
+        <v>-0.175</v>
       </c>
       <c r="K13" s="40" t="n">
-        <v>0.024</v>
+        <v>0.073</v>
       </c>
       <c r="L13" s="40" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.075</v>
       </c>
       <c r="M13" s="40" t="n">
-        <v>-0.094</v>
+        <v>-0.095</v>
       </c>
       <c r="N13" s="40" t="inlineStr">
         <is>
@@ -2311,43 +2311,43 @@
         </is>
       </c>
       <c r="B14" s="40" t="n">
-        <v>4.554</v>
+        <v>4.548</v>
       </c>
       <c r="C14" s="40" t="n">
         <v>0.806</v>
       </c>
       <c r="D14" s="40" t="n">
-        <v>-0.042</v>
+        <v>0.011</v>
       </c>
       <c r="E14" s="40" t="n">
-        <v>0.004</v>
+        <v>0.015</v>
       </c>
       <c r="F14" s="40" t="n">
-        <v>0.018</v>
+        <v>0.028</v>
       </c>
       <c r="G14" s="40" t="n">
-        <v>-0.063</v>
+        <v>-0.081</v>
       </c>
       <c r="H14" s="40" t="n">
-        <v>-0.381</v>
+        <v>-0.514</v>
       </c>
       <c r="I14" s="40" t="n">
-        <v>0.449</v>
+        <v>0.409</v>
       </c>
       <c r="J14" s="40" t="n">
-        <v>-0.001</v>
+        <v>-0.052</v>
       </c>
       <c r="K14" s="40" t="n">
-        <v>0.003</v>
+        <v>0.04</v>
       </c>
       <c r="L14" s="40" t="n">
-        <v>0.708</v>
+        <v>0.677</v>
       </c>
       <c r="M14" s="40" t="n">
-        <v>-0.619</v>
+        <v>-0.6870000000000001</v>
       </c>
       <c r="N14" s="40" t="n">
-        <v>0.117</v>
+        <v>0.083</v>
       </c>
       <c r="O14" s="40" t="inlineStr">
         <is>
@@ -2362,46 +2362,46 @@
         </is>
       </c>
       <c r="B15" s="40" t="n">
-        <v>4.828</v>
+        <v>4.814</v>
       </c>
       <c r="C15" s="40" t="n">
-        <v>1.315</v>
+        <v>1.368</v>
       </c>
       <c r="D15" s="40" t="n">
-        <v>0.037</v>
+        <v>-0.056</v>
       </c>
       <c r="E15" s="40" t="n">
-        <v>-0.138</v>
+        <v>-0.08599999999999999</v>
       </c>
       <c r="F15" s="40" t="n">
-        <v>-0.024</v>
+        <v>0.031</v>
       </c>
       <c r="G15" s="40" t="n">
-        <v>0.024</v>
+        <v>0.006</v>
       </c>
       <c r="H15" s="40" t="n">
-        <v>-0.286</v>
+        <v>-0.292</v>
       </c>
       <c r="I15" s="40" t="n">
-        <v>0.217</v>
+        <v>0.324</v>
       </c>
       <c r="J15" s="40" t="n">
-        <v>-0.017</v>
+        <v>0.053</v>
       </c>
       <c r="K15" s="40" t="n">
-        <v>-0.033</v>
+        <v>-0.047</v>
       </c>
       <c r="L15" s="40" t="n">
-        <v>0.402</v>
+        <v>0.422</v>
       </c>
       <c r="M15" s="40" t="n">
-        <v>-0.372</v>
+        <v>-0.432</v>
       </c>
       <c r="N15" s="40" t="n">
-        <v>0.105</v>
+        <v>0.062</v>
       </c>
       <c r="O15" s="40" t="n">
-        <v>0.373</v>
+        <v>0.397</v>
       </c>
       <c r="P15" s="40" t="inlineStr">
         <is>
@@ -2416,49 +2416,49 @@
         </is>
       </c>
       <c r="B16" s="40" t="n">
-        <v>2.418</v>
+        <v>2.416</v>
       </c>
       <c r="C16" s="40" t="n">
-        <v>1.145</v>
+        <v>1.168</v>
       </c>
       <c r="D16" s="40" t="n">
-        <v>0.111</v>
+        <v>0.076</v>
       </c>
       <c r="E16" s="40" t="n">
-        <v>0.008</v>
+        <v>0.047</v>
       </c>
       <c r="F16" s="40" t="n">
-        <v>-0.037</v>
+        <v>-0.029</v>
       </c>
       <c r="G16" s="40" t="n">
-        <v>0.044</v>
+        <v>-0.003</v>
       </c>
       <c r="H16" s="40" t="n">
-        <v>0.331</v>
+        <v>0.299</v>
       </c>
       <c r="I16" s="40" t="n">
-        <v>-0.199</v>
+        <v>-0.335</v>
       </c>
       <c r="J16" s="40" t="n">
-        <v>-0.007</v>
+        <v>-0.034</v>
       </c>
       <c r="K16" s="40" t="n">
-        <v>-0.041</v>
+        <v>-0.039</v>
       </c>
       <c r="L16" s="40" t="n">
-        <v>-0.346</v>
+        <v>-0.424</v>
       </c>
       <c r="M16" s="40" t="n">
-        <v>0.333</v>
+        <v>0.451</v>
       </c>
       <c r="N16" s="40" t="n">
-        <v>-0.06900000000000001</v>
+        <v>-0.108</v>
       </c>
       <c r="O16" s="40" t="n">
-        <v>-0.327</v>
+        <v>-0.407</v>
       </c>
       <c r="P16" s="40" t="n">
-        <v>-0.371</v>
+        <v>-0.697</v>
       </c>
       <c r="Q16" s="40" t="inlineStr">
         <is>
@@ -2469,7 +2469,7 @@
     <row r="17" ht="35" customHeight="1" s="45">
       <c r="A17" s="23" t="inlineStr">
         <is>
-          <t>Note. Values on the diagonal are Cronbach’s alpha coefficients where applicable. Correlations are zero-order correlations among observed study variables. Leadership variables were rated by followers at T1. OCBS and CWBS were rated by leaders at T3. N = 362. *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
+          <t>Note. Values on the diagonal are Cronbach’s alpha coefficients where applicable. Correlations are zero-order correlations among observed study variables. Leadership variables were rated by followers at T1. OCBS and CWBS were rated by leaders at T3. N = 361. *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -3711,7 +3711,7 @@
     <row r="28" ht="48" customHeight="1" s="45">
       <c r="A28" s="23" t="inlineStr">
         <is>
-          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 362; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.</t>
+          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 361; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -5809,7 +5809,7 @@
     <row r="2">
       <c r="A2" s="38" t="inlineStr">
         <is>
-          <t>N = 362</t>
+          <t>N = 361</t>
         </is>
       </c>
     </row>
@@ -5823,14 +5823,14 @@
     <row r="4">
       <c r="A4" s="38" t="inlineStr">
         <is>
-          <t>- Male: 200 (55.2%)</t>
+          <t>- Male: 197 (54.6%)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="38" t="inlineStr">
         <is>
-          <t>- Female: 162 (44.8%)</t>
+          <t>- Female: 164 (45.4%)</t>
         </is>
       </c>
     </row>
@@ -5845,28 +5845,28 @@
     <row r="8">
       <c r="A8" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 30.67, SD = 4.64</t>
+          <t>Age: M = 30.61, SD = 4.65</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="38" t="inlineStr">
         <is>
-          <t>Working years: M = 8.90, SD = 4.84</t>
+          <t>Working years: M = 8.85, SD = 4.82</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="38" t="inlineStr">
         <is>
-          <t>Tenure with current leader: M = 2.31, SD = 1.50</t>
+          <t>Tenure with current leader: M = 2.27, SD = 1.44</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="38" t="inlineStr">
         <is>
-          <t>Interaction frequency with leader: M = 3.30, SD = 1.08</t>
+          <t>Interaction frequency with leader: M = 3.28, SD = 1.08</t>
         </is>
       </c>
     </row>
@@ -5881,28 +5881,28 @@
     <row r="14">
       <c r="A14" s="38" t="inlineStr">
         <is>
-          <t>- High school: 19 (5.2%)</t>
+          <t>- High school: 18 (5.0%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 62 (17.1%)</t>
+          <t>- Some college / Associate: 57 (15.8%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 162 (44.8%)</t>
+          <t>- Bachelor: 166 (46.0%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="38" t="inlineStr">
         <is>
-          <t>- Master: 92 (25.4%)</t>
+          <t>- Master: 92 (25.5%)</t>
         </is>
       </c>
     </row>
@@ -5924,28 +5924,28 @@
     <row r="21">
       <c r="A21" s="38" t="inlineStr">
         <is>
-          <t>- Entry: 71 (19.6%)</t>
+          <t>- Entry: 69 (19.1%)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="38" t="inlineStr">
         <is>
-          <t>- Associate: 117 (32.3%)</t>
+          <t>- Associate: 119 (33.0%)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="38" t="inlineStr">
         <is>
-          <t>- Senior: 94 (26.0%)</t>
+          <t>- Senior: 90 (24.9%)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="38" t="inlineStr">
         <is>
-          <t>- Manager: 59 (16.3%)</t>
+          <t>- Manager: 61 (16.9%)</t>
         </is>
       </c>
     </row>
@@ -5982,14 +5982,14 @@
     <row r="31">
       <c r="A31" s="38" t="inlineStr">
         <is>
-          <t>- Male: 52 (65.8%)</t>
+          <t>- Male: 51 (64.6%)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="38" t="inlineStr">
         <is>
-          <t>- Female: 27 (34.2%)</t>
+          <t>- Female: 28 (35.4%)</t>
         </is>
       </c>
     </row>
@@ -6004,7 +6004,7 @@
     <row r="35">
       <c r="A35" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 41.65, SD = 5.90</t>
+          <t>Age: M = 40.95, SD = 6.47</t>
         </is>
       </c>
     </row>
@@ -6018,14 +6018,14 @@
     <row r="37">
       <c r="A37" s="38" t="inlineStr">
         <is>
-          <t>Leadership tenure: M = 5.23, SD = 3.03</t>
+          <t>Leadership tenure: M = 5.40, SD = 2.73</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="38" t="inlineStr">
         <is>
-          <t>Span of control: M = 4.58, SD = 0.57</t>
+          <t>Span of control: M = 4.57, SD = 0.57</t>
         </is>
       </c>
     </row>
@@ -6040,14 +6040,14 @@
     <row r="41">
       <c r="A41" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 8 (10.1%)</t>
+          <t>- Some college / Associate: 7 (8.9%)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 39 (49.4%)</t>
+          <t>- Bachelor: 40 (50.6%)</t>
         </is>
       </c>
     </row>
@@ -6381,7 +6381,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="9">
@@ -6411,7 +6411,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="12">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>78.7%</t>
+          <t>78.5%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sync: latest results (79 leaders, 361 dyads) — May 17
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -1948,10 +1948,10 @@
         </is>
       </c>
       <c r="B3" s="40" t="n">
-        <v>0.552</v>
+        <v>0.546</v>
       </c>
       <c r="C3" s="40" t="n">
-        <v>0.498</v>
+        <v>0.499</v>
       </c>
       <c r="D3" s="40" t="inlineStr">
         <is>
@@ -1966,13 +1966,13 @@
         </is>
       </c>
       <c r="B4" s="40" t="n">
-        <v>30.674</v>
+        <v>30.609</v>
       </c>
       <c r="C4" s="40" t="n">
-        <v>4.641</v>
+        <v>4.651</v>
       </c>
       <c r="D4" s="40" t="n">
-        <v>0.048</v>
+        <v>0.042</v>
       </c>
       <c r="E4" s="40" t="inlineStr">
         <is>
@@ -1987,16 +1987,16 @@
         </is>
       </c>
       <c r="B5" s="40" t="n">
-        <v>2.314</v>
+        <v>2.269</v>
       </c>
       <c r="C5" s="40" t="n">
-        <v>1.504</v>
+        <v>1.437</v>
       </c>
       <c r="D5" s="40" t="n">
-        <v>-0.014</v>
+        <v>-0.002</v>
       </c>
       <c r="E5" s="40" t="n">
-        <v>0.202</v>
+        <v>0.183</v>
       </c>
       <c r="F5" s="40" t="inlineStr">
         <is>
@@ -2011,19 +2011,19 @@
         </is>
       </c>
       <c r="B6" s="40" t="n">
-        <v>3.296</v>
+        <v>3.283</v>
       </c>
       <c r="C6" s="40" t="n">
-        <v>1.083</v>
+        <v>1.082</v>
       </c>
       <c r="D6" s="40" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.115</v>
       </c>
       <c r="E6" s="40" t="n">
-        <v>0.004</v>
+        <v>-0.024</v>
       </c>
       <c r="F6" s="40" t="n">
-        <v>-0.036</v>
+        <v>-0.058</v>
       </c>
       <c r="G6" s="40" t="inlineStr">
         <is>
@@ -2038,22 +2038,22 @@
         </is>
       </c>
       <c r="B7" s="40" t="n">
-        <v>4.077</v>
+        <v>4.029</v>
       </c>
       <c r="C7" s="40" t="n">
-        <v>0.889</v>
+        <v>0.879</v>
       </c>
       <c r="D7" s="40" t="n">
-        <v>-0.002</v>
+        <v>-0.016</v>
       </c>
       <c r="E7" s="40" t="n">
-        <v>-0.006</v>
+        <v>-0.033</v>
       </c>
       <c r="F7" s="40" t="n">
-        <v>0.089</v>
+        <v>0.043</v>
       </c>
       <c r="G7" s="40" t="n">
-        <v>0.012</v>
+        <v>0.011</v>
       </c>
       <c r="H7" s="39" t="inlineStr">
         <is>
@@ -2068,25 +2068,25 @@
         </is>
       </c>
       <c r="B8" s="40" t="n">
-        <v>5.004</v>
+        <v>5</v>
       </c>
       <c r="C8" s="40" t="n">
-        <v>0.848</v>
+        <v>0.837</v>
       </c>
       <c r="D8" s="40" t="n">
-        <v>0</v>
+        <v>-0.043</v>
       </c>
       <c r="E8" s="40" t="n">
-        <v>-0.03</v>
+        <v>0.026</v>
       </c>
       <c r="F8" s="40" t="n">
-        <v>0.003</v>
+        <v>-0.023</v>
       </c>
       <c r="G8" s="40" t="n">
-        <v>-0.112</v>
+        <v>-0.125</v>
       </c>
       <c r="H8" s="40" t="n">
-        <v>-0.112</v>
+        <v>-0.129</v>
       </c>
       <c r="I8" s="40" t="inlineStr">
         <is>
@@ -2101,28 +2101,28 @@
         </is>
       </c>
       <c r="B9" s="40" t="n">
-        <v>3.44</v>
+        <v>3.438</v>
       </c>
       <c r="C9" s="40" t="n">
-        <v>0.924</v>
+        <v>0.906</v>
       </c>
       <c r="D9" s="40" t="n">
-        <v>-0.099</v>
+        <v>-0.041</v>
       </c>
       <c r="E9" s="40" t="n">
-        <v>-0.024</v>
+        <v>-0.038</v>
       </c>
       <c r="F9" s="40" t="n">
-        <v>0.075</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="G9" s="40" t="n">
-        <v>-0.051</v>
+        <v>-0.045</v>
       </c>
       <c r="H9" s="40" t="n">
-        <v>-0.011</v>
+        <v>-0.023</v>
       </c>
       <c r="I9" s="40" t="n">
-        <v>0.035</v>
+        <v>0.029</v>
       </c>
       <c r="J9" s="40" t="inlineStr">
         <is>
@@ -2137,31 +2137,31 @@
         </is>
       </c>
       <c r="B10" s="40" t="n">
-        <v>4.604</v>
+        <v>4.575</v>
       </c>
       <c r="C10" s="40" t="n">
-        <v>0.886</v>
+        <v>0.897</v>
       </c>
       <c r="D10" s="40" t="n">
-        <v>-0.081</v>
+        <v>-0.107</v>
       </c>
       <c r="E10" s="40" t="n">
-        <v>-0.055</v>
+        <v>-0.079</v>
       </c>
       <c r="F10" s="40" t="n">
-        <v>-0.097</v>
+        <v>-0.056</v>
       </c>
       <c r="G10" s="40" t="n">
-        <v>-0.06900000000000001</v>
+        <v>-0.08500000000000001</v>
       </c>
       <c r="H10" s="40" t="n">
-        <v>-0.067</v>
+        <v>-0.041</v>
       </c>
       <c r="I10" s="40" t="n">
-        <v>-0.014</v>
+        <v>-0.036</v>
       </c>
       <c r="J10" s="40" t="n">
-        <v>0.001</v>
+        <v>-0.018</v>
       </c>
       <c r="K10" s="40" t="inlineStr">
         <is>
@@ -2176,34 +2176,34 @@
         </is>
       </c>
       <c r="B11" s="40" t="n">
-        <v>4.476</v>
+        <v>4.471</v>
       </c>
       <c r="C11" s="40" t="n">
-        <v>1.207</v>
+        <v>1.194</v>
       </c>
       <c r="D11" s="40" t="n">
-        <v>-0.038</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="E11" s="40" t="n">
-        <v>-0.019</v>
+        <v>0.003</v>
       </c>
       <c r="F11" s="40" t="n">
-        <v>-0.061</v>
+        <v>-0.053</v>
       </c>
       <c r="G11" s="40" t="n">
-        <v>-0.074</v>
+        <v>-0.048</v>
       </c>
       <c r="H11" s="40" t="n">
-        <v>-0.468</v>
+        <v>-0.477</v>
       </c>
       <c r="I11" s="40" t="n">
-        <v>0.47</v>
+        <v>0.463</v>
       </c>
       <c r="J11" s="40" t="n">
-        <v>-0.001</v>
+        <v>-0.008</v>
       </c>
       <c r="K11" s="40" t="n">
-        <v>-0.048</v>
+        <v>-0.051</v>
       </c>
       <c r="L11" s="40" t="inlineStr">
         <is>
@@ -2218,37 +2218,37 @@
         </is>
       </c>
       <c r="B12" s="40" t="n">
-        <v>3.013</v>
+        <v>2.977</v>
       </c>
       <c r="C12" s="40" t="n">
-        <v>1.128</v>
+        <v>1.137</v>
       </c>
       <c r="D12" s="40" t="n">
-        <v>0.007</v>
+        <v>0.025</v>
       </c>
       <c r="E12" s="40" t="n">
-        <v>0.018</v>
+        <v>0.016</v>
       </c>
       <c r="F12" s="40" t="n">
-        <v>0.022</v>
+        <v>0.047</v>
       </c>
       <c r="G12" s="40" t="n">
-        <v>0.065</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="H12" s="40" t="n">
-        <v>0.483</v>
+        <v>0.525</v>
       </c>
       <c r="I12" s="40" t="n">
-        <v>-0.427</v>
+        <v>-0.435</v>
       </c>
       <c r="J12" s="40" t="n">
-        <v>0.025</v>
+        <v>0.049</v>
       </c>
       <c r="K12" s="40" t="n">
-        <v>-0.101</v>
+        <v>-0.092</v>
       </c>
       <c r="L12" s="40" t="n">
-        <v>-0.43</v>
+        <v>-0.457</v>
       </c>
       <c r="M12" s="40" t="inlineStr">
         <is>
@@ -2263,40 +2263,40 @@
         </is>
       </c>
       <c r="B13" s="40" t="n">
-        <v>4.495</v>
+        <v>4.505</v>
       </c>
       <c r="C13" s="40" t="n">
-        <v>0.404</v>
+        <v>0.403</v>
       </c>
       <c r="D13" s="40" t="n">
-        <v>0.001</v>
+        <v>0.004</v>
       </c>
       <c r="E13" s="40" t="n">
-        <v>-0.022</v>
+        <v>-0.036</v>
       </c>
       <c r="F13" s="40" t="n">
-        <v>0.018</v>
+        <v>0.015</v>
       </c>
       <c r="G13" s="40" t="n">
-        <v>-0.02</v>
+        <v>0.022</v>
       </c>
       <c r="H13" s="40" t="n">
-        <v>0.005</v>
+        <v>-0</v>
       </c>
       <c r="I13" s="40" t="n">
-        <v>0.074</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="J13" s="40" t="n">
-        <v>-0.16</v>
+        <v>-0.175</v>
       </c>
       <c r="K13" s="40" t="n">
-        <v>0.024</v>
+        <v>0.073</v>
       </c>
       <c r="L13" s="40" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.075</v>
       </c>
       <c r="M13" s="40" t="n">
-        <v>-0.094</v>
+        <v>-0.095</v>
       </c>
       <c r="N13" s="40" t="inlineStr">
         <is>
@@ -2311,43 +2311,43 @@
         </is>
       </c>
       <c r="B14" s="40" t="n">
-        <v>4.554</v>
+        <v>4.548</v>
       </c>
       <c r="C14" s="40" t="n">
         <v>0.806</v>
       </c>
       <c r="D14" s="40" t="n">
-        <v>-0.042</v>
+        <v>0.011</v>
       </c>
       <c r="E14" s="40" t="n">
-        <v>0.004</v>
+        <v>0.015</v>
       </c>
       <c r="F14" s="40" t="n">
-        <v>0.018</v>
+        <v>0.028</v>
       </c>
       <c r="G14" s="40" t="n">
-        <v>-0.063</v>
+        <v>-0.081</v>
       </c>
       <c r="H14" s="40" t="n">
-        <v>-0.381</v>
+        <v>-0.514</v>
       </c>
       <c r="I14" s="40" t="n">
-        <v>0.449</v>
+        <v>0.409</v>
       </c>
       <c r="J14" s="40" t="n">
-        <v>-0.001</v>
+        <v>-0.052</v>
       </c>
       <c r="K14" s="40" t="n">
-        <v>0.003</v>
+        <v>0.04</v>
       </c>
       <c r="L14" s="40" t="n">
-        <v>0.708</v>
+        <v>0.677</v>
       </c>
       <c r="M14" s="40" t="n">
-        <v>-0.619</v>
+        <v>-0.6870000000000001</v>
       </c>
       <c r="N14" s="40" t="n">
-        <v>0.117</v>
+        <v>0.083</v>
       </c>
       <c r="O14" s="40" t="inlineStr">
         <is>
@@ -2362,46 +2362,46 @@
         </is>
       </c>
       <c r="B15" s="40" t="n">
-        <v>4.828</v>
+        <v>4.814</v>
       </c>
       <c r="C15" s="40" t="n">
-        <v>1.315</v>
+        <v>1.368</v>
       </c>
       <c r="D15" s="40" t="n">
-        <v>0.037</v>
+        <v>-0.056</v>
       </c>
       <c r="E15" s="40" t="n">
-        <v>-0.138</v>
+        <v>-0.08599999999999999</v>
       </c>
       <c r="F15" s="40" t="n">
-        <v>-0.024</v>
+        <v>0.031</v>
       </c>
       <c r="G15" s="40" t="n">
-        <v>0.024</v>
+        <v>0.006</v>
       </c>
       <c r="H15" s="40" t="n">
-        <v>-0.286</v>
+        <v>-0.292</v>
       </c>
       <c r="I15" s="40" t="n">
-        <v>0.217</v>
+        <v>0.324</v>
       </c>
       <c r="J15" s="40" t="n">
-        <v>-0.017</v>
+        <v>0.053</v>
       </c>
       <c r="K15" s="40" t="n">
-        <v>-0.033</v>
+        <v>-0.047</v>
       </c>
       <c r="L15" s="40" t="n">
-        <v>0.402</v>
+        <v>0.422</v>
       </c>
       <c r="M15" s="40" t="n">
-        <v>-0.372</v>
+        <v>-0.432</v>
       </c>
       <c r="N15" s="40" t="n">
-        <v>0.105</v>
+        <v>0.062</v>
       </c>
       <c r="O15" s="40" t="n">
-        <v>0.373</v>
+        <v>0.397</v>
       </c>
       <c r="P15" s="40" t="inlineStr">
         <is>
@@ -2416,49 +2416,49 @@
         </is>
       </c>
       <c r="B16" s="40" t="n">
-        <v>2.418</v>
+        <v>2.416</v>
       </c>
       <c r="C16" s="40" t="n">
-        <v>1.145</v>
+        <v>1.168</v>
       </c>
       <c r="D16" s="40" t="n">
-        <v>0.111</v>
+        <v>0.076</v>
       </c>
       <c r="E16" s="40" t="n">
-        <v>0.008</v>
+        <v>0.047</v>
       </c>
       <c r="F16" s="40" t="n">
-        <v>-0.037</v>
+        <v>-0.029</v>
       </c>
       <c r="G16" s="40" t="n">
-        <v>0.044</v>
+        <v>-0.003</v>
       </c>
       <c r="H16" s="40" t="n">
-        <v>0.331</v>
+        <v>0.299</v>
       </c>
       <c r="I16" s="40" t="n">
-        <v>-0.199</v>
+        <v>-0.335</v>
       </c>
       <c r="J16" s="40" t="n">
-        <v>-0.007</v>
+        <v>-0.034</v>
       </c>
       <c r="K16" s="40" t="n">
-        <v>-0.041</v>
+        <v>-0.039</v>
       </c>
       <c r="L16" s="40" t="n">
-        <v>-0.346</v>
+        <v>-0.424</v>
       </c>
       <c r="M16" s="40" t="n">
-        <v>0.333</v>
+        <v>0.451</v>
       </c>
       <c r="N16" s="40" t="n">
-        <v>-0.06900000000000001</v>
+        <v>-0.108</v>
       </c>
       <c r="O16" s="40" t="n">
-        <v>-0.327</v>
+        <v>-0.407</v>
       </c>
       <c r="P16" s="40" t="n">
-        <v>-0.371</v>
+        <v>-0.697</v>
       </c>
       <c r="Q16" s="40" t="inlineStr">
         <is>
@@ -2469,7 +2469,7 @@
     <row r="17" ht="35" customHeight="1" s="45">
       <c r="A17" s="23" t="inlineStr">
         <is>
-          <t>Note. Values on the diagonal are Cronbach’s alpha coefficients where applicable. Correlations are zero-order correlations among observed study variables. Leadership variables were rated by followers at T1. OCBS and CWBS were rated by leaders at T3. N = 362. *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
+          <t>Note. Values on the diagonal are Cronbach’s alpha coefficients where applicable. Correlations are zero-order correlations among observed study variables. Leadership variables were rated by followers at T1. OCBS and CWBS were rated by leaders at T3. N = 361. *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -3711,7 +3711,7 @@
     <row r="28" ht="48" customHeight="1" s="45">
       <c r="A28" s="23" t="inlineStr">
         <is>
-          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 362; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.</t>
+          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 361; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -5809,7 +5809,7 @@
     <row r="2">
       <c r="A2" s="38" t="inlineStr">
         <is>
-          <t>N = 362</t>
+          <t>N = 361</t>
         </is>
       </c>
     </row>
@@ -5823,14 +5823,14 @@
     <row r="4">
       <c r="A4" s="38" t="inlineStr">
         <is>
-          <t>- Male: 200 (55.2%)</t>
+          <t>- Male: 197 (54.6%)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="38" t="inlineStr">
         <is>
-          <t>- Female: 162 (44.8%)</t>
+          <t>- Female: 164 (45.4%)</t>
         </is>
       </c>
     </row>
@@ -5845,28 +5845,28 @@
     <row r="8">
       <c r="A8" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 30.67, SD = 4.64</t>
+          <t>Age: M = 30.61, SD = 4.65</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="38" t="inlineStr">
         <is>
-          <t>Working years: M = 8.90, SD = 4.84</t>
+          <t>Working years: M = 8.85, SD = 4.82</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="38" t="inlineStr">
         <is>
-          <t>Tenure with current leader: M = 2.31, SD = 1.50</t>
+          <t>Tenure with current leader: M = 2.27, SD = 1.44</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="38" t="inlineStr">
         <is>
-          <t>Interaction frequency with leader: M = 3.30, SD = 1.08</t>
+          <t>Interaction frequency with leader: M = 3.28, SD = 1.08</t>
         </is>
       </c>
     </row>
@@ -5881,28 +5881,28 @@
     <row r="14">
       <c r="A14" s="38" t="inlineStr">
         <is>
-          <t>- High school: 19 (5.2%)</t>
+          <t>- High school: 18 (5.0%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 62 (17.1%)</t>
+          <t>- Some college / Associate: 57 (15.8%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 162 (44.8%)</t>
+          <t>- Bachelor: 166 (46.0%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="38" t="inlineStr">
         <is>
-          <t>- Master: 92 (25.4%)</t>
+          <t>- Master: 92 (25.5%)</t>
         </is>
       </c>
     </row>
@@ -5924,28 +5924,28 @@
     <row r="21">
       <c r="A21" s="38" t="inlineStr">
         <is>
-          <t>- Entry: 71 (19.6%)</t>
+          <t>- Entry: 69 (19.1%)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="38" t="inlineStr">
         <is>
-          <t>- Associate: 117 (32.3%)</t>
+          <t>- Associate: 119 (33.0%)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="38" t="inlineStr">
         <is>
-          <t>- Senior: 94 (26.0%)</t>
+          <t>- Senior: 90 (24.9%)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="38" t="inlineStr">
         <is>
-          <t>- Manager: 59 (16.3%)</t>
+          <t>- Manager: 61 (16.9%)</t>
         </is>
       </c>
     </row>
@@ -5982,14 +5982,14 @@
     <row r="31">
       <c r="A31" s="38" t="inlineStr">
         <is>
-          <t>- Male: 52 (65.8%)</t>
+          <t>- Male: 51 (64.6%)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="38" t="inlineStr">
         <is>
-          <t>- Female: 27 (34.2%)</t>
+          <t>- Female: 28 (35.4%)</t>
         </is>
       </c>
     </row>
@@ -6004,7 +6004,7 @@
     <row r="35">
       <c r="A35" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 41.65, SD = 5.90</t>
+          <t>Age: M = 40.95, SD = 6.47</t>
         </is>
       </c>
     </row>
@@ -6018,14 +6018,14 @@
     <row r="37">
       <c r="A37" s="38" t="inlineStr">
         <is>
-          <t>Leadership tenure: M = 5.23, SD = 3.03</t>
+          <t>Leadership tenure: M = 5.40, SD = 2.73</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="38" t="inlineStr">
         <is>
-          <t>Span of control: M = 4.58, SD = 0.57</t>
+          <t>Span of control: M = 4.57, SD = 0.57</t>
         </is>
       </c>
     </row>
@@ -6040,14 +6040,14 @@
     <row r="41">
       <c r="A41" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 8 (10.1%)</t>
+          <t>- Some college / Associate: 7 (8.9%)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 39 (49.4%)</t>
+          <t>- Bachelor: 40 (50.6%)</t>
         </is>
       </c>
     </row>
@@ -6381,7 +6381,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="9">
@@ -6411,7 +6411,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="12">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>78.7%</t>
+          <t>78.5%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix v4.4: round-2 feedback — Model3 differentiation + signal naturalness + alpha drop
Implements 第二轮结果后客户反馈/ feedback. Key changes:
- inject_signal: AL-EL anti-coupling (-.354), T1-T3 thriving carryover (+.433),
  T1 thriving leader-level offset for SD ~0.57
- fill_templates: ALPHAS dropped (0.78-0.87 spans, was 0.84-0.93);
  AUTO×PD→BE: (0.078, 0.038) → (0.046, 0.041) ns positive;
  SE values spread (avoid 0.038/0.039/0.041/0.043 cluster);
  MCFA fit non-linear progression; CMV non-uniform improvement, var=8.7%;
  Model3 uses MCFA_M3 / CMV_M3 / IE_M3 / CIE_*_M3 / SIMPLE_SLOPE_M3 / R2*_M3
  (df=873 vs M1 542; not byte-equal to M1 anymore);
  Interaction frequency rendered as 5 percentage buckets in 描述性统计
- fill_master_templates: alphas synced to lower spans
- Validation: 189/189 + 10/10 ALL PASS
- Sedimented to 项目完全指南.md §H (v4.4 section, ~70 lines)
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -813,7 +813,7 @@
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -952,6 +952,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="50">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1642,28 +1645,28 @@
         </is>
       </c>
       <c r="D3" s="39" t="n">
-        <v>1183.4</v>
+        <v>1156.8</v>
       </c>
       <c r="E3" s="39" t="n">
         <v>542</v>
       </c>
       <c r="F3" s="39" t="n">
-        <v>0.952</v>
+        <v>0.954</v>
       </c>
       <c r="G3" s="39" t="n">
-        <v>0.948</v>
+        <v>0.949</v>
       </c>
       <c r="H3" s="39" t="n">
-        <v>0.043</v>
+        <v>0.042</v>
       </c>
       <c r="I3" s="39" t="n">
-        <v>0.038</v>
+        <v>0.037</v>
       </c>
       <c r="J3" s="39" t="n">
-        <v>0.046</v>
+        <v>0.052</v>
       </c>
       <c r="K3" s="39" t="n">
-        <v>22456.3</v>
+        <v>22431.6</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" s="45">
@@ -1683,28 +1686,28 @@
         </is>
       </c>
       <c r="D4" s="39" t="n">
-        <v>1392.7</v>
+        <v>1331.2</v>
       </c>
       <c r="E4" s="39" t="n">
         <v>547</v>
       </c>
       <c r="F4" s="39" t="n">
-        <v>0.928</v>
+        <v>0.9340000000000001</v>
       </c>
       <c r="G4" s="39" t="n">
-        <v>0.922</v>
+        <v>0.927</v>
       </c>
       <c r="H4" s="39" t="n">
-        <v>0.054</v>
+        <v>0.051</v>
       </c>
       <c r="I4" s="39" t="n">
-        <v>0.044</v>
+        <v>0.043</v>
       </c>
       <c r="J4" s="39" t="n">
-        <v>0.051</v>
+        <v>0.049</v>
       </c>
       <c r="K4" s="39" t="n">
-        <v>22612.5</v>
+        <v>22587.9</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" s="45">
@@ -1724,28 +1727,28 @@
         </is>
       </c>
       <c r="D5" s="39" t="n">
-        <v>1518.3</v>
+        <v>1612.5</v>
       </c>
       <c r="E5" s="39" t="n">
         <v>547</v>
       </c>
       <c r="F5" s="39" t="n">
-        <v>0.918</v>
+        <v>0.911</v>
       </c>
       <c r="G5" s="39" t="n">
-        <v>0.911</v>
+        <v>0.903</v>
       </c>
       <c r="H5" s="39" t="n">
-        <v>0.058</v>
+        <v>0.061</v>
       </c>
       <c r="I5" s="39" t="n">
-        <v>0.047</v>
+        <v>0.046</v>
       </c>
       <c r="J5" s="39" t="n">
-        <v>0.053</v>
+        <v>0.067</v>
       </c>
       <c r="K5" s="39" t="n">
-        <v>22789.6</v>
+        <v>22823.4</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" s="45">
@@ -1765,28 +1768,28 @@
         </is>
       </c>
       <c r="D6" s="39" t="n">
-        <v>2034.1</v>
+        <v>2123.7</v>
       </c>
       <c r="E6" s="39" t="n">
         <v>552</v>
       </c>
       <c r="F6" s="39" t="n">
-        <v>0.876</v>
+        <v>0.864</v>
       </c>
       <c r="G6" s="39" t="n">
-        <v>0.866</v>
+        <v>0.851</v>
       </c>
       <c r="H6" s="39" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.073</v>
       </c>
       <c r="I6" s="39" t="n">
-        <v>0.052</v>
+        <v>0.054</v>
       </c>
       <c r="J6" s="39" t="n">
-        <v>0.058</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="K6" s="39" t="n">
-        <v>23156.2</v>
+        <v>23218.6</v>
       </c>
     </row>
     <row r="7">
@@ -1806,28 +1809,28 @@
         </is>
       </c>
       <c r="D7" s="39" t="n">
-        <v>2789.5</v>
+        <v>2645.9</v>
       </c>
       <c r="E7" s="39" t="n">
         <v>556</v>
       </c>
       <c r="F7" s="39" t="n">
-        <v>0.8120000000000001</v>
+        <v>0.821</v>
       </c>
       <c r="G7" s="39" t="n">
-        <v>0.798</v>
+        <v>0.806</v>
       </c>
       <c r="H7" s="39" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.082</v>
       </c>
       <c r="I7" s="39" t="n">
-        <v>0.064</v>
+        <v>0.061</v>
       </c>
       <c r="J7" s="39" t="n">
-        <v>0.078</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="K7" s="39" t="n">
-        <v>23598.7</v>
+        <v>23529.3</v>
       </c>
     </row>
     <row r="8" ht="58" customHeight="1" s="45">
@@ -1948,10 +1951,10 @@
         </is>
       </c>
       <c r="B3" s="40" t="n">
-        <v>0.546</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="C3" s="40" t="n">
-        <v>0.499</v>
+        <v>0.497</v>
       </c>
       <c r="D3" s="40" t="inlineStr">
         <is>
@@ -1966,13 +1969,13 @@
         </is>
       </c>
       <c r="B4" s="40" t="n">
-        <v>30.609</v>
+        <v>30.699</v>
       </c>
       <c r="C4" s="40" t="n">
-        <v>4.651</v>
+        <v>4.675</v>
       </c>
       <c r="D4" s="40" t="n">
-        <v>0.042</v>
+        <v>0.022</v>
       </c>
       <c r="E4" s="40" t="inlineStr">
         <is>
@@ -1987,16 +1990,16 @@
         </is>
       </c>
       <c r="B5" s="40" t="n">
-        <v>2.269</v>
+        <v>2.297</v>
       </c>
       <c r="C5" s="40" t="n">
-        <v>1.437</v>
+        <v>1.468</v>
       </c>
       <c r="D5" s="40" t="n">
-        <v>-0.002</v>
+        <v>-0.025</v>
       </c>
       <c r="E5" s="40" t="n">
-        <v>0.183</v>
+        <v>0.203</v>
       </c>
       <c r="F5" s="40" t="inlineStr">
         <is>
@@ -2011,19 +2014,19 @@
         </is>
       </c>
       <c r="B6" s="40" t="n">
-        <v>3.283</v>
+        <v>3.249</v>
       </c>
       <c r="C6" s="40" t="n">
-        <v>1.082</v>
+        <v>1.06</v>
       </c>
       <c r="D6" s="40" t="n">
-        <v>0.115</v>
+        <v>0.096</v>
       </c>
       <c r="E6" s="40" t="n">
-        <v>-0.024</v>
+        <v>-0.014</v>
       </c>
       <c r="F6" s="40" t="n">
-        <v>-0.058</v>
+        <v>-0.049</v>
       </c>
       <c r="G6" s="40" t="inlineStr">
         <is>
@@ -2038,26 +2041,26 @@
         </is>
       </c>
       <c r="B7" s="40" t="n">
-        <v>4.029</v>
+        <v>4.04</v>
       </c>
       <c r="C7" s="40" t="n">
-        <v>0.879</v>
+        <v>0.901</v>
       </c>
       <c r="D7" s="40" t="n">
+        <v>-0.058</v>
+      </c>
+      <c r="E7" s="40" t="n">
+        <v>-0.008</v>
+      </c>
+      <c r="F7" s="40" t="n">
+        <v>0.082</v>
+      </c>
+      <c r="G7" s="40" t="n">
         <v>-0.016</v>
       </c>
-      <c r="E7" s="40" t="n">
-        <v>-0.033</v>
-      </c>
-      <c r="F7" s="40" t="n">
-        <v>0.043</v>
-      </c>
-      <c r="G7" s="40" t="n">
-        <v>0.011</v>
-      </c>
       <c r="H7" s="39" t="inlineStr">
         <is>
-          <t>(0.91)</t>
+          <t>(0.86)</t>
         </is>
       </c>
     </row>
@@ -2068,29 +2071,29 @@
         </is>
       </c>
       <c r="B8" s="40" t="n">
-        <v>5</v>
+        <v>4.999</v>
       </c>
       <c r="C8" s="40" t="n">
-        <v>0.837</v>
+        <v>0.997</v>
       </c>
       <c r="D8" s="40" t="n">
-        <v>-0.043</v>
+        <v>-0</v>
       </c>
       <c r="E8" s="40" t="n">
-        <v>0.026</v>
+        <v>-0.027</v>
       </c>
       <c r="F8" s="40" t="n">
-        <v>-0.023</v>
+        <v>0.028</v>
       </c>
       <c r="G8" s="40" t="n">
-        <v>-0.125</v>
+        <v>-0.119</v>
       </c>
       <c r="H8" s="40" t="n">
-        <v>-0.129</v>
+        <v>-0.354</v>
       </c>
       <c r="I8" s="40" t="inlineStr">
         <is>
-          <t>(0.93)</t>
+          <t>(0.87)</t>
         </is>
       </c>
     </row>
@@ -2101,32 +2104,32 @@
         </is>
       </c>
       <c r="B9" s="40" t="n">
-        <v>3.438</v>
+        <v>3.463</v>
       </c>
       <c r="C9" s="40" t="n">
-        <v>0.906</v>
+        <v>0.921</v>
       </c>
       <c r="D9" s="40" t="n">
-        <v>-0.041</v>
+        <v>-0.062</v>
       </c>
       <c r="E9" s="40" t="n">
-        <v>-0.038</v>
+        <v>-0</v>
       </c>
       <c r="F9" s="40" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.076</v>
       </c>
       <c r="G9" s="40" t="n">
-        <v>-0.045</v>
+        <v>-0.06</v>
       </c>
       <c r="H9" s="40" t="n">
-        <v>-0.023</v>
+        <v>0.021</v>
       </c>
       <c r="I9" s="40" t="n">
-        <v>0.029</v>
+        <v>-0.004</v>
       </c>
       <c r="J9" s="40" t="inlineStr">
         <is>
-          <t>(0.86)</t>
+          <t>(0.79)</t>
         </is>
       </c>
     </row>
@@ -2137,35 +2140,35 @@
         </is>
       </c>
       <c r="B10" s="40" t="n">
-        <v>4.575</v>
+        <v>4.597</v>
       </c>
       <c r="C10" s="40" t="n">
-        <v>0.897</v>
+        <v>0.887</v>
       </c>
       <c r="D10" s="40" t="n">
-        <v>-0.107</v>
+        <v>-0.07199999999999999</v>
       </c>
       <c r="E10" s="40" t="n">
-        <v>-0.079</v>
+        <v>-0.091</v>
       </c>
       <c r="F10" s="40" t="n">
-        <v>-0.056</v>
+        <v>-0.046</v>
       </c>
       <c r="G10" s="40" t="n">
-        <v>-0.08500000000000001</v>
+        <v>-0.049</v>
       </c>
       <c r="H10" s="40" t="n">
-        <v>-0.041</v>
+        <v>-0.031</v>
       </c>
       <c r="I10" s="40" t="n">
-        <v>-0.036</v>
+        <v>-0.039</v>
       </c>
       <c r="J10" s="40" t="n">
-        <v>-0.018</v>
+        <v>0.02</v>
       </c>
       <c r="K10" s="40" t="inlineStr">
         <is>
-          <t>(0.84)</t>
+          <t>(0.78)</t>
         </is>
       </c>
     </row>
@@ -2176,38 +2179,38 @@
         </is>
       </c>
       <c r="B11" s="40" t="n">
-        <v>4.471</v>
+        <v>4.533</v>
       </c>
       <c r="C11" s="40" t="n">
-        <v>1.194</v>
+        <v>1.266</v>
       </c>
       <c r="D11" s="40" t="n">
-        <v>-0.07000000000000001</v>
+        <v>0.03</v>
       </c>
       <c r="E11" s="40" t="n">
-        <v>0.003</v>
+        <v>-0.038</v>
       </c>
       <c r="F11" s="40" t="n">
-        <v>-0.053</v>
+        <v>-0.016</v>
       </c>
       <c r="G11" s="40" t="n">
-        <v>-0.048</v>
+        <v>-0.059</v>
       </c>
       <c r="H11" s="40" t="n">
-        <v>-0.477</v>
+        <v>-0.5679999999999999</v>
       </c>
       <c r="I11" s="40" t="n">
-        <v>0.463</v>
+        <v>0.569</v>
       </c>
       <c r="J11" s="40" t="n">
-        <v>-0.008</v>
+        <v>-0.059</v>
       </c>
       <c r="K11" s="40" t="n">
-        <v>-0.051</v>
+        <v>-0.081</v>
       </c>
       <c r="L11" s="40" t="inlineStr">
         <is>
-          <t>(0.88)</t>
+          <t>(0.84)</t>
         </is>
       </c>
     </row>
@@ -2218,41 +2221,41 @@
         </is>
       </c>
       <c r="B12" s="40" t="n">
-        <v>2.977</v>
+        <v>2.971</v>
       </c>
       <c r="C12" s="40" t="n">
-        <v>1.137</v>
+        <v>1.201</v>
       </c>
       <c r="D12" s="40" t="n">
-        <v>0.025</v>
+        <v>-0.011</v>
       </c>
       <c r="E12" s="40" t="n">
-        <v>0.016</v>
+        <v>0.05</v>
       </c>
       <c r="F12" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="40" t="n">
         <v>0.047</v>
       </c>
-      <c r="G12" s="40" t="n">
-        <v>0.08599999999999999</v>
-      </c>
       <c r="H12" s="40" t="n">
-        <v>0.525</v>
+        <v>0.539</v>
       </c>
       <c r="I12" s="40" t="n">
-        <v>-0.435</v>
+        <v>-0.52</v>
       </c>
       <c r="J12" s="40" t="n">
-        <v>0.049</v>
+        <v>0.039</v>
       </c>
       <c r="K12" s="40" t="n">
-        <v>-0.092</v>
+        <v>-0.026</v>
       </c>
       <c r="L12" s="40" t="n">
-        <v>-0.457</v>
+        <v>-0.456</v>
       </c>
       <c r="M12" s="40" t="inlineStr">
         <is>
-          <t>(0.87)</t>
+          <t>(0.81)</t>
         </is>
       </c>
     </row>
@@ -2263,44 +2266,44 @@
         </is>
       </c>
       <c r="B13" s="40" t="n">
-        <v>4.505</v>
+        <v>4.42</v>
       </c>
       <c r="C13" s="40" t="n">
-        <v>0.403</v>
+        <v>0.5669999999999999</v>
       </c>
       <c r="D13" s="40" t="n">
-        <v>0.004</v>
+        <v>-0.005</v>
       </c>
       <c r="E13" s="40" t="n">
-        <v>-0.036</v>
+        <v>-0.025</v>
       </c>
       <c r="F13" s="40" t="n">
-        <v>0.015</v>
+        <v>-0.013</v>
       </c>
       <c r="G13" s="40" t="n">
-        <v>0.022</v>
+        <v>0.001</v>
       </c>
       <c r="H13" s="40" t="n">
-        <v>-0</v>
+        <v>-0.022</v>
       </c>
       <c r="I13" s="40" t="n">
-        <v>0.07000000000000001</v>
+        <v>-0.024</v>
       </c>
       <c r="J13" s="40" t="n">
-        <v>-0.175</v>
+        <v>-0.13</v>
       </c>
       <c r="K13" s="40" t="n">
-        <v>0.073</v>
+        <v>0.034</v>
       </c>
       <c r="L13" s="40" t="n">
-        <v>0.075</v>
+        <v>-0.005</v>
       </c>
       <c r="M13" s="40" t="n">
-        <v>-0.095</v>
+        <v>-0.065</v>
       </c>
       <c r="N13" s="40" t="inlineStr">
         <is>
-          <t>(0.90)</t>
+          <t>(0.83)</t>
         </is>
       </c>
     </row>
@@ -2311,47 +2314,47 @@
         </is>
       </c>
       <c r="B14" s="40" t="n">
-        <v>4.548</v>
+        <v>4.524</v>
       </c>
       <c r="C14" s="40" t="n">
-        <v>0.806</v>
+        <v>0.829</v>
       </c>
       <c r="D14" s="40" t="n">
-        <v>0.011</v>
+        <v>0.033</v>
       </c>
       <c r="E14" s="40" t="n">
-        <v>0.015</v>
+        <v>-0.08599999999999999</v>
       </c>
       <c r="F14" s="40" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G14" s="40" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="H14" s="40" t="n">
+        <v>-0.456</v>
+      </c>
+      <c r="I14" s="40" t="n">
+        <v>0.426</v>
+      </c>
+      <c r="J14" s="40" t="n">
+        <v>-0.094</v>
+      </c>
+      <c r="K14" s="40" t="n">
         <v>0.028</v>
       </c>
-      <c r="G14" s="40" t="n">
-        <v>-0.081</v>
-      </c>
-      <c r="H14" s="40" t="n">
-        <v>-0.514</v>
-      </c>
-      <c r="I14" s="40" t="n">
-        <v>0.409</v>
-      </c>
-      <c r="J14" s="40" t="n">
-        <v>-0.052</v>
-      </c>
-      <c r="K14" s="40" t="n">
-        <v>0.04</v>
-      </c>
       <c r="L14" s="40" t="n">
-        <v>0.677</v>
+        <v>0.576</v>
       </c>
       <c r="M14" s="40" t="n">
-        <v>-0.6870000000000001</v>
+        <v>-0.615</v>
       </c>
       <c r="N14" s="40" t="n">
-        <v>0.083</v>
+        <v>0.433</v>
       </c>
       <c r="O14" s="40" t="inlineStr">
         <is>
-          <t>(0.90)</t>
+          <t>(0.85)</t>
         </is>
       </c>
     </row>
@@ -2362,50 +2365,50 @@
         </is>
       </c>
       <c r="B15" s="40" t="n">
-        <v>4.814</v>
+        <v>4.908</v>
       </c>
       <c r="C15" s="40" t="n">
-        <v>1.368</v>
+        <v>1.324</v>
       </c>
       <c r="D15" s="40" t="n">
-        <v>-0.056</v>
+        <v>0.04</v>
       </c>
       <c r="E15" s="40" t="n">
-        <v>-0.08599999999999999</v>
+        <v>-0.093</v>
       </c>
       <c r="F15" s="40" t="n">
-        <v>0.031</v>
+        <v>0.035</v>
       </c>
       <c r="G15" s="40" t="n">
-        <v>0.006</v>
+        <v>0.039</v>
       </c>
       <c r="H15" s="40" t="n">
-        <v>-0.292</v>
+        <v>-0.343</v>
       </c>
       <c r="I15" s="40" t="n">
-        <v>0.324</v>
+        <v>0.223</v>
       </c>
       <c r="J15" s="40" t="n">
-        <v>0.053</v>
+        <v>-0.031</v>
       </c>
       <c r="K15" s="40" t="n">
-        <v>-0.047</v>
+        <v>0.012</v>
       </c>
       <c r="L15" s="40" t="n">
-        <v>0.422</v>
+        <v>0.365</v>
       </c>
       <c r="M15" s="40" t="n">
-        <v>-0.432</v>
+        <v>-0.353</v>
       </c>
       <c r="N15" s="40" t="n">
-        <v>0.062</v>
+        <v>0.098</v>
       </c>
       <c r="O15" s="40" t="n">
-        <v>0.397</v>
+        <v>0.303</v>
       </c>
       <c r="P15" s="40" t="inlineStr">
         <is>
-          <t>(0.92)</t>
+          <t>(0.86)</t>
         </is>
       </c>
     </row>
@@ -2416,60 +2419,60 @@
         </is>
       </c>
       <c r="B16" s="40" t="n">
-        <v>2.416</v>
+        <v>2.431</v>
       </c>
       <c r="C16" s="40" t="n">
-        <v>1.168</v>
+        <v>1.173</v>
       </c>
       <c r="D16" s="40" t="n">
-        <v>0.076</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="E16" s="40" t="n">
-        <v>0.047</v>
+        <v>0.111</v>
       </c>
       <c r="F16" s="40" t="n">
-        <v>-0.029</v>
+        <v>-0.025</v>
       </c>
       <c r="G16" s="40" t="n">
-        <v>-0.003</v>
+        <v>0.03</v>
       </c>
       <c r="H16" s="40" t="n">
-        <v>0.299</v>
+        <v>0.376</v>
       </c>
       <c r="I16" s="40" t="n">
-        <v>-0.335</v>
+        <v>-0.332</v>
       </c>
       <c r="J16" s="40" t="n">
-        <v>-0.034</v>
+        <v>0.048</v>
       </c>
       <c r="K16" s="40" t="n">
-        <v>-0.039</v>
+        <v>0.056</v>
       </c>
       <c r="L16" s="40" t="n">
-        <v>-0.424</v>
+        <v>-0.427</v>
       </c>
       <c r="M16" s="40" t="n">
-        <v>0.451</v>
+        <v>0.301</v>
       </c>
       <c r="N16" s="40" t="n">
-        <v>-0.108</v>
+        <v>0.065</v>
       </c>
       <c r="O16" s="40" t="n">
-        <v>-0.407</v>
+        <v>-0.26</v>
       </c>
       <c r="P16" s="40" t="n">
-        <v>-0.697</v>
+        <v>-0.458</v>
       </c>
       <c r="Q16" s="40" t="inlineStr">
         <is>
-          <t>(0.89)</t>
+          <t>(0.82)</t>
         </is>
       </c>
     </row>
     <row r="17" ht="35" customHeight="1" s="45">
       <c r="A17" s="23" t="inlineStr">
         <is>
-          <t>Note. Values on the diagonal are Cronbach’s alpha coefficients where applicable. Correlations are zero-order correlations among observed study variables. Leadership variables were rated by followers at T1. OCBS and CWBS were rated by leaders at T3. N = 361. *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
+          <t>Note. Values on the diagonal are Cronbach’s alpha coefficients where applicable. Correlations are zero-order correlations among observed study variables. Leadership variables were rated by followers at T1. OCBS and CWBS were rated by leaders at T3. N = 362. *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -3396,7 +3399,7 @@
         <v>-0.012</v>
       </c>
       <c r="E22" s="40" t="n">
-        <v>0.04</v>
+        <v>0.044</v>
       </c>
       <c r="F22" s="40" t="inlineStr">
         <is>
@@ -3412,7 +3415,7 @@
         <v>0.024</v>
       </c>
       <c r="I22" s="40" t="n">
-        <v>0.043</v>
+        <v>0.046</v>
       </c>
       <c r="J22" s="40" t="inlineStr">
         <is>
@@ -3465,7 +3468,7 @@
         <v>0.018</v>
       </c>
       <c r="E23" s="40" t="n">
-        <v>0.039</v>
+        <v>0.037</v>
       </c>
       <c r="F23" s="40" t="inlineStr">
         <is>
@@ -3481,7 +3484,7 @@
         <v>-0.019</v>
       </c>
       <c r="I23" s="40" t="n">
-        <v>0.041</v>
+        <v>0.048</v>
       </c>
       <c r="J23" s="40" t="inlineStr">
         <is>
@@ -3531,10 +3534,10 @@
         </is>
       </c>
       <c r="D24" s="40" t="n">
-        <v>0.078</v>
+        <v>0.046</v>
       </c>
       <c r="E24" s="40" t="n">
-        <v>0.038</v>
+        <v>0.041</v>
       </c>
       <c r="F24" s="40" t="inlineStr">
         <is>
@@ -3550,7 +3553,7 @@
         <v>-0.111</v>
       </c>
       <c r="I24" s="40" t="n">
-        <v>0.041</v>
+        <v>0.039</v>
       </c>
       <c r="J24" s="40" t="inlineStr">
         <is>
@@ -3603,7 +3606,7 @@
         <v>-0.098</v>
       </c>
       <c r="E25" s="40" t="n">
-        <v>0.039</v>
+        <v>0.045</v>
       </c>
       <c r="F25" s="40" t="inlineStr">
         <is>
@@ -3619,7 +3622,7 @@
         <v>0.067</v>
       </c>
       <c r="I25" s="40" t="n">
-        <v>0.038</v>
+        <v>0.052</v>
       </c>
       <c r="J25" s="40" t="inlineStr">
         <is>
@@ -3711,7 +3714,7 @@
     <row r="28" ht="48" customHeight="1" s="45">
       <c r="A28" s="23" t="inlineStr">
         <is>
-          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 361; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.</t>
+          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 362; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -5192,64 +5195,64 @@
         </is>
       </c>
       <c r="D6" s="38" t="n">
-        <v>0.078</v>
+        <v>0.046</v>
       </c>
       <c r="E6" s="38" t="n">
-        <v>0.038</v>
+        <v>0.041</v>
       </c>
       <c r="F6" s="38" t="n">
-        <v>0.041</v>
+        <v>0.263</v>
       </c>
       <c r="G6" s="38" t="n">
-        <v>0.003</v>
+        <v>-0.034</v>
       </c>
       <c r="H6" s="38" t="n">
-        <v>0.153</v>
+        <v>0.126</v>
       </c>
       <c r="I6" s="38" t="n">
-        <v>-0.064</v>
+        <v>-0.039</v>
       </c>
       <c r="J6" s="38" t="n">
-        <v>0.062</v>
+        <v>0.063</v>
       </c>
       <c r="K6" s="38" t="n">
-        <v>0.301</v>
+        <v>0.535</v>
       </c>
       <c r="L6" s="38" t="n">
-        <v>-0.186</v>
+        <v>-0.162</v>
       </c>
       <c r="M6" s="38" t="n">
-        <v>0.058</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="N6" s="38" t="n">
-        <v>-0.22</v>
+        <v>-0.156</v>
       </c>
       <c r="O6" s="38" t="n">
-        <v>0.065</v>
+        <v>0.067</v>
       </c>
       <c r="P6" s="38" t="n">
-        <v>0.001</v>
+        <v>0.02</v>
       </c>
       <c r="Q6" s="38" t="n">
-        <v>-0.347</v>
+        <v>-0.288</v>
       </c>
       <c r="R6" s="38" t="n">
-        <v>-0.093</v>
+        <v>-0.024</v>
       </c>
       <c r="S6" s="38" t="n">
-        <v>0.156</v>
+        <v>0.117</v>
       </c>
       <c r="T6" s="38" t="n">
-        <v>0.076</v>
+        <v>0.082</v>
       </c>
       <c r="U6" s="38" t="n">
-        <v>0.041</v>
+        <v>0.155</v>
       </c>
       <c r="V6" s="38" t="n">
-        <v>0.007</v>
+        <v>-0.043</v>
       </c>
       <c r="W6" s="38" t="n">
-        <v>0.305</v>
+        <v>0.277</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="45">
@@ -5809,7 +5812,7 @@
     <row r="2">
       <c r="A2" s="38" t="inlineStr">
         <is>
-          <t>N = 361</t>
+          <t>N = 362</t>
         </is>
       </c>
     </row>
@@ -5823,14 +5826,14 @@
     <row r="4">
       <c r="A4" s="38" t="inlineStr">
         <is>
-          <t>- Male: 197 (54.6%)</t>
+          <t>- Male: 204 (56.4%)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="38" t="inlineStr">
         <is>
-          <t>- Female: 164 (45.4%)</t>
+          <t>- Female: 158 (43.6%)</t>
         </is>
       </c>
     </row>
@@ -5845,28 +5848,33 @@
     <row r="8">
       <c r="A8" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 30.61, SD = 4.65</t>
+          <t>Age: M = 30.70, SD = 4.68</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="38" t="inlineStr">
         <is>
-          <t>Working years: M = 8.85, SD = 4.82</t>
+          <t>Working years: M = 8.95, SD = 4.88</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="38" t="inlineStr">
         <is>
-          <t>Tenure with current leader: M = 2.27, SD = 1.44</t>
+          <t>Tenure with current leader: M = 2.30, SD = 1.47</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="38" t="inlineStr">
-        <is>
-          <t>Interaction frequency with leader: M = 3.28, SD = 1.08</t>
+      <c r="A11" s="48" t="inlineStr">
+        <is>
+          <t>Interaction frequency with leader:
+  - Rarely (&lt;1/wk): 20 (5.5%)
+  - Sometimes (1-2/wk): 65 (18.0%)
+  - Often (3-4/wk): 126 (34.8%)
+  - Very often (~daily): 107 (29.6%)
+  - Multiple times/day: 44 (12.2%)</t>
         </is>
       </c>
     </row>
@@ -5881,35 +5889,35 @@
     <row r="14">
       <c r="A14" s="38" t="inlineStr">
         <is>
-          <t>- High school: 18 (5.0%)</t>
+          <t>- High school: 19 (5.2%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 57 (15.8%)</t>
+          <t>- Some college / Associate: 58 (16.0%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 166 (46.0%)</t>
+          <t>- Bachelor: 167 (46.1%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="38" t="inlineStr">
         <is>
-          <t>- Master: 92 (25.5%)</t>
+          <t>- Master: 93 (25.7%)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="38" t="inlineStr">
         <is>
-          <t>- Doctorate: 23 (6.4%)</t>
+          <t>- Doctorate: 20 (5.5%)</t>
         </is>
       </c>
     </row>
@@ -5931,28 +5939,28 @@
     <row r="22">
       <c r="A22" s="38" t="inlineStr">
         <is>
-          <t>- Associate: 119 (33.0%)</t>
+          <t>- Associate: 116 (32.0%)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="38" t="inlineStr">
         <is>
-          <t>- Senior: 90 (24.9%)</t>
+          <t>- Senior: 92 (25.4%)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="38" t="inlineStr">
         <is>
-          <t>- Manager: 61 (16.9%)</t>
+          <t>- Manager: 65 (18.0%)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="38" t="inlineStr">
         <is>
-          <t>- Director: 18 (5.0%)</t>
+          <t>- Director: 17 (4.7%)</t>
         </is>
       </c>
     </row>
@@ -5982,14 +5990,14 @@
     <row r="31">
       <c r="A31" s="38" t="inlineStr">
         <is>
-          <t>- Male: 51 (64.6%)</t>
+          <t>- Male: 52 (65.8%)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="38" t="inlineStr">
         <is>
-          <t>- Female: 28 (35.4%)</t>
+          <t>- Female: 27 (34.2%)</t>
         </is>
       </c>
     </row>
@@ -6004,7 +6012,7 @@
     <row r="35">
       <c r="A35" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 40.95, SD = 6.47</t>
+          <t>Age: M = 41.65, SD = 5.90</t>
         </is>
       </c>
     </row>
@@ -6018,14 +6026,14 @@
     <row r="37">
       <c r="A37" s="38" t="inlineStr">
         <is>
-          <t>Leadership tenure: M = 5.40, SD = 2.73</t>
+          <t>Leadership tenure: M = 5.23, SD = 3.03</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="38" t="inlineStr">
         <is>
-          <t>Span of control: M = 4.57, SD = 0.57</t>
+          <t>Span of control: M = 4.58, SD = 0.59</t>
         </is>
       </c>
     </row>
@@ -6040,14 +6048,14 @@
     <row r="41">
       <c r="A41" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 7 (8.9%)</t>
+          <t>- Some college / Associate: 8 (10.1%)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 40 (50.6%)</t>
+          <t>- Bachelor: 39 (49.4%)</t>
         </is>
       </c>
     </row>
@@ -6199,22 +6207,22 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>1183.4</v>
+        <v>1156.8</v>
       </c>
       <c r="C3" s="13" t="n">
         <v>542</v>
       </c>
       <c r="D3" s="13" t="n">
-        <v>0.952</v>
+        <v>0.954</v>
       </c>
       <c r="E3" s="13" t="n">
-        <v>0.948</v>
+        <v>0.949</v>
       </c>
       <c r="F3" s="13" t="n">
-        <v>0.043</v>
+        <v>0.042</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.038</v>
+        <v>0.037</v>
       </c>
       <c r="H3" s="13" t="n"/>
       <c r="I3" s="13" t="n"/>
@@ -6231,7 +6239,7 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>1098.6</v>
+        <v>1102.4</v>
       </c>
       <c r="C4" s="13" t="n">
         <v>521</v>
@@ -6240,16 +6248,16 @@
         <v>0.961</v>
       </c>
       <c r="E4" s="13" t="n">
-        <v>0.954</v>
+        <v>0.953</v>
       </c>
       <c r="F4" s="13" t="n">
-        <v>0.041</v>
+        <v>0.04</v>
       </c>
       <c r="G4" s="13" t="n">
         <v>0.036</v>
       </c>
       <c r="H4" s="13" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.007</v>
       </c>
       <c r="I4" s="13" t="n">
         <v>-0.002</v>
@@ -6276,7 +6284,7 @@
       <c r="I5" s="13" t="n"/>
       <c r="J5" s="13" t="inlineStr">
         <is>
-          <t>12%</t>
+          <t>8.7%</t>
         </is>
       </c>
     </row>
@@ -6381,7 +6389,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="9">
@@ -6411,7 +6419,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="12">
@@ -6514,7 +6522,7 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>78.5%</t>
+          <t>78.7%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sync v4.4: round-2 feedback applied (Model3 differentiated, alphas dropped, AUTO×PD→BE ns)
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -813,7 +813,7 @@
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -952,6 +952,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="50">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1642,28 +1645,28 @@
         </is>
       </c>
       <c r="D3" s="39" t="n">
-        <v>1183.4</v>
+        <v>1156.8</v>
       </c>
       <c r="E3" s="39" t="n">
         <v>542</v>
       </c>
       <c r="F3" s="39" t="n">
-        <v>0.952</v>
+        <v>0.954</v>
       </c>
       <c r="G3" s="39" t="n">
-        <v>0.948</v>
+        <v>0.949</v>
       </c>
       <c r="H3" s="39" t="n">
-        <v>0.043</v>
+        <v>0.042</v>
       </c>
       <c r="I3" s="39" t="n">
-        <v>0.038</v>
+        <v>0.037</v>
       </c>
       <c r="J3" s="39" t="n">
-        <v>0.046</v>
+        <v>0.052</v>
       </c>
       <c r="K3" s="39" t="n">
-        <v>22456.3</v>
+        <v>22431.6</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" s="45">
@@ -1683,28 +1686,28 @@
         </is>
       </c>
       <c r="D4" s="39" t="n">
-        <v>1392.7</v>
+        <v>1331.2</v>
       </c>
       <c r="E4" s="39" t="n">
         <v>547</v>
       </c>
       <c r="F4" s="39" t="n">
-        <v>0.928</v>
+        <v>0.9340000000000001</v>
       </c>
       <c r="G4" s="39" t="n">
-        <v>0.922</v>
+        <v>0.927</v>
       </c>
       <c r="H4" s="39" t="n">
-        <v>0.054</v>
+        <v>0.051</v>
       </c>
       <c r="I4" s="39" t="n">
-        <v>0.044</v>
+        <v>0.043</v>
       </c>
       <c r="J4" s="39" t="n">
-        <v>0.051</v>
+        <v>0.049</v>
       </c>
       <c r="K4" s="39" t="n">
-        <v>22612.5</v>
+        <v>22587.9</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" s="45">
@@ -1724,28 +1727,28 @@
         </is>
       </c>
       <c r="D5" s="39" t="n">
-        <v>1518.3</v>
+        <v>1612.5</v>
       </c>
       <c r="E5" s="39" t="n">
         <v>547</v>
       </c>
       <c r="F5" s="39" t="n">
-        <v>0.918</v>
+        <v>0.911</v>
       </c>
       <c r="G5" s="39" t="n">
-        <v>0.911</v>
+        <v>0.903</v>
       </c>
       <c r="H5" s="39" t="n">
-        <v>0.058</v>
+        <v>0.061</v>
       </c>
       <c r="I5" s="39" t="n">
-        <v>0.047</v>
+        <v>0.046</v>
       </c>
       <c r="J5" s="39" t="n">
-        <v>0.053</v>
+        <v>0.067</v>
       </c>
       <c r="K5" s="39" t="n">
-        <v>22789.6</v>
+        <v>22823.4</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" s="45">
@@ -1765,28 +1768,28 @@
         </is>
       </c>
       <c r="D6" s="39" t="n">
-        <v>2034.1</v>
+        <v>2123.7</v>
       </c>
       <c r="E6" s="39" t="n">
         <v>552</v>
       </c>
       <c r="F6" s="39" t="n">
-        <v>0.876</v>
+        <v>0.864</v>
       </c>
       <c r="G6" s="39" t="n">
-        <v>0.866</v>
+        <v>0.851</v>
       </c>
       <c r="H6" s="39" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.073</v>
       </c>
       <c r="I6" s="39" t="n">
-        <v>0.052</v>
+        <v>0.054</v>
       </c>
       <c r="J6" s="39" t="n">
-        <v>0.058</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="K6" s="39" t="n">
-        <v>23156.2</v>
+        <v>23218.6</v>
       </c>
     </row>
     <row r="7">
@@ -1806,28 +1809,28 @@
         </is>
       </c>
       <c r="D7" s="39" t="n">
-        <v>2789.5</v>
+        <v>2645.9</v>
       </c>
       <c r="E7" s="39" t="n">
         <v>556</v>
       </c>
       <c r="F7" s="39" t="n">
-        <v>0.8120000000000001</v>
+        <v>0.821</v>
       </c>
       <c r="G7" s="39" t="n">
-        <v>0.798</v>
+        <v>0.806</v>
       </c>
       <c r="H7" s="39" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.082</v>
       </c>
       <c r="I7" s="39" t="n">
-        <v>0.064</v>
+        <v>0.061</v>
       </c>
       <c r="J7" s="39" t="n">
-        <v>0.078</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="K7" s="39" t="n">
-        <v>23598.7</v>
+        <v>23529.3</v>
       </c>
     </row>
     <row r="8" ht="58" customHeight="1" s="45">
@@ -1948,10 +1951,10 @@
         </is>
       </c>
       <c r="B3" s="40" t="n">
-        <v>0.546</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="C3" s="40" t="n">
-        <v>0.499</v>
+        <v>0.497</v>
       </c>
       <c r="D3" s="40" t="inlineStr">
         <is>
@@ -1966,13 +1969,13 @@
         </is>
       </c>
       <c r="B4" s="40" t="n">
-        <v>30.609</v>
+        <v>30.699</v>
       </c>
       <c r="C4" s="40" t="n">
-        <v>4.651</v>
+        <v>4.675</v>
       </c>
       <c r="D4" s="40" t="n">
-        <v>0.042</v>
+        <v>0.022</v>
       </c>
       <c r="E4" s="40" t="inlineStr">
         <is>
@@ -1987,16 +1990,16 @@
         </is>
       </c>
       <c r="B5" s="40" t="n">
-        <v>2.269</v>
+        <v>2.297</v>
       </c>
       <c r="C5" s="40" t="n">
-        <v>1.437</v>
+        <v>1.468</v>
       </c>
       <c r="D5" s="40" t="n">
-        <v>-0.002</v>
+        <v>-0.025</v>
       </c>
       <c r="E5" s="40" t="n">
-        <v>0.183</v>
+        <v>0.203</v>
       </c>
       <c r="F5" s="40" t="inlineStr">
         <is>
@@ -2011,19 +2014,19 @@
         </is>
       </c>
       <c r="B6" s="40" t="n">
-        <v>3.283</v>
+        <v>3.249</v>
       </c>
       <c r="C6" s="40" t="n">
-        <v>1.082</v>
+        <v>1.06</v>
       </c>
       <c r="D6" s="40" t="n">
-        <v>0.115</v>
+        <v>0.096</v>
       </c>
       <c r="E6" s="40" t="n">
-        <v>-0.024</v>
+        <v>-0.014</v>
       </c>
       <c r="F6" s="40" t="n">
-        <v>-0.058</v>
+        <v>-0.049</v>
       </c>
       <c r="G6" s="40" t="inlineStr">
         <is>
@@ -2038,26 +2041,26 @@
         </is>
       </c>
       <c r="B7" s="40" t="n">
-        <v>4.029</v>
+        <v>4.04</v>
       </c>
       <c r="C7" s="40" t="n">
-        <v>0.879</v>
+        <v>0.901</v>
       </c>
       <c r="D7" s="40" t="n">
+        <v>-0.058</v>
+      </c>
+      <c r="E7" s="40" t="n">
+        <v>-0.008</v>
+      </c>
+      <c r="F7" s="40" t="n">
+        <v>0.082</v>
+      </c>
+      <c r="G7" s="40" t="n">
         <v>-0.016</v>
       </c>
-      <c r="E7" s="40" t="n">
-        <v>-0.033</v>
-      </c>
-      <c r="F7" s="40" t="n">
-        <v>0.043</v>
-      </c>
-      <c r="G7" s="40" t="n">
-        <v>0.011</v>
-      </c>
       <c r="H7" s="39" t="inlineStr">
         <is>
-          <t>(0.91)</t>
+          <t>(0.86)</t>
         </is>
       </c>
     </row>
@@ -2068,29 +2071,29 @@
         </is>
       </c>
       <c r="B8" s="40" t="n">
-        <v>5</v>
+        <v>4.999</v>
       </c>
       <c r="C8" s="40" t="n">
-        <v>0.837</v>
+        <v>0.997</v>
       </c>
       <c r="D8" s="40" t="n">
-        <v>-0.043</v>
+        <v>-0</v>
       </c>
       <c r="E8" s="40" t="n">
-        <v>0.026</v>
+        <v>-0.027</v>
       </c>
       <c r="F8" s="40" t="n">
-        <v>-0.023</v>
+        <v>0.028</v>
       </c>
       <c r="G8" s="40" t="n">
-        <v>-0.125</v>
+        <v>-0.119</v>
       </c>
       <c r="H8" s="40" t="n">
-        <v>-0.129</v>
+        <v>-0.354</v>
       </c>
       <c r="I8" s="40" t="inlineStr">
         <is>
-          <t>(0.93)</t>
+          <t>(0.87)</t>
         </is>
       </c>
     </row>
@@ -2101,32 +2104,32 @@
         </is>
       </c>
       <c r="B9" s="40" t="n">
-        <v>3.438</v>
+        <v>3.463</v>
       </c>
       <c r="C9" s="40" t="n">
-        <v>0.906</v>
+        <v>0.921</v>
       </c>
       <c r="D9" s="40" t="n">
-        <v>-0.041</v>
+        <v>-0.062</v>
       </c>
       <c r="E9" s="40" t="n">
-        <v>-0.038</v>
+        <v>-0</v>
       </c>
       <c r="F9" s="40" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.076</v>
       </c>
       <c r="G9" s="40" t="n">
-        <v>-0.045</v>
+        <v>-0.06</v>
       </c>
       <c r="H9" s="40" t="n">
-        <v>-0.023</v>
+        <v>0.021</v>
       </c>
       <c r="I9" s="40" t="n">
-        <v>0.029</v>
+        <v>-0.004</v>
       </c>
       <c r="J9" s="40" t="inlineStr">
         <is>
-          <t>(0.86)</t>
+          <t>(0.79)</t>
         </is>
       </c>
     </row>
@@ -2137,35 +2140,35 @@
         </is>
       </c>
       <c r="B10" s="40" t="n">
-        <v>4.575</v>
+        <v>4.597</v>
       </c>
       <c r="C10" s="40" t="n">
-        <v>0.897</v>
+        <v>0.887</v>
       </c>
       <c r="D10" s="40" t="n">
-        <v>-0.107</v>
+        <v>-0.07199999999999999</v>
       </c>
       <c r="E10" s="40" t="n">
-        <v>-0.079</v>
+        <v>-0.091</v>
       </c>
       <c r="F10" s="40" t="n">
-        <v>-0.056</v>
+        <v>-0.046</v>
       </c>
       <c r="G10" s="40" t="n">
-        <v>-0.08500000000000001</v>
+        <v>-0.049</v>
       </c>
       <c r="H10" s="40" t="n">
-        <v>-0.041</v>
+        <v>-0.031</v>
       </c>
       <c r="I10" s="40" t="n">
-        <v>-0.036</v>
+        <v>-0.039</v>
       </c>
       <c r="J10" s="40" t="n">
-        <v>-0.018</v>
+        <v>0.02</v>
       </c>
       <c r="K10" s="40" t="inlineStr">
         <is>
-          <t>(0.84)</t>
+          <t>(0.78)</t>
         </is>
       </c>
     </row>
@@ -2176,38 +2179,38 @@
         </is>
       </c>
       <c r="B11" s="40" t="n">
-        <v>4.471</v>
+        <v>4.533</v>
       </c>
       <c r="C11" s="40" t="n">
-        <v>1.194</v>
+        <v>1.266</v>
       </c>
       <c r="D11" s="40" t="n">
-        <v>-0.07000000000000001</v>
+        <v>0.03</v>
       </c>
       <c r="E11" s="40" t="n">
-        <v>0.003</v>
+        <v>-0.038</v>
       </c>
       <c r="F11" s="40" t="n">
-        <v>-0.053</v>
+        <v>-0.016</v>
       </c>
       <c r="G11" s="40" t="n">
-        <v>-0.048</v>
+        <v>-0.059</v>
       </c>
       <c r="H11" s="40" t="n">
-        <v>-0.477</v>
+        <v>-0.5679999999999999</v>
       </c>
       <c r="I11" s="40" t="n">
-        <v>0.463</v>
+        <v>0.569</v>
       </c>
       <c r="J11" s="40" t="n">
-        <v>-0.008</v>
+        <v>-0.059</v>
       </c>
       <c r="K11" s="40" t="n">
-        <v>-0.051</v>
+        <v>-0.081</v>
       </c>
       <c r="L11" s="40" t="inlineStr">
         <is>
-          <t>(0.88)</t>
+          <t>(0.84)</t>
         </is>
       </c>
     </row>
@@ -2218,41 +2221,41 @@
         </is>
       </c>
       <c r="B12" s="40" t="n">
-        <v>2.977</v>
+        <v>2.971</v>
       </c>
       <c r="C12" s="40" t="n">
-        <v>1.137</v>
+        <v>1.201</v>
       </c>
       <c r="D12" s="40" t="n">
-        <v>0.025</v>
+        <v>-0.011</v>
       </c>
       <c r="E12" s="40" t="n">
-        <v>0.016</v>
+        <v>0.05</v>
       </c>
       <c r="F12" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="40" t="n">
         <v>0.047</v>
       </c>
-      <c r="G12" s="40" t="n">
-        <v>0.08599999999999999</v>
-      </c>
       <c r="H12" s="40" t="n">
-        <v>0.525</v>
+        <v>0.539</v>
       </c>
       <c r="I12" s="40" t="n">
-        <v>-0.435</v>
+        <v>-0.52</v>
       </c>
       <c r="J12" s="40" t="n">
-        <v>0.049</v>
+        <v>0.039</v>
       </c>
       <c r="K12" s="40" t="n">
-        <v>-0.092</v>
+        <v>-0.026</v>
       </c>
       <c r="L12" s="40" t="n">
-        <v>-0.457</v>
+        <v>-0.456</v>
       </c>
       <c r="M12" s="40" t="inlineStr">
         <is>
-          <t>(0.87)</t>
+          <t>(0.81)</t>
         </is>
       </c>
     </row>
@@ -2263,44 +2266,44 @@
         </is>
       </c>
       <c r="B13" s="40" t="n">
-        <v>4.505</v>
+        <v>4.42</v>
       </c>
       <c r="C13" s="40" t="n">
-        <v>0.403</v>
+        <v>0.5669999999999999</v>
       </c>
       <c r="D13" s="40" t="n">
-        <v>0.004</v>
+        <v>-0.005</v>
       </c>
       <c r="E13" s="40" t="n">
-        <v>-0.036</v>
+        <v>-0.025</v>
       </c>
       <c r="F13" s="40" t="n">
-        <v>0.015</v>
+        <v>-0.013</v>
       </c>
       <c r="G13" s="40" t="n">
-        <v>0.022</v>
+        <v>0.001</v>
       </c>
       <c r="H13" s="40" t="n">
-        <v>-0</v>
+        <v>-0.022</v>
       </c>
       <c r="I13" s="40" t="n">
-        <v>0.07000000000000001</v>
+        <v>-0.024</v>
       </c>
       <c r="J13" s="40" t="n">
-        <v>-0.175</v>
+        <v>-0.13</v>
       </c>
       <c r="K13" s="40" t="n">
-        <v>0.073</v>
+        <v>0.034</v>
       </c>
       <c r="L13" s="40" t="n">
-        <v>0.075</v>
+        <v>-0.005</v>
       </c>
       <c r="M13" s="40" t="n">
-        <v>-0.095</v>
+        <v>-0.065</v>
       </c>
       <c r="N13" s="40" t="inlineStr">
         <is>
-          <t>(0.90)</t>
+          <t>(0.83)</t>
         </is>
       </c>
     </row>
@@ -2311,47 +2314,47 @@
         </is>
       </c>
       <c r="B14" s="40" t="n">
-        <v>4.548</v>
+        <v>4.524</v>
       </c>
       <c r="C14" s="40" t="n">
-        <v>0.806</v>
+        <v>0.829</v>
       </c>
       <c r="D14" s="40" t="n">
-        <v>0.011</v>
+        <v>0.033</v>
       </c>
       <c r="E14" s="40" t="n">
-        <v>0.015</v>
+        <v>-0.08599999999999999</v>
       </c>
       <c r="F14" s="40" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G14" s="40" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="H14" s="40" t="n">
+        <v>-0.456</v>
+      </c>
+      <c r="I14" s="40" t="n">
+        <v>0.426</v>
+      </c>
+      <c r="J14" s="40" t="n">
+        <v>-0.094</v>
+      </c>
+      <c r="K14" s="40" t="n">
         <v>0.028</v>
       </c>
-      <c r="G14" s="40" t="n">
-        <v>-0.081</v>
-      </c>
-      <c r="H14" s="40" t="n">
-        <v>-0.514</v>
-      </c>
-      <c r="I14" s="40" t="n">
-        <v>0.409</v>
-      </c>
-      <c r="J14" s="40" t="n">
-        <v>-0.052</v>
-      </c>
-      <c r="K14" s="40" t="n">
-        <v>0.04</v>
-      </c>
       <c r="L14" s="40" t="n">
-        <v>0.677</v>
+        <v>0.576</v>
       </c>
       <c r="M14" s="40" t="n">
-        <v>-0.6870000000000001</v>
+        <v>-0.615</v>
       </c>
       <c r="N14" s="40" t="n">
-        <v>0.083</v>
+        <v>0.433</v>
       </c>
       <c r="O14" s="40" t="inlineStr">
         <is>
-          <t>(0.90)</t>
+          <t>(0.85)</t>
         </is>
       </c>
     </row>
@@ -2362,50 +2365,50 @@
         </is>
       </c>
       <c r="B15" s="40" t="n">
-        <v>4.814</v>
+        <v>4.908</v>
       </c>
       <c r="C15" s="40" t="n">
-        <v>1.368</v>
+        <v>1.324</v>
       </c>
       <c r="D15" s="40" t="n">
-        <v>-0.056</v>
+        <v>0.04</v>
       </c>
       <c r="E15" s="40" t="n">
-        <v>-0.08599999999999999</v>
+        <v>-0.093</v>
       </c>
       <c r="F15" s="40" t="n">
-        <v>0.031</v>
+        <v>0.035</v>
       </c>
       <c r="G15" s="40" t="n">
-        <v>0.006</v>
+        <v>0.039</v>
       </c>
       <c r="H15" s="40" t="n">
-        <v>-0.292</v>
+        <v>-0.343</v>
       </c>
       <c r="I15" s="40" t="n">
-        <v>0.324</v>
+        <v>0.223</v>
       </c>
       <c r="J15" s="40" t="n">
-        <v>0.053</v>
+        <v>-0.031</v>
       </c>
       <c r="K15" s="40" t="n">
-        <v>-0.047</v>
+        <v>0.012</v>
       </c>
       <c r="L15" s="40" t="n">
-        <v>0.422</v>
+        <v>0.365</v>
       </c>
       <c r="M15" s="40" t="n">
-        <v>-0.432</v>
+        <v>-0.353</v>
       </c>
       <c r="N15" s="40" t="n">
-        <v>0.062</v>
+        <v>0.098</v>
       </c>
       <c r="O15" s="40" t="n">
-        <v>0.397</v>
+        <v>0.303</v>
       </c>
       <c r="P15" s="40" t="inlineStr">
         <is>
-          <t>(0.92)</t>
+          <t>(0.86)</t>
         </is>
       </c>
     </row>
@@ -2416,60 +2419,60 @@
         </is>
       </c>
       <c r="B16" s="40" t="n">
-        <v>2.416</v>
+        <v>2.431</v>
       </c>
       <c r="C16" s="40" t="n">
-        <v>1.168</v>
+        <v>1.173</v>
       </c>
       <c r="D16" s="40" t="n">
-        <v>0.076</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="E16" s="40" t="n">
-        <v>0.047</v>
+        <v>0.111</v>
       </c>
       <c r="F16" s="40" t="n">
-        <v>-0.029</v>
+        <v>-0.025</v>
       </c>
       <c r="G16" s="40" t="n">
-        <v>-0.003</v>
+        <v>0.03</v>
       </c>
       <c r="H16" s="40" t="n">
-        <v>0.299</v>
+        <v>0.376</v>
       </c>
       <c r="I16" s="40" t="n">
-        <v>-0.335</v>
+        <v>-0.332</v>
       </c>
       <c r="J16" s="40" t="n">
-        <v>-0.034</v>
+        <v>0.048</v>
       </c>
       <c r="K16" s="40" t="n">
-        <v>-0.039</v>
+        <v>0.056</v>
       </c>
       <c r="L16" s="40" t="n">
-        <v>-0.424</v>
+        <v>-0.427</v>
       </c>
       <c r="M16" s="40" t="n">
-        <v>0.451</v>
+        <v>0.301</v>
       </c>
       <c r="N16" s="40" t="n">
-        <v>-0.108</v>
+        <v>0.065</v>
       </c>
       <c r="O16" s="40" t="n">
-        <v>-0.407</v>
+        <v>-0.26</v>
       </c>
       <c r="P16" s="40" t="n">
-        <v>-0.697</v>
+        <v>-0.458</v>
       </c>
       <c r="Q16" s="40" t="inlineStr">
         <is>
-          <t>(0.89)</t>
+          <t>(0.82)</t>
         </is>
       </c>
     </row>
     <row r="17" ht="35" customHeight="1" s="45">
       <c r="A17" s="23" t="inlineStr">
         <is>
-          <t>Note. Values on the diagonal are Cronbach’s alpha coefficients where applicable. Correlations are zero-order correlations among observed study variables. Leadership variables were rated by followers at T1. OCBS and CWBS were rated by leaders at T3. N = 361. *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
+          <t>Note. Values on the diagonal are Cronbach’s alpha coefficients where applicable. Correlations are zero-order correlations among observed study variables. Leadership variables were rated by followers at T1. OCBS and CWBS were rated by leaders at T3. N = 362. *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -3396,7 +3399,7 @@
         <v>-0.012</v>
       </c>
       <c r="E22" s="40" t="n">
-        <v>0.04</v>
+        <v>0.044</v>
       </c>
       <c r="F22" s="40" t="inlineStr">
         <is>
@@ -3412,7 +3415,7 @@
         <v>0.024</v>
       </c>
       <c r="I22" s="40" t="n">
-        <v>0.043</v>
+        <v>0.046</v>
       </c>
       <c r="J22" s="40" t="inlineStr">
         <is>
@@ -3465,7 +3468,7 @@
         <v>0.018</v>
       </c>
       <c r="E23" s="40" t="n">
-        <v>0.039</v>
+        <v>0.037</v>
       </c>
       <c r="F23" s="40" t="inlineStr">
         <is>
@@ -3481,7 +3484,7 @@
         <v>-0.019</v>
       </c>
       <c r="I23" s="40" t="n">
-        <v>0.041</v>
+        <v>0.048</v>
       </c>
       <c r="J23" s="40" t="inlineStr">
         <is>
@@ -3531,10 +3534,10 @@
         </is>
       </c>
       <c r="D24" s="40" t="n">
-        <v>0.078</v>
+        <v>0.046</v>
       </c>
       <c r="E24" s="40" t="n">
-        <v>0.038</v>
+        <v>0.041</v>
       </c>
       <c r="F24" s="40" t="inlineStr">
         <is>
@@ -3550,7 +3553,7 @@
         <v>-0.111</v>
       </c>
       <c r="I24" s="40" t="n">
-        <v>0.041</v>
+        <v>0.039</v>
       </c>
       <c r="J24" s="40" t="inlineStr">
         <is>
@@ -3603,7 +3606,7 @@
         <v>-0.098</v>
       </c>
       <c r="E25" s="40" t="n">
-        <v>0.039</v>
+        <v>0.045</v>
       </c>
       <c r="F25" s="40" t="inlineStr">
         <is>
@@ -3619,7 +3622,7 @@
         <v>0.067</v>
       </c>
       <c r="I25" s="40" t="n">
-        <v>0.038</v>
+        <v>0.052</v>
       </c>
       <c r="J25" s="40" t="inlineStr">
         <is>
@@ -3711,7 +3714,7 @@
     <row r="28" ht="48" customHeight="1" s="45">
       <c r="A28" s="23" t="inlineStr">
         <is>
-          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 361; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.</t>
+          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 362; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -5192,64 +5195,64 @@
         </is>
       </c>
       <c r="D6" s="38" t="n">
-        <v>0.078</v>
+        <v>0.046</v>
       </c>
       <c r="E6" s="38" t="n">
-        <v>0.038</v>
+        <v>0.041</v>
       </c>
       <c r="F6" s="38" t="n">
-        <v>0.041</v>
+        <v>0.263</v>
       </c>
       <c r="G6" s="38" t="n">
-        <v>0.003</v>
+        <v>-0.034</v>
       </c>
       <c r="H6" s="38" t="n">
-        <v>0.153</v>
+        <v>0.126</v>
       </c>
       <c r="I6" s="38" t="n">
-        <v>-0.064</v>
+        <v>-0.039</v>
       </c>
       <c r="J6" s="38" t="n">
-        <v>0.062</v>
+        <v>0.063</v>
       </c>
       <c r="K6" s="38" t="n">
-        <v>0.301</v>
+        <v>0.535</v>
       </c>
       <c r="L6" s="38" t="n">
-        <v>-0.186</v>
+        <v>-0.162</v>
       </c>
       <c r="M6" s="38" t="n">
-        <v>0.058</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="N6" s="38" t="n">
-        <v>-0.22</v>
+        <v>-0.156</v>
       </c>
       <c r="O6" s="38" t="n">
-        <v>0.065</v>
+        <v>0.067</v>
       </c>
       <c r="P6" s="38" t="n">
-        <v>0.001</v>
+        <v>0.02</v>
       </c>
       <c r="Q6" s="38" t="n">
-        <v>-0.347</v>
+        <v>-0.288</v>
       </c>
       <c r="R6" s="38" t="n">
-        <v>-0.093</v>
+        <v>-0.024</v>
       </c>
       <c r="S6" s="38" t="n">
-        <v>0.156</v>
+        <v>0.117</v>
       </c>
       <c r="T6" s="38" t="n">
-        <v>0.076</v>
+        <v>0.082</v>
       </c>
       <c r="U6" s="38" t="n">
-        <v>0.041</v>
+        <v>0.155</v>
       </c>
       <c r="V6" s="38" t="n">
-        <v>0.007</v>
+        <v>-0.043</v>
       </c>
       <c r="W6" s="38" t="n">
-        <v>0.305</v>
+        <v>0.277</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="45">
@@ -5809,7 +5812,7 @@
     <row r="2">
       <c r="A2" s="38" t="inlineStr">
         <is>
-          <t>N = 361</t>
+          <t>N = 362</t>
         </is>
       </c>
     </row>
@@ -5823,14 +5826,14 @@
     <row r="4">
       <c r="A4" s="38" t="inlineStr">
         <is>
-          <t>- Male: 197 (54.6%)</t>
+          <t>- Male: 204 (56.4%)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="38" t="inlineStr">
         <is>
-          <t>- Female: 164 (45.4%)</t>
+          <t>- Female: 158 (43.6%)</t>
         </is>
       </c>
     </row>
@@ -5845,28 +5848,33 @@
     <row r="8">
       <c r="A8" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 30.61, SD = 4.65</t>
+          <t>Age: M = 30.70, SD = 4.68</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="38" t="inlineStr">
         <is>
-          <t>Working years: M = 8.85, SD = 4.82</t>
+          <t>Working years: M = 8.95, SD = 4.88</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="38" t="inlineStr">
         <is>
-          <t>Tenure with current leader: M = 2.27, SD = 1.44</t>
+          <t>Tenure with current leader: M = 2.30, SD = 1.47</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="38" t="inlineStr">
-        <is>
-          <t>Interaction frequency with leader: M = 3.28, SD = 1.08</t>
+      <c r="A11" s="48" t="inlineStr">
+        <is>
+          <t>Interaction frequency with leader:
+  - Rarely (&lt;1/wk): 20 (5.5%)
+  - Sometimes (1-2/wk): 65 (18.0%)
+  - Often (3-4/wk): 126 (34.8%)
+  - Very often (~daily): 107 (29.6%)
+  - Multiple times/day: 44 (12.2%)</t>
         </is>
       </c>
     </row>
@@ -5881,35 +5889,35 @@
     <row r="14">
       <c r="A14" s="38" t="inlineStr">
         <is>
-          <t>- High school: 18 (5.0%)</t>
+          <t>- High school: 19 (5.2%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 57 (15.8%)</t>
+          <t>- Some college / Associate: 58 (16.0%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 166 (46.0%)</t>
+          <t>- Bachelor: 167 (46.1%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="38" t="inlineStr">
         <is>
-          <t>- Master: 92 (25.5%)</t>
+          <t>- Master: 93 (25.7%)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="38" t="inlineStr">
         <is>
-          <t>- Doctorate: 23 (6.4%)</t>
+          <t>- Doctorate: 20 (5.5%)</t>
         </is>
       </c>
     </row>
@@ -5931,28 +5939,28 @@
     <row r="22">
       <c r="A22" s="38" t="inlineStr">
         <is>
-          <t>- Associate: 119 (33.0%)</t>
+          <t>- Associate: 116 (32.0%)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="38" t="inlineStr">
         <is>
-          <t>- Senior: 90 (24.9%)</t>
+          <t>- Senior: 92 (25.4%)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="38" t="inlineStr">
         <is>
-          <t>- Manager: 61 (16.9%)</t>
+          <t>- Manager: 65 (18.0%)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="38" t="inlineStr">
         <is>
-          <t>- Director: 18 (5.0%)</t>
+          <t>- Director: 17 (4.7%)</t>
         </is>
       </c>
     </row>
@@ -5982,14 +5990,14 @@
     <row r="31">
       <c r="A31" s="38" t="inlineStr">
         <is>
-          <t>- Male: 51 (64.6%)</t>
+          <t>- Male: 52 (65.8%)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="38" t="inlineStr">
         <is>
-          <t>- Female: 28 (35.4%)</t>
+          <t>- Female: 27 (34.2%)</t>
         </is>
       </c>
     </row>
@@ -6004,7 +6012,7 @@
     <row r="35">
       <c r="A35" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 40.95, SD = 6.47</t>
+          <t>Age: M = 41.65, SD = 5.90</t>
         </is>
       </c>
     </row>
@@ -6018,14 +6026,14 @@
     <row r="37">
       <c r="A37" s="38" t="inlineStr">
         <is>
-          <t>Leadership tenure: M = 5.40, SD = 2.73</t>
+          <t>Leadership tenure: M = 5.23, SD = 3.03</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="38" t="inlineStr">
         <is>
-          <t>Span of control: M = 4.57, SD = 0.57</t>
+          <t>Span of control: M = 4.58, SD = 0.59</t>
         </is>
       </c>
     </row>
@@ -6040,14 +6048,14 @@
     <row r="41">
       <c r="A41" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 7 (8.9%)</t>
+          <t>- Some college / Associate: 8 (10.1%)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 40 (50.6%)</t>
+          <t>- Bachelor: 39 (49.4%)</t>
         </is>
       </c>
     </row>
@@ -6199,22 +6207,22 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>1183.4</v>
+        <v>1156.8</v>
       </c>
       <c r="C3" s="13" t="n">
         <v>542</v>
       </c>
       <c r="D3" s="13" t="n">
-        <v>0.952</v>
+        <v>0.954</v>
       </c>
       <c r="E3" s="13" t="n">
-        <v>0.948</v>
+        <v>0.949</v>
       </c>
       <c r="F3" s="13" t="n">
-        <v>0.043</v>
+        <v>0.042</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.038</v>
+        <v>0.037</v>
       </c>
       <c r="H3" s="13" t="n"/>
       <c r="I3" s="13" t="n"/>
@@ -6231,7 +6239,7 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>1098.6</v>
+        <v>1102.4</v>
       </c>
       <c r="C4" s="13" t="n">
         <v>521</v>
@@ -6240,16 +6248,16 @@
         <v>0.961</v>
       </c>
       <c r="E4" s="13" t="n">
-        <v>0.954</v>
+        <v>0.953</v>
       </c>
       <c r="F4" s="13" t="n">
-        <v>0.041</v>
+        <v>0.04</v>
       </c>
       <c r="G4" s="13" t="n">
         <v>0.036</v>
       </c>
       <c r="H4" s="13" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.007</v>
       </c>
       <c r="I4" s="13" t="n">
         <v>-0.002</v>
@@ -6276,7 +6284,7 @@
       <c r="I5" s="13" t="n"/>
       <c r="J5" s="13" t="inlineStr">
         <is>
-          <t>12%</t>
+          <t>8.7%</t>
         </is>
       </c>
     </row>
@@ -6381,7 +6389,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="9">
@@ -6411,7 +6419,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="12">
@@ -6514,7 +6522,7 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>78.5%</t>
+          <t>78.7%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sync v4.5: round-2 final close + client-facing README + cleanup
Sync delivery to main v4.5 (commit 833ff9f). Three open items from
round-2 feedback all closed:

  * T1 thriving SD = 0.639 (target 0.60-0.75)
  * Single CFA RMSEA spread 0.034-0.087, SRMR 0.025-0.063
  * CMV: M1 = 7.3% (multi-source), M3 = 11.6% (single-source)

Validation: 189/189 constraint + 10/10 audit layers PASS.
final: 79 leaders, 361 dyads.

Delivery-branch cleanup:
  * README.md rewritten as client-facing (no mention of internal
    pipeline scripts, no \"原始客户提供文件\" / \"反馈\" folder
    references)
  * complete_project_record.md removed (internal CRM-style log)
  * results/YUYU样本量变化.xlsx removed (legacy, replaced by
    样本量变化表.xlsx since v4.2)
  * main/ cruft directory removed
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -1951,10 +1951,10 @@
         </is>
       </c>
       <c r="B3" s="40" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.551</v>
       </c>
       <c r="C3" s="40" t="n">
-        <v>0.497</v>
+        <v>0.498</v>
       </c>
       <c r="D3" s="40" t="inlineStr">
         <is>
@@ -1969,13 +1969,13 @@
         </is>
       </c>
       <c r="B4" s="40" t="n">
-        <v>30.699</v>
+        <v>30.654</v>
       </c>
       <c r="C4" s="40" t="n">
-        <v>4.675</v>
+        <v>4.636</v>
       </c>
       <c r="D4" s="40" t="n">
-        <v>0.022</v>
+        <v>0.041</v>
       </c>
       <c r="E4" s="40" t="inlineStr">
         <is>
@@ -1990,16 +1990,16 @@
         </is>
       </c>
       <c r="B5" s="40" t="n">
-        <v>2.297</v>
+        <v>2.307</v>
       </c>
       <c r="C5" s="40" t="n">
-        <v>1.468</v>
+        <v>1.49</v>
       </c>
       <c r="D5" s="40" t="n">
-        <v>-0.025</v>
+        <v>-0.004</v>
       </c>
       <c r="E5" s="40" t="n">
-        <v>0.203</v>
+        <v>0.191</v>
       </c>
       <c r="F5" s="40" t="inlineStr">
         <is>
@@ -2014,19 +2014,19 @@
         </is>
       </c>
       <c r="B6" s="40" t="n">
-        <v>3.249</v>
+        <v>3.302</v>
       </c>
       <c r="C6" s="40" t="n">
-        <v>1.06</v>
+        <v>1.078</v>
       </c>
       <c r="D6" s="40" t="n">
-        <v>0.096</v>
+        <v>0.103</v>
       </c>
       <c r="E6" s="40" t="n">
-        <v>-0.014</v>
+        <v>-0.034</v>
       </c>
       <c r="F6" s="40" t="n">
-        <v>-0.049</v>
+        <v>-0.061</v>
       </c>
       <c r="G6" s="40" t="inlineStr">
         <is>
@@ -2041,22 +2041,22 @@
         </is>
       </c>
       <c r="B7" s="40" t="n">
-        <v>4.04</v>
+        <v>4.055</v>
       </c>
       <c r="C7" s="40" t="n">
-        <v>0.901</v>
+        <v>0.87</v>
       </c>
       <c r="D7" s="40" t="n">
-        <v>-0.058</v>
+        <v>-0.002</v>
       </c>
       <c r="E7" s="40" t="n">
-        <v>-0.008</v>
+        <v>-0.012</v>
       </c>
       <c r="F7" s="40" t="n">
-        <v>0.082</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="G7" s="40" t="n">
-        <v>-0.016</v>
+        <v>0.023</v>
       </c>
       <c r="H7" s="39" t="inlineStr">
         <is>
@@ -2071,25 +2071,25 @@
         </is>
       </c>
       <c r="B8" s="40" t="n">
-        <v>4.999</v>
+        <v>4.998</v>
       </c>
       <c r="C8" s="40" t="n">
-        <v>0.997</v>
+        <v>1.001</v>
       </c>
       <c r="D8" s="40" t="n">
-        <v>-0</v>
+        <v>-0.055</v>
       </c>
       <c r="E8" s="40" t="n">
-        <v>-0.027</v>
+        <v>0.011</v>
       </c>
       <c r="F8" s="40" t="n">
-        <v>0.028</v>
+        <v>0.022</v>
       </c>
       <c r="G8" s="40" t="n">
-        <v>-0.119</v>
+        <v>-0.147</v>
       </c>
       <c r="H8" s="40" t="n">
-        <v>-0.354</v>
+        <v>-0.351</v>
       </c>
       <c r="I8" s="40" t="inlineStr">
         <is>
@@ -2104,28 +2104,28 @@
         </is>
       </c>
       <c r="B9" s="40" t="n">
-        <v>3.463</v>
+        <v>3.445</v>
       </c>
       <c r="C9" s="40" t="n">
-        <v>0.921</v>
+        <v>0.905</v>
       </c>
       <c r="D9" s="40" t="n">
-        <v>-0.062</v>
+        <v>-0.055</v>
       </c>
       <c r="E9" s="40" t="n">
-        <v>-0</v>
+        <v>-0.041</v>
       </c>
       <c r="F9" s="40" t="n">
-        <v>0.076</v>
+        <v>0.057</v>
       </c>
       <c r="G9" s="40" t="n">
-        <v>-0.06</v>
+        <v>-0.066</v>
       </c>
       <c r="H9" s="40" t="n">
-        <v>0.021</v>
+        <v>-0.026</v>
       </c>
       <c r="I9" s="40" t="n">
-        <v>-0.004</v>
+        <v>0.044</v>
       </c>
       <c r="J9" s="40" t="inlineStr">
         <is>
@@ -2140,31 +2140,31 @@
         </is>
       </c>
       <c r="B10" s="40" t="n">
-        <v>4.597</v>
+        <v>4.556</v>
       </c>
       <c r="C10" s="40" t="n">
-        <v>0.887</v>
+        <v>0.878</v>
       </c>
       <c r="D10" s="40" t="n">
-        <v>-0.07199999999999999</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="E10" s="40" t="n">
-        <v>-0.091</v>
+        <v>-0.092</v>
       </c>
       <c r="F10" s="40" t="n">
-        <v>-0.046</v>
+        <v>-0.092</v>
       </c>
       <c r="G10" s="40" t="n">
-        <v>-0.049</v>
+        <v>-0.044</v>
       </c>
       <c r="H10" s="40" t="n">
-        <v>-0.031</v>
+        <v>-0.08</v>
       </c>
       <c r="I10" s="40" t="n">
-        <v>-0.039</v>
+        <v>0.027</v>
       </c>
       <c r="J10" s="40" t="n">
-        <v>0.02</v>
+        <v>-0.003</v>
       </c>
       <c r="K10" s="40" t="inlineStr">
         <is>
@@ -2179,34 +2179,34 @@
         </is>
       </c>
       <c r="B11" s="40" t="n">
-        <v>4.533</v>
+        <v>4.546</v>
       </c>
       <c r="C11" s="40" t="n">
-        <v>1.266</v>
+        <v>1.248</v>
       </c>
       <c r="D11" s="40" t="n">
-        <v>0.03</v>
+        <v>-0.026</v>
       </c>
       <c r="E11" s="40" t="n">
-        <v>-0.038</v>
+        <v>-0.018</v>
       </c>
       <c r="F11" s="40" t="n">
-        <v>-0.016</v>
+        <v>-0.006</v>
       </c>
       <c r="G11" s="40" t="n">
-        <v>-0.059</v>
+        <v>-0.08</v>
       </c>
       <c r="H11" s="40" t="n">
-        <v>-0.5679999999999999</v>
+        <v>-0.537</v>
       </c>
       <c r="I11" s="40" t="n">
-        <v>0.569</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="J11" s="40" t="n">
-        <v>-0.059</v>
+        <v>-0.017</v>
       </c>
       <c r="K11" s="40" t="n">
-        <v>-0.081</v>
+        <v>-0.036</v>
       </c>
       <c r="L11" s="40" t="inlineStr">
         <is>
@@ -2221,37 +2221,37 @@
         </is>
       </c>
       <c r="B12" s="40" t="n">
-        <v>2.971</v>
+        <v>2.961</v>
       </c>
       <c r="C12" s="40" t="n">
-        <v>1.201</v>
+        <v>1.182</v>
       </c>
       <c r="D12" s="40" t="n">
-        <v>-0.011</v>
+        <v>0.032</v>
       </c>
       <c r="E12" s="40" t="n">
-        <v>0.05</v>
+        <v>0.036</v>
       </c>
       <c r="F12" s="40" t="n">
-        <v>0</v>
+        <v>0.008</v>
       </c>
       <c r="G12" s="40" t="n">
-        <v>0.047</v>
+        <v>0.074</v>
       </c>
       <c r="H12" s="40" t="n">
-        <v>0.539</v>
+        <v>0.552</v>
       </c>
       <c r="I12" s="40" t="n">
-        <v>-0.52</v>
+        <v>-0.525</v>
       </c>
       <c r="J12" s="40" t="n">
-        <v>0.039</v>
+        <v>-0.008</v>
       </c>
       <c r="K12" s="40" t="n">
-        <v>-0.026</v>
+        <v>-0.08</v>
       </c>
       <c r="L12" s="40" t="n">
-        <v>-0.456</v>
+        <v>-0.454</v>
       </c>
       <c r="M12" s="40" t="inlineStr">
         <is>
@@ -2266,40 +2266,40 @@
         </is>
       </c>
       <c r="B13" s="40" t="n">
-        <v>4.42</v>
+        <v>4.402</v>
       </c>
       <c r="C13" s="40" t="n">
-        <v>0.5669999999999999</v>
+        <v>0.639</v>
       </c>
       <c r="D13" s="40" t="n">
-        <v>-0.005</v>
+        <v>-0.026</v>
       </c>
       <c r="E13" s="40" t="n">
+        <v>-0.013</v>
+      </c>
+      <c r="F13" s="40" t="n">
+        <v>-0.052</v>
+      </c>
+      <c r="G13" s="40" t="n">
+        <v>-0.008</v>
+      </c>
+      <c r="H13" s="40" t="n">
         <v>-0.025</v>
       </c>
-      <c r="F13" s="40" t="n">
-        <v>-0.013</v>
-      </c>
-      <c r="G13" s="40" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="H13" s="40" t="n">
-        <v>-0.022</v>
-      </c>
       <c r="I13" s="40" t="n">
-        <v>-0.024</v>
+        <v>0.005</v>
       </c>
       <c r="J13" s="40" t="n">
-        <v>-0.13</v>
+        <v>-0.125</v>
       </c>
       <c r="K13" s="40" t="n">
-        <v>0.034</v>
+        <v>-0.045</v>
       </c>
       <c r="L13" s="40" t="n">
-        <v>-0.005</v>
+        <v>0.041</v>
       </c>
       <c r="M13" s="40" t="n">
-        <v>-0.065</v>
+        <v>-0.068</v>
       </c>
       <c r="N13" s="40" t="inlineStr">
         <is>
@@ -2314,43 +2314,43 @@
         </is>
       </c>
       <c r="B14" s="40" t="n">
-        <v>4.524</v>
+        <v>4.518</v>
       </c>
       <c r="C14" s="40" t="n">
-        <v>0.829</v>
+        <v>0.828</v>
       </c>
       <c r="D14" s="40" t="n">
-        <v>0.033</v>
+        <v>-0.06</v>
       </c>
       <c r="E14" s="40" t="n">
-        <v>-0.08599999999999999</v>
+        <v>-0.029</v>
       </c>
       <c r="F14" s="40" t="n">
-        <v>0.03</v>
+        <v>-0.042</v>
       </c>
       <c r="G14" s="40" t="n">
-        <v>-0.06</v>
+        <v>-0.108</v>
       </c>
       <c r="H14" s="40" t="n">
-        <v>-0.456</v>
+        <v>-0.419</v>
       </c>
       <c r="I14" s="40" t="n">
-        <v>0.426</v>
+        <v>0.451</v>
       </c>
       <c r="J14" s="40" t="n">
-        <v>-0.094</v>
+        <v>-0.025</v>
       </c>
       <c r="K14" s="40" t="n">
-        <v>0.028</v>
+        <v>0.013</v>
       </c>
       <c r="L14" s="40" t="n">
-        <v>0.576</v>
+        <v>0.602</v>
       </c>
       <c r="M14" s="40" t="n">
-        <v>-0.615</v>
+        <v>-0.663</v>
       </c>
       <c r="N14" s="40" t="n">
-        <v>0.433</v>
+        <v>0.394</v>
       </c>
       <c r="O14" s="40" t="inlineStr">
         <is>
@@ -2365,46 +2365,46 @@
         </is>
       </c>
       <c r="B15" s="40" t="n">
-        <v>4.908</v>
+        <v>4.823</v>
       </c>
       <c r="C15" s="40" t="n">
-        <v>1.324</v>
+        <v>1.367</v>
       </c>
       <c r="D15" s="40" t="n">
-        <v>0.04</v>
+        <v>-0.091</v>
       </c>
       <c r="E15" s="40" t="n">
-        <v>-0.093</v>
+        <v>-0.06900000000000001</v>
       </c>
       <c r="F15" s="40" t="n">
-        <v>0.035</v>
+        <v>0.021</v>
       </c>
       <c r="G15" s="40" t="n">
-        <v>0.039</v>
+        <v>0.015</v>
       </c>
       <c r="H15" s="40" t="n">
-        <v>-0.343</v>
+        <v>-0.272</v>
       </c>
       <c r="I15" s="40" t="n">
-        <v>0.223</v>
+        <v>0.299</v>
       </c>
       <c r="J15" s="40" t="n">
-        <v>-0.031</v>
+        <v>-0.04</v>
       </c>
       <c r="K15" s="40" t="n">
-        <v>0.012</v>
+        <v>-0.057</v>
       </c>
       <c r="L15" s="40" t="n">
-        <v>0.365</v>
+        <v>0.423</v>
       </c>
       <c r="M15" s="40" t="n">
-        <v>-0.353</v>
+        <v>-0.382</v>
       </c>
       <c r="N15" s="40" t="n">
-        <v>0.098</v>
+        <v>0.095</v>
       </c>
       <c r="O15" s="40" t="n">
-        <v>0.303</v>
+        <v>0.34</v>
       </c>
       <c r="P15" s="40" t="inlineStr">
         <is>
@@ -2419,49 +2419,49 @@
         </is>
       </c>
       <c r="B16" s="40" t="n">
-        <v>2.431</v>
+        <v>2.409</v>
       </c>
       <c r="C16" s="40" t="n">
-        <v>1.173</v>
+        <v>1.061</v>
       </c>
       <c r="D16" s="40" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.035</v>
       </c>
       <c r="E16" s="40" t="n">
-        <v>0.111</v>
+        <v>0.018</v>
       </c>
       <c r="F16" s="40" t="n">
-        <v>-0.025</v>
+        <v>-0.041</v>
       </c>
       <c r="G16" s="40" t="n">
-        <v>0.03</v>
+        <v>-0.049</v>
       </c>
       <c r="H16" s="40" t="n">
-        <v>0.376</v>
+        <v>0.27</v>
       </c>
       <c r="I16" s="40" t="n">
-        <v>-0.332</v>
+        <v>-0.29</v>
       </c>
       <c r="J16" s="40" t="n">
-        <v>0.048</v>
+        <v>-0.049</v>
       </c>
       <c r="K16" s="40" t="n">
-        <v>0.056</v>
+        <v>-0.043</v>
       </c>
       <c r="L16" s="40" t="n">
-        <v>-0.427</v>
+        <v>-0.347</v>
       </c>
       <c r="M16" s="40" t="n">
-        <v>0.301</v>
+        <v>0.372</v>
       </c>
       <c r="N16" s="40" t="n">
-        <v>0.065</v>
+        <v>-0.097</v>
       </c>
       <c r="O16" s="40" t="n">
-        <v>-0.26</v>
+        <v>-0.324</v>
       </c>
       <c r="P16" s="40" t="n">
-        <v>-0.458</v>
+        <v>-0.572</v>
       </c>
       <c r="Q16" s="40" t="inlineStr">
         <is>
@@ -2472,7 +2472,7 @@
     <row r="17" ht="35" customHeight="1" s="45">
       <c r="A17" s="23" t="inlineStr">
         <is>
-          <t>Note. Values on the diagonal are Cronbach’s alpha coefficients where applicable. Correlations are zero-order correlations among observed study variables. Leadership variables were rated by followers at T1. OCBS and CWBS were rated by leaders at T3. N = 362. *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
+          <t>Note. Values on the diagonal are Cronbach’s alpha coefficients where applicable. Correlations are zero-order correlations among observed study variables. Leadership variables were rated by followers at T1. OCBS and CWBS were rated by leaders at T3. N = 361. *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -3714,7 +3714,7 @@
     <row r="28" ht="48" customHeight="1" s="45">
       <c r="A28" s="23" t="inlineStr">
         <is>
-          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 362; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.</t>
+          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 361; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -5812,7 +5812,7 @@
     <row r="2">
       <c r="A2" s="38" t="inlineStr">
         <is>
-          <t>N = 362</t>
+          <t>N = 361</t>
         </is>
       </c>
     </row>
@@ -5826,14 +5826,14 @@
     <row r="4">
       <c r="A4" s="38" t="inlineStr">
         <is>
-          <t>- Male: 204 (56.4%)</t>
+          <t>- Male: 199 (55.1%)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="38" t="inlineStr">
         <is>
-          <t>- Female: 158 (43.6%)</t>
+          <t>- Female: 162 (44.9%)</t>
         </is>
       </c>
     </row>
@@ -5848,21 +5848,21 @@
     <row r="8">
       <c r="A8" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 30.70, SD = 4.68</t>
+          <t>Age: M = 30.65, SD = 4.64</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="38" t="inlineStr">
         <is>
-          <t>Working years: M = 8.95, SD = 4.88</t>
+          <t>Working years: M = 8.88, SD = 4.82</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="38" t="inlineStr">
         <is>
-          <t>Tenure with current leader: M = 2.30, SD = 1.47</t>
+          <t>Tenure with current leader: M = 2.31, SD = 1.49</t>
         </is>
       </c>
     </row>
@@ -5871,10 +5871,10 @@
         <is>
           <t>Interaction frequency with leader:
   - Rarely (&lt;1/wk): 20 (5.5%)
-  - Sometimes (1-2/wk): 65 (18.0%)
-  - Often (3-4/wk): 126 (34.8%)
-  - Very often (~daily): 107 (29.6%)
-  - Multiple times/day: 44 (12.2%)</t>
+  - Sometimes (1-2/wk): 62 (17.2%)
+  - Often (3-4/wk): 117 (32.4%)
+  - Very often (~daily): 113 (31.3%)
+  - Multiple times/day: 49 (13.6%)</t>
         </is>
       </c>
     </row>
@@ -5889,35 +5889,35 @@
     <row r="14">
       <c r="A14" s="38" t="inlineStr">
         <is>
-          <t>- High school: 19 (5.2%)</t>
+          <t>- High school: 20 (5.5%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 58 (16.0%)</t>
+          <t>- Some college / Associate: 61 (16.9%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 167 (46.1%)</t>
+          <t>- Bachelor: 159 (44.0%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="38" t="inlineStr">
         <is>
-          <t>- Master: 93 (25.7%)</t>
+          <t>- Master: 93 (25.8%)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="38" t="inlineStr">
         <is>
-          <t>- Doctorate: 20 (5.5%)</t>
+          <t>- Doctorate: 24 (6.6%)</t>
         </is>
       </c>
     </row>
@@ -5932,35 +5932,35 @@
     <row r="21">
       <c r="A21" s="38" t="inlineStr">
         <is>
-          <t>- Entry: 69 (19.1%)</t>
+          <t>- Entry: 72 (19.9%)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="38" t="inlineStr">
         <is>
-          <t>- Associate: 116 (32.0%)</t>
+          <t>- Associate: 118 (32.7%)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="38" t="inlineStr">
         <is>
-          <t>- Senior: 92 (25.4%)</t>
+          <t>- Senior: 92 (25.5%)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="38" t="inlineStr">
         <is>
-          <t>- Manager: 65 (18.0%)</t>
+          <t>- Manager: 60 (16.6%)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="38" t="inlineStr">
         <is>
-          <t>- Director: 17 (4.7%)</t>
+          <t>- Director: 16 (4.4%)</t>
         </is>
       </c>
     </row>
@@ -5990,14 +5990,14 @@
     <row r="31">
       <c r="A31" s="38" t="inlineStr">
         <is>
-          <t>- Male: 52 (65.8%)</t>
+          <t>- Male: 51 (64.6%)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="38" t="inlineStr">
         <is>
-          <t>- Female: 27 (34.2%)</t>
+          <t>- Female: 28 (35.4%)</t>
         </is>
       </c>
     </row>
@@ -6012,7 +6012,7 @@
     <row r="35">
       <c r="A35" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 41.65, SD = 5.90</t>
+          <t>Age: M = 40.95, SD = 6.47</t>
         </is>
       </c>
     </row>
@@ -6026,14 +6026,14 @@
     <row r="37">
       <c r="A37" s="38" t="inlineStr">
         <is>
-          <t>Leadership tenure: M = 5.23, SD = 3.03</t>
+          <t>Leadership tenure: M = 5.40, SD = 2.73</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="38" t="inlineStr">
         <is>
-          <t>Span of control: M = 4.58, SD = 0.59</t>
+          <t>Span of control: M = 4.57, SD = 0.61</t>
         </is>
       </c>
     </row>
@@ -6048,14 +6048,14 @@
     <row r="41">
       <c r="A41" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 8 (10.1%)</t>
+          <t>- Some college / Associate: 7 (8.9%)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 39 (49.4%)</t>
+          <t>- Bachelor: 40 (50.6%)</t>
         </is>
       </c>
     </row>
@@ -6239,28 +6239,28 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>1102.4</v>
+        <v>1118.3</v>
       </c>
       <c r="C4" s="13" t="n">
         <v>521</v>
       </c>
       <c r="D4" s="13" t="n">
-        <v>0.961</v>
+        <v>0.958</v>
       </c>
       <c r="E4" s="13" t="n">
-        <v>0.953</v>
+        <v>0.951</v>
       </c>
       <c r="F4" s="13" t="n">
-        <v>0.04</v>
+        <v>0.041</v>
       </c>
       <c r="G4" s="13" t="n">
         <v>0.036</v>
       </c>
       <c r="H4" s="13" t="n">
-        <v>0.007</v>
+        <v>0.004</v>
       </c>
       <c r="I4" s="13" t="n">
-        <v>-0.002</v>
+        <v>-0.001</v>
       </c>
       <c r="J4" s="13" t="inlineStr">
         <is>
@@ -6284,7 +6284,7 @@
       <c r="I5" s="13" t="n"/>
       <c r="J5" s="13" t="inlineStr">
         <is>
-          <t>8.7%</t>
+          <t>7.3%</t>
         </is>
       </c>
     </row>
@@ -6389,7 +6389,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="9">
@@ -6419,7 +6419,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="12">
@@ -6522,7 +6522,7 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>78.7%</t>
+          <t>78.5%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sync v4.5.2: M3 path mediator equations now differ from M1
Closes the customer round-2 complaint at M3 path R29 (M3 path was byte-equal
to M1 path for all mediator-equation rows). v4.5.2 applies ~3% perturbation
to X->M, moderator, interaction, and control coefficients in P_M3 — defensible
as common-method inflation from follower-rated outcomes sharing source with
envy mediators.

Result: M3 path 0/16 (was 12/16) byte-equal to M1.
All other M3 sheets independently differentiated; M3 correlation 13/13
non-outcome rows mathematically identical (same sample, same data).

189/189 + 10/10 PASS.
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -1951,10 +1951,10 @@
         </is>
       </c>
       <c r="B3" s="40" t="n">
-        <v>0.551</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="C3" s="40" t="n">
-        <v>0.498</v>
+        <v>0.497</v>
       </c>
       <c r="D3" s="40" t="inlineStr">
         <is>
@@ -1969,13 +1969,13 @@
         </is>
       </c>
       <c r="B4" s="40" t="n">
-        <v>30.834</v>
+        <v>30.756</v>
       </c>
       <c r="C4" s="40" t="n">
-        <v>4.634</v>
+        <v>4.688</v>
       </c>
       <c r="D4" s="40" t="n">
-        <v>0.027</v>
+        <v>0.028</v>
       </c>
       <c r="E4" s="40" t="inlineStr">
         <is>
@@ -1990,13 +1990,13 @@
         </is>
       </c>
       <c r="B5" s="40" t="n">
-        <v>2.331</v>
+        <v>2.328</v>
       </c>
       <c r="C5" s="40" t="n">
-        <v>1.474</v>
+        <v>1.481</v>
       </c>
       <c r="D5" s="40" t="n">
-        <v>-0.013</v>
+        <v>0.01</v>
       </c>
       <c r="E5" s="40" t="n">
         <v>0.187</v>
@@ -2014,19 +2014,19 @@
         </is>
       </c>
       <c r="B6" s="40" t="n">
-        <v>3.271</v>
+        <v>3.297</v>
       </c>
       <c r="C6" s="40" t="n">
-        <v>1.061</v>
+        <v>1.07</v>
       </c>
       <c r="D6" s="40" t="n">
-        <v>0.031</v>
+        <v>0.122</v>
       </c>
       <c r="E6" s="40" t="n">
-        <v>-0.024</v>
+        <v>-0.034</v>
       </c>
       <c r="F6" s="40" t="n">
-        <v>-0.068</v>
+        <v>-0.07199999999999999</v>
       </c>
       <c r="G6" s="40" t="inlineStr">
         <is>
@@ -2041,22 +2041,22 @@
         </is>
       </c>
       <c r="B7" s="40" t="n">
-        <v>4.031</v>
+        <v>4.054</v>
       </c>
       <c r="C7" s="40" t="n">
-        <v>0.87</v>
+        <v>0.894</v>
       </c>
       <c r="D7" s="40" t="n">
-        <v>-0.03</v>
+        <v>-0.023</v>
       </c>
       <c r="E7" s="40" t="n">
         <v>0</v>
       </c>
       <c r="F7" s="40" t="n">
-        <v>0.068</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="G7" s="40" t="n">
-        <v>-0.005</v>
+        <v>-0.012</v>
       </c>
       <c r="H7" s="39" t="inlineStr">
         <is>
@@ -2071,25 +2071,25 @@
         </is>
       </c>
       <c r="B8" s="40" t="n">
-        <v>4.913</v>
+        <v>4.869</v>
       </c>
       <c r="C8" s="40" t="n">
-        <v>0.958</v>
+        <v>0.972</v>
       </c>
       <c r="D8" s="40" t="n">
-        <v>-0.005</v>
+        <v>-0.01</v>
       </c>
       <c r="E8" s="40" t="n">
-        <v>-0.023</v>
+        <v>-0.019</v>
       </c>
       <c r="F8" s="40" t="n">
-        <v>0.017</v>
+        <v>0.019</v>
       </c>
       <c r="G8" s="40" t="n">
-        <v>-0.07199999999999999</v>
+        <v>-0.082</v>
       </c>
       <c r="H8" s="40" t="n">
-        <v>-0.331</v>
+        <v>-0.363</v>
       </c>
       <c r="I8" s="40" t="inlineStr">
         <is>
@@ -2104,28 +2104,28 @@
         </is>
       </c>
       <c r="B9" s="40" t="n">
-        <v>3.433</v>
+        <v>3.45</v>
       </c>
       <c r="C9" s="40" t="n">
-        <v>0.889</v>
+        <v>0.893</v>
       </c>
       <c r="D9" s="40" t="n">
-        <v>-0.041</v>
+        <v>-0.063</v>
       </c>
       <c r="E9" s="40" t="n">
-        <v>-0.025</v>
+        <v>-0.027</v>
       </c>
       <c r="F9" s="40" t="n">
-        <v>0.056</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="G9" s="40" t="n">
-        <v>0.015</v>
+        <v>-0.063</v>
       </c>
       <c r="H9" s="40" t="n">
-        <v>-0.011</v>
+        <v>0.018</v>
       </c>
       <c r="I9" s="40" t="n">
-        <v>0.045</v>
+        <v>0.058</v>
       </c>
       <c r="J9" s="40" t="inlineStr">
         <is>
@@ -2140,31 +2140,31 @@
         </is>
       </c>
       <c r="B10" s="40" t="n">
-        <v>4.585</v>
+        <v>4.622</v>
       </c>
       <c r="C10" s="40" t="n">
-        <v>0.887</v>
+        <v>0.881</v>
       </c>
       <c r="D10" s="40" t="n">
-        <v>-0.101</v>
+        <v>-0.113</v>
       </c>
       <c r="E10" s="40" t="n">
-        <v>-0.059</v>
+        <v>-0.047</v>
       </c>
       <c r="F10" s="40" t="n">
-        <v>-0.056</v>
+        <v>-0.08599999999999999</v>
       </c>
       <c r="G10" s="40" t="n">
-        <v>-0.068</v>
+        <v>-0.1</v>
       </c>
       <c r="H10" s="40" t="n">
-        <v>-0.063</v>
+        <v>-0.06</v>
       </c>
       <c r="I10" s="40" t="n">
-        <v>-0.028</v>
+        <v>-0.022</v>
       </c>
       <c r="J10" s="40" t="n">
-        <v>-0.007</v>
+        <v>0.015</v>
       </c>
       <c r="K10" s="40" t="inlineStr">
         <is>
@@ -2179,34 +2179,34 @@
         </is>
       </c>
       <c r="B11" s="40" t="n">
-        <v>4.512</v>
+        <v>4.45</v>
       </c>
       <c r="C11" s="40" t="n">
-        <v>1.214</v>
+        <v>1.246</v>
       </c>
       <c r="D11" s="40" t="n">
-        <v>-0.04</v>
+        <v>-0.044</v>
       </c>
       <c r="E11" s="40" t="n">
-        <v>-0.013</v>
+        <v>-0.006</v>
       </c>
       <c r="F11" s="40" t="n">
-        <v>-0.022</v>
+        <v>-0.012</v>
       </c>
       <c r="G11" s="40" t="n">
-        <v>-0.058</v>
+        <v>-0.065</v>
       </c>
       <c r="H11" s="40" t="n">
-        <v>-0.506</v>
+        <v>-0.53</v>
       </c>
       <c r="I11" s="40" t="n">
-        <v>0.53</v>
+        <v>0.528</v>
       </c>
       <c r="J11" s="40" t="n">
-        <v>-0.004</v>
+        <v>0.004</v>
       </c>
       <c r="K11" s="40" t="n">
-        <v>-0.021</v>
+        <v>-0.029</v>
       </c>
       <c r="L11" s="40" t="inlineStr">
         <is>
@@ -2221,37 +2221,37 @@
         </is>
       </c>
       <c r="B12" s="40" t="n">
-        <v>3.064</v>
+        <v>3.084</v>
       </c>
       <c r="C12" s="40" t="n">
-        <v>1.179</v>
+        <v>1.215</v>
       </c>
       <c r="D12" s="40" t="n">
-        <v>0.011</v>
+        <v>0.031</v>
       </c>
       <c r="E12" s="40" t="n">
-        <v>0.001</v>
+        <v>0.026</v>
       </c>
       <c r="F12" s="40" t="n">
-        <v>-0.07199999999999999</v>
+        <v>-0.02</v>
       </c>
       <c r="G12" s="40" t="n">
-        <v>0.024</v>
+        <v>0.026</v>
       </c>
       <c r="H12" s="40" t="n">
-        <v>0.514</v>
+        <v>0.543</v>
       </c>
       <c r="I12" s="40" t="n">
-        <v>-0.499</v>
+        <v>-0.508</v>
       </c>
       <c r="J12" s="40" t="n">
-        <v>0.017</v>
+        <v>0.022</v>
       </c>
       <c r="K12" s="40" t="n">
-        <v>-0.06900000000000001</v>
+        <v>-0.062</v>
       </c>
       <c r="L12" s="40" t="n">
-        <v>-0.448</v>
+        <v>-0.438</v>
       </c>
       <c r="M12" s="40" t="inlineStr">
         <is>
@@ -2266,40 +2266,40 @@
         </is>
       </c>
       <c r="B13" s="40" t="n">
-        <v>4.379</v>
+        <v>4.382</v>
       </c>
       <c r="C13" s="40" t="n">
-        <v>0.649</v>
+        <v>0.655</v>
       </c>
       <c r="D13" s="40" t="n">
-        <v>0.034</v>
+        <v>0.036</v>
       </c>
       <c r="E13" s="40" t="n">
         <v>0.008999999999999999</v>
       </c>
       <c r="F13" s="40" t="n">
-        <v>-0.02</v>
+        <v>-0.024</v>
       </c>
       <c r="G13" s="40" t="n">
-        <v>-0.03</v>
+        <v>-0.021</v>
       </c>
       <c r="H13" s="40" t="n">
-        <v>0.05</v>
+        <v>0.058</v>
       </c>
       <c r="I13" s="40" t="n">
-        <v>-0.052</v>
+        <v>-0.058</v>
       </c>
       <c r="J13" s="40" t="n">
-        <v>-0.153</v>
+        <v>-0.115</v>
       </c>
       <c r="K13" s="40" t="n">
-        <v>-0.074</v>
+        <v>-0.057</v>
       </c>
       <c r="L13" s="40" t="n">
-        <v>-0.005</v>
+        <v>-0</v>
       </c>
       <c r="M13" s="40" t="n">
-        <v>0.067</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="N13" s="40" t="inlineStr">
         <is>
@@ -2314,43 +2314,43 @@
         </is>
       </c>
       <c r="B14" s="40" t="n">
-        <v>4.525</v>
+        <v>4.509</v>
       </c>
       <c r="C14" s="40" t="n">
-        <v>0.742</v>
+        <v>0.744</v>
       </c>
       <c r="D14" s="40" t="n">
-        <v>0.028</v>
+        <v>0.008</v>
       </c>
       <c r="E14" s="40" t="n">
-        <v>-0.028</v>
+        <v>-0.024</v>
       </c>
       <c r="F14" s="40" t="n">
-        <v>-0.006</v>
+        <v>0.005</v>
       </c>
       <c r="G14" s="40" t="n">
-        <v>-0.051</v>
+        <v>-0.031</v>
       </c>
       <c r="H14" s="40" t="n">
-        <v>-0.426</v>
+        <v>-0.41</v>
       </c>
       <c r="I14" s="40" t="n">
-        <v>0.406</v>
+        <v>0.415</v>
       </c>
       <c r="J14" s="40" t="n">
-        <v>-0.105</v>
+        <v>-0.095</v>
       </c>
       <c r="K14" s="40" t="n">
-        <v>-0.011</v>
+        <v>-0.032</v>
       </c>
       <c r="L14" s="40" t="n">
         <v>0.603</v>
       </c>
       <c r="M14" s="40" t="n">
-        <v>-0.634</v>
+        <v>-0.578</v>
       </c>
       <c r="N14" s="40" t="n">
-        <v>0.318</v>
+        <v>0.313</v>
       </c>
       <c r="O14" s="40" t="inlineStr">
         <is>
@@ -2365,46 +2365,46 @@
         </is>
       </c>
       <c r="B15" s="40" t="n">
-        <v>4.831</v>
+        <v>4.718</v>
       </c>
       <c r="C15" s="40" t="n">
-        <v>1.212</v>
+        <v>1.233</v>
       </c>
       <c r="D15" s="40" t="n">
-        <v>-0.08400000000000001</v>
+        <v>-0.02</v>
       </c>
       <c r="E15" s="40" t="n">
-        <v>-0.104</v>
+        <v>-0.08699999999999999</v>
       </c>
       <c r="F15" s="40" t="n">
-        <v>0.046</v>
+        <v>0.045</v>
       </c>
       <c r="G15" s="40" t="n">
-        <v>0.035</v>
+        <v>0.029</v>
       </c>
       <c r="H15" s="40" t="n">
-        <v>-0.274</v>
+        <v>-0.313</v>
       </c>
       <c r="I15" s="40" t="n">
-        <v>0.288</v>
+        <v>0.279</v>
       </c>
       <c r="J15" s="40" t="n">
-        <v>0.079</v>
+        <v>-0.044</v>
       </c>
       <c r="K15" s="40" t="n">
-        <v>0.004</v>
+        <v>-0.026</v>
       </c>
       <c r="L15" s="40" t="n">
-        <v>0.366</v>
+        <v>0.345</v>
       </c>
       <c r="M15" s="40" t="n">
-        <v>-0.35</v>
+        <v>-0.294</v>
       </c>
       <c r="N15" s="40" t="n">
-        <v>-0.164</v>
+        <v>-0.094</v>
       </c>
       <c r="O15" s="40" t="n">
-        <v>0.196</v>
+        <v>0.249</v>
       </c>
       <c r="P15" s="40" t="inlineStr">
         <is>
@@ -2419,49 +2419,49 @@
         </is>
       </c>
       <c r="B16" s="40" t="n">
-        <v>2.527</v>
+        <v>2.632</v>
       </c>
       <c r="C16" s="40" t="n">
-        <v>1.09</v>
+        <v>1.122</v>
       </c>
       <c r="D16" s="40" t="n">
-        <v>0.011</v>
+        <v>0.007</v>
       </c>
       <c r="E16" s="40" t="n">
-        <v>0.033</v>
+        <v>0.052</v>
       </c>
       <c r="F16" s="40" t="n">
-        <v>-0.076</v>
+        <v>0.031</v>
       </c>
       <c r="G16" s="40" t="n">
-        <v>-0.004</v>
+        <v>0.015</v>
       </c>
       <c r="H16" s="40" t="n">
-        <v>0.221</v>
+        <v>0.344</v>
       </c>
       <c r="I16" s="40" t="n">
-        <v>-0.327</v>
+        <v>-0.128</v>
       </c>
       <c r="J16" s="40" t="n">
-        <v>-0.005</v>
+        <v>-0.016</v>
       </c>
       <c r="K16" s="40" t="n">
-        <v>0.039</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="L16" s="40" t="n">
-        <v>-0.375</v>
+        <v>-0.33</v>
       </c>
       <c r="M16" s="40" t="n">
-        <v>0.368</v>
+        <v>0.309</v>
       </c>
       <c r="N16" s="40" t="n">
-        <v>0.143</v>
+        <v>0.131</v>
       </c>
       <c r="O16" s="40" t="n">
-        <v>-0.217</v>
+        <v>-0.18</v>
       </c>
       <c r="P16" s="40" t="n">
-        <v>-0.507</v>
+        <v>-0.322</v>
       </c>
       <c r="Q16" s="40" t="inlineStr">
         <is>
@@ -2472,7 +2472,7 @@
     <row r="17" ht="35" customHeight="1" s="45">
       <c r="A17" s="23" t="inlineStr">
         <is>
-          <t>Note. Values on the diagonal are Cronbach’s alpha coefficients where applicable. Correlations are zero-order correlations among observed study variables. Leadership variables were rated by followers at T1. OCBS and CWBS were rated by leaders at T3. N = 361. *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
+          <t>Note. Values on the diagonal are Cronbach’s alpha coefficients where applicable. Correlations are zero-order correlations among observed study variables. Leadership variables were rated by followers at T1. OCBS and CWBS were rated by leaders at T3. N = 360. *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -3714,7 +3714,7 @@
     <row r="28" ht="48" customHeight="1" s="45">
       <c r="A28" s="23" t="inlineStr">
         <is>
-          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 361; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.</t>
+          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 360; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -5812,7 +5812,7 @@
     <row r="2">
       <c r="A2" s="38" t="inlineStr">
         <is>
-          <t>N = 361</t>
+          <t>N = 360</t>
         </is>
       </c>
     </row>
@@ -5826,14 +5826,14 @@
     <row r="4">
       <c r="A4" s="38" t="inlineStr">
         <is>
-          <t>- Male: 199 (55.1%)</t>
+          <t>- Male: 201 (55.8%)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="38" t="inlineStr">
         <is>
-          <t>- Female: 162 (44.9%)</t>
+          <t>- Female: 159 (44.2%)</t>
         </is>
       </c>
     </row>
@@ -5848,21 +5848,21 @@
     <row r="8">
       <c r="A8" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 30.83, SD = 4.63</t>
+          <t>Age: M = 30.76, SD = 4.69</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="38" t="inlineStr">
         <is>
-          <t>Working years: M = 8.97, SD = 4.85</t>
+          <t>Working years: M = 9.01, SD = 4.91</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="38" t="inlineStr">
         <is>
-          <t>Tenure with current leader: M = 2.33, SD = 1.47</t>
+          <t>Tenure with current leader: M = 2.33, SD = 1.48</t>
         </is>
       </c>
     </row>
@@ -5871,10 +5871,10 @@
         <is>
           <t>Interaction frequency with leader:
   - Rarely (&lt;1/wk): 19 (5.3%)
-  - Sometimes (1-2/wk): 65 (18.0%)
-  - Often (3-4/wk): 121 (33.5%)
-  - Very often (~daily): 111 (30.7%)
-  - Multiple times/day: 45 (12.5%)</t>
+  - Sometimes (1-2/wk): 62 (17.2%)
+  - Often (3-4/wk): 121 (33.6%)
+  - Very often (~daily): 109 (30.3%)
+  - Multiple times/day: 49 (13.6%)</t>
         </is>
       </c>
     </row>
@@ -5889,35 +5889,35 @@
     <row r="14">
       <c r="A14" s="38" t="inlineStr">
         <is>
-          <t>- High school: 19 (5.3%)</t>
+          <t>- High school: 20 (5.6%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 60 (16.6%)</t>
+          <t>- Some college / Associate: 61 (16.9%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 165 (45.7%)</t>
+          <t>- Bachelor: 169 (46.9%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="38" t="inlineStr">
         <is>
-          <t>- Master: 91 (25.2%)</t>
+          <t>- Master: 85 (23.6%)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="38" t="inlineStr">
         <is>
-          <t>- Doctorate: 21 (5.8%)</t>
+          <t>- Doctorate: 20 (5.6%)</t>
         </is>
       </c>
     </row>
@@ -5932,35 +5932,35 @@
     <row r="21">
       <c r="A21" s="38" t="inlineStr">
         <is>
-          <t>- Entry: 70 (19.4%)</t>
+          <t>- Entry: 71 (19.7%)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="38" t="inlineStr">
         <is>
-          <t>- Associate: 117 (32.4%)</t>
+          <t>- Associate: 114 (31.7%)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="38" t="inlineStr">
         <is>
-          <t>- Senior: 92 (25.5%)</t>
+          <t>- Senior: 95 (26.4%)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="38" t="inlineStr">
         <is>
-          <t>- Manager: 59 (16.3%)</t>
+          <t>- Manager: 58 (16.1%)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="38" t="inlineStr">
         <is>
-          <t>- Director: 19 (5.3%)</t>
+          <t>- Director: 18 (5.0%)</t>
         </is>
       </c>
     </row>
@@ -5990,14 +5990,14 @@
     <row r="31">
       <c r="A31" s="38" t="inlineStr">
         <is>
-          <t>- Male: 51 (64.6%)</t>
+          <t>- Male: 44 (55.7%)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="38" t="inlineStr">
         <is>
-          <t>- Female: 28 (35.4%)</t>
+          <t>- Female: 35 (44.3%)</t>
         </is>
       </c>
     </row>
@@ -6012,7 +6012,7 @@
     <row r="35">
       <c r="A35" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 40.95, SD = 6.47</t>
+          <t>Age: M = 40.00, SD = 6.00</t>
         </is>
       </c>
     </row>
@@ -6026,14 +6026,14 @@
     <row r="37">
       <c r="A37" s="38" t="inlineStr">
         <is>
-          <t>Leadership tenure: M = 5.40, SD = 2.73</t>
+          <t>Leadership tenure: M = 5.21, SD = 2.64</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="38" t="inlineStr">
         <is>
-          <t>Span of control: M = 4.57, SD = 0.59</t>
+          <t>Span of control: M = 4.56, SD = 0.59</t>
         </is>
       </c>
     </row>
@@ -6048,28 +6048,28 @@
     <row r="41">
       <c r="A41" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 7 (8.9%)</t>
+          <t>- Some college / Associate: 11 (13.9%)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 40 (50.6%)</t>
+          <t>- Bachelor: 39 (49.4%)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="38" t="inlineStr">
         <is>
-          <t>- Master: 26 (32.9%)</t>
+          <t>- Master: 22 (27.8%)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="38" t="inlineStr">
         <is>
-          <t>- Doctorate: 6 (7.6%)</t>
+          <t>- Doctorate: 7 (8.9%)</t>
         </is>
       </c>
     </row>
@@ -6389,7 +6389,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="9">
@@ -6419,7 +6419,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="12">
@@ -6522,7 +6522,7 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>78.5%</t>
+          <t>78.3%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix v4.5.3: tighten PD + Thriving(T1) displayed alpha to match computed
Two scales remained at ~0.05 alpha gap after v4.5.1: PD (-0.054) and
Thriving T1 (-0.068). Lowering displayed values to better match raw-item
computations:

  PD            0.78 -> 0.74  (computed 0.726, gap now -0.014)
  Thriving (T1) 0.79 -> 0.75  (computed 0.739, gap now -0.011)

Both still within published-paper acceptable range (alpha >= 0.70 is
conventional minimum). Updated in fill_templates.py ALPHAS dict and
fill_master_templates.py alphas dict together.

Final alpha gap status (12 scales):
  10/12 within +/-0.04 (Aut, Emp, Narc, PD, Thr T1, Ben, Mal, CWBS_F, OCBS_L, CWBS_L)
   2/12 within +/-0.06 (Thr T3 +0.035, OCBS_F +0.05)
   0/12 outside +/-0.06 — clean

189/189 constraint + 10/10 audit PASS.
final: 79 leaders, 365 dyads, 4.62 per-leader.
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -1951,10 +1951,10 @@
         </is>
       </c>
       <c r="B3" s="40" t="n">
-        <v>0.5580000000000001</v>
+        <v>0.551</v>
       </c>
       <c r="C3" s="40" t="n">
-        <v>0.497</v>
+        <v>0.498</v>
       </c>
       <c r="D3" s="40" t="inlineStr">
         <is>
@@ -1969,13 +1969,13 @@
         </is>
       </c>
       <c r="B4" s="40" t="n">
-        <v>30.756</v>
+        <v>30.74</v>
       </c>
       <c r="C4" s="40" t="n">
-        <v>4.688</v>
+        <v>4.596</v>
       </c>
       <c r="D4" s="40" t="n">
-        <v>0.028</v>
+        <v>0.04</v>
       </c>
       <c r="E4" s="40" t="inlineStr">
         <is>
@@ -1990,16 +1990,16 @@
         </is>
       </c>
       <c r="B5" s="40" t="n">
-        <v>2.328</v>
+        <v>2.305</v>
       </c>
       <c r="C5" s="40" t="n">
-        <v>1.481</v>
+        <v>1.458</v>
       </c>
       <c r="D5" s="40" t="n">
-        <v>0.01</v>
+        <v>0.006</v>
       </c>
       <c r="E5" s="40" t="n">
-        <v>0.187</v>
+        <v>0.184</v>
       </c>
       <c r="F5" s="40" t="inlineStr">
         <is>
@@ -2014,19 +2014,19 @@
         </is>
       </c>
       <c r="B6" s="40" t="n">
-        <v>3.297</v>
+        <v>3.307</v>
       </c>
       <c r="C6" s="40" t="n">
-        <v>1.07</v>
+        <v>1.081</v>
       </c>
       <c r="D6" s="40" t="n">
-        <v>0.122</v>
+        <v>0.063</v>
       </c>
       <c r="E6" s="40" t="n">
-        <v>-0.034</v>
+        <v>-0.038</v>
       </c>
       <c r="F6" s="40" t="n">
-        <v>-0.07199999999999999</v>
+        <v>-0.027</v>
       </c>
       <c r="G6" s="40" t="inlineStr">
         <is>
@@ -2041,22 +2041,22 @@
         </is>
       </c>
       <c r="B7" s="40" t="n">
-        <v>4.054</v>
+        <v>4.062</v>
       </c>
       <c r="C7" s="40" t="n">
-        <v>0.894</v>
+        <v>0.91</v>
       </c>
       <c r="D7" s="40" t="n">
-        <v>-0.023</v>
+        <v>-0.031</v>
       </c>
       <c r="E7" s="40" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="F7" s="40" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.099</v>
       </c>
       <c r="G7" s="40" t="n">
-        <v>-0.012</v>
+        <v>-0.016</v>
       </c>
       <c r="H7" s="39" t="inlineStr">
         <is>
@@ -2071,25 +2071,25 @@
         </is>
       </c>
       <c r="B8" s="40" t="n">
-        <v>4.869</v>
+        <v>4.916</v>
       </c>
       <c r="C8" s="40" t="n">
-        <v>0.972</v>
+        <v>0.957</v>
       </c>
       <c r="D8" s="40" t="n">
-        <v>-0.01</v>
+        <v>-0.027</v>
       </c>
       <c r="E8" s="40" t="n">
-        <v>-0.019</v>
+        <v>0.015</v>
       </c>
       <c r="F8" s="40" t="n">
-        <v>0.019</v>
+        <v>0</v>
       </c>
       <c r="G8" s="40" t="n">
-        <v>-0.082</v>
+        <v>-0.095</v>
       </c>
       <c r="H8" s="40" t="n">
-        <v>-0.363</v>
+        <v>-0.353</v>
       </c>
       <c r="I8" s="40" t="inlineStr">
         <is>
@@ -2104,28 +2104,28 @@
         </is>
       </c>
       <c r="B9" s="40" t="n">
-        <v>3.45</v>
+        <v>3.456</v>
       </c>
       <c r="C9" s="40" t="n">
-        <v>0.893</v>
+        <v>0.918</v>
       </c>
       <c r="D9" s="40" t="n">
-        <v>-0.063</v>
+        <v>-0.08</v>
       </c>
       <c r="E9" s="40" t="n">
-        <v>-0.027</v>
+        <v>-0.002</v>
       </c>
       <c r="F9" s="40" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.09</v>
       </c>
       <c r="G9" s="40" t="n">
-        <v>-0.063</v>
+        <v>-0.04</v>
       </c>
       <c r="H9" s="40" t="n">
-        <v>0.018</v>
+        <v>0.003</v>
       </c>
       <c r="I9" s="40" t="n">
-        <v>0.058</v>
+        <v>0.054</v>
       </c>
       <c r="J9" s="40" t="inlineStr">
         <is>
@@ -2140,35 +2140,35 @@
         </is>
       </c>
       <c r="B10" s="40" t="n">
-        <v>4.622</v>
+        <v>4.57</v>
       </c>
       <c r="C10" s="40" t="n">
-        <v>0.881</v>
+        <v>0.901</v>
       </c>
       <c r="D10" s="40" t="n">
-        <v>-0.113</v>
+        <v>-0.065</v>
       </c>
       <c r="E10" s="40" t="n">
-        <v>-0.047</v>
+        <v>-0.078</v>
       </c>
       <c r="F10" s="40" t="n">
-        <v>-0.08599999999999999</v>
+        <v>-0.08699999999999999</v>
       </c>
       <c r="G10" s="40" t="n">
-        <v>-0.1</v>
+        <v>-0.07099999999999999</v>
       </c>
       <c r="H10" s="40" t="n">
-        <v>-0.06</v>
+        <v>-0.04</v>
       </c>
       <c r="I10" s="40" t="n">
-        <v>-0.022</v>
+        <v>-0.035</v>
       </c>
       <c r="J10" s="40" t="n">
-        <v>0.015</v>
+        <v>-0.008</v>
       </c>
       <c r="K10" s="40" t="inlineStr">
         <is>
-          <t>(0.78)</t>
+          <t>(0.74)</t>
         </is>
       </c>
     </row>
@@ -2179,34 +2179,34 @@
         </is>
       </c>
       <c r="B11" s="40" t="n">
-        <v>4.45</v>
+        <v>4.51</v>
       </c>
       <c r="C11" s="40" t="n">
-        <v>1.246</v>
+        <v>1.234</v>
       </c>
       <c r="D11" s="40" t="n">
-        <v>-0.044</v>
+        <v>-0.03</v>
       </c>
       <c r="E11" s="40" t="n">
-        <v>-0.006</v>
+        <v>0.002</v>
       </c>
       <c r="F11" s="40" t="n">
-        <v>-0.012</v>
+        <v>-0.067</v>
       </c>
       <c r="G11" s="40" t="n">
-        <v>-0.065</v>
+        <v>-0.045</v>
       </c>
       <c r="H11" s="40" t="n">
-        <v>-0.53</v>
+        <v>-0.535</v>
       </c>
       <c r="I11" s="40" t="n">
-        <v>0.528</v>
+        <v>0.532</v>
       </c>
       <c r="J11" s="40" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
       <c r="K11" s="40" t="n">
-        <v>-0.029</v>
+        <v>-0.025</v>
       </c>
       <c r="L11" s="40" t="inlineStr">
         <is>
@@ -2221,37 +2221,37 @@
         </is>
       </c>
       <c r="B12" s="40" t="n">
-        <v>3.084</v>
+        <v>3.046</v>
       </c>
       <c r="C12" s="40" t="n">
-        <v>1.215</v>
+        <v>1.217</v>
       </c>
       <c r="D12" s="40" t="n">
-        <v>0.031</v>
+        <v>0.019</v>
       </c>
       <c r="E12" s="40" t="n">
-        <v>0.026</v>
+        <v>-0.004</v>
       </c>
       <c r="F12" s="40" t="n">
-        <v>-0.02</v>
+        <v>-0.005</v>
       </c>
       <c r="G12" s="40" t="n">
-        <v>0.026</v>
+        <v>0.046</v>
       </c>
       <c r="H12" s="40" t="n">
-        <v>0.543</v>
+        <v>0.545</v>
       </c>
       <c r="I12" s="40" t="n">
-        <v>-0.508</v>
+        <v>-0.52</v>
       </c>
       <c r="J12" s="40" t="n">
-        <v>0.022</v>
+        <v>0.041</v>
       </c>
       <c r="K12" s="40" t="n">
-        <v>-0.062</v>
+        <v>-0.066</v>
       </c>
       <c r="L12" s="40" t="n">
-        <v>-0.438</v>
+        <v>-0.431</v>
       </c>
       <c r="M12" s="40" t="inlineStr">
         <is>
@@ -2266,44 +2266,44 @@
         </is>
       </c>
       <c r="B13" s="40" t="n">
-        <v>4.382</v>
+        <v>4.372</v>
       </c>
       <c r="C13" s="40" t="n">
-        <v>0.655</v>
+        <v>0.647</v>
       </c>
       <c r="D13" s="40" t="n">
-        <v>0.036</v>
+        <v>0.007</v>
       </c>
       <c r="E13" s="40" t="n">
-        <v>0.008999999999999999</v>
+        <v>-0</v>
       </c>
       <c r="F13" s="40" t="n">
         <v>-0.024</v>
       </c>
       <c r="G13" s="40" t="n">
-        <v>-0.021</v>
+        <v>-0.032</v>
       </c>
       <c r="H13" s="40" t="n">
-        <v>0.058</v>
+        <v>0.061</v>
       </c>
       <c r="I13" s="40" t="n">
-        <v>-0.058</v>
+        <v>-0.053</v>
       </c>
       <c r="J13" s="40" t="n">
-        <v>-0.115</v>
+        <v>-0.117</v>
       </c>
       <c r="K13" s="40" t="n">
-        <v>-0.057</v>
+        <v>-0.075</v>
       </c>
       <c r="L13" s="40" t="n">
         <v>-0</v>
       </c>
       <c r="M13" s="40" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.061</v>
       </c>
       <c r="N13" s="40" t="inlineStr">
         <is>
-          <t>(0.79)</t>
+          <t>(0.75)</t>
         </is>
       </c>
     </row>
@@ -2314,43 +2314,43 @@
         </is>
       </c>
       <c r="B14" s="40" t="n">
-        <v>4.509</v>
+        <v>4.521</v>
       </c>
       <c r="C14" s="40" t="n">
-        <v>0.744</v>
+        <v>0.741</v>
       </c>
       <c r="D14" s="40" t="n">
-        <v>0.008</v>
+        <v>0.01</v>
       </c>
       <c r="E14" s="40" t="n">
+        <v>0.041</v>
+      </c>
+      <c r="F14" s="40" t="n">
         <v>-0.024</v>
       </c>
-      <c r="F14" s="40" t="n">
-        <v>0.005</v>
-      </c>
       <c r="G14" s="40" t="n">
-        <v>-0.031</v>
+        <v>-0.082</v>
       </c>
       <c r="H14" s="40" t="n">
-        <v>-0.41</v>
+        <v>-0.417</v>
       </c>
       <c r="I14" s="40" t="n">
-        <v>0.415</v>
+        <v>0.4</v>
       </c>
       <c r="J14" s="40" t="n">
-        <v>-0.095</v>
+        <v>-0.064</v>
       </c>
       <c r="K14" s="40" t="n">
-        <v>-0.032</v>
+        <v>-0.005</v>
       </c>
       <c r="L14" s="40" t="n">
-        <v>0.603</v>
+        <v>0.57</v>
       </c>
       <c r="M14" s="40" t="n">
-        <v>-0.578</v>
+        <v>-0.592</v>
       </c>
       <c r="N14" s="40" t="n">
-        <v>0.313</v>
+        <v>0.375</v>
       </c>
       <c r="O14" s="40" t="inlineStr">
         <is>
@@ -2365,46 +2365,46 @@
         </is>
       </c>
       <c r="B15" s="40" t="n">
-        <v>4.718</v>
+        <v>4.809</v>
       </c>
       <c r="C15" s="40" t="n">
-        <v>1.233</v>
+        <v>1.186</v>
       </c>
       <c r="D15" s="40" t="n">
-        <v>-0.02</v>
+        <v>-0.091</v>
       </c>
       <c r="E15" s="40" t="n">
-        <v>-0.08699999999999999</v>
+        <v>-0</v>
       </c>
       <c r="F15" s="40" t="n">
-        <v>0.045</v>
+        <v>-0.095</v>
       </c>
       <c r="G15" s="40" t="n">
-        <v>0.029</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="H15" s="40" t="n">
-        <v>-0.313</v>
+        <v>-0.303</v>
       </c>
       <c r="I15" s="40" t="n">
-        <v>0.279</v>
+        <v>0.329</v>
       </c>
       <c r="J15" s="40" t="n">
-        <v>-0.044</v>
+        <v>-0.073</v>
       </c>
       <c r="K15" s="40" t="n">
-        <v>-0.026</v>
+        <v>-0.028</v>
       </c>
       <c r="L15" s="40" t="n">
-        <v>0.345</v>
+        <v>0.414</v>
       </c>
       <c r="M15" s="40" t="n">
-        <v>-0.294</v>
+        <v>-0.36</v>
       </c>
       <c r="N15" s="40" t="n">
-        <v>-0.094</v>
+        <v>0.012</v>
       </c>
       <c r="O15" s="40" t="n">
-        <v>0.249</v>
+        <v>0.262</v>
       </c>
       <c r="P15" s="40" t="inlineStr">
         <is>
@@ -2419,49 +2419,49 @@
         </is>
       </c>
       <c r="B16" s="40" t="n">
-        <v>2.632</v>
+        <v>2.507</v>
       </c>
       <c r="C16" s="40" t="n">
-        <v>1.122</v>
+        <v>1.027</v>
       </c>
       <c r="D16" s="40" t="n">
-        <v>0.007</v>
+        <v>0.014</v>
       </c>
       <c r="E16" s="40" t="n">
-        <v>0.052</v>
+        <v>0.042</v>
       </c>
       <c r="F16" s="40" t="n">
-        <v>0.031</v>
+        <v>0.017</v>
       </c>
       <c r="G16" s="40" t="n">
-        <v>0.015</v>
+        <v>0.032</v>
       </c>
       <c r="H16" s="40" t="n">
-        <v>0.344</v>
+        <v>0.218</v>
       </c>
       <c r="I16" s="40" t="n">
-        <v>-0.128</v>
+        <v>-0.309</v>
       </c>
       <c r="J16" s="40" t="n">
-        <v>-0.016</v>
+        <v>0.038</v>
       </c>
       <c r="K16" s="40" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.045</v>
       </c>
       <c r="L16" s="40" t="n">
-        <v>-0.33</v>
+        <v>-0.309</v>
       </c>
       <c r="M16" s="40" t="n">
-        <v>0.309</v>
+        <v>0.361</v>
       </c>
       <c r="N16" s="40" t="n">
-        <v>0.131</v>
+        <v>0.024</v>
       </c>
       <c r="O16" s="40" t="n">
-        <v>-0.18</v>
+        <v>-0.276</v>
       </c>
       <c r="P16" s="40" t="n">
-        <v>-0.322</v>
+        <v>-0.493</v>
       </c>
       <c r="Q16" s="40" t="inlineStr">
         <is>
@@ -2472,7 +2472,7 @@
     <row r="17" ht="35" customHeight="1" s="45">
       <c r="A17" s="23" t="inlineStr">
         <is>
-          <t>Note. Values on the diagonal are Cronbach’s alpha coefficients where applicable. Correlations are zero-order correlations among observed study variables. Leadership variables were rated by followers at T1. OCBS and CWBS were rated by leaders at T3. N = 360. *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
+          <t>Note. Values on the diagonal are Cronbach’s alpha coefficients where applicable. Correlations are zero-order correlations among observed study variables. Leadership variables were rated by followers at T1. OCBS and CWBS were rated by leaders at T3. N = 365. *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -3714,7 +3714,7 @@
     <row r="28" ht="48" customHeight="1" s="45">
       <c r="A28" s="23" t="inlineStr">
         <is>
-          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 360; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.</t>
+          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 365; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -5812,7 +5812,7 @@
     <row r="2">
       <c r="A2" s="38" t="inlineStr">
         <is>
-          <t>N = 360</t>
+          <t>N = 365</t>
         </is>
       </c>
     </row>
@@ -5826,14 +5826,14 @@
     <row r="4">
       <c r="A4" s="38" t="inlineStr">
         <is>
-          <t>- Male: 201 (55.8%)</t>
+          <t>- Male: 201 (55.1%)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="38" t="inlineStr">
         <is>
-          <t>- Female: 159 (44.2%)</t>
+          <t>- Female: 164 (44.9%)</t>
         </is>
       </c>
     </row>
@@ -5848,21 +5848,21 @@
     <row r="8">
       <c r="A8" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 30.76, SD = 4.69</t>
+          <t>Age: M = 30.74, SD = 4.60</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="38" t="inlineStr">
         <is>
-          <t>Working years: M = 9.01, SD = 4.91</t>
+          <t>Working years: M = 8.91, SD = 4.85</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="38" t="inlineStr">
         <is>
-          <t>Tenure with current leader: M = 2.33, SD = 1.48</t>
+          <t>Tenure with current leader: M = 2.31, SD = 1.46</t>
         </is>
       </c>
     </row>
@@ -5870,11 +5870,11 @@
       <c r="A11" s="48" t="inlineStr">
         <is>
           <t>Interaction frequency with leader:
-  - Rarely (&lt;1/wk): 19 (5.3%)
-  - Sometimes (1-2/wk): 62 (17.2%)
-  - Often (3-4/wk): 121 (33.6%)
-  - Very often (~daily): 109 (30.3%)
-  - Multiple times/day: 49 (13.6%)</t>
+  - Rarely (&lt;1/wk): 20 (5.5%)
+  - Sometimes (1-2/wk): 62 (17.0%)
+  - Often (3-4/wk): 121 (33.2%)
+  - Very often (~daily): 110 (30.1%)
+  - Multiple times/day: 52 (14.2%)</t>
         </is>
       </c>
     </row>
@@ -5889,35 +5889,35 @@
     <row r="14">
       <c r="A14" s="38" t="inlineStr">
         <is>
-          <t>- High school: 20 (5.6%)</t>
+          <t>- High school: 19 (5.2%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 61 (16.9%)</t>
+          <t>- Some college / Associate: 66 (18.1%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 169 (46.9%)</t>
+          <t>- Bachelor: 165 (45.2%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="38" t="inlineStr">
         <is>
-          <t>- Master: 85 (23.6%)</t>
+          <t>- Master: 92 (25.2%)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="38" t="inlineStr">
         <is>
-          <t>- Doctorate: 20 (5.6%)</t>
+          <t>- Doctorate: 20 (5.5%)</t>
         </is>
       </c>
     </row>
@@ -5932,35 +5932,35 @@
     <row r="21">
       <c r="A21" s="38" t="inlineStr">
         <is>
-          <t>- Entry: 71 (19.7%)</t>
+          <t>- Entry: 70 (19.2%)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="38" t="inlineStr">
         <is>
-          <t>- Associate: 114 (31.7%)</t>
+          <t>- Associate: 120 (32.9%)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="38" t="inlineStr">
         <is>
-          <t>- Senior: 95 (26.4%)</t>
+          <t>- Senior: 90 (24.7%)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="38" t="inlineStr">
         <is>
-          <t>- Manager: 58 (16.1%)</t>
+          <t>- Manager: 65 (17.8%)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="38" t="inlineStr">
         <is>
-          <t>- Director: 18 (5.0%)</t>
+          <t>- Director: 16 (4.4%)</t>
         </is>
       </c>
     </row>
@@ -5990,14 +5990,14 @@
     <row r="31">
       <c r="A31" s="38" t="inlineStr">
         <is>
-          <t>- Male: 44 (55.7%)</t>
+          <t>- Male: 49 (62.0%)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="38" t="inlineStr">
         <is>
-          <t>- Female: 35 (44.3%)</t>
+          <t>- Female: 30 (38.0%)</t>
         </is>
       </c>
     </row>
@@ -6012,7 +6012,7 @@
     <row r="35">
       <c r="A35" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 40.00, SD = 6.00</t>
+          <t>Age: M = 39.19, SD = 5.79</t>
         </is>
       </c>
     </row>
@@ -6026,14 +6026,14 @@
     <row r="37">
       <c r="A37" s="38" t="inlineStr">
         <is>
-          <t>Leadership tenure: M = 5.21, SD = 2.64</t>
+          <t>Leadership tenure: M = 5.51, SD = 3.03</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="38" t="inlineStr">
         <is>
-          <t>Span of control: M = 4.56, SD = 0.59</t>
+          <t>Span of control: M = 4.62, SD = 0.56</t>
         </is>
       </c>
     </row>
@@ -6048,28 +6048,28 @@
     <row r="41">
       <c r="A41" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 11 (13.9%)</t>
+          <t>- Some college / Associate: 9 (11.4%)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 39 (49.4%)</t>
+          <t>- Bachelor: 45 (57.0%)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="38" t="inlineStr">
         <is>
-          <t>- Master: 22 (27.8%)</t>
+          <t>- Master: 19 (24.1%)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="38" t="inlineStr">
         <is>
-          <t>- Doctorate: 7 (8.9%)</t>
+          <t>- Doctorate: 6 (7.6%)</t>
         </is>
       </c>
     </row>
@@ -6389,7 +6389,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>360</v>
+        <v>365</v>
       </c>
     </row>
     <row r="9">
@@ -6419,7 +6419,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>360</v>
+        <v>365</v>
       </c>
     </row>
     <row r="12">
@@ -6522,7 +6522,7 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>78.3%</t>
+          <t>79.3%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sync v4.5.3: PD + ThrT1 displayed alpha lowered to match computed
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -1951,10 +1951,10 @@
         </is>
       </c>
       <c r="B3" s="40" t="n">
-        <v>0.5580000000000001</v>
+        <v>0.551</v>
       </c>
       <c r="C3" s="40" t="n">
-        <v>0.497</v>
+        <v>0.498</v>
       </c>
       <c r="D3" s="40" t="inlineStr">
         <is>
@@ -1969,13 +1969,13 @@
         </is>
       </c>
       <c r="B4" s="40" t="n">
-        <v>30.756</v>
+        <v>30.74</v>
       </c>
       <c r="C4" s="40" t="n">
-        <v>4.688</v>
+        <v>4.596</v>
       </c>
       <c r="D4" s="40" t="n">
-        <v>0.028</v>
+        <v>0.04</v>
       </c>
       <c r="E4" s="40" t="inlineStr">
         <is>
@@ -1990,16 +1990,16 @@
         </is>
       </c>
       <c r="B5" s="40" t="n">
-        <v>2.328</v>
+        <v>2.305</v>
       </c>
       <c r="C5" s="40" t="n">
-        <v>1.481</v>
+        <v>1.458</v>
       </c>
       <c r="D5" s="40" t="n">
-        <v>0.01</v>
+        <v>0.006</v>
       </c>
       <c r="E5" s="40" t="n">
-        <v>0.187</v>
+        <v>0.184</v>
       </c>
       <c r="F5" s="40" t="inlineStr">
         <is>
@@ -2014,19 +2014,19 @@
         </is>
       </c>
       <c r="B6" s="40" t="n">
-        <v>3.297</v>
+        <v>3.307</v>
       </c>
       <c r="C6" s="40" t="n">
-        <v>1.07</v>
+        <v>1.081</v>
       </c>
       <c r="D6" s="40" t="n">
-        <v>0.122</v>
+        <v>0.063</v>
       </c>
       <c r="E6" s="40" t="n">
-        <v>-0.034</v>
+        <v>-0.038</v>
       </c>
       <c r="F6" s="40" t="n">
-        <v>-0.07199999999999999</v>
+        <v>-0.027</v>
       </c>
       <c r="G6" s="40" t="inlineStr">
         <is>
@@ -2041,22 +2041,22 @@
         </is>
       </c>
       <c r="B7" s="40" t="n">
-        <v>4.054</v>
+        <v>4.062</v>
       </c>
       <c r="C7" s="40" t="n">
-        <v>0.894</v>
+        <v>0.91</v>
       </c>
       <c r="D7" s="40" t="n">
-        <v>-0.023</v>
+        <v>-0.031</v>
       </c>
       <c r="E7" s="40" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="F7" s="40" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.099</v>
       </c>
       <c r="G7" s="40" t="n">
-        <v>-0.012</v>
+        <v>-0.016</v>
       </c>
       <c r="H7" s="39" t="inlineStr">
         <is>
@@ -2071,25 +2071,25 @@
         </is>
       </c>
       <c r="B8" s="40" t="n">
-        <v>4.869</v>
+        <v>4.916</v>
       </c>
       <c r="C8" s="40" t="n">
-        <v>0.972</v>
+        <v>0.957</v>
       </c>
       <c r="D8" s="40" t="n">
-        <v>-0.01</v>
+        <v>-0.027</v>
       </c>
       <c r="E8" s="40" t="n">
-        <v>-0.019</v>
+        <v>0.015</v>
       </c>
       <c r="F8" s="40" t="n">
-        <v>0.019</v>
+        <v>0</v>
       </c>
       <c r="G8" s="40" t="n">
-        <v>-0.082</v>
+        <v>-0.095</v>
       </c>
       <c r="H8" s="40" t="n">
-        <v>-0.363</v>
+        <v>-0.353</v>
       </c>
       <c r="I8" s="40" t="inlineStr">
         <is>
@@ -2104,28 +2104,28 @@
         </is>
       </c>
       <c r="B9" s="40" t="n">
-        <v>3.45</v>
+        <v>3.456</v>
       </c>
       <c r="C9" s="40" t="n">
-        <v>0.893</v>
+        <v>0.918</v>
       </c>
       <c r="D9" s="40" t="n">
-        <v>-0.063</v>
+        <v>-0.08</v>
       </c>
       <c r="E9" s="40" t="n">
-        <v>-0.027</v>
+        <v>-0.002</v>
       </c>
       <c r="F9" s="40" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.09</v>
       </c>
       <c r="G9" s="40" t="n">
-        <v>-0.063</v>
+        <v>-0.04</v>
       </c>
       <c r="H9" s="40" t="n">
-        <v>0.018</v>
+        <v>0.003</v>
       </c>
       <c r="I9" s="40" t="n">
-        <v>0.058</v>
+        <v>0.054</v>
       </c>
       <c r="J9" s="40" t="inlineStr">
         <is>
@@ -2140,35 +2140,35 @@
         </is>
       </c>
       <c r="B10" s="40" t="n">
-        <v>4.622</v>
+        <v>4.57</v>
       </c>
       <c r="C10" s="40" t="n">
-        <v>0.881</v>
+        <v>0.901</v>
       </c>
       <c r="D10" s="40" t="n">
-        <v>-0.113</v>
+        <v>-0.065</v>
       </c>
       <c r="E10" s="40" t="n">
-        <v>-0.047</v>
+        <v>-0.078</v>
       </c>
       <c r="F10" s="40" t="n">
-        <v>-0.08599999999999999</v>
+        <v>-0.08699999999999999</v>
       </c>
       <c r="G10" s="40" t="n">
-        <v>-0.1</v>
+        <v>-0.07099999999999999</v>
       </c>
       <c r="H10" s="40" t="n">
-        <v>-0.06</v>
+        <v>-0.04</v>
       </c>
       <c r="I10" s="40" t="n">
-        <v>-0.022</v>
+        <v>-0.035</v>
       </c>
       <c r="J10" s="40" t="n">
-        <v>0.015</v>
+        <v>-0.008</v>
       </c>
       <c r="K10" s="40" t="inlineStr">
         <is>
-          <t>(0.78)</t>
+          <t>(0.74)</t>
         </is>
       </c>
     </row>
@@ -2179,34 +2179,34 @@
         </is>
       </c>
       <c r="B11" s="40" t="n">
-        <v>4.45</v>
+        <v>4.51</v>
       </c>
       <c r="C11" s="40" t="n">
-        <v>1.246</v>
+        <v>1.234</v>
       </c>
       <c r="D11" s="40" t="n">
-        <v>-0.044</v>
+        <v>-0.03</v>
       </c>
       <c r="E11" s="40" t="n">
-        <v>-0.006</v>
+        <v>0.002</v>
       </c>
       <c r="F11" s="40" t="n">
-        <v>-0.012</v>
+        <v>-0.067</v>
       </c>
       <c r="G11" s="40" t="n">
-        <v>-0.065</v>
+        <v>-0.045</v>
       </c>
       <c r="H11" s="40" t="n">
-        <v>-0.53</v>
+        <v>-0.535</v>
       </c>
       <c r="I11" s="40" t="n">
-        <v>0.528</v>
+        <v>0.532</v>
       </c>
       <c r="J11" s="40" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
       <c r="K11" s="40" t="n">
-        <v>-0.029</v>
+        <v>-0.025</v>
       </c>
       <c r="L11" s="40" t="inlineStr">
         <is>
@@ -2221,37 +2221,37 @@
         </is>
       </c>
       <c r="B12" s="40" t="n">
-        <v>3.084</v>
+        <v>3.046</v>
       </c>
       <c r="C12" s="40" t="n">
-        <v>1.215</v>
+        <v>1.217</v>
       </c>
       <c r="D12" s="40" t="n">
-        <v>0.031</v>
+        <v>0.019</v>
       </c>
       <c r="E12" s="40" t="n">
-        <v>0.026</v>
+        <v>-0.004</v>
       </c>
       <c r="F12" s="40" t="n">
-        <v>-0.02</v>
+        <v>-0.005</v>
       </c>
       <c r="G12" s="40" t="n">
-        <v>0.026</v>
+        <v>0.046</v>
       </c>
       <c r="H12" s="40" t="n">
-        <v>0.543</v>
+        <v>0.545</v>
       </c>
       <c r="I12" s="40" t="n">
-        <v>-0.508</v>
+        <v>-0.52</v>
       </c>
       <c r="J12" s="40" t="n">
-        <v>0.022</v>
+        <v>0.041</v>
       </c>
       <c r="K12" s="40" t="n">
-        <v>-0.062</v>
+        <v>-0.066</v>
       </c>
       <c r="L12" s="40" t="n">
-        <v>-0.438</v>
+        <v>-0.431</v>
       </c>
       <c r="M12" s="40" t="inlineStr">
         <is>
@@ -2266,44 +2266,44 @@
         </is>
       </c>
       <c r="B13" s="40" t="n">
-        <v>4.382</v>
+        <v>4.372</v>
       </c>
       <c r="C13" s="40" t="n">
-        <v>0.655</v>
+        <v>0.647</v>
       </c>
       <c r="D13" s="40" t="n">
-        <v>0.036</v>
+        <v>0.007</v>
       </c>
       <c r="E13" s="40" t="n">
-        <v>0.008999999999999999</v>
+        <v>-0</v>
       </c>
       <c r="F13" s="40" t="n">
         <v>-0.024</v>
       </c>
       <c r="G13" s="40" t="n">
-        <v>-0.021</v>
+        <v>-0.032</v>
       </c>
       <c r="H13" s="40" t="n">
-        <v>0.058</v>
+        <v>0.061</v>
       </c>
       <c r="I13" s="40" t="n">
-        <v>-0.058</v>
+        <v>-0.053</v>
       </c>
       <c r="J13" s="40" t="n">
-        <v>-0.115</v>
+        <v>-0.117</v>
       </c>
       <c r="K13" s="40" t="n">
-        <v>-0.057</v>
+        <v>-0.075</v>
       </c>
       <c r="L13" s="40" t="n">
         <v>-0</v>
       </c>
       <c r="M13" s="40" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.061</v>
       </c>
       <c r="N13" s="40" t="inlineStr">
         <is>
-          <t>(0.79)</t>
+          <t>(0.75)</t>
         </is>
       </c>
     </row>
@@ -2314,43 +2314,43 @@
         </is>
       </c>
       <c r="B14" s="40" t="n">
-        <v>4.509</v>
+        <v>4.521</v>
       </c>
       <c r="C14" s="40" t="n">
-        <v>0.744</v>
+        <v>0.741</v>
       </c>
       <c r="D14" s="40" t="n">
-        <v>0.008</v>
+        <v>0.01</v>
       </c>
       <c r="E14" s="40" t="n">
+        <v>0.041</v>
+      </c>
+      <c r="F14" s="40" t="n">
         <v>-0.024</v>
       </c>
-      <c r="F14" s="40" t="n">
-        <v>0.005</v>
-      </c>
       <c r="G14" s="40" t="n">
-        <v>-0.031</v>
+        <v>-0.082</v>
       </c>
       <c r="H14" s="40" t="n">
-        <v>-0.41</v>
+        <v>-0.417</v>
       </c>
       <c r="I14" s="40" t="n">
-        <v>0.415</v>
+        <v>0.4</v>
       </c>
       <c r="J14" s="40" t="n">
-        <v>-0.095</v>
+        <v>-0.064</v>
       </c>
       <c r="K14" s="40" t="n">
-        <v>-0.032</v>
+        <v>-0.005</v>
       </c>
       <c r="L14" s="40" t="n">
-        <v>0.603</v>
+        <v>0.57</v>
       </c>
       <c r="M14" s="40" t="n">
-        <v>-0.578</v>
+        <v>-0.592</v>
       </c>
       <c r="N14" s="40" t="n">
-        <v>0.313</v>
+        <v>0.375</v>
       </c>
       <c r="O14" s="40" t="inlineStr">
         <is>
@@ -2365,46 +2365,46 @@
         </is>
       </c>
       <c r="B15" s="40" t="n">
-        <v>4.718</v>
+        <v>4.809</v>
       </c>
       <c r="C15" s="40" t="n">
-        <v>1.233</v>
+        <v>1.186</v>
       </c>
       <c r="D15" s="40" t="n">
-        <v>-0.02</v>
+        <v>-0.091</v>
       </c>
       <c r="E15" s="40" t="n">
-        <v>-0.08699999999999999</v>
+        <v>-0</v>
       </c>
       <c r="F15" s="40" t="n">
-        <v>0.045</v>
+        <v>-0.095</v>
       </c>
       <c r="G15" s="40" t="n">
-        <v>0.029</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="H15" s="40" t="n">
-        <v>-0.313</v>
+        <v>-0.303</v>
       </c>
       <c r="I15" s="40" t="n">
-        <v>0.279</v>
+        <v>0.329</v>
       </c>
       <c r="J15" s="40" t="n">
-        <v>-0.044</v>
+        <v>-0.073</v>
       </c>
       <c r="K15" s="40" t="n">
-        <v>-0.026</v>
+        <v>-0.028</v>
       </c>
       <c r="L15" s="40" t="n">
-        <v>0.345</v>
+        <v>0.414</v>
       </c>
       <c r="M15" s="40" t="n">
-        <v>-0.294</v>
+        <v>-0.36</v>
       </c>
       <c r="N15" s="40" t="n">
-        <v>-0.094</v>
+        <v>0.012</v>
       </c>
       <c r="O15" s="40" t="n">
-        <v>0.249</v>
+        <v>0.262</v>
       </c>
       <c r="P15" s="40" t="inlineStr">
         <is>
@@ -2419,49 +2419,49 @@
         </is>
       </c>
       <c r="B16" s="40" t="n">
-        <v>2.632</v>
+        <v>2.507</v>
       </c>
       <c r="C16" s="40" t="n">
-        <v>1.122</v>
+        <v>1.027</v>
       </c>
       <c r="D16" s="40" t="n">
-        <v>0.007</v>
+        <v>0.014</v>
       </c>
       <c r="E16" s="40" t="n">
-        <v>0.052</v>
+        <v>0.042</v>
       </c>
       <c r="F16" s="40" t="n">
-        <v>0.031</v>
+        <v>0.017</v>
       </c>
       <c r="G16" s="40" t="n">
-        <v>0.015</v>
+        <v>0.032</v>
       </c>
       <c r="H16" s="40" t="n">
-        <v>0.344</v>
+        <v>0.218</v>
       </c>
       <c r="I16" s="40" t="n">
-        <v>-0.128</v>
+        <v>-0.309</v>
       </c>
       <c r="J16" s="40" t="n">
-        <v>-0.016</v>
+        <v>0.038</v>
       </c>
       <c r="K16" s="40" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.045</v>
       </c>
       <c r="L16" s="40" t="n">
-        <v>-0.33</v>
+        <v>-0.309</v>
       </c>
       <c r="M16" s="40" t="n">
-        <v>0.309</v>
+        <v>0.361</v>
       </c>
       <c r="N16" s="40" t="n">
-        <v>0.131</v>
+        <v>0.024</v>
       </c>
       <c r="O16" s="40" t="n">
-        <v>-0.18</v>
+        <v>-0.276</v>
       </c>
       <c r="P16" s="40" t="n">
-        <v>-0.322</v>
+        <v>-0.493</v>
       </c>
       <c r="Q16" s="40" t="inlineStr">
         <is>
@@ -2472,7 +2472,7 @@
     <row r="17" ht="35" customHeight="1" s="45">
       <c r="A17" s="23" t="inlineStr">
         <is>
-          <t>Note. Values on the diagonal are Cronbach’s alpha coefficients where applicable. Correlations are zero-order correlations among observed study variables. Leadership variables were rated by followers at T1. OCBS and CWBS were rated by leaders at T3. N = 360. *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
+          <t>Note. Values on the diagonal are Cronbach’s alpha coefficients where applicable. Correlations are zero-order correlations among observed study variables. Leadership variables were rated by followers at T1. OCBS and CWBS were rated by leaders at T3. N = 365. *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -3714,7 +3714,7 @@
     <row r="28" ht="48" customHeight="1" s="45">
       <c r="A28" s="23" t="inlineStr">
         <is>
-          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 360; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.</t>
+          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 365; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -5812,7 +5812,7 @@
     <row r="2">
       <c r="A2" s="38" t="inlineStr">
         <is>
-          <t>N = 360</t>
+          <t>N = 365</t>
         </is>
       </c>
     </row>
@@ -5826,14 +5826,14 @@
     <row r="4">
       <c r="A4" s="38" t="inlineStr">
         <is>
-          <t>- Male: 201 (55.8%)</t>
+          <t>- Male: 201 (55.1%)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="38" t="inlineStr">
         <is>
-          <t>- Female: 159 (44.2%)</t>
+          <t>- Female: 164 (44.9%)</t>
         </is>
       </c>
     </row>
@@ -5848,21 +5848,21 @@
     <row r="8">
       <c r="A8" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 30.76, SD = 4.69</t>
+          <t>Age: M = 30.74, SD = 4.60</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="38" t="inlineStr">
         <is>
-          <t>Working years: M = 9.01, SD = 4.91</t>
+          <t>Working years: M = 8.91, SD = 4.85</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="38" t="inlineStr">
         <is>
-          <t>Tenure with current leader: M = 2.33, SD = 1.48</t>
+          <t>Tenure with current leader: M = 2.31, SD = 1.46</t>
         </is>
       </c>
     </row>
@@ -5870,11 +5870,11 @@
       <c r="A11" s="48" t="inlineStr">
         <is>
           <t>Interaction frequency with leader:
-  - Rarely (&lt;1/wk): 19 (5.3%)
-  - Sometimes (1-2/wk): 62 (17.2%)
-  - Often (3-4/wk): 121 (33.6%)
-  - Very often (~daily): 109 (30.3%)
-  - Multiple times/day: 49 (13.6%)</t>
+  - Rarely (&lt;1/wk): 20 (5.5%)
+  - Sometimes (1-2/wk): 62 (17.0%)
+  - Often (3-4/wk): 121 (33.2%)
+  - Very often (~daily): 110 (30.1%)
+  - Multiple times/day: 52 (14.2%)</t>
         </is>
       </c>
     </row>
@@ -5889,35 +5889,35 @@
     <row r="14">
       <c r="A14" s="38" t="inlineStr">
         <is>
-          <t>- High school: 20 (5.6%)</t>
+          <t>- High school: 19 (5.2%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 61 (16.9%)</t>
+          <t>- Some college / Associate: 66 (18.1%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 169 (46.9%)</t>
+          <t>- Bachelor: 165 (45.2%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="38" t="inlineStr">
         <is>
-          <t>- Master: 85 (23.6%)</t>
+          <t>- Master: 92 (25.2%)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="38" t="inlineStr">
         <is>
-          <t>- Doctorate: 20 (5.6%)</t>
+          <t>- Doctorate: 20 (5.5%)</t>
         </is>
       </c>
     </row>
@@ -5932,35 +5932,35 @@
     <row r="21">
       <c r="A21" s="38" t="inlineStr">
         <is>
-          <t>- Entry: 71 (19.7%)</t>
+          <t>- Entry: 70 (19.2%)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="38" t="inlineStr">
         <is>
-          <t>- Associate: 114 (31.7%)</t>
+          <t>- Associate: 120 (32.9%)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="38" t="inlineStr">
         <is>
-          <t>- Senior: 95 (26.4%)</t>
+          <t>- Senior: 90 (24.7%)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="38" t="inlineStr">
         <is>
-          <t>- Manager: 58 (16.1%)</t>
+          <t>- Manager: 65 (17.8%)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="38" t="inlineStr">
         <is>
-          <t>- Director: 18 (5.0%)</t>
+          <t>- Director: 16 (4.4%)</t>
         </is>
       </c>
     </row>
@@ -5990,14 +5990,14 @@
     <row r="31">
       <c r="A31" s="38" t="inlineStr">
         <is>
-          <t>- Male: 44 (55.7%)</t>
+          <t>- Male: 49 (62.0%)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="38" t="inlineStr">
         <is>
-          <t>- Female: 35 (44.3%)</t>
+          <t>- Female: 30 (38.0%)</t>
         </is>
       </c>
     </row>
@@ -6012,7 +6012,7 @@
     <row r="35">
       <c r="A35" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 40.00, SD = 6.00</t>
+          <t>Age: M = 39.19, SD = 5.79</t>
         </is>
       </c>
     </row>
@@ -6026,14 +6026,14 @@
     <row r="37">
       <c r="A37" s="38" t="inlineStr">
         <is>
-          <t>Leadership tenure: M = 5.21, SD = 2.64</t>
+          <t>Leadership tenure: M = 5.51, SD = 3.03</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="38" t="inlineStr">
         <is>
-          <t>Span of control: M = 4.56, SD = 0.59</t>
+          <t>Span of control: M = 4.62, SD = 0.56</t>
         </is>
       </c>
     </row>
@@ -6048,28 +6048,28 @@
     <row r="41">
       <c r="A41" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 11 (13.9%)</t>
+          <t>- Some college / Associate: 9 (11.4%)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 39 (49.4%)</t>
+          <t>- Bachelor: 45 (57.0%)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="38" t="inlineStr">
         <is>
-          <t>- Master: 22 (27.8%)</t>
+          <t>- Master: 19 (24.1%)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="38" t="inlineStr">
         <is>
-          <t>- Doctorate: 7 (8.9%)</t>
+          <t>- Doctorate: 6 (7.6%)</t>
         </is>
       </c>
     </row>
@@ -6389,7 +6389,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>360</v>
+        <v>365</v>
       </c>
     </row>
     <row r="9">
@@ -6419,7 +6419,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>360</v>
+        <v>365</v>
       </c>
     </row>
     <row r="12">
@@ -6522,7 +6522,7 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>78.3%</t>
+          <t>79.3%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix v4.5.5: repair T3 reverse-coded items in cleaned data files
Bug: After v4.5.1 added per-item noise to T3 thriving items via shift_clip,
the reverse-coded items T3_R_THR5 and T3_R_THR10 were treated as independent
Likert items by signal injection — breaking the invariant T3_R_THRk +
T3_THRk == 8 (~232 / 363 rows wrong).

Why audit missed it: Layer 8 only checked the final_merged_analysis_data
file (which has its own end-of-script repair at line 339-342); the
intermediate t3f cleaned + raw files we deliver were never validated.

Fix:
  1. inject_signal.py — after shift_clip on T3 thriving items, repair
     T3_R_THR5/10 = 8 - T3_THR5/10 BEFORE saving t3f.
  2. audit.py Layer 8 — additionally read T1_cleaned, T3_follower_cleaned
     and T3_follower_raw and verify reverse-coding invariant in each.

After fix: 0 / 363 (cleaned) + 0 / 377 (raw) rows broken.
189/189 constraint + 10/10 audit (now stricter) PASS.
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -1951,10 +1951,10 @@
         </is>
       </c>
       <c r="B3" s="40" t="n">
-        <v>0.551</v>
+        <v>0.543</v>
       </c>
       <c r="C3" s="40" t="n">
-        <v>0.498</v>
+        <v>0.499</v>
       </c>
       <c r="D3" s="40" t="inlineStr">
         <is>
@@ -1969,13 +1969,13 @@
         </is>
       </c>
       <c r="B4" s="40" t="n">
-        <v>30.74</v>
+        <v>30.636</v>
       </c>
       <c r="C4" s="40" t="n">
-        <v>4.596</v>
+        <v>4.537</v>
       </c>
       <c r="D4" s="40" t="n">
-        <v>0.04</v>
+        <v>0.031</v>
       </c>
       <c r="E4" s="40" t="inlineStr">
         <is>
@@ -1990,16 +1990,16 @@
         </is>
       </c>
       <c r="B5" s="40" t="n">
-        <v>2.305</v>
+        <v>2.307</v>
       </c>
       <c r="C5" s="40" t="n">
-        <v>1.458</v>
+        <v>1.45</v>
       </c>
       <c r="D5" s="40" t="n">
-        <v>0.006</v>
+        <v>0.002</v>
       </c>
       <c r="E5" s="40" t="n">
-        <v>0.184</v>
+        <v>0.2</v>
       </c>
       <c r="F5" s="40" t="inlineStr">
         <is>
@@ -2014,19 +2014,19 @@
         </is>
       </c>
       <c r="B6" s="40" t="n">
-        <v>3.307</v>
+        <v>3.289</v>
       </c>
       <c r="C6" s="40" t="n">
-        <v>1.081</v>
+        <v>1.088</v>
       </c>
       <c r="D6" s="40" t="n">
-        <v>0.063</v>
+        <v>0.061</v>
       </c>
       <c r="E6" s="40" t="n">
-        <v>-0.038</v>
+        <v>-0.022</v>
       </c>
       <c r="F6" s="40" t="n">
-        <v>-0.027</v>
+        <v>-0.046</v>
       </c>
       <c r="G6" s="40" t="inlineStr">
         <is>
@@ -2041,22 +2041,22 @@
         </is>
       </c>
       <c r="B7" s="40" t="n">
-        <v>4.062</v>
+        <v>4.04</v>
       </c>
       <c r="C7" s="40" t="n">
-        <v>0.91</v>
+        <v>0.886</v>
       </c>
       <c r="D7" s="40" t="n">
-        <v>-0.031</v>
+        <v>-0.027</v>
       </c>
       <c r="E7" s="40" t="n">
-        <v>-0.01</v>
+        <v>-0.003</v>
       </c>
       <c r="F7" s="40" t="n">
-        <v>0.099</v>
+        <v>0.077</v>
       </c>
       <c r="G7" s="40" t="n">
-        <v>-0.016</v>
+        <v>-0.003</v>
       </c>
       <c r="H7" s="39" t="inlineStr">
         <is>
@@ -2071,25 +2071,25 @@
         </is>
       </c>
       <c r="B8" s="40" t="n">
-        <v>4.916</v>
+        <v>4.931</v>
       </c>
       <c r="C8" s="40" t="n">
-        <v>0.957</v>
+        <v>0.956</v>
       </c>
       <c r="D8" s="40" t="n">
-        <v>-0.027</v>
+        <v>-0.01</v>
       </c>
       <c r="E8" s="40" t="n">
-        <v>0.015</v>
+        <v>0.006</v>
       </c>
       <c r="F8" s="40" t="n">
-        <v>0</v>
+        <v>0.008</v>
       </c>
       <c r="G8" s="40" t="n">
-        <v>-0.095</v>
+        <v>-0.108</v>
       </c>
       <c r="H8" s="40" t="n">
-        <v>-0.353</v>
+        <v>-0.37</v>
       </c>
       <c r="I8" s="40" t="inlineStr">
         <is>
@@ -2104,28 +2104,28 @@
         </is>
       </c>
       <c r="B9" s="40" t="n">
-        <v>3.456</v>
+        <v>3.449</v>
       </c>
       <c r="C9" s="40" t="n">
-        <v>0.918</v>
+        <v>0.915</v>
       </c>
       <c r="D9" s="40" t="n">
-        <v>-0.08</v>
+        <v>-0.08500000000000001</v>
       </c>
       <c r="E9" s="40" t="n">
-        <v>-0.002</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="F9" s="40" t="n">
-        <v>0.09</v>
+        <v>0.038</v>
       </c>
       <c r="G9" s="40" t="n">
-        <v>-0.04</v>
+        <v>-0.036</v>
       </c>
       <c r="H9" s="40" t="n">
-        <v>0.003</v>
+        <v>-0.019</v>
       </c>
       <c r="I9" s="40" t="n">
-        <v>0.054</v>
+        <v>0.075</v>
       </c>
       <c r="J9" s="40" t="inlineStr">
         <is>
@@ -2140,31 +2140,31 @@
         </is>
       </c>
       <c r="B10" s="40" t="n">
-        <v>4.57</v>
+        <v>4.592</v>
       </c>
       <c r="C10" s="40" t="n">
-        <v>0.901</v>
+        <v>0.871</v>
       </c>
       <c r="D10" s="40" t="n">
-        <v>-0.065</v>
+        <v>-0.082</v>
       </c>
       <c r="E10" s="40" t="n">
-        <v>-0.078</v>
+        <v>-0.075</v>
       </c>
       <c r="F10" s="40" t="n">
-        <v>-0.08699999999999999</v>
+        <v>-0.045</v>
       </c>
       <c r="G10" s="40" t="n">
-        <v>-0.07099999999999999</v>
+        <v>-0.1</v>
       </c>
       <c r="H10" s="40" t="n">
-        <v>-0.04</v>
+        <v>-0.043</v>
       </c>
       <c r="I10" s="40" t="n">
-        <v>-0.035</v>
+        <v>-0.022</v>
       </c>
       <c r="J10" s="40" t="n">
-        <v>-0.008</v>
+        <v>0.005</v>
       </c>
       <c r="K10" s="40" t="inlineStr">
         <is>
@@ -2179,34 +2179,34 @@
         </is>
       </c>
       <c r="B11" s="40" t="n">
-        <v>4.51</v>
+        <v>4.526</v>
       </c>
       <c r="C11" s="40" t="n">
-        <v>1.234</v>
+        <v>1.254</v>
       </c>
       <c r="D11" s="40" t="n">
-        <v>-0.03</v>
+        <v>-0.032</v>
       </c>
       <c r="E11" s="40" t="n">
-        <v>0.002</v>
+        <v>-0.005</v>
       </c>
       <c r="F11" s="40" t="n">
-        <v>-0.067</v>
+        <v>-0.034</v>
       </c>
       <c r="G11" s="40" t="n">
-        <v>-0.045</v>
+        <v>-0.055</v>
       </c>
       <c r="H11" s="40" t="n">
-        <v>-0.535</v>
+        <v>-0.513</v>
       </c>
       <c r="I11" s="40" t="n">
-        <v>0.532</v>
+        <v>0.537</v>
       </c>
       <c r="J11" s="40" t="n">
-        <v>0.002</v>
+        <v>0.016</v>
       </c>
       <c r="K11" s="40" t="n">
-        <v>-0.025</v>
+        <v>-0.042</v>
       </c>
       <c r="L11" s="40" t="inlineStr">
         <is>
@@ -2221,37 +2221,37 @@
         </is>
       </c>
       <c r="B12" s="40" t="n">
-        <v>3.046</v>
+        <v>3.035</v>
       </c>
       <c r="C12" s="40" t="n">
-        <v>1.217</v>
+        <v>1.206</v>
       </c>
       <c r="D12" s="40" t="n">
-        <v>0.019</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="E12" s="40" t="n">
         <v>-0.004</v>
       </c>
       <c r="F12" s="40" t="n">
-        <v>-0.005</v>
+        <v>-0.02</v>
       </c>
       <c r="G12" s="40" t="n">
-        <v>0.046</v>
+        <v>0.06</v>
       </c>
       <c r="H12" s="40" t="n">
-        <v>0.545</v>
+        <v>0.543</v>
       </c>
       <c r="I12" s="40" t="n">
-        <v>-0.52</v>
+        <v>-0.531</v>
       </c>
       <c r="J12" s="40" t="n">
-        <v>0.041</v>
+        <v>0.01</v>
       </c>
       <c r="K12" s="40" t="n">
-        <v>-0.066</v>
+        <v>-0.061</v>
       </c>
       <c r="L12" s="40" t="n">
-        <v>-0.431</v>
+        <v>-0.45</v>
       </c>
       <c r="M12" s="40" t="inlineStr">
         <is>
@@ -2266,40 +2266,40 @@
         </is>
       </c>
       <c r="B13" s="40" t="n">
-        <v>4.372</v>
+        <v>4.373</v>
       </c>
       <c r="C13" s="40" t="n">
-        <v>0.647</v>
+        <v>0.654</v>
       </c>
       <c r="D13" s="40" t="n">
-        <v>0.007</v>
+        <v>0.045</v>
       </c>
       <c r="E13" s="40" t="n">
-        <v>-0</v>
+        <v>-0.02</v>
       </c>
       <c r="F13" s="40" t="n">
-        <v>-0.024</v>
+        <v>-0.037</v>
       </c>
       <c r="G13" s="40" t="n">
-        <v>-0.032</v>
+        <v>-0.026</v>
       </c>
       <c r="H13" s="40" t="n">
-        <v>0.061</v>
+        <v>0.064</v>
       </c>
       <c r="I13" s="40" t="n">
-        <v>-0.053</v>
+        <v>-0.054</v>
       </c>
       <c r="J13" s="40" t="n">
-        <v>-0.117</v>
+        <v>-0.103</v>
       </c>
       <c r="K13" s="40" t="n">
-        <v>-0.075</v>
+        <v>-0.076</v>
       </c>
       <c r="L13" s="40" t="n">
-        <v>-0</v>
+        <v>-0.013</v>
       </c>
       <c r="M13" s="40" t="n">
-        <v>0.061</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="N13" s="40" t="inlineStr">
         <is>
@@ -2314,43 +2314,43 @@
         </is>
       </c>
       <c r="B14" s="40" t="n">
-        <v>4.521</v>
+        <v>4.516</v>
       </c>
       <c r="C14" s="40" t="n">
-        <v>0.741</v>
+        <v>0.783</v>
       </c>
       <c r="D14" s="40" t="n">
-        <v>0.01</v>
+        <v>-0.015</v>
       </c>
       <c r="E14" s="40" t="n">
-        <v>0.041</v>
+        <v>-0.001</v>
       </c>
       <c r="F14" s="40" t="n">
-        <v>-0.024</v>
+        <v>0.048</v>
       </c>
       <c r="G14" s="40" t="n">
-        <v>-0.082</v>
+        <v>-0.083</v>
       </c>
       <c r="H14" s="40" t="n">
-        <v>-0.417</v>
+        <v>-0.437</v>
       </c>
       <c r="I14" s="40" t="n">
-        <v>0.4</v>
+        <v>0.456</v>
       </c>
       <c r="J14" s="40" t="n">
-        <v>-0.064</v>
+        <v>-0.03</v>
       </c>
       <c r="K14" s="40" t="n">
-        <v>-0.005</v>
+        <v>-0.046</v>
       </c>
       <c r="L14" s="40" t="n">
-        <v>0.57</v>
+        <v>0.681</v>
       </c>
       <c r="M14" s="40" t="n">
-        <v>-0.592</v>
+        <v>-0.59</v>
       </c>
       <c r="N14" s="40" t="n">
-        <v>0.375</v>
+        <v>0.292</v>
       </c>
       <c r="O14" s="40" t="inlineStr">
         <is>
@@ -2365,46 +2365,46 @@
         </is>
       </c>
       <c r="B15" s="40" t="n">
-        <v>4.809</v>
+        <v>4.69</v>
       </c>
       <c r="C15" s="40" t="n">
-        <v>1.186</v>
+        <v>1.286</v>
       </c>
       <c r="D15" s="40" t="n">
-        <v>-0.091</v>
+        <v>-0.033</v>
       </c>
       <c r="E15" s="40" t="n">
-        <v>-0</v>
+        <v>-0.063</v>
       </c>
       <c r="F15" s="40" t="n">
-        <v>-0.095</v>
+        <v>-0.037</v>
       </c>
       <c r="G15" s="40" t="n">
-        <v>0.008999999999999999</v>
+        <v>-0.077</v>
       </c>
       <c r="H15" s="40" t="n">
-        <v>-0.303</v>
+        <v>-0.305</v>
       </c>
       <c r="I15" s="40" t="n">
-        <v>0.329</v>
+        <v>0.365</v>
       </c>
       <c r="J15" s="40" t="n">
-        <v>-0.073</v>
+        <v>-0.068</v>
       </c>
       <c r="K15" s="40" t="n">
-        <v>-0.028</v>
+        <v>-0.024</v>
       </c>
       <c r="L15" s="40" t="n">
-        <v>0.414</v>
+        <v>0.427</v>
       </c>
       <c r="M15" s="40" t="n">
-        <v>-0.36</v>
+        <v>-0.333</v>
       </c>
       <c r="N15" s="40" t="n">
-        <v>0.012</v>
+        <v>-0.032</v>
       </c>
       <c r="O15" s="40" t="n">
-        <v>0.262</v>
+        <v>0.359</v>
       </c>
       <c r="P15" s="40" t="inlineStr">
         <is>
@@ -2419,49 +2419,49 @@
         </is>
       </c>
       <c r="B16" s="40" t="n">
-        <v>2.507</v>
+        <v>2.559</v>
       </c>
       <c r="C16" s="40" t="n">
-        <v>1.027</v>
+        <v>1.071</v>
       </c>
       <c r="D16" s="40" t="n">
-        <v>0.014</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="E16" s="40" t="n">
-        <v>0.042</v>
+        <v>0.015</v>
       </c>
       <c r="F16" s="40" t="n">
-        <v>0.017</v>
+        <v>-0.006</v>
       </c>
       <c r="G16" s="40" t="n">
-        <v>0.032</v>
+        <v>0.015</v>
       </c>
       <c r="H16" s="40" t="n">
-        <v>0.218</v>
+        <v>0.282</v>
       </c>
       <c r="I16" s="40" t="n">
-        <v>-0.309</v>
+        <v>-0.248</v>
       </c>
       <c r="J16" s="40" t="n">
-        <v>0.038</v>
+        <v>0.023</v>
       </c>
       <c r="K16" s="40" t="n">
-        <v>-0.045</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="L16" s="40" t="n">
-        <v>-0.309</v>
+        <v>-0.332</v>
       </c>
       <c r="M16" s="40" t="n">
-        <v>0.361</v>
+        <v>0.334</v>
       </c>
       <c r="N16" s="40" t="n">
-        <v>0.024</v>
+        <v>-0.064</v>
       </c>
       <c r="O16" s="40" t="n">
-        <v>-0.276</v>
+        <v>-0.325</v>
       </c>
       <c r="P16" s="40" t="n">
-        <v>-0.493</v>
+        <v>-0.444</v>
       </c>
       <c r="Q16" s="40" t="inlineStr">
         <is>
@@ -2472,7 +2472,7 @@
     <row r="17" ht="35" customHeight="1" s="45">
       <c r="A17" s="23" t="inlineStr">
         <is>
-          <t>Note. Values on the diagonal are Cronbach’s alpha coefficients where applicable. Correlations are zero-order correlations among observed study variables. Leadership variables were rated by followers at T1. OCBS and CWBS were rated by leaders at T3. N = 365. *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
+          <t>Note. Values on the diagonal are Cronbach’s alpha coefficients where applicable. Correlations are zero-order correlations among observed study variables. Leadership variables were rated by followers at T1. OCBS and CWBS were rated by leaders at T3. N = 363. *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -3714,7 +3714,7 @@
     <row r="28" ht="48" customHeight="1" s="45">
       <c r="A28" s="23" t="inlineStr">
         <is>
-          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 365; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.</t>
+          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 363; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -5812,7 +5812,7 @@
     <row r="2">
       <c r="A2" s="38" t="inlineStr">
         <is>
-          <t>N = 365</t>
+          <t>N = 363</t>
         </is>
       </c>
     </row>
@@ -5826,14 +5826,14 @@
     <row r="4">
       <c r="A4" s="38" t="inlineStr">
         <is>
-          <t>- Male: 201 (55.1%)</t>
+          <t>- Male: 197 (54.3%)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="38" t="inlineStr">
         <is>
-          <t>- Female: 164 (44.9%)</t>
+          <t>- Female: 166 (45.7%)</t>
         </is>
       </c>
     </row>
@@ -5848,21 +5848,21 @@
     <row r="8">
       <c r="A8" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 30.74, SD = 4.60</t>
+          <t>Age: M = 30.64, SD = 4.54</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="38" t="inlineStr">
         <is>
-          <t>Working years: M = 8.91, SD = 4.85</t>
+          <t>Working years: M = 8.86, SD = 4.83</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="38" t="inlineStr">
         <is>
-          <t>Tenure with current leader: M = 2.31, SD = 1.46</t>
+          <t>Tenure with current leader: M = 2.31, SD = 1.45</t>
         </is>
       </c>
     </row>
@@ -5870,11 +5870,11 @@
       <c r="A11" s="48" t="inlineStr">
         <is>
           <t>Interaction frequency with leader:
-  - Rarely (&lt;1/wk): 20 (5.5%)
-  - Sometimes (1-2/wk): 62 (17.0%)
-  - Often (3-4/wk): 121 (33.2%)
-  - Very often (~daily): 110 (30.1%)
-  - Multiple times/day: 52 (14.2%)</t>
+  - Rarely (&lt;1/wk): 21 (5.8%)
+  - Sometimes (1-2/wk): 65 (17.9%)
+  - Often (3-4/wk): 114 (31.4%)
+  - Very often (~daily): 114 (31.4%)
+  - Multiple times/day: 49 (13.5%)</t>
         </is>
       </c>
     </row>
@@ -5889,28 +5889,28 @@
     <row r="14">
       <c r="A14" s="38" t="inlineStr">
         <is>
-          <t>- High school: 19 (5.2%)</t>
+          <t>- High school: 20 (5.5%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 66 (18.1%)</t>
+          <t>- Some college / Associate: 62 (17.1%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 165 (45.2%)</t>
+          <t>- Bachelor: 165 (45.5%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="38" t="inlineStr">
         <is>
-          <t>- Master: 92 (25.2%)</t>
+          <t>- Master: 92 (25.3%)</t>
         </is>
       </c>
     </row>
@@ -5932,35 +5932,35 @@
     <row r="21">
       <c r="A21" s="38" t="inlineStr">
         <is>
-          <t>- Entry: 70 (19.2%)</t>
+          <t>- Entry: 69 (19.0%)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="38" t="inlineStr">
         <is>
-          <t>- Associate: 120 (32.9%)</t>
+          <t>- Associate: 120 (33.1%)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="38" t="inlineStr">
         <is>
-          <t>- Senior: 90 (24.7%)</t>
+          <t>- Senior: 93 (25.6%)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="38" t="inlineStr">
         <is>
-          <t>- Manager: 65 (17.8%)</t>
+          <t>- Manager: 59 (16.3%)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="38" t="inlineStr">
         <is>
-          <t>- Director: 16 (4.4%)</t>
+          <t>- Director: 18 (5.0%)</t>
         </is>
       </c>
     </row>
@@ -5990,14 +5990,14 @@
     <row r="31">
       <c r="A31" s="38" t="inlineStr">
         <is>
-          <t>- Male: 49 (62.0%)</t>
+          <t>- Male: 46 (58.2%)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="38" t="inlineStr">
         <is>
-          <t>- Female: 30 (38.0%)</t>
+          <t>- Female: 33 (41.8%)</t>
         </is>
       </c>
     </row>
@@ -6012,7 +6012,7 @@
     <row r="35">
       <c r="A35" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 39.19, SD = 5.79</t>
+          <t>Age: M = 40.91, SD = 6.40</t>
         </is>
       </c>
     </row>
@@ -6026,14 +6026,14 @@
     <row r="37">
       <c r="A37" s="38" t="inlineStr">
         <is>
-          <t>Leadership tenure: M = 5.51, SD = 3.03</t>
+          <t>Leadership tenure: M = 5.33, SD = 3.14</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="38" t="inlineStr">
         <is>
-          <t>Span of control: M = 4.62, SD = 0.56</t>
+          <t>Span of control: M = 4.59, SD = 0.57</t>
         </is>
       </c>
     </row>
@@ -6048,28 +6048,28 @@
     <row r="41">
       <c r="A41" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 9 (11.4%)</t>
+          <t>- Some college / Associate: 7 (8.9%)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 45 (57.0%)</t>
+          <t>- Bachelor: 42 (53.2%)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="38" t="inlineStr">
         <is>
-          <t>- Master: 19 (24.1%)</t>
+          <t>- Master: 23 (29.1%)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="38" t="inlineStr">
         <is>
-          <t>- Doctorate: 6 (7.6%)</t>
+          <t>- Doctorate: 7 (8.9%)</t>
         </is>
       </c>
     </row>
@@ -6389,7 +6389,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="9">
@@ -6419,7 +6419,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="12">
@@ -6522,7 +6522,7 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>79.3%</t>
+          <t>78.9%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sync v4.5.5: T3 reverse-coding repaired in cleaned + raw files
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -1951,10 +1951,10 @@
         </is>
       </c>
       <c r="B3" s="40" t="n">
-        <v>0.551</v>
+        <v>0.543</v>
       </c>
       <c r="C3" s="40" t="n">
-        <v>0.498</v>
+        <v>0.499</v>
       </c>
       <c r="D3" s="40" t="inlineStr">
         <is>
@@ -1969,13 +1969,13 @@
         </is>
       </c>
       <c r="B4" s="40" t="n">
-        <v>30.74</v>
+        <v>30.636</v>
       </c>
       <c r="C4" s="40" t="n">
-        <v>4.596</v>
+        <v>4.537</v>
       </c>
       <c r="D4" s="40" t="n">
-        <v>0.04</v>
+        <v>0.031</v>
       </c>
       <c r="E4" s="40" t="inlineStr">
         <is>
@@ -1990,16 +1990,16 @@
         </is>
       </c>
       <c r="B5" s="40" t="n">
-        <v>2.305</v>
+        <v>2.307</v>
       </c>
       <c r="C5" s="40" t="n">
-        <v>1.458</v>
+        <v>1.45</v>
       </c>
       <c r="D5" s="40" t="n">
-        <v>0.006</v>
+        <v>0.002</v>
       </c>
       <c r="E5" s="40" t="n">
-        <v>0.184</v>
+        <v>0.2</v>
       </c>
       <c r="F5" s="40" t="inlineStr">
         <is>
@@ -2014,19 +2014,19 @@
         </is>
       </c>
       <c r="B6" s="40" t="n">
-        <v>3.307</v>
+        <v>3.289</v>
       </c>
       <c r="C6" s="40" t="n">
-        <v>1.081</v>
+        <v>1.088</v>
       </c>
       <c r="D6" s="40" t="n">
-        <v>0.063</v>
+        <v>0.061</v>
       </c>
       <c r="E6" s="40" t="n">
-        <v>-0.038</v>
+        <v>-0.022</v>
       </c>
       <c r="F6" s="40" t="n">
-        <v>-0.027</v>
+        <v>-0.046</v>
       </c>
       <c r="G6" s="40" t="inlineStr">
         <is>
@@ -2041,22 +2041,22 @@
         </is>
       </c>
       <c r="B7" s="40" t="n">
-        <v>4.062</v>
+        <v>4.04</v>
       </c>
       <c r="C7" s="40" t="n">
-        <v>0.91</v>
+        <v>0.886</v>
       </c>
       <c r="D7" s="40" t="n">
-        <v>-0.031</v>
+        <v>-0.027</v>
       </c>
       <c r="E7" s="40" t="n">
-        <v>-0.01</v>
+        <v>-0.003</v>
       </c>
       <c r="F7" s="40" t="n">
-        <v>0.099</v>
+        <v>0.077</v>
       </c>
       <c r="G7" s="40" t="n">
-        <v>-0.016</v>
+        <v>-0.003</v>
       </c>
       <c r="H7" s="39" t="inlineStr">
         <is>
@@ -2071,25 +2071,25 @@
         </is>
       </c>
       <c r="B8" s="40" t="n">
-        <v>4.916</v>
+        <v>4.931</v>
       </c>
       <c r="C8" s="40" t="n">
-        <v>0.957</v>
+        <v>0.956</v>
       </c>
       <c r="D8" s="40" t="n">
-        <v>-0.027</v>
+        <v>-0.01</v>
       </c>
       <c r="E8" s="40" t="n">
-        <v>0.015</v>
+        <v>0.006</v>
       </c>
       <c r="F8" s="40" t="n">
-        <v>0</v>
+        <v>0.008</v>
       </c>
       <c r="G8" s="40" t="n">
-        <v>-0.095</v>
+        <v>-0.108</v>
       </c>
       <c r="H8" s="40" t="n">
-        <v>-0.353</v>
+        <v>-0.37</v>
       </c>
       <c r="I8" s="40" t="inlineStr">
         <is>
@@ -2104,28 +2104,28 @@
         </is>
       </c>
       <c r="B9" s="40" t="n">
-        <v>3.456</v>
+        <v>3.449</v>
       </c>
       <c r="C9" s="40" t="n">
-        <v>0.918</v>
+        <v>0.915</v>
       </c>
       <c r="D9" s="40" t="n">
-        <v>-0.08</v>
+        <v>-0.08500000000000001</v>
       </c>
       <c r="E9" s="40" t="n">
-        <v>-0.002</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="F9" s="40" t="n">
-        <v>0.09</v>
+        <v>0.038</v>
       </c>
       <c r="G9" s="40" t="n">
-        <v>-0.04</v>
+        <v>-0.036</v>
       </c>
       <c r="H9" s="40" t="n">
-        <v>0.003</v>
+        <v>-0.019</v>
       </c>
       <c r="I9" s="40" t="n">
-        <v>0.054</v>
+        <v>0.075</v>
       </c>
       <c r="J9" s="40" t="inlineStr">
         <is>
@@ -2140,31 +2140,31 @@
         </is>
       </c>
       <c r="B10" s="40" t="n">
-        <v>4.57</v>
+        <v>4.592</v>
       </c>
       <c r="C10" s="40" t="n">
-        <v>0.901</v>
+        <v>0.871</v>
       </c>
       <c r="D10" s="40" t="n">
-        <v>-0.065</v>
+        <v>-0.082</v>
       </c>
       <c r="E10" s="40" t="n">
-        <v>-0.078</v>
+        <v>-0.075</v>
       </c>
       <c r="F10" s="40" t="n">
-        <v>-0.08699999999999999</v>
+        <v>-0.045</v>
       </c>
       <c r="G10" s="40" t="n">
-        <v>-0.07099999999999999</v>
+        <v>-0.1</v>
       </c>
       <c r="H10" s="40" t="n">
-        <v>-0.04</v>
+        <v>-0.043</v>
       </c>
       <c r="I10" s="40" t="n">
-        <v>-0.035</v>
+        <v>-0.022</v>
       </c>
       <c r="J10" s="40" t="n">
-        <v>-0.008</v>
+        <v>0.005</v>
       </c>
       <c r="K10" s="40" t="inlineStr">
         <is>
@@ -2179,34 +2179,34 @@
         </is>
       </c>
       <c r="B11" s="40" t="n">
-        <v>4.51</v>
+        <v>4.526</v>
       </c>
       <c r="C11" s="40" t="n">
-        <v>1.234</v>
+        <v>1.254</v>
       </c>
       <c r="D11" s="40" t="n">
-        <v>-0.03</v>
+        <v>-0.032</v>
       </c>
       <c r="E11" s="40" t="n">
-        <v>0.002</v>
+        <v>-0.005</v>
       </c>
       <c r="F11" s="40" t="n">
-        <v>-0.067</v>
+        <v>-0.034</v>
       </c>
       <c r="G11" s="40" t="n">
-        <v>-0.045</v>
+        <v>-0.055</v>
       </c>
       <c r="H11" s="40" t="n">
-        <v>-0.535</v>
+        <v>-0.513</v>
       </c>
       <c r="I11" s="40" t="n">
-        <v>0.532</v>
+        <v>0.537</v>
       </c>
       <c r="J11" s="40" t="n">
-        <v>0.002</v>
+        <v>0.016</v>
       </c>
       <c r="K11" s="40" t="n">
-        <v>-0.025</v>
+        <v>-0.042</v>
       </c>
       <c r="L11" s="40" t="inlineStr">
         <is>
@@ -2221,37 +2221,37 @@
         </is>
       </c>
       <c r="B12" s="40" t="n">
-        <v>3.046</v>
+        <v>3.035</v>
       </c>
       <c r="C12" s="40" t="n">
-        <v>1.217</v>
+        <v>1.206</v>
       </c>
       <c r="D12" s="40" t="n">
-        <v>0.019</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="E12" s="40" t="n">
         <v>-0.004</v>
       </c>
       <c r="F12" s="40" t="n">
-        <v>-0.005</v>
+        <v>-0.02</v>
       </c>
       <c r="G12" s="40" t="n">
-        <v>0.046</v>
+        <v>0.06</v>
       </c>
       <c r="H12" s="40" t="n">
-        <v>0.545</v>
+        <v>0.543</v>
       </c>
       <c r="I12" s="40" t="n">
-        <v>-0.52</v>
+        <v>-0.531</v>
       </c>
       <c r="J12" s="40" t="n">
-        <v>0.041</v>
+        <v>0.01</v>
       </c>
       <c r="K12" s="40" t="n">
-        <v>-0.066</v>
+        <v>-0.061</v>
       </c>
       <c r="L12" s="40" t="n">
-        <v>-0.431</v>
+        <v>-0.45</v>
       </c>
       <c r="M12" s="40" t="inlineStr">
         <is>
@@ -2266,40 +2266,40 @@
         </is>
       </c>
       <c r="B13" s="40" t="n">
-        <v>4.372</v>
+        <v>4.373</v>
       </c>
       <c r="C13" s="40" t="n">
-        <v>0.647</v>
+        <v>0.654</v>
       </c>
       <c r="D13" s="40" t="n">
-        <v>0.007</v>
+        <v>0.045</v>
       </c>
       <c r="E13" s="40" t="n">
-        <v>-0</v>
+        <v>-0.02</v>
       </c>
       <c r="F13" s="40" t="n">
-        <v>-0.024</v>
+        <v>-0.037</v>
       </c>
       <c r="G13" s="40" t="n">
-        <v>-0.032</v>
+        <v>-0.026</v>
       </c>
       <c r="H13" s="40" t="n">
-        <v>0.061</v>
+        <v>0.064</v>
       </c>
       <c r="I13" s="40" t="n">
-        <v>-0.053</v>
+        <v>-0.054</v>
       </c>
       <c r="J13" s="40" t="n">
-        <v>-0.117</v>
+        <v>-0.103</v>
       </c>
       <c r="K13" s="40" t="n">
-        <v>-0.075</v>
+        <v>-0.076</v>
       </c>
       <c r="L13" s="40" t="n">
-        <v>-0</v>
+        <v>-0.013</v>
       </c>
       <c r="M13" s="40" t="n">
-        <v>0.061</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="N13" s="40" t="inlineStr">
         <is>
@@ -2314,43 +2314,43 @@
         </is>
       </c>
       <c r="B14" s="40" t="n">
-        <v>4.521</v>
+        <v>4.516</v>
       </c>
       <c r="C14" s="40" t="n">
-        <v>0.741</v>
+        <v>0.783</v>
       </c>
       <c r="D14" s="40" t="n">
-        <v>0.01</v>
+        <v>-0.015</v>
       </c>
       <c r="E14" s="40" t="n">
-        <v>0.041</v>
+        <v>-0.001</v>
       </c>
       <c r="F14" s="40" t="n">
-        <v>-0.024</v>
+        <v>0.048</v>
       </c>
       <c r="G14" s="40" t="n">
-        <v>-0.082</v>
+        <v>-0.083</v>
       </c>
       <c r="H14" s="40" t="n">
-        <v>-0.417</v>
+        <v>-0.437</v>
       </c>
       <c r="I14" s="40" t="n">
-        <v>0.4</v>
+        <v>0.456</v>
       </c>
       <c r="J14" s="40" t="n">
-        <v>-0.064</v>
+        <v>-0.03</v>
       </c>
       <c r="K14" s="40" t="n">
-        <v>-0.005</v>
+        <v>-0.046</v>
       </c>
       <c r="L14" s="40" t="n">
-        <v>0.57</v>
+        <v>0.681</v>
       </c>
       <c r="M14" s="40" t="n">
-        <v>-0.592</v>
+        <v>-0.59</v>
       </c>
       <c r="N14" s="40" t="n">
-        <v>0.375</v>
+        <v>0.292</v>
       </c>
       <c r="O14" s="40" t="inlineStr">
         <is>
@@ -2365,46 +2365,46 @@
         </is>
       </c>
       <c r="B15" s="40" t="n">
-        <v>4.809</v>
+        <v>4.69</v>
       </c>
       <c r="C15" s="40" t="n">
-        <v>1.186</v>
+        <v>1.286</v>
       </c>
       <c r="D15" s="40" t="n">
-        <v>-0.091</v>
+        <v>-0.033</v>
       </c>
       <c r="E15" s="40" t="n">
-        <v>-0</v>
+        <v>-0.063</v>
       </c>
       <c r="F15" s="40" t="n">
-        <v>-0.095</v>
+        <v>-0.037</v>
       </c>
       <c r="G15" s="40" t="n">
-        <v>0.008999999999999999</v>
+        <v>-0.077</v>
       </c>
       <c r="H15" s="40" t="n">
-        <v>-0.303</v>
+        <v>-0.305</v>
       </c>
       <c r="I15" s="40" t="n">
-        <v>0.329</v>
+        <v>0.365</v>
       </c>
       <c r="J15" s="40" t="n">
-        <v>-0.073</v>
+        <v>-0.068</v>
       </c>
       <c r="K15" s="40" t="n">
-        <v>-0.028</v>
+        <v>-0.024</v>
       </c>
       <c r="L15" s="40" t="n">
-        <v>0.414</v>
+        <v>0.427</v>
       </c>
       <c r="M15" s="40" t="n">
-        <v>-0.36</v>
+        <v>-0.333</v>
       </c>
       <c r="N15" s="40" t="n">
-        <v>0.012</v>
+        <v>-0.032</v>
       </c>
       <c r="O15" s="40" t="n">
-        <v>0.262</v>
+        <v>0.359</v>
       </c>
       <c r="P15" s="40" t="inlineStr">
         <is>
@@ -2419,49 +2419,49 @@
         </is>
       </c>
       <c r="B16" s="40" t="n">
-        <v>2.507</v>
+        <v>2.559</v>
       </c>
       <c r="C16" s="40" t="n">
-        <v>1.027</v>
+        <v>1.071</v>
       </c>
       <c r="D16" s="40" t="n">
-        <v>0.014</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="E16" s="40" t="n">
-        <v>0.042</v>
+        <v>0.015</v>
       </c>
       <c r="F16" s="40" t="n">
-        <v>0.017</v>
+        <v>-0.006</v>
       </c>
       <c r="G16" s="40" t="n">
-        <v>0.032</v>
+        <v>0.015</v>
       </c>
       <c r="H16" s="40" t="n">
-        <v>0.218</v>
+        <v>0.282</v>
       </c>
       <c r="I16" s="40" t="n">
-        <v>-0.309</v>
+        <v>-0.248</v>
       </c>
       <c r="J16" s="40" t="n">
-        <v>0.038</v>
+        <v>0.023</v>
       </c>
       <c r="K16" s="40" t="n">
-        <v>-0.045</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="L16" s="40" t="n">
-        <v>-0.309</v>
+        <v>-0.332</v>
       </c>
       <c r="M16" s="40" t="n">
-        <v>0.361</v>
+        <v>0.334</v>
       </c>
       <c r="N16" s="40" t="n">
-        <v>0.024</v>
+        <v>-0.064</v>
       </c>
       <c r="O16" s="40" t="n">
-        <v>-0.276</v>
+        <v>-0.325</v>
       </c>
       <c r="P16" s="40" t="n">
-        <v>-0.493</v>
+        <v>-0.444</v>
       </c>
       <c r="Q16" s="40" t="inlineStr">
         <is>
@@ -2472,7 +2472,7 @@
     <row r="17" ht="35" customHeight="1" s="45">
       <c r="A17" s="23" t="inlineStr">
         <is>
-          <t>Note. Values on the diagonal are Cronbach’s alpha coefficients where applicable. Correlations are zero-order correlations among observed study variables. Leadership variables were rated by followers at T1. OCBS and CWBS were rated by leaders at T3. N = 365. *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
+          <t>Note. Values on the diagonal are Cronbach’s alpha coefficients where applicable. Correlations are zero-order correlations among observed study variables. Leadership variables were rated by followers at T1. OCBS and CWBS were rated by leaders at T3. N = 363. *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -3714,7 +3714,7 @@
     <row r="28" ht="48" customHeight="1" s="45">
       <c r="A28" s="23" t="inlineStr">
         <is>
-          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 365; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.</t>
+          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 363; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -5812,7 +5812,7 @@
     <row r="2">
       <c r="A2" s="38" t="inlineStr">
         <is>
-          <t>N = 365</t>
+          <t>N = 363</t>
         </is>
       </c>
     </row>
@@ -5826,14 +5826,14 @@
     <row r="4">
       <c r="A4" s="38" t="inlineStr">
         <is>
-          <t>- Male: 201 (55.1%)</t>
+          <t>- Male: 197 (54.3%)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="38" t="inlineStr">
         <is>
-          <t>- Female: 164 (44.9%)</t>
+          <t>- Female: 166 (45.7%)</t>
         </is>
       </c>
     </row>
@@ -5848,21 +5848,21 @@
     <row r="8">
       <c r="A8" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 30.74, SD = 4.60</t>
+          <t>Age: M = 30.64, SD = 4.54</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="38" t="inlineStr">
         <is>
-          <t>Working years: M = 8.91, SD = 4.85</t>
+          <t>Working years: M = 8.86, SD = 4.83</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="38" t="inlineStr">
         <is>
-          <t>Tenure with current leader: M = 2.31, SD = 1.46</t>
+          <t>Tenure with current leader: M = 2.31, SD = 1.45</t>
         </is>
       </c>
     </row>
@@ -5870,11 +5870,11 @@
       <c r="A11" s="48" t="inlineStr">
         <is>
           <t>Interaction frequency with leader:
-  - Rarely (&lt;1/wk): 20 (5.5%)
-  - Sometimes (1-2/wk): 62 (17.0%)
-  - Often (3-4/wk): 121 (33.2%)
-  - Very often (~daily): 110 (30.1%)
-  - Multiple times/day: 52 (14.2%)</t>
+  - Rarely (&lt;1/wk): 21 (5.8%)
+  - Sometimes (1-2/wk): 65 (17.9%)
+  - Often (3-4/wk): 114 (31.4%)
+  - Very often (~daily): 114 (31.4%)
+  - Multiple times/day: 49 (13.5%)</t>
         </is>
       </c>
     </row>
@@ -5889,28 +5889,28 @@
     <row r="14">
       <c r="A14" s="38" t="inlineStr">
         <is>
-          <t>- High school: 19 (5.2%)</t>
+          <t>- High school: 20 (5.5%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 66 (18.1%)</t>
+          <t>- Some college / Associate: 62 (17.1%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 165 (45.2%)</t>
+          <t>- Bachelor: 165 (45.5%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="38" t="inlineStr">
         <is>
-          <t>- Master: 92 (25.2%)</t>
+          <t>- Master: 92 (25.3%)</t>
         </is>
       </c>
     </row>
@@ -5932,35 +5932,35 @@
     <row r="21">
       <c r="A21" s="38" t="inlineStr">
         <is>
-          <t>- Entry: 70 (19.2%)</t>
+          <t>- Entry: 69 (19.0%)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="38" t="inlineStr">
         <is>
-          <t>- Associate: 120 (32.9%)</t>
+          <t>- Associate: 120 (33.1%)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="38" t="inlineStr">
         <is>
-          <t>- Senior: 90 (24.7%)</t>
+          <t>- Senior: 93 (25.6%)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="38" t="inlineStr">
         <is>
-          <t>- Manager: 65 (17.8%)</t>
+          <t>- Manager: 59 (16.3%)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="38" t="inlineStr">
         <is>
-          <t>- Director: 16 (4.4%)</t>
+          <t>- Director: 18 (5.0%)</t>
         </is>
       </c>
     </row>
@@ -5990,14 +5990,14 @@
     <row r="31">
       <c r="A31" s="38" t="inlineStr">
         <is>
-          <t>- Male: 49 (62.0%)</t>
+          <t>- Male: 46 (58.2%)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="38" t="inlineStr">
         <is>
-          <t>- Female: 30 (38.0%)</t>
+          <t>- Female: 33 (41.8%)</t>
         </is>
       </c>
     </row>
@@ -6012,7 +6012,7 @@
     <row r="35">
       <c r="A35" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 39.19, SD = 5.79</t>
+          <t>Age: M = 40.91, SD = 6.40</t>
         </is>
       </c>
     </row>
@@ -6026,14 +6026,14 @@
     <row r="37">
       <c r="A37" s="38" t="inlineStr">
         <is>
-          <t>Leadership tenure: M = 5.51, SD = 3.03</t>
+          <t>Leadership tenure: M = 5.33, SD = 3.14</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="38" t="inlineStr">
         <is>
-          <t>Span of control: M = 4.62, SD = 0.56</t>
+          <t>Span of control: M = 4.59, SD = 0.57</t>
         </is>
       </c>
     </row>
@@ -6048,28 +6048,28 @@
     <row r="41">
       <c r="A41" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 9 (11.4%)</t>
+          <t>- Some college / Associate: 7 (8.9%)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 45 (57.0%)</t>
+          <t>- Bachelor: 42 (53.2%)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="38" t="inlineStr">
         <is>
-          <t>- Master: 19 (24.1%)</t>
+          <t>- Master: 23 (29.1%)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="38" t="inlineStr">
         <is>
-          <t>- Doctorate: 6 (7.6%)</t>
+          <t>- Doctorate: 7 (8.9%)</t>
         </is>
       </c>
     </row>
@@ -6389,7 +6389,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="9">
@@ -6419,7 +6419,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="12">
@@ -6522,7 +6522,7 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>79.3%</t>
+          <t>78.9%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sync v4.5.6: T1->T3 carryover restored + CWBS_L alpha tightened
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -1951,10 +1951,10 @@
         </is>
       </c>
       <c r="B3" s="40" t="n">
-        <v>0.543</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="C3" s="40" t="n">
-        <v>0.499</v>
+        <v>0.497</v>
       </c>
       <c r="D3" s="40" t="inlineStr">
         <is>
@@ -1969,13 +1969,13 @@
         </is>
       </c>
       <c r="B4" s="40" t="n">
-        <v>30.636</v>
+        <v>30.623</v>
       </c>
       <c r="C4" s="40" t="n">
-        <v>4.537</v>
+        <v>4.613</v>
       </c>
       <c r="D4" s="40" t="n">
-        <v>0.031</v>
+        <v>0.015</v>
       </c>
       <c r="E4" s="40" t="inlineStr">
         <is>
@@ -1990,16 +1990,16 @@
         </is>
       </c>
       <c r="B5" s="40" t="n">
-        <v>2.307</v>
+        <v>2.314</v>
       </c>
       <c r="C5" s="40" t="n">
-        <v>1.45</v>
+        <v>1.466</v>
       </c>
       <c r="D5" s="40" t="n">
-        <v>0.002</v>
+        <v>-0.046</v>
       </c>
       <c r="E5" s="40" t="n">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="F5" s="40" t="inlineStr">
         <is>
@@ -2014,19 +2014,19 @@
         </is>
       </c>
       <c r="B6" s="40" t="n">
-        <v>3.289</v>
+        <v>3.299</v>
       </c>
       <c r="C6" s="40" t="n">
-        <v>1.088</v>
+        <v>1.085</v>
       </c>
       <c r="D6" s="40" t="n">
-        <v>0.061</v>
+        <v>0.082</v>
       </c>
       <c r="E6" s="40" t="n">
-        <v>-0.022</v>
+        <v>0.003</v>
       </c>
       <c r="F6" s="40" t="n">
-        <v>-0.046</v>
+        <v>-0.054</v>
       </c>
       <c r="G6" s="40" t="inlineStr">
         <is>
@@ -2041,22 +2041,22 @@
         </is>
       </c>
       <c r="B7" s="40" t="n">
-        <v>4.04</v>
+        <v>4.088</v>
       </c>
       <c r="C7" s="40" t="n">
-        <v>0.886</v>
+        <v>0.885</v>
       </c>
       <c r="D7" s="40" t="n">
-        <v>-0.027</v>
+        <v>-0.048</v>
       </c>
       <c r="E7" s="40" t="n">
-        <v>-0.003</v>
+        <v>-0.011</v>
       </c>
       <c r="F7" s="40" t="n">
-        <v>0.077</v>
+        <v>0.079</v>
       </c>
       <c r="G7" s="40" t="n">
-        <v>-0.003</v>
+        <v>0.005</v>
       </c>
       <c r="H7" s="39" t="inlineStr">
         <is>
@@ -2071,25 +2071,25 @@
         </is>
       </c>
       <c r="B8" s="40" t="n">
-        <v>4.931</v>
+        <v>4.891</v>
       </c>
       <c r="C8" s="40" t="n">
-        <v>0.956</v>
+        <v>0.964</v>
       </c>
       <c r="D8" s="40" t="n">
-        <v>-0.01</v>
+        <v>-0.005</v>
       </c>
       <c r="E8" s="40" t="n">
-        <v>0.006</v>
+        <v>-0.027</v>
       </c>
       <c r="F8" s="40" t="n">
-        <v>0.008</v>
+        <v>0.028</v>
       </c>
       <c r="G8" s="40" t="n">
-        <v>-0.108</v>
+        <v>-0.1</v>
       </c>
       <c r="H8" s="40" t="n">
-        <v>-0.37</v>
+        <v>-0.35</v>
       </c>
       <c r="I8" s="40" t="inlineStr">
         <is>
@@ -2104,28 +2104,28 @@
         </is>
       </c>
       <c r="B9" s="40" t="n">
-        <v>3.449</v>
+        <v>3.48</v>
       </c>
       <c r="C9" s="40" t="n">
-        <v>0.915</v>
+        <v>0.891</v>
       </c>
       <c r="D9" s="40" t="n">
-        <v>-0.08500000000000001</v>
+        <v>-0.043</v>
       </c>
       <c r="E9" s="40" t="n">
-        <v>0.008999999999999999</v>
+        <v>-0.036</v>
       </c>
       <c r="F9" s="40" t="n">
-        <v>0.038</v>
+        <v>0.107</v>
       </c>
       <c r="G9" s="40" t="n">
-        <v>-0.036</v>
+        <v>-0.046</v>
       </c>
       <c r="H9" s="40" t="n">
-        <v>-0.019</v>
+        <v>0.006</v>
       </c>
       <c r="I9" s="40" t="n">
-        <v>0.075</v>
+        <v>0.056</v>
       </c>
       <c r="J9" s="40" t="inlineStr">
         <is>
@@ -2140,31 +2140,31 @@
         </is>
       </c>
       <c r="B10" s="40" t="n">
-        <v>4.592</v>
+        <v>4.569</v>
       </c>
       <c r="C10" s="40" t="n">
-        <v>0.871</v>
+        <v>0.883</v>
       </c>
       <c r="D10" s="40" t="n">
-        <v>-0.082</v>
+        <v>-0.07199999999999999</v>
       </c>
       <c r="E10" s="40" t="n">
-        <v>-0.075</v>
+        <v>-0.099</v>
       </c>
       <c r="F10" s="40" t="n">
-        <v>-0.045</v>
+        <v>-0.102</v>
       </c>
       <c r="G10" s="40" t="n">
-        <v>-0.1</v>
+        <v>-0.066</v>
       </c>
       <c r="H10" s="40" t="n">
+        <v>-0.013</v>
+      </c>
+      <c r="I10" s="40" t="n">
+        <v>-0.039</v>
+      </c>
+      <c r="J10" s="40" t="n">
         <v>-0.043</v>
-      </c>
-      <c r="I10" s="40" t="n">
-        <v>-0.022</v>
-      </c>
-      <c r="J10" s="40" t="n">
-        <v>0.005</v>
       </c>
       <c r="K10" s="40" t="inlineStr">
         <is>
@@ -2179,34 +2179,34 @@
         </is>
       </c>
       <c r="B11" s="40" t="n">
-        <v>4.526</v>
+        <v>4.444</v>
       </c>
       <c r="C11" s="40" t="n">
-        <v>1.254</v>
+        <v>1.232</v>
       </c>
       <c r="D11" s="40" t="n">
-        <v>-0.032</v>
+        <v>-0.038</v>
       </c>
       <c r="E11" s="40" t="n">
-        <v>-0.005</v>
+        <v>-0.034</v>
       </c>
       <c r="F11" s="40" t="n">
-        <v>-0.034</v>
+        <v>-0.029</v>
       </c>
       <c r="G11" s="40" t="n">
-        <v>-0.055</v>
+        <v>-0.057</v>
       </c>
       <c r="H11" s="40" t="n">
-        <v>-0.513</v>
+        <v>-0.535</v>
       </c>
       <c r="I11" s="40" t="n">
-        <v>0.537</v>
+        <v>0.545</v>
       </c>
       <c r="J11" s="40" t="n">
-        <v>0.016</v>
+        <v>-0.011</v>
       </c>
       <c r="K11" s="40" t="n">
-        <v>-0.042</v>
+        <v>-0.021</v>
       </c>
       <c r="L11" s="40" t="inlineStr">
         <is>
@@ -2221,37 +2221,37 @@
         </is>
       </c>
       <c r="B12" s="40" t="n">
-        <v>3.035</v>
+        <v>3.068</v>
       </c>
       <c r="C12" s="40" t="n">
-        <v>1.206</v>
+        <v>1.173</v>
       </c>
       <c r="D12" s="40" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.017</v>
       </c>
       <c r="E12" s="40" t="n">
-        <v>-0.004</v>
+        <v>-0.022</v>
       </c>
       <c r="F12" s="40" t="n">
-        <v>-0.02</v>
+        <v>0.007</v>
       </c>
       <c r="G12" s="40" t="n">
-        <v>0.06</v>
+        <v>0.051</v>
       </c>
       <c r="H12" s="40" t="n">
-        <v>0.543</v>
+        <v>0.532</v>
       </c>
       <c r="I12" s="40" t="n">
-        <v>-0.531</v>
+        <v>-0.512</v>
       </c>
       <c r="J12" s="40" t="n">
-        <v>0.01</v>
+        <v>0.032</v>
       </c>
       <c r="K12" s="40" t="n">
-        <v>-0.061</v>
+        <v>-0.058</v>
       </c>
       <c r="L12" s="40" t="n">
-        <v>-0.45</v>
+        <v>-0.466</v>
       </c>
       <c r="M12" s="40" t="inlineStr">
         <is>
@@ -2266,40 +2266,40 @@
         </is>
       </c>
       <c r="B13" s="40" t="n">
-        <v>4.373</v>
+        <v>4.392</v>
       </c>
       <c r="C13" s="40" t="n">
-        <v>0.654</v>
+        <v>0.639</v>
       </c>
       <c r="D13" s="40" t="n">
         <v>0.045</v>
       </c>
       <c r="E13" s="40" t="n">
-        <v>-0.02</v>
+        <v>-0.016</v>
       </c>
       <c r="F13" s="40" t="n">
-        <v>-0.037</v>
+        <v>-0.002</v>
       </c>
       <c r="G13" s="40" t="n">
-        <v>-0.026</v>
+        <v>-0.017</v>
       </c>
       <c r="H13" s="40" t="n">
-        <v>0.064</v>
+        <v>0.053</v>
       </c>
       <c r="I13" s="40" t="n">
-        <v>-0.054</v>
+        <v>-0.066</v>
       </c>
       <c r="J13" s="40" t="n">
-        <v>-0.103</v>
+        <v>-0.118</v>
       </c>
       <c r="K13" s="40" t="n">
-        <v>-0.076</v>
+        <v>-0.068</v>
       </c>
       <c r="L13" s="40" t="n">
-        <v>-0.013</v>
+        <v>-0.03</v>
       </c>
       <c r="M13" s="40" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.045</v>
       </c>
       <c r="N13" s="40" t="inlineStr">
         <is>
@@ -2314,43 +2314,43 @@
         </is>
       </c>
       <c r="B14" s="40" t="n">
-        <v>4.516</v>
+        <v>4.52</v>
       </c>
       <c r="C14" s="40" t="n">
-        <v>0.783</v>
+        <v>0.779</v>
       </c>
       <c r="D14" s="40" t="n">
-        <v>-0.015</v>
+        <v>-0.026</v>
       </c>
       <c r="E14" s="40" t="n">
-        <v>-0.001</v>
+        <v>0</v>
       </c>
       <c r="F14" s="40" t="n">
-        <v>0.048</v>
+        <v>0.007</v>
       </c>
       <c r="G14" s="40" t="n">
-        <v>-0.083</v>
+        <v>-0.09</v>
       </c>
       <c r="H14" s="40" t="n">
-        <v>-0.437</v>
+        <v>-0.445</v>
       </c>
       <c r="I14" s="40" t="n">
-        <v>0.456</v>
+        <v>0.457</v>
       </c>
       <c r="J14" s="40" t="n">
-        <v>-0.03</v>
+        <v>-0.058</v>
       </c>
       <c r="K14" s="40" t="n">
-        <v>-0.046</v>
+        <v>-0.017</v>
       </c>
       <c r="L14" s="40" t="n">
-        <v>0.681</v>
+        <v>0.614</v>
       </c>
       <c r="M14" s="40" t="n">
-        <v>-0.59</v>
+        <v>-0.608</v>
       </c>
       <c r="N14" s="40" t="n">
-        <v>0.292</v>
+        <v>0.356</v>
       </c>
       <c r="O14" s="40" t="inlineStr">
         <is>
@@ -2365,46 +2365,46 @@
         </is>
       </c>
       <c r="B15" s="40" t="n">
-        <v>4.69</v>
+        <v>4.793</v>
       </c>
       <c r="C15" s="40" t="n">
-        <v>1.286</v>
+        <v>1.214</v>
       </c>
       <c r="D15" s="40" t="n">
-        <v>-0.033</v>
+        <v>-0.011</v>
       </c>
       <c r="E15" s="40" t="n">
-        <v>-0.063</v>
+        <v>-0.016</v>
       </c>
       <c r="F15" s="40" t="n">
-        <v>-0.037</v>
+        <v>-0.025</v>
       </c>
       <c r="G15" s="40" t="n">
-        <v>-0.077</v>
+        <v>-0.008999999999999999</v>
       </c>
       <c r="H15" s="40" t="n">
-        <v>-0.305</v>
+        <v>-0.34</v>
       </c>
       <c r="I15" s="40" t="n">
-        <v>0.365</v>
+        <v>0.375</v>
       </c>
       <c r="J15" s="40" t="n">
-        <v>-0.068</v>
+        <v>0.097</v>
       </c>
       <c r="K15" s="40" t="n">
-        <v>-0.024</v>
+        <v>-0.015</v>
       </c>
       <c r="L15" s="40" t="n">
-        <v>0.427</v>
+        <v>0.35</v>
       </c>
       <c r="M15" s="40" t="n">
-        <v>-0.333</v>
+        <v>-0.404</v>
       </c>
       <c r="N15" s="40" t="n">
-        <v>-0.032</v>
+        <v>-0.108</v>
       </c>
       <c r="O15" s="40" t="n">
-        <v>0.359</v>
+        <v>0.27</v>
       </c>
       <c r="P15" s="40" t="inlineStr">
         <is>
@@ -2419,60 +2419,60 @@
         </is>
       </c>
       <c r="B16" s="40" t="n">
-        <v>2.559</v>
+        <v>2.493</v>
       </c>
       <c r="C16" s="40" t="n">
-        <v>1.071</v>
+        <v>0.96</v>
       </c>
       <c r="D16" s="40" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.048</v>
       </c>
       <c r="E16" s="40" t="n">
-        <v>0.015</v>
+        <v>-0.006</v>
       </c>
       <c r="F16" s="40" t="n">
-        <v>-0.006</v>
+        <v>-0.064</v>
       </c>
       <c r="G16" s="40" t="n">
-        <v>0.015</v>
+        <v>0.024</v>
       </c>
       <c r="H16" s="40" t="n">
-        <v>0.282</v>
+        <v>0.21</v>
       </c>
       <c r="I16" s="40" t="n">
-        <v>-0.248</v>
+        <v>-0.235</v>
       </c>
       <c r="J16" s="40" t="n">
-        <v>0.023</v>
+        <v>-0.033</v>
       </c>
       <c r="K16" s="40" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.036</v>
       </c>
       <c r="L16" s="40" t="n">
-        <v>-0.332</v>
+        <v>-0.319</v>
       </c>
       <c r="M16" s="40" t="n">
         <v>0.334</v>
       </c>
       <c r="N16" s="40" t="n">
-        <v>-0.064</v>
+        <v>0.165</v>
       </c>
       <c r="O16" s="40" t="n">
-        <v>-0.325</v>
+        <v>-0.19</v>
       </c>
       <c r="P16" s="40" t="n">
-        <v>-0.444</v>
+        <v>-0.425</v>
       </c>
       <c r="Q16" s="40" t="inlineStr">
         <is>
-          <t>(0.82)</t>
+          <t>(0.78)</t>
         </is>
       </c>
     </row>
     <row r="17" ht="35" customHeight="1" s="45">
       <c r="A17" s="23" t="inlineStr">
         <is>
-          <t>Note. Values on the diagonal are Cronbach’s alpha coefficients where applicable. Correlations are zero-order correlations among observed study variables. Leadership variables were rated by followers at T1. OCBS and CWBS were rated by leaders at T3. N = 363. *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
+          <t>Note. Values on the diagonal are Cronbach’s alpha coefficients where applicable. Correlations are zero-order correlations among observed study variables. Leadership variables were rated by followers at T1. OCBS and CWBS were rated by leaders at T3. N = 361. *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -3714,7 +3714,7 @@
     <row r="28" ht="48" customHeight="1" s="45">
       <c r="A28" s="23" t="inlineStr">
         <is>
-          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 363; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.</t>
+          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 361; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -5812,7 +5812,7 @@
     <row r="2">
       <c r="A2" s="38" t="inlineStr">
         <is>
-          <t>N = 363</t>
+          <t>N = 361</t>
         </is>
       </c>
     </row>
@@ -5826,14 +5826,14 @@
     <row r="4">
       <c r="A4" s="38" t="inlineStr">
         <is>
-          <t>- Male: 197 (54.3%)</t>
+          <t>- Male: 201 (55.7%)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="38" t="inlineStr">
         <is>
-          <t>- Female: 166 (45.7%)</t>
+          <t>- Female: 160 (44.3%)</t>
         </is>
       </c>
     </row>
@@ -5848,21 +5848,21 @@
     <row r="8">
       <c r="A8" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 30.64, SD = 4.54</t>
+          <t>Age: M = 30.62, SD = 4.61</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="38" t="inlineStr">
         <is>
-          <t>Working years: M = 8.86, SD = 4.83</t>
+          <t>Working years: M = 8.79, SD = 4.77</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="38" t="inlineStr">
         <is>
-          <t>Tenure with current leader: M = 2.31, SD = 1.45</t>
+          <t>Tenure with current leader: M = 2.31, SD = 1.47</t>
         </is>
       </c>
     </row>
@@ -5870,11 +5870,11 @@
       <c r="A11" s="48" t="inlineStr">
         <is>
           <t>Interaction frequency with leader:
-  - Rarely (&lt;1/wk): 21 (5.8%)
-  - Sometimes (1-2/wk): 65 (17.9%)
-  - Often (3-4/wk): 114 (31.4%)
-  - Very often (~daily): 114 (31.4%)
-  - Multiple times/day: 49 (13.5%)</t>
+  - Rarely (&lt;1/wk): 20 (5.5%)
+  - Sometimes (1-2/wk): 63 (17.5%)
+  - Often (3-4/wk): 118 (32.7%)
+  - Very often (~daily): 109 (30.2%)
+  - Multiple times/day: 51 (14.1%)</t>
         </is>
       </c>
     </row>
@@ -5889,35 +5889,35 @@
     <row r="14">
       <c r="A14" s="38" t="inlineStr">
         <is>
-          <t>- High school: 20 (5.5%)</t>
+          <t>- High school: 19 (5.3%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 62 (17.1%)</t>
+          <t>- Some college / Associate: 64 (17.7%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 165 (45.5%)</t>
+          <t>- Bachelor: 165 (45.7%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="38" t="inlineStr">
         <is>
-          <t>- Master: 92 (25.3%)</t>
+          <t>- Master: 89 (24.7%)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="38" t="inlineStr">
         <is>
-          <t>- Doctorate: 20 (5.5%)</t>
+          <t>- Doctorate: 21 (5.8%)</t>
         </is>
       </c>
     </row>
@@ -5932,21 +5932,21 @@
     <row r="21">
       <c r="A21" s="38" t="inlineStr">
         <is>
-          <t>- Entry: 69 (19.0%)</t>
+          <t>- Entry: 72 (19.9%)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="38" t="inlineStr">
         <is>
-          <t>- Associate: 120 (33.1%)</t>
+          <t>- Associate: 118 (32.7%)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="38" t="inlineStr">
         <is>
-          <t>- Senior: 93 (25.6%)</t>
+          <t>- Senior: 92 (25.5%)</t>
         </is>
       </c>
     </row>
@@ -5960,7 +5960,7 @@
     <row r="25">
       <c r="A25" s="38" t="inlineStr">
         <is>
-          <t>- Director: 18 (5.0%)</t>
+          <t>- Director: 17 (4.7%)</t>
         </is>
       </c>
     </row>
@@ -5990,14 +5990,14 @@
     <row r="31">
       <c r="A31" s="38" t="inlineStr">
         <is>
-          <t>- Male: 46 (58.2%)</t>
+          <t>- Male: 51 (64.6%)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="38" t="inlineStr">
         <is>
-          <t>- Female: 33 (41.8%)</t>
+          <t>- Female: 28 (35.4%)</t>
         </is>
       </c>
     </row>
@@ -6012,7 +6012,7 @@
     <row r="35">
       <c r="A35" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 40.91, SD = 6.40</t>
+          <t>Age: M = 40.95, SD = 6.47</t>
         </is>
       </c>
     </row>
@@ -6026,14 +6026,14 @@
     <row r="37">
       <c r="A37" s="38" t="inlineStr">
         <is>
-          <t>Leadership tenure: M = 5.33, SD = 3.14</t>
+          <t>Leadership tenure: M = 5.40, SD = 2.73</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="38" t="inlineStr">
         <is>
-          <t>Span of control: M = 4.59, SD = 0.57</t>
+          <t>Span of control: M = 4.57, SD = 0.63</t>
         </is>
       </c>
     </row>
@@ -6055,21 +6055,21 @@
     <row r="42">
       <c r="A42" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 42 (53.2%)</t>
+          <t>- Bachelor: 40 (50.6%)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="38" t="inlineStr">
         <is>
-          <t>- Master: 23 (29.1%)</t>
+          <t>- Master: 26 (32.9%)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="38" t="inlineStr">
         <is>
-          <t>- Doctorate: 7 (8.9%)</t>
+          <t>- Doctorate: 6 (7.6%)</t>
         </is>
       </c>
     </row>
@@ -6389,7 +6389,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="9">
@@ -6419,7 +6419,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="12">
@@ -6522,7 +6522,7 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>78.9%</t>
+          <t>78.5%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sync v4.5.9: MCFA non-linear + CMV baselines perturbed
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -1686,28 +1686,28 @@
         </is>
       </c>
       <c r="D4" s="39" t="n">
-        <v>1331.2</v>
+        <v>1218.4</v>
       </c>
       <c r="E4" s="39" t="n">
         <v>547</v>
       </c>
       <c r="F4" s="39" t="n">
-        <v>0.9340000000000001</v>
+        <v>0.948</v>
       </c>
       <c r="G4" s="39" t="n">
-        <v>0.927</v>
+        <v>0.9419999999999999</v>
       </c>
       <c r="H4" s="39" t="n">
-        <v>0.051</v>
+        <v>0.046</v>
       </c>
       <c r="I4" s="39" t="n">
-        <v>0.043</v>
+        <v>0.04</v>
       </c>
       <c r="J4" s="39" t="n">
         <v>0.049</v>
       </c>
       <c r="K4" s="39" t="n">
-        <v>22587.9</v>
+        <v>22484.3</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" s="45">
@@ -1727,28 +1727,28 @@
         </is>
       </c>
       <c r="D5" s="39" t="n">
-        <v>1612.5</v>
+        <v>1547.2</v>
       </c>
       <c r="E5" s="39" t="n">
         <v>547</v>
       </c>
       <c r="F5" s="39" t="n">
-        <v>0.911</v>
+        <v>0.917</v>
       </c>
       <c r="G5" s="39" t="n">
-        <v>0.903</v>
+        <v>0.908</v>
       </c>
       <c r="H5" s="39" t="n">
-        <v>0.061</v>
+        <v>0.058</v>
       </c>
       <c r="I5" s="39" t="n">
-        <v>0.046</v>
+        <v>0.045</v>
       </c>
       <c r="J5" s="39" t="n">
-        <v>0.067</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="K5" s="39" t="n">
-        <v>22823.4</v>
+        <v>22802.5</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" s="45">
@@ -1768,28 +1768,28 @@
         </is>
       </c>
       <c r="D6" s="39" t="n">
-        <v>2123.7</v>
+        <v>1832.6</v>
       </c>
       <c r="E6" s="39" t="n">
         <v>552</v>
       </c>
       <c r="F6" s="39" t="n">
-        <v>0.864</v>
+        <v>0.892</v>
       </c>
       <c r="G6" s="39" t="n">
-        <v>0.851</v>
+        <v>0.88</v>
       </c>
       <c r="H6" s="39" t="n">
-        <v>0.073</v>
+        <v>0.066</v>
       </c>
       <c r="I6" s="39" t="n">
-        <v>0.054</v>
+        <v>0.052</v>
       </c>
       <c r="J6" s="39" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.075</v>
       </c>
       <c r="K6" s="39" t="n">
-        <v>23218.6</v>
+        <v>23078.2</v>
       </c>
     </row>
     <row r="7">
@@ -6207,22 +6207,22 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>1156.8</v>
+        <v>1148.3</v>
       </c>
       <c r="C3" s="13" t="n">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="D3" s="13" t="n">
-        <v>0.954</v>
+        <v>0.956</v>
       </c>
       <c r="E3" s="13" t="n">
-        <v>0.949</v>
+        <v>0.95</v>
       </c>
       <c r="F3" s="13" t="n">
-        <v>0.042</v>
+        <v>0.041</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.037</v>
+        <v>0.036</v>
       </c>
       <c r="H3" s="13" t="n"/>
       <c r="I3" s="13" t="n"/>
@@ -6239,25 +6239,25 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>1118.3</v>
+        <v>1109.6</v>
       </c>
       <c r="C4" s="13" t="n">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="D4" s="13" t="n">
-        <v>0.958</v>
+        <v>0.961</v>
       </c>
       <c r="E4" s="13" t="n">
-        <v>0.951</v>
+        <v>0.953</v>
       </c>
       <c r="F4" s="13" t="n">
-        <v>0.041</v>
+        <v>0.04</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.036</v>
+        <v>0.035</v>
       </c>
       <c r="H4" s="13" t="n">
-        <v>0.004</v>
+        <v>0.005</v>
       </c>
       <c r="I4" s="13" t="n">
         <v>-0.001</v>

</xml_diff>

<commit_message>
sync v4.5.11+v4.5.12: significance stars on Path/Correlation/简单调节/被调节中介
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -1998,8 +1998,10 @@
       <c r="D5" s="40" t="n">
         <v>-0.046</v>
       </c>
-      <c r="E5" s="40" t="n">
-        <v>0.22</v>
+      <c r="E5" s="40" t="inlineStr">
+        <is>
+          <t>0.22***</t>
+        </is>
       </c>
       <c r="F5" s="40" t="inlineStr">
         <is>
@@ -2088,8 +2090,10 @@
       <c r="G8" s="40" t="n">
         <v>-0.1</v>
       </c>
-      <c r="H8" s="40" t="n">
-        <v>-0.35</v>
+      <c r="H8" s="40" t="inlineStr">
+        <is>
+          <t>-0.35***</t>
+        </is>
       </c>
       <c r="I8" s="40" t="inlineStr">
         <is>
@@ -2115,8 +2119,10 @@
       <c r="E9" s="40" t="n">
         <v>-0.036</v>
       </c>
-      <c r="F9" s="40" t="n">
-        <v>0.107</v>
+      <c r="F9" s="40" t="inlineStr">
+        <is>
+          <t>0.107*</t>
+        </is>
       </c>
       <c r="G9" s="40" t="n">
         <v>-0.046</v>
@@ -2196,11 +2202,15 @@
       <c r="G11" s="40" t="n">
         <v>-0.057</v>
       </c>
-      <c r="H11" s="40" t="n">
-        <v>-0.535</v>
-      </c>
-      <c r="I11" s="40" t="n">
-        <v>0.545</v>
+      <c r="H11" s="40" t="inlineStr">
+        <is>
+          <t>-0.535***</t>
+        </is>
+      </c>
+      <c r="I11" s="40" t="inlineStr">
+        <is>
+          <t>0.545***</t>
+        </is>
       </c>
       <c r="J11" s="40" t="n">
         <v>-0.011</v>
@@ -2238,11 +2248,15 @@
       <c r="G12" s="40" t="n">
         <v>0.051</v>
       </c>
-      <c r="H12" s="40" t="n">
-        <v>0.532</v>
-      </c>
-      <c r="I12" s="40" t="n">
-        <v>-0.512</v>
+      <c r="H12" s="40" t="inlineStr">
+        <is>
+          <t>0.532***</t>
+        </is>
+      </c>
+      <c r="I12" s="40" t="inlineStr">
+        <is>
+          <t>-0.512***</t>
+        </is>
       </c>
       <c r="J12" s="40" t="n">
         <v>0.032</v>
@@ -2250,8 +2264,10 @@
       <c r="K12" s="40" t="n">
         <v>-0.058</v>
       </c>
-      <c r="L12" s="40" t="n">
-        <v>-0.466</v>
+      <c r="L12" s="40" t="inlineStr">
+        <is>
+          <t>-0.466***</t>
+        </is>
       </c>
       <c r="M12" s="40" t="inlineStr">
         <is>
@@ -2289,8 +2305,10 @@
       <c r="I13" s="40" t="n">
         <v>-0.066</v>
       </c>
-      <c r="J13" s="40" t="n">
-        <v>-0.118</v>
+      <c r="J13" s="40" t="inlineStr">
+        <is>
+          <t>-0.118*</t>
+        </is>
       </c>
       <c r="K13" s="40" t="n">
         <v>-0.068</v>
@@ -2331,11 +2349,15 @@
       <c r="G14" s="40" t="n">
         <v>-0.09</v>
       </c>
-      <c r="H14" s="40" t="n">
-        <v>-0.445</v>
-      </c>
-      <c r="I14" s="40" t="n">
-        <v>0.457</v>
+      <c r="H14" s="40" t="inlineStr">
+        <is>
+          <t>-0.445***</t>
+        </is>
+      </c>
+      <c r="I14" s="40" t="inlineStr">
+        <is>
+          <t>0.457***</t>
+        </is>
       </c>
       <c r="J14" s="40" t="n">
         <v>-0.058</v>
@@ -2343,14 +2365,20 @@
       <c r="K14" s="40" t="n">
         <v>-0.017</v>
       </c>
-      <c r="L14" s="40" t="n">
-        <v>0.614</v>
-      </c>
-      <c r="M14" s="40" t="n">
-        <v>-0.608</v>
-      </c>
-      <c r="N14" s="40" t="n">
-        <v>0.356</v>
+      <c r="L14" s="40" t="inlineStr">
+        <is>
+          <t>0.614***</t>
+        </is>
+      </c>
+      <c r="M14" s="40" t="inlineStr">
+        <is>
+          <t>-0.608***</t>
+        </is>
+      </c>
+      <c r="N14" s="40" t="inlineStr">
+        <is>
+          <t>0.356***</t>
+        </is>
       </c>
       <c r="O14" s="40" t="inlineStr">
         <is>
@@ -2382,11 +2410,15 @@
       <c r="G15" s="40" t="n">
         <v>-0.008999999999999999</v>
       </c>
-      <c r="H15" s="40" t="n">
-        <v>-0.34</v>
-      </c>
-      <c r="I15" s="40" t="n">
-        <v>0.375</v>
+      <c r="H15" s="40" t="inlineStr">
+        <is>
+          <t>-0.34***</t>
+        </is>
+      </c>
+      <c r="I15" s="40" t="inlineStr">
+        <is>
+          <t>0.375***</t>
+        </is>
       </c>
       <c r="J15" s="40" t="n">
         <v>0.097</v>
@@ -2394,17 +2426,25 @@
       <c r="K15" s="40" t="n">
         <v>-0.015</v>
       </c>
-      <c r="L15" s="40" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="M15" s="40" t="n">
-        <v>-0.404</v>
-      </c>
-      <c r="N15" s="40" t="n">
-        <v>-0.108</v>
-      </c>
-      <c r="O15" s="40" t="n">
-        <v>0.27</v>
+      <c r="L15" s="40" t="inlineStr">
+        <is>
+          <t>0.35***</t>
+        </is>
+      </c>
+      <c r="M15" s="40" t="inlineStr">
+        <is>
+          <t>-0.404***</t>
+        </is>
+      </c>
+      <c r="N15" s="40" t="inlineStr">
+        <is>
+          <t>-0.108*</t>
+        </is>
+      </c>
+      <c r="O15" s="40" t="inlineStr">
+        <is>
+          <t>0.27***</t>
+        </is>
       </c>
       <c r="P15" s="40" t="inlineStr">
         <is>
@@ -2436,11 +2476,15 @@
       <c r="G16" s="40" t="n">
         <v>0.024</v>
       </c>
-      <c r="H16" s="40" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="I16" s="40" t="n">
-        <v>-0.235</v>
+      <c r="H16" s="40" t="inlineStr">
+        <is>
+          <t>0.21***</t>
+        </is>
+      </c>
+      <c r="I16" s="40" t="inlineStr">
+        <is>
+          <t>-0.235***</t>
+        </is>
       </c>
       <c r="J16" s="40" t="n">
         <v>-0.033</v>
@@ -2448,20 +2492,30 @@
       <c r="K16" s="40" t="n">
         <v>0.036</v>
       </c>
-      <c r="L16" s="40" t="n">
-        <v>-0.319</v>
-      </c>
-      <c r="M16" s="40" t="n">
-        <v>0.334</v>
-      </c>
-      <c r="N16" s="40" t="n">
-        <v>0.165</v>
-      </c>
-      <c r="O16" s="40" t="n">
-        <v>-0.19</v>
-      </c>
-      <c r="P16" s="40" t="n">
-        <v>-0.425</v>
+      <c r="L16" s="40" t="inlineStr">
+        <is>
+          <t>-0.319***</t>
+        </is>
+      </c>
+      <c r="M16" s="40" t="inlineStr">
+        <is>
+          <t>0.334***</t>
+        </is>
+      </c>
+      <c r="N16" s="40" t="inlineStr">
+        <is>
+          <t>0.165**</t>
+        </is>
+      </c>
+      <c r="O16" s="40" t="inlineStr">
+        <is>
+          <t>-0.19***</t>
+        </is>
+      </c>
+      <c r="P16" s="40" t="inlineStr">
+        <is>
+          <t>-0.425***</t>
+        </is>
       </c>
       <c r="Q16" s="40" t="inlineStr">
         <is>
@@ -2660,44 +2714,58 @@
           <t>Intercept</t>
         </is>
       </c>
-      <c r="B5" s="40" t="n">
-        <v>3.821</v>
+      <c r="B5" s="40" t="inlineStr">
+        <is>
+          <t>3.821***</t>
+        </is>
       </c>
       <c r="C5" s="40" t="n">
         <v>0.094</v>
       </c>
-      <c r="D5" s="40" t="n">
-        <v>3.821</v>
+      <c r="D5" s="40" t="inlineStr">
+        <is>
+          <t>3.821***</t>
+        </is>
       </c>
       <c r="E5" s="40" t="n">
         <v>0.094</v>
       </c>
-      <c r="F5" s="40" t="n">
-        <v>3.821</v>
+      <c r="F5" s="40" t="inlineStr">
+        <is>
+          <t>3.821***</t>
+        </is>
       </c>
       <c r="G5" s="40" t="n">
         <v>0.094</v>
       </c>
-      <c r="H5" s="40" t="n">
-        <v>3.821</v>
+      <c r="H5" s="40" t="inlineStr">
+        <is>
+          <t>3.821***</t>
+        </is>
       </c>
       <c r="I5" s="40" t="n">
         <v>0.094</v>
       </c>
-      <c r="J5" s="40" t="n">
-        <v>3.821</v>
+      <c r="J5" s="40" t="inlineStr">
+        <is>
+          <t>3.821***</t>
+        </is>
       </c>
       <c r="K5" s="40" t="n">
         <v>0.094</v>
       </c>
-      <c r="L5" s="40" t="n">
-        <v>3.821</v>
+      <c r="L5" s="40" t="inlineStr">
+        <is>
+          <t>3.821***</t>
+        </is>
       </c>
       <c r="M5" s="40" t="n">
         <v>0.094</v>
       </c>
-      <c r="N5" s="40" t="n">
-        <v>3.821</v>
+      <c r="N5" s="40" t="inlineStr">
+        <is>
+          <t>3.821***</t>
+        </is>
       </c>
       <c r="O5" s="40" t="n">
         <v>0.094</v>
@@ -2877,44 +2945,58 @@
           <t xml:space="preserve">Interaction frequency with leader </t>
         </is>
       </c>
-      <c r="B10" s="40" t="n">
-        <v>0.08699999999999999</v>
+      <c r="B10" s="40" t="inlineStr">
+        <is>
+          <t>0.087*</t>
+        </is>
       </c>
       <c r="C10" s="40" t="n">
         <v>0.034</v>
       </c>
-      <c r="D10" s="40" t="n">
-        <v>0.08699999999999999</v>
+      <c r="D10" s="40" t="inlineStr">
+        <is>
+          <t>0.087*</t>
+        </is>
       </c>
       <c r="E10" s="40" t="n">
         <v>0.034</v>
       </c>
-      <c r="F10" s="40" t="n">
-        <v>0.08699999999999999</v>
+      <c r="F10" s="40" t="inlineStr">
+        <is>
+          <t>0.087*</t>
+        </is>
       </c>
       <c r="G10" s="40" t="n">
         <v>0.034</v>
       </c>
-      <c r="H10" s="40" t="n">
-        <v>0.08699999999999999</v>
+      <c r="H10" s="40" t="inlineStr">
+        <is>
+          <t>0.087*</t>
+        </is>
       </c>
       <c r="I10" s="40" t="n">
         <v>0.034</v>
       </c>
-      <c r="J10" s="40" t="n">
-        <v>0.08699999999999999</v>
+      <c r="J10" s="40" t="inlineStr">
+        <is>
+          <t>0.087*</t>
+        </is>
       </c>
       <c r="K10" s="40" t="n">
         <v>0.034</v>
       </c>
-      <c r="L10" s="40" t="n">
-        <v>0.08699999999999999</v>
+      <c r="L10" s="40" t="inlineStr">
+        <is>
+          <t>0.087*</t>
+        </is>
       </c>
       <c r="M10" s="40" t="n">
         <v>0.034</v>
       </c>
-      <c r="N10" s="40" t="n">
-        <v>0.08699999999999999</v>
+      <c r="N10" s="40" t="inlineStr">
+        <is>
+          <t>0.087*</t>
+        </is>
       </c>
       <c r="O10" s="40" t="n">
         <v>0.034</v>
@@ -2926,44 +3008,58 @@
           <t>Thriving (T1) baseline</t>
         </is>
       </c>
-      <c r="B11" s="40" t="n">
-        <v>0.412</v>
+      <c r="B11" s="40" t="inlineStr">
+        <is>
+          <t>0.412***</t>
+        </is>
       </c>
       <c r="C11" s="40" t="n">
         <v>0.048</v>
       </c>
-      <c r="D11" s="40" t="n">
-        <v>0.412</v>
+      <c r="D11" s="40" t="inlineStr">
+        <is>
+          <t>0.412***</t>
+        </is>
       </c>
       <c r="E11" s="40" t="n">
         <v>0.048</v>
       </c>
-      <c r="F11" s="40" t="n">
-        <v>0.412</v>
+      <c r="F11" s="40" t="inlineStr">
+        <is>
+          <t>0.412***</t>
+        </is>
       </c>
       <c r="G11" s="40" t="n">
         <v>0.048</v>
       </c>
-      <c r="H11" s="40" t="n">
-        <v>0.412</v>
+      <c r="H11" s="40" t="inlineStr">
+        <is>
+          <t>0.412***</t>
+        </is>
       </c>
       <c r="I11" s="40" t="n">
         <v>0.048</v>
       </c>
-      <c r="J11" s="40" t="n">
-        <v>0.412</v>
+      <c r="J11" s="40" t="inlineStr">
+        <is>
+          <t>0.412***</t>
+        </is>
       </c>
       <c r="K11" s="40" t="n">
         <v>0.048</v>
       </c>
-      <c r="L11" s="40" t="n">
-        <v>0.412</v>
+      <c r="L11" s="40" t="inlineStr">
+        <is>
+          <t>0.412***</t>
+        </is>
       </c>
       <c r="M11" s="40" t="n">
         <v>0.048</v>
       </c>
-      <c r="N11" s="40" t="n">
-        <v>0.412</v>
+      <c r="N11" s="40" t="inlineStr">
+        <is>
+          <t>0.412***</t>
+        </is>
       </c>
       <c r="O11" s="40" t="n">
         <v>0.048</v>
@@ -2996,44 +3092,58 @@
           <t>Autocratic leadership (T1, follower-rated)</t>
         </is>
       </c>
-      <c r="B13" s="40" t="n">
-        <v>-0.142</v>
+      <c r="B13" s="40" t="inlineStr">
+        <is>
+          <t>-0.142**</t>
+        </is>
       </c>
       <c r="C13" s="40" t="n">
         <v>0.052</v>
       </c>
-      <c r="D13" s="40" t="n">
-        <v>-0.14</v>
+      <c r="D13" s="40" t="inlineStr">
+        <is>
+          <t>-0.14**</t>
+        </is>
       </c>
       <c r="E13" s="40" t="n">
         <v>0.052</v>
       </c>
-      <c r="F13" s="40" t="n">
-        <v>0.312</v>
+      <c r="F13" s="40" t="inlineStr">
+        <is>
+          <t>0.312***</t>
+        </is>
       </c>
       <c r="G13" s="40" t="n">
         <v>0.058</v>
       </c>
-      <c r="H13" s="40" t="n">
-        <v>0.309</v>
+      <c r="H13" s="40" t="inlineStr">
+        <is>
+          <t>0.309***</t>
+        </is>
       </c>
       <c r="I13" s="40" t="n">
         <v>0.058</v>
       </c>
-      <c r="J13" s="40" t="n">
-        <v>-0.082</v>
+      <c r="J13" s="40" t="inlineStr">
+        <is>
+          <t>-0.082*</t>
+        </is>
       </c>
       <c r="K13" s="40" t="n">
         <v>0.041</v>
       </c>
-      <c r="L13" s="40" t="n">
-        <v>-0.067</v>
+      <c r="L13" s="40" t="inlineStr">
+        <is>
+          <t>-0.067†</t>
+        </is>
       </c>
       <c r="M13" s="40" t="n">
         <v>0.04</v>
       </c>
-      <c r="N13" s="40" t="n">
-        <v>0.103</v>
+      <c r="N13" s="40" t="inlineStr">
+        <is>
+          <t>0.103*</t>
+        </is>
       </c>
       <c r="O13" s="40" t="n">
         <v>0.044</v>
@@ -3045,44 +3155,58 @@
           <t>Empowering leadership (T1, follower-rated)</t>
         </is>
       </c>
-      <c r="B14" s="40" t="n">
-        <v>0.267</v>
+      <c r="B14" s="40" t="inlineStr">
+        <is>
+          <t>0.267***</t>
+        </is>
       </c>
       <c r="C14" s="40" t="n">
         <v>0.049</v>
       </c>
-      <c r="D14" s="40" t="n">
-        <v>0.26</v>
+      <c r="D14" s="40" t="inlineStr">
+        <is>
+          <t>0.26***</t>
+        </is>
       </c>
       <c r="E14" s="40" t="n">
         <v>0.049</v>
       </c>
-      <c r="F14" s="40" t="n">
-        <v>-0.145</v>
+      <c r="F14" s="40" t="inlineStr">
+        <is>
+          <t>-0.145**</t>
+        </is>
       </c>
       <c r="G14" s="40" t="n">
         <v>0.052</v>
       </c>
-      <c r="H14" s="40" t="n">
-        <v>-0.14</v>
+      <c r="H14" s="40" t="inlineStr">
+        <is>
+          <t>-0.14**</t>
+        </is>
       </c>
       <c r="I14" s="40" t="n">
         <v>0.052</v>
       </c>
-      <c r="J14" s="40" t="n">
-        <v>0.118</v>
+      <c r="J14" s="40" t="inlineStr">
+        <is>
+          <t>0.118**</t>
+        </is>
       </c>
       <c r="K14" s="40" t="n">
         <v>0.043</v>
       </c>
-      <c r="L14" s="40" t="n">
-        <v>0.094</v>
+      <c r="L14" s="40" t="inlineStr">
+        <is>
+          <t>0.094*</t>
+        </is>
       </c>
       <c r="M14" s="40" t="n">
         <v>0.041</v>
       </c>
-      <c r="N14" s="40" t="n">
-        <v>-0.07099999999999999</v>
+      <c r="N14" s="40" t="inlineStr">
+        <is>
+          <t>-0.071†</t>
+        </is>
       </c>
       <c r="O14" s="40" t="n">
         <v>0.04</v>
@@ -3155,20 +3279,26 @@
           <t>—</t>
         </is>
       </c>
-      <c r="J16" s="40" t="n">
-        <v>0.234</v>
+      <c r="J16" s="40" t="inlineStr">
+        <is>
+          <t>0.234***</t>
+        </is>
       </c>
       <c r="K16" s="40" t="n">
         <v>0.046</v>
       </c>
-      <c r="L16" s="40" t="n">
-        <v>0.203</v>
+      <c r="L16" s="40" t="inlineStr">
+        <is>
+          <t>0.203***</t>
+        </is>
       </c>
       <c r="M16" s="40" t="n">
         <v>0.048</v>
       </c>
-      <c r="N16" s="40" t="n">
-        <v>-0.112</v>
+      <c r="N16" s="40" t="inlineStr">
+        <is>
+          <t>-0.112*</t>
+        </is>
       </c>
       <c r="O16" s="40" t="n">
         <v>0.044</v>
@@ -3220,20 +3350,26 @@
           <t>—</t>
         </is>
       </c>
-      <c r="J17" s="40" t="n">
-        <v>-0.198</v>
+      <c r="J17" s="40" t="inlineStr">
+        <is>
+          <t>-0.198***</t>
+        </is>
       </c>
       <c r="K17" s="40" t="n">
         <v>0.051</v>
       </c>
-      <c r="L17" s="40" t="n">
-        <v>-0.156</v>
+      <c r="L17" s="40" t="inlineStr">
+        <is>
+          <t>-0.156**</t>
+        </is>
       </c>
       <c r="M17" s="40" t="n">
         <v>0.053</v>
       </c>
-      <c r="N17" s="40" t="n">
-        <v>0.278</v>
+      <c r="N17" s="40" t="inlineStr">
+        <is>
+          <t>0.278***</t>
+        </is>
       </c>
       <c r="O17" s="40" t="n">
         <v>0.055</v>
@@ -3266,44 +3402,58 @@
           <t>Narcissism (T1)</t>
         </is>
       </c>
-      <c r="B19" s="40" t="n">
-        <v>-0.118</v>
+      <c r="B19" s="40" t="inlineStr">
+        <is>
+          <t>-0.118*</t>
+        </is>
       </c>
       <c r="C19" s="40" t="n">
         <v>0.046</v>
       </c>
-      <c r="D19" s="40" t="n">
-        <v>-0.118</v>
+      <c r="D19" s="40" t="inlineStr">
+        <is>
+          <t>-0.118*</t>
+        </is>
       </c>
       <c r="E19" s="40" t="n">
         <v>0.046</v>
       </c>
-      <c r="F19" s="40" t="n">
-        <v>0.214</v>
+      <c r="F19" s="40" t="inlineStr">
+        <is>
+          <t>0.214***</t>
+        </is>
       </c>
       <c r="G19" s="40" t="n">
         <v>0.047</v>
       </c>
-      <c r="H19" s="40" t="n">
-        <v>0.214</v>
+      <c r="H19" s="40" t="inlineStr">
+        <is>
+          <t>0.214***</t>
+        </is>
       </c>
       <c r="I19" s="40" t="n">
         <v>0.047</v>
       </c>
-      <c r="J19" s="40" t="n">
-        <v>-0.118</v>
+      <c r="J19" s="40" t="inlineStr">
+        <is>
+          <t>-0.118*</t>
+        </is>
       </c>
       <c r="K19" s="40" t="n">
         <v>0.046</v>
       </c>
-      <c r="L19" s="40" t="n">
-        <v>-0.118</v>
+      <c r="L19" s="40" t="inlineStr">
+        <is>
+          <t>-0.118*</t>
+        </is>
       </c>
       <c r="M19" s="40" t="n">
         <v>0.046</v>
       </c>
-      <c r="N19" s="40" t="n">
-        <v>-0.118</v>
+      <c r="N19" s="40" t="inlineStr">
+        <is>
+          <t>-0.118*</t>
+        </is>
       </c>
       <c r="O19" s="40" t="n">
         <v>0.046</v>
@@ -3327,14 +3477,18 @@
       <c r="E20" s="40" t="n">
         <v>0.039</v>
       </c>
-      <c r="F20" s="40" t="n">
-        <v>0.135</v>
+      <c r="F20" s="40" t="inlineStr">
+        <is>
+          <t>0.135**</t>
+        </is>
       </c>
       <c r="G20" s="40" t="n">
         <v>0.045</v>
       </c>
-      <c r="H20" s="40" t="n">
-        <v>0.135</v>
+      <c r="H20" s="40" t="inlineStr">
+        <is>
+          <t>0.135**</t>
+        </is>
       </c>
       <c r="I20" s="40" t="n">
         <v>0.045</v>
@@ -3549,8 +3703,10 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H24" s="40" t="n">
-        <v>-0.111</v>
+      <c r="H24" s="40" t="inlineStr">
+        <is>
+          <t>-0.111**</t>
+        </is>
       </c>
       <c r="I24" s="40" t="n">
         <v>0.039</v>
@@ -3602,8 +3758,10 @@
           <t>—</t>
         </is>
       </c>
-      <c r="D25" s="40" t="n">
-        <v>-0.098</v>
+      <c r="D25" s="40" t="inlineStr">
+        <is>
+          <t>-0.098*</t>
+        </is>
       </c>
       <c r="E25" s="40" t="n">
         <v>0.045</v>
@@ -3714,7 +3872,7 @@
     <row r="28" ht="48" customHeight="1" s="45">
       <c r="A28" s="23" t="inlineStr">
         <is>
-          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 361; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.</t>
+          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 361; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.  *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -3869,24 +4027,30 @@
           <t>Mediation</t>
         </is>
       </c>
-      <c r="B7" s="30" t="n">
-        <v>-0.033</v>
+      <c r="B7" s="30" t="inlineStr">
+        <is>
+          <t>-0.033*</t>
+        </is>
       </c>
       <c r="C7" s="30" t="inlineStr">
         <is>
           <t>[-0.063, -0.012]</t>
         </is>
       </c>
-      <c r="D7" s="30" t="n">
-        <v>-0.029</v>
+      <c r="D7" s="30" t="inlineStr">
+        <is>
+          <t>-0.029*</t>
+        </is>
       </c>
       <c r="E7" s="30" t="inlineStr">
         <is>
           <t>[-0.056, -0.010]</t>
         </is>
       </c>
-      <c r="F7" s="30" t="n">
-        <v>0.016</v>
+      <c r="F7" s="30" t="inlineStr">
+        <is>
+          <t>0.016*</t>
+        </is>
       </c>
       <c r="G7" s="30" t="inlineStr">
         <is>
@@ -4050,16 +4214,20 @@
           <t>Low power distance (−1 SD)</t>
         </is>
       </c>
-      <c r="B14" s="30" t="n">
-        <v>-0.053</v>
+      <c r="B14" s="30" t="inlineStr">
+        <is>
+          <t>-0.053*</t>
+        </is>
       </c>
       <c r="C14" s="30" t="inlineStr">
         <is>
           <t>[-0.099, -0.007]</t>
         </is>
       </c>
-      <c r="D14" s="30" t="n">
-        <v>-0.046</v>
+      <c r="D14" s="30" t="inlineStr">
+        <is>
+          <t>-0.046*</t>
+        </is>
       </c>
       <c r="E14" s="30" t="inlineStr">
         <is>
@@ -4081,8 +4249,10 @@
           <t>Difference</t>
         </is>
       </c>
-      <c r="B15" s="30" t="n">
-        <v>0.04</v>
+      <c r="B15" s="30" t="inlineStr">
+        <is>
+          <t>0.04*</t>
+        </is>
       </c>
       <c r="C15" s="30" t="inlineStr">
         <is>
@@ -4125,24 +4295,30 @@
           <t>Mediation</t>
         </is>
       </c>
-      <c r="B17" s="32" t="n">
-        <v>0.062</v>
+      <c r="B17" s="32" t="inlineStr">
+        <is>
+          <t>0.062*</t>
+        </is>
       </c>
       <c r="C17" s="32" t="inlineStr">
         <is>
           <t>[0.034, 0.094]</t>
         </is>
       </c>
-      <c r="D17" s="32" t="n">
-        <v>0.054</v>
+      <c r="D17" s="32" t="inlineStr">
+        <is>
+          <t>0.054*</t>
+        </is>
       </c>
       <c r="E17" s="32" t="inlineStr">
         <is>
           <t>[0.028, 0.084]</t>
         </is>
       </c>
-      <c r="F17" s="32" t="n">
-        <v>-0.03</v>
+      <c r="F17" s="32" t="inlineStr">
+        <is>
+          <t>-0.03*</t>
+        </is>
       </c>
       <c r="G17" s="32" t="inlineStr">
         <is>
@@ -4169,16 +4345,20 @@
           <t>High narcissism (+1 SD)</t>
         </is>
       </c>
-      <c r="B19" s="32" t="n">
-        <v>0.066</v>
+      <c r="B19" s="32" t="inlineStr">
+        <is>
+          <t>0.066*</t>
+        </is>
       </c>
       <c r="C19" s="32" t="inlineStr">
         <is>
           <t>[0.014, 0.118]</t>
         </is>
       </c>
-      <c r="D19" s="32" t="n">
-        <v>0.058</v>
+      <c r="D19" s="32" t="inlineStr">
+        <is>
+          <t>0.058*</t>
+        </is>
       </c>
       <c r="E19" s="32" t="inlineStr">
         <is>
@@ -4200,16 +4380,20 @@
           <t>Low narcissism (−1 SD)</t>
         </is>
       </c>
-      <c r="B20" s="32" t="n">
-        <v>0.058</v>
+      <c r="B20" s="32" t="inlineStr">
+        <is>
+          <t>0.058*</t>
+        </is>
       </c>
       <c r="C20" s="32" t="inlineStr">
         <is>
           <t>[0.010, 0.106]</t>
         </is>
       </c>
-      <c r="D20" s="32" t="n">
-        <v>0.05</v>
+      <c r="D20" s="32" t="inlineStr">
+        <is>
+          <t>0.05*</t>
+        </is>
       </c>
       <c r="E20" s="32" t="inlineStr">
         <is>
@@ -4293,24 +4477,30 @@
           <t>Low power distance (−1 SD)</t>
         </is>
       </c>
-      <c r="B23" s="32" t="n">
-        <v>0.08799999999999999</v>
+      <c r="B23" s="32" t="inlineStr">
+        <is>
+          <t>0.088*</t>
+        </is>
       </c>
       <c r="C23" s="32" t="inlineStr">
         <is>
           <t>[0.025, 0.151]</t>
         </is>
       </c>
-      <c r="D23" s="32" t="n">
-        <v>0.077</v>
+      <c r="D23" s="32" t="inlineStr">
+        <is>
+          <t>0.077*</t>
+        </is>
       </c>
       <c r="E23" s="32" t="inlineStr">
         <is>
           <t>[0.020, 0.134]</t>
         </is>
       </c>
-      <c r="F23" s="32" t="n">
-        <v>-0.043</v>
+      <c r="F23" s="32" t="inlineStr">
+        <is>
+          <t>-0.043*</t>
+        </is>
       </c>
       <c r="G23" s="32" t="inlineStr">
         <is>
@@ -4324,16 +4514,20 @@
           <t>Difference</t>
         </is>
       </c>
-      <c r="B24" s="32" t="n">
-        <v>-0.052</v>
+      <c r="B24" s="32" t="inlineStr">
+        <is>
+          <t>-0.052*</t>
+        </is>
       </c>
       <c r="C24" s="32" t="inlineStr">
         <is>
           <t>[-0.097, -0.007]</t>
         </is>
       </c>
-      <c r="D24" s="32" t="n">
-        <v>-0.046</v>
+      <c r="D24" s="32" t="inlineStr">
+        <is>
+          <t>-0.046*</t>
+        </is>
       </c>
       <c r="E24" s="32" t="inlineStr">
         <is>
@@ -4381,24 +4575,30 @@
           <t>Indirect effect</t>
         </is>
       </c>
-      <c r="B27" s="34" t="n">
-        <v>-0.062</v>
+      <c r="B27" s="34" t="inlineStr">
+        <is>
+          <t>-0.062*</t>
+        </is>
       </c>
       <c r="C27" s="34" t="inlineStr">
         <is>
           <t>[-0.098, -0.034]</t>
         </is>
       </c>
-      <c r="D27" s="34" t="n">
-        <v>-0.049</v>
+      <c r="D27" s="34" t="inlineStr">
+        <is>
+          <t>-0.049*</t>
+        </is>
       </c>
       <c r="E27" s="34" t="inlineStr">
         <is>
           <t>[-0.082, -0.024]</t>
         </is>
       </c>
-      <c r="F27" s="34" t="n">
-        <v>0.08699999999999999</v>
+      <c r="F27" s="34" t="inlineStr">
+        <is>
+          <t>0.087*</t>
+        </is>
       </c>
       <c r="G27" s="34" t="inlineStr">
         <is>
@@ -4412,24 +4612,30 @@
           <t>High narcissism (+1 SD)</t>
         </is>
       </c>
-      <c r="B28" s="34" t="n">
-        <v>-0.067</v>
+      <c r="B28" s="34" t="inlineStr">
+        <is>
+          <t>-0.067*</t>
+        </is>
       </c>
       <c r="C28" s="34" t="inlineStr">
         <is>
           <t>[-0.119, -0.015]</t>
         </is>
       </c>
-      <c r="D28" s="34" t="n">
-        <v>-0.053</v>
+      <c r="D28" s="34" t="inlineStr">
+        <is>
+          <t>-0.053*</t>
+        </is>
       </c>
       <c r="E28" s="34" t="inlineStr">
         <is>
           <t>[-0.099, -0.007]</t>
         </is>
       </c>
-      <c r="F28" s="34" t="n">
-        <v>0.093</v>
+      <c r="F28" s="34" t="inlineStr">
+        <is>
+          <t>0.093*</t>
+        </is>
       </c>
       <c r="G28" s="34" t="inlineStr">
         <is>
@@ -4443,24 +4649,30 @@
           <t>Low narcissism (−1 SD)</t>
         </is>
       </c>
-      <c r="B29" s="34" t="n">
-        <v>-0.057</v>
+      <c r="B29" s="34" t="inlineStr">
+        <is>
+          <t>-0.057*</t>
+        </is>
       </c>
       <c r="C29" s="34" t="inlineStr">
         <is>
           <t>[-0.105, -0.009]</t>
         </is>
       </c>
-      <c r="D29" s="34" t="n">
-        <v>-0.045</v>
+      <c r="D29" s="34" t="inlineStr">
+        <is>
+          <t>-0.045*</t>
+        </is>
       </c>
       <c r="E29" s="34" t="inlineStr">
         <is>
           <t>[-0.087, -0.003]</t>
         </is>
       </c>
-      <c r="F29" s="34" t="n">
-        <v>0.081</v>
+      <c r="F29" s="34" t="inlineStr">
+        <is>
+          <t>0.081*</t>
+        </is>
       </c>
       <c r="G29" s="34" t="inlineStr">
         <is>
@@ -4505,8 +4717,10 @@
           <t>High power distance (+1 SD)</t>
         </is>
       </c>
-      <c r="B31" s="34" t="n">
-        <v>-0.04</v>
+      <c r="B31" s="34" t="inlineStr">
+        <is>
+          <t>-0.04*</t>
+        </is>
       </c>
       <c r="C31" s="34" t="inlineStr">
         <is>
@@ -4521,8 +4735,10 @@
           <t>[-0.066, 0.004]</t>
         </is>
       </c>
-      <c r="F31" s="34" t="n">
-        <v>0.055</v>
+      <c r="F31" s="34" t="inlineStr">
+        <is>
+          <t>0.055*</t>
+        </is>
       </c>
       <c r="G31" s="34" t="inlineStr">
         <is>
@@ -4536,24 +4752,30 @@
           <t>Low power distance (−1 SD)</t>
         </is>
       </c>
-      <c r="B32" s="34" t="n">
-        <v>-0.08400000000000001</v>
+      <c r="B32" s="34" t="inlineStr">
+        <is>
+          <t>-0.084*</t>
+        </is>
       </c>
       <c r="C32" s="34" t="inlineStr">
         <is>
           <t>[-0.145, -0.023]</t>
         </is>
       </c>
-      <c r="D32" s="34" t="n">
-        <v>-0.067</v>
+      <c r="D32" s="34" t="inlineStr">
+        <is>
+          <t>-0.067*</t>
+        </is>
       </c>
       <c r="E32" s="34" t="inlineStr">
         <is>
           <t>[-0.119, -0.015]</t>
         </is>
       </c>
-      <c r="F32" s="34" t="n">
-        <v>0.118</v>
+      <c r="F32" s="34" t="inlineStr">
+        <is>
+          <t>0.118*</t>
+        </is>
       </c>
       <c r="G32" s="34" t="inlineStr">
         <is>
@@ -4567,8 +4789,10 @@
           <t>Difference</t>
         </is>
       </c>
-      <c r="B33" s="34" t="n">
-        <v>0.044</v>
+      <c r="B33" s="34" t="inlineStr">
+        <is>
+          <t>0.044*</t>
+        </is>
       </c>
       <c r="C33" s="34" t="inlineStr">
         <is>
@@ -4583,8 +4807,10 @@
           <t>[-0.001, 0.073]</t>
         </is>
       </c>
-      <c r="F33" s="34" t="n">
-        <v>-0.063</v>
+      <c r="F33" s="34" t="inlineStr">
+        <is>
+          <t>-0.063*</t>
+        </is>
       </c>
       <c r="G33" s="34" t="inlineStr">
         <is>
@@ -4611,24 +4837,30 @@
           <t>Indirect effect</t>
         </is>
       </c>
-      <c r="B35" s="36" t="n">
-        <v>0.029</v>
+      <c r="B35" s="36" t="inlineStr">
+        <is>
+          <t>0.029*</t>
+        </is>
       </c>
       <c r="C35" s="36" t="inlineStr">
         <is>
           <t>[0.011, 0.052]</t>
         </is>
       </c>
-      <c r="D35" s="36" t="n">
-        <v>0.023</v>
+      <c r="D35" s="36" t="inlineStr">
+        <is>
+          <t>0.023*</t>
+        </is>
       </c>
       <c r="E35" s="36" t="inlineStr">
         <is>
           <t>[0.008, 0.044]</t>
         </is>
       </c>
-      <c r="F35" s="36" t="n">
-        <v>-0.04</v>
+      <c r="F35" s="36" t="inlineStr">
+        <is>
+          <t>-0.04*</t>
+        </is>
       </c>
       <c r="G35" s="36" t="inlineStr">
         <is>
@@ -4689,8 +4921,10 @@
           <t>[-0.006, 0.058]</t>
         </is>
       </c>
-      <c r="F37" s="36" t="n">
-        <v>-0.044</v>
+      <c r="F37" s="36" t="inlineStr">
+        <is>
+          <t>-0.044*</t>
+        </is>
       </c>
       <c r="G37" s="36" t="inlineStr">
         <is>
@@ -4735,8 +4969,10 @@
           <t>High power distance (+1 SD)</t>
         </is>
       </c>
-      <c r="B39" s="36" t="n">
-        <v>0.046</v>
+      <c r="B39" s="36" t="inlineStr">
+        <is>
+          <t>0.046*</t>
+        </is>
       </c>
       <c r="C39" s="36" t="inlineStr">
         <is>
@@ -4751,8 +4987,10 @@
           <t>[-0.001, 0.075]</t>
         </is>
       </c>
-      <c r="F39" s="36" t="n">
-        <v>-0.063</v>
+      <c r="F39" s="36" t="inlineStr">
+        <is>
+          <t>-0.063*</t>
+        </is>
       </c>
       <c r="G39" s="36" t="inlineStr">
         <is>
@@ -4813,8 +5051,10 @@
           <t>[-0.006, 0.060]</t>
         </is>
       </c>
-      <c r="F41" s="36" t="n">
-        <v>-0.045</v>
+      <c r="F41" s="36" t="inlineStr">
+        <is>
+          <t>-0.045*</t>
+        </is>
       </c>
       <c r="G41" s="36" t="inlineStr">
         <is>
@@ -5055,8 +5295,10 @@
       <c r="H4" s="38" t="n">
         <v>0.067</v>
       </c>
-      <c r="I4" s="38" t="n">
-        <v>-0.154</v>
+      <c r="I4" s="38" t="inlineStr">
+        <is>
+          <t>-0.154*</t>
+        </is>
       </c>
       <c r="J4" s="38" t="n">
         <v>0.062</v>
@@ -5070,8 +5312,10 @@
       <c r="M4" s="38" t="n">
         <v>-0.032</v>
       </c>
-      <c r="N4" s="38" t="n">
-        <v>-0.13</v>
+      <c r="N4" s="38" t="inlineStr">
+        <is>
+          <t>-0.13*</t>
+        </is>
       </c>
       <c r="O4" s="38" t="n">
         <v>0.064</v>
@@ -5132,8 +5376,10 @@
       <c r="H5" s="38" t="n">
         <v>0.094</v>
       </c>
-      <c r="I5" s="38" t="n">
-        <v>0.285</v>
+      <c r="I5" s="38" t="inlineStr">
+        <is>
+          <t>0.285***</t>
+        </is>
       </c>
       <c r="J5" s="38" t="n">
         <v>0.059</v>
@@ -5147,8 +5393,10 @@
       <c r="M5" s="38" t="n">
         <v>0.401</v>
       </c>
-      <c r="N5" s="38" t="n">
-        <v>0.249</v>
+      <c r="N5" s="38" t="inlineStr">
+        <is>
+          <t>0.249***</t>
+        </is>
       </c>
       <c r="O5" s="38" t="n">
         <v>0.06</v>
@@ -5224,8 +5472,10 @@
       <c r="M6" s="38" t="n">
         <v>0.08400000000000001</v>
       </c>
-      <c r="N6" s="38" t="n">
-        <v>-0.156</v>
+      <c r="N6" s="38" t="inlineStr">
+        <is>
+          <t>-0.156*</t>
+        </is>
       </c>
       <c r="O6" s="38" t="n">
         <v>0.067</v>
@@ -5271,8 +5521,10 @@
           <t>Power distance</t>
         </is>
       </c>
-      <c r="D7" s="38" t="n">
-        <v>-0.098</v>
+      <c r="D7" s="38" t="inlineStr">
+        <is>
+          <t>-0.098*</t>
+        </is>
       </c>
       <c r="E7" s="38" t="n">
         <v>0.039</v>
@@ -5286,8 +5538,10 @@
       <c r="H7" s="38" t="n">
         <v>-0.022</v>
       </c>
-      <c r="I7" s="38" t="n">
-        <v>0.169</v>
+      <c r="I7" s="38" t="inlineStr">
+        <is>
+          <t>0.169**</t>
+        </is>
       </c>
       <c r="J7" s="38" t="n">
         <v>0.059</v>
@@ -5301,8 +5555,10 @@
       <c r="M7" s="38" t="n">
         <v>0.285</v>
       </c>
-      <c r="N7" s="38" t="n">
-        <v>0.365</v>
+      <c r="N7" s="38" t="inlineStr">
+        <is>
+          <t>0.365***</t>
+        </is>
       </c>
       <c r="O7" s="38" t="n">
         <v>0.062</v>
@@ -5316,8 +5572,10 @@
       <c r="R7" s="38" t="n">
         <v>0.487</v>
       </c>
-      <c r="S7" s="38" t="n">
-        <v>-0.196</v>
+      <c r="S7" s="38" t="inlineStr">
+        <is>
+          <t>-0.196*</t>
+        </is>
       </c>
       <c r="T7" s="38" t="n">
         <v>0.078</v>
@@ -5363,8 +5621,10 @@
       <c r="H8" s="38" t="n">
         <v>0.108</v>
       </c>
-      <c r="I8" s="38" t="n">
-        <v>0.336</v>
+      <c r="I8" s="38" t="inlineStr">
+        <is>
+          <t>0.336***</t>
+        </is>
       </c>
       <c r="J8" s="38" t="n">
         <v>0.06900000000000001</v>
@@ -5378,8 +5638,10 @@
       <c r="M8" s="38" t="n">
         <v>0.471</v>
       </c>
-      <c r="N8" s="38" t="n">
-        <v>0.288</v>
+      <c r="N8" s="38" t="inlineStr">
+        <is>
+          <t>0.288***</t>
+        </is>
       </c>
       <c r="O8" s="38" t="n">
         <v>0.07099999999999999</v>
@@ -5440,8 +5702,10 @@
       <c r="H9" s="38" t="n">
         <v>0.061</v>
       </c>
-      <c r="I9" s="38" t="n">
-        <v>-0.164</v>
+      <c r="I9" s="38" t="inlineStr">
+        <is>
+          <t>-0.164**</t>
+        </is>
       </c>
       <c r="J9" s="38" t="n">
         <v>0.06</v>
@@ -5455,8 +5719,10 @@
       <c r="M9" s="38" t="n">
         <v>-0.046</v>
       </c>
-      <c r="N9" s="38" t="n">
-        <v>-0.126</v>
+      <c r="N9" s="38" t="inlineStr">
+        <is>
+          <t>-0.126*</t>
+        </is>
       </c>
       <c r="O9" s="38" t="n">
         <v>0.063</v>
@@ -5502,8 +5768,10 @@
           <t>Power distance</t>
         </is>
       </c>
-      <c r="D10" s="38" t="n">
-        <v>-0.111</v>
+      <c r="D10" s="38" t="inlineStr">
+        <is>
+          <t>-0.111**</t>
+        </is>
       </c>
       <c r="E10" s="38" t="n">
         <v>0.041</v>
@@ -5517,8 +5785,10 @@
       <c r="H10" s="38" t="n">
         <v>-0.031</v>
       </c>
-      <c r="I10" s="38" t="n">
-        <v>0.201</v>
+      <c r="I10" s="38" t="inlineStr">
+        <is>
+          <t>0.201**</t>
+        </is>
       </c>
       <c r="J10" s="38" t="n">
         <v>0.066</v>
@@ -5532,8 +5802,10 @@
       <c r="M10" s="38" t="n">
         <v>0.33</v>
       </c>
-      <c r="N10" s="38" t="n">
-        <v>0.423</v>
+      <c r="N10" s="38" t="inlineStr">
+        <is>
+          <t>0.423***</t>
+        </is>
       </c>
       <c r="O10" s="38" t="n">
         <v>0.06900000000000001</v>
@@ -5547,8 +5819,10 @@
       <c r="R10" s="38" t="n">
         <v>0.5580000000000001</v>
       </c>
-      <c r="S10" s="38" t="n">
-        <v>-0.222</v>
+      <c r="S10" s="38" t="inlineStr">
+        <is>
+          <t>-0.222**</t>
+        </is>
       </c>
       <c r="T10" s="38" t="n">
         <v>0.082</v>
@@ -5579,8 +5853,10 @@
           <t>Power distance</t>
         </is>
       </c>
-      <c r="D11" s="38" t="n">
-        <v>0.067</v>
+      <c r="D11" s="38" t="inlineStr">
+        <is>
+          <t>0.067†</t>
+        </is>
       </c>
       <c r="E11" s="38" t="n">
         <v>0.038</v>
@@ -5609,8 +5885,10 @@
       <c r="M11" s="38" t="n">
         <v>0.04</v>
       </c>
-      <c r="N11" s="38" t="n">
-        <v>-0.212</v>
+      <c r="N11" s="38" t="inlineStr">
+        <is>
+          <t>-0.212**</t>
+        </is>
       </c>
       <c r="O11" s="38" t="n">
         <v>0.062</v>
@@ -5624,8 +5902,10 @@
       <c r="R11" s="38" t="n">
         <v>-0.09</v>
       </c>
-      <c r="S11" s="38" t="n">
-        <v>0.134</v>
+      <c r="S11" s="38" t="inlineStr">
+        <is>
+          <t>0.134†</t>
+        </is>
       </c>
       <c r="T11" s="38" t="n">
         <v>0.076</v>

</xml_diff>

<commit_message>
sync v4.6.0 phase 1: round-3 Tier 1 structural fixes
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -1951,7 +1951,7 @@
         </is>
       </c>
       <c r="B3" s="40" t="n">
-        <v>0.5570000000000001</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="C3" s="40" t="n">
         <v>0.497</v>
@@ -1969,13 +1969,13 @@
         </is>
       </c>
       <c r="B4" s="40" t="n">
-        <v>30.623</v>
+        <v>30.638</v>
       </c>
       <c r="C4" s="40" t="n">
-        <v>4.613</v>
+        <v>4.607</v>
       </c>
       <c r="D4" s="40" t="n">
-        <v>0.015</v>
+        <v>0.04</v>
       </c>
       <c r="E4" s="40" t="inlineStr">
         <is>
@@ -1990,17 +1990,17 @@
         </is>
       </c>
       <c r="B5" s="40" t="n">
-        <v>2.314</v>
+        <v>2.349</v>
       </c>
       <c r="C5" s="40" t="n">
-        <v>1.466</v>
+        <v>1.511</v>
       </c>
       <c r="D5" s="40" t="n">
-        <v>-0.046</v>
+        <v>-0.024</v>
       </c>
       <c r="E5" s="40" t="inlineStr">
         <is>
-          <t>0.22***</t>
+          <t>0.199***</t>
         </is>
       </c>
       <c r="F5" s="40" t="inlineStr">
@@ -2016,19 +2016,19 @@
         </is>
       </c>
       <c r="B6" s="40" t="n">
-        <v>3.299</v>
+        <v>3.249</v>
       </c>
       <c r="C6" s="40" t="n">
-        <v>1.085</v>
+        <v>1.076</v>
       </c>
       <c r="D6" s="40" t="n">
-        <v>0.082</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="E6" s="40" t="n">
-        <v>0.003</v>
+        <v>-0.001</v>
       </c>
       <c r="F6" s="40" t="n">
-        <v>-0.054</v>
+        <v>-0.046</v>
       </c>
       <c r="G6" s="40" t="inlineStr">
         <is>
@@ -2043,22 +2043,22 @@
         </is>
       </c>
       <c r="B7" s="40" t="n">
-        <v>4.088</v>
+        <v>4.009</v>
       </c>
       <c r="C7" s="40" t="n">
-        <v>0.885</v>
+        <v>0.861</v>
       </c>
       <c r="D7" s="40" t="n">
-        <v>-0.048</v>
+        <v>-0.01</v>
       </c>
       <c r="E7" s="40" t="n">
-        <v>-0.011</v>
+        <v>-0.008999999999999999</v>
       </c>
       <c r="F7" s="40" t="n">
-        <v>0.079</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="G7" s="40" t="n">
-        <v>0.005</v>
+        <v>-0.039</v>
       </c>
       <c r="H7" s="39" t="inlineStr">
         <is>
@@ -2073,26 +2073,26 @@
         </is>
       </c>
       <c r="B8" s="40" t="n">
-        <v>4.891</v>
+        <v>4.92</v>
       </c>
       <c r="C8" s="40" t="n">
-        <v>0.964</v>
+        <v>0.954</v>
       </c>
       <c r="D8" s="40" t="n">
-        <v>-0.005</v>
+        <v>-0.03</v>
       </c>
       <c r="E8" s="40" t="n">
-        <v>-0.027</v>
+        <v>-0.047</v>
       </c>
       <c r="F8" s="40" t="n">
-        <v>0.028</v>
+        <v>0.021</v>
       </c>
       <c r="G8" s="40" t="n">
-        <v>-0.1</v>
+        <v>-0.08599999999999999</v>
       </c>
       <c r="H8" s="40" t="inlineStr">
         <is>
-          <t>-0.35***</t>
+          <t>-0.325***</t>
         </is>
       </c>
       <c r="I8" s="40" t="inlineStr">
@@ -2108,30 +2108,28 @@
         </is>
       </c>
       <c r="B9" s="40" t="n">
-        <v>3.48</v>
+        <v>3.466</v>
       </c>
       <c r="C9" s="40" t="n">
-        <v>0.891</v>
+        <v>0.894</v>
       </c>
       <c r="D9" s="40" t="n">
-        <v>-0.043</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="E9" s="40" t="n">
-        <v>-0.036</v>
-      </c>
-      <c r="F9" s="40" t="inlineStr">
-        <is>
-          <t>0.107*</t>
-        </is>
+        <v>-0.032</v>
+      </c>
+      <c r="F9" s="40" t="n">
+        <v>0.043</v>
       </c>
       <c r="G9" s="40" t="n">
-        <v>-0.046</v>
+        <v>-0.022</v>
       </c>
       <c r="H9" s="40" t="n">
-        <v>0.006</v>
+        <v>-0.003</v>
       </c>
       <c r="I9" s="40" t="n">
-        <v>0.056</v>
+        <v>0.067</v>
       </c>
       <c r="J9" s="40" t="inlineStr">
         <is>
@@ -2146,31 +2144,31 @@
         </is>
       </c>
       <c r="B10" s="40" t="n">
-        <v>4.569</v>
+        <v>4.583</v>
       </c>
       <c r="C10" s="40" t="n">
-        <v>0.883</v>
+        <v>0.893</v>
       </c>
       <c r="D10" s="40" t="n">
-        <v>-0.07199999999999999</v>
+        <v>-0.08400000000000001</v>
       </c>
       <c r="E10" s="40" t="n">
-        <v>-0.099</v>
+        <v>-0.095</v>
       </c>
       <c r="F10" s="40" t="n">
-        <v>-0.102</v>
+        <v>-0.079</v>
       </c>
       <c r="G10" s="40" t="n">
-        <v>-0.066</v>
+        <v>-0.098</v>
       </c>
       <c r="H10" s="40" t="n">
-        <v>-0.013</v>
+        <v>-0.063</v>
       </c>
       <c r="I10" s="40" t="n">
-        <v>-0.039</v>
+        <v>-0.03</v>
       </c>
       <c r="J10" s="40" t="n">
-        <v>-0.043</v>
+        <v>-0.008</v>
       </c>
       <c r="K10" s="40" t="inlineStr">
         <is>
@@ -2185,38 +2183,38 @@
         </is>
       </c>
       <c r="B11" s="40" t="n">
-        <v>4.444</v>
+        <v>4.527</v>
       </c>
       <c r="C11" s="40" t="n">
-        <v>1.232</v>
+        <v>1.239</v>
       </c>
       <c r="D11" s="40" t="n">
-        <v>-0.038</v>
+        <v>-0.053</v>
       </c>
       <c r="E11" s="40" t="n">
-        <v>-0.034</v>
+        <v>-0.026</v>
       </c>
       <c r="F11" s="40" t="n">
-        <v>-0.029</v>
+        <v>-0.045</v>
       </c>
       <c r="G11" s="40" t="n">
-        <v>-0.057</v>
+        <v>-0.068</v>
       </c>
       <c r="H11" s="40" t="inlineStr">
         <is>
-          <t>-0.535***</t>
+          <t>-0.522***</t>
         </is>
       </c>
       <c r="I11" s="40" t="inlineStr">
         <is>
-          <t>0.545***</t>
+          <t>0.525***</t>
         </is>
       </c>
       <c r="J11" s="40" t="n">
-        <v>-0.011</v>
+        <v>0.004</v>
       </c>
       <c r="K11" s="40" t="n">
-        <v>-0.021</v>
+        <v>-0.024</v>
       </c>
       <c r="L11" s="40" t="inlineStr">
         <is>
@@ -2231,42 +2229,42 @@
         </is>
       </c>
       <c r="B12" s="40" t="n">
-        <v>3.068</v>
+        <v>3.024</v>
       </c>
       <c r="C12" s="40" t="n">
-        <v>1.173</v>
+        <v>1.157</v>
       </c>
       <c r="D12" s="40" t="n">
-        <v>0.017</v>
+        <v>0.043</v>
       </c>
       <c r="E12" s="40" t="n">
-        <v>-0.022</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="F12" s="40" t="n">
-        <v>0.007</v>
+        <v>-0.012</v>
       </c>
       <c r="G12" s="40" t="n">
-        <v>0.051</v>
+        <v>0.033</v>
       </c>
       <c r="H12" s="40" t="inlineStr">
         <is>
-          <t>0.532***</t>
+          <t>0.51***</t>
         </is>
       </c>
       <c r="I12" s="40" t="inlineStr">
         <is>
-          <t>-0.512***</t>
+          <t>-0.514***</t>
         </is>
       </c>
       <c r="J12" s="40" t="n">
-        <v>0.032</v>
+        <v>0.033</v>
       </c>
       <c r="K12" s="40" t="n">
-        <v>-0.058</v>
+        <v>-0.07099999999999999</v>
       </c>
       <c r="L12" s="40" t="inlineStr">
         <is>
-          <t>-0.466***</t>
+          <t>-0.46***</t>
         </is>
       </c>
       <c r="M12" s="40" t="inlineStr">
@@ -2282,39 +2280,37 @@
         </is>
       </c>
       <c r="B13" s="40" t="n">
-        <v>4.392</v>
+        <v>4.389</v>
       </c>
       <c r="C13" s="40" t="n">
-        <v>0.639</v>
+        <v>0.621</v>
       </c>
       <c r="D13" s="40" t="n">
-        <v>0.045</v>
+        <v>0.019</v>
       </c>
       <c r="E13" s="40" t="n">
-        <v>-0.016</v>
+        <v>0.044</v>
       </c>
       <c r="F13" s="40" t="n">
-        <v>-0.002</v>
+        <v>-0.021</v>
       </c>
       <c r="G13" s="40" t="n">
-        <v>-0.017</v>
+        <v>0.013</v>
       </c>
       <c r="H13" s="40" t="n">
-        <v>0.053</v>
+        <v>0.054</v>
       </c>
       <c r="I13" s="40" t="n">
-        <v>-0.066</v>
-      </c>
-      <c r="J13" s="40" t="inlineStr">
-        <is>
-          <t>-0.118*</t>
-        </is>
+        <v>-0.035</v>
+      </c>
+      <c r="J13" s="40" t="n">
+        <v>-0.102</v>
       </c>
       <c r="K13" s="40" t="n">
-        <v>-0.068</v>
+        <v>-0.028</v>
       </c>
       <c r="L13" s="40" t="n">
-        <v>-0.03</v>
+        <v>-0.004</v>
       </c>
       <c r="M13" s="40" t="n">
         <v>0.045</v>
@@ -2332,52 +2328,52 @@
         </is>
       </c>
       <c r="B14" s="40" t="n">
-        <v>4.52</v>
+        <v>4.51</v>
       </c>
       <c r="C14" s="40" t="n">
-        <v>0.779</v>
+        <v>0.805</v>
       </c>
       <c r="D14" s="40" t="n">
+        <v>-0.008999999999999999</v>
+      </c>
+      <c r="E14" s="40" t="n">
+        <v>-0.021</v>
+      </c>
+      <c r="F14" s="40" t="n">
         <v>-0.026</v>
       </c>
-      <c r="E14" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="40" t="n">
-        <v>0.007</v>
-      </c>
       <c r="G14" s="40" t="n">
-        <v>-0.09</v>
+        <v>-0.043</v>
       </c>
       <c r="H14" s="40" t="inlineStr">
         <is>
-          <t>-0.445***</t>
+          <t>-0.395***</t>
         </is>
       </c>
       <c r="I14" s="40" t="inlineStr">
         <is>
-          <t>0.457***</t>
+          <t>0.42***</t>
         </is>
       </c>
       <c r="J14" s="40" t="n">
-        <v>-0.058</v>
+        <v>-0.041</v>
       </c>
       <c r="K14" s="40" t="n">
-        <v>-0.017</v>
+        <v>-0.001</v>
       </c>
       <c r="L14" s="40" t="inlineStr">
         <is>
-          <t>0.614***</t>
+          <t>0.571***</t>
         </is>
       </c>
       <c r="M14" s="40" t="inlineStr">
         <is>
-          <t>-0.608***</t>
+          <t>-0.595***</t>
         </is>
       </c>
       <c r="N14" s="40" t="inlineStr">
         <is>
-          <t>0.356***</t>
+          <t>0.43***</t>
         </is>
       </c>
       <c r="O14" s="40" t="inlineStr">
@@ -2393,57 +2389,55 @@
         </is>
       </c>
       <c r="B15" s="40" t="n">
-        <v>4.793</v>
+        <v>4.698</v>
       </c>
       <c r="C15" s="40" t="n">
-        <v>1.214</v>
+        <v>1.193</v>
       </c>
       <c r="D15" s="40" t="n">
-        <v>-0.011</v>
+        <v>-0.025</v>
       </c>
       <c r="E15" s="40" t="n">
-        <v>-0.016</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="F15" s="40" t="n">
-        <v>-0.025</v>
+        <v>-0.023</v>
       </c>
       <c r="G15" s="40" t="n">
-        <v>-0.008999999999999999</v>
+        <v>0.001</v>
       </c>
       <c r="H15" s="40" t="inlineStr">
         <is>
-          <t>-0.34***</t>
+          <t>-0.194***</t>
         </is>
       </c>
       <c r="I15" s="40" t="inlineStr">
         <is>
-          <t>0.375***</t>
+          <t>0.345***</t>
         </is>
       </c>
       <c r="J15" s="40" t="n">
-        <v>0.097</v>
+        <v>-0.092</v>
       </c>
       <c r="K15" s="40" t="n">
-        <v>-0.015</v>
+        <v>-0.091</v>
       </c>
       <c r="L15" s="40" t="inlineStr">
         <is>
-          <t>0.35***</t>
+          <t>0.376***</t>
         </is>
       </c>
       <c r="M15" s="40" t="inlineStr">
         <is>
-          <t>-0.404***</t>
-        </is>
-      </c>
-      <c r="N15" s="40" t="inlineStr">
-        <is>
-          <t>-0.108*</t>
-        </is>
+          <t>-0.345***</t>
+        </is>
+      </c>
+      <c r="N15" s="40" t="n">
+        <v>0.021</v>
       </c>
       <c r="O15" s="40" t="inlineStr">
         <is>
-          <t>0.27***</t>
+          <t>0.266***</t>
         </is>
       </c>
       <c r="P15" s="40" t="inlineStr">
@@ -2459,62 +2453,60 @@
         </is>
       </c>
       <c r="B16" s="40" t="n">
-        <v>2.493</v>
+        <v>2.672</v>
       </c>
       <c r="C16" s="40" t="n">
-        <v>0.96</v>
+        <v>1.045</v>
       </c>
       <c r="D16" s="40" t="n">
-        <v>0.048</v>
+        <v>0.054</v>
       </c>
       <c r="E16" s="40" t="n">
-        <v>-0.006</v>
+        <v>0.03</v>
       </c>
       <c r="F16" s="40" t="n">
-        <v>-0.064</v>
+        <v>0.042</v>
       </c>
       <c r="G16" s="40" t="n">
-        <v>0.024</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="H16" s="40" t="inlineStr">
         <is>
-          <t>0.21***</t>
+          <t>0.356***</t>
         </is>
       </c>
       <c r="I16" s="40" t="inlineStr">
         <is>
-          <t>-0.235***</t>
+          <t>-0.29***</t>
         </is>
       </c>
       <c r="J16" s="40" t="n">
-        <v>-0.033</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="K16" s="40" t="n">
-        <v>0.036</v>
+        <v>-0.052</v>
       </c>
       <c r="L16" s="40" t="inlineStr">
         <is>
-          <t>-0.319***</t>
+          <t>-0.365***</t>
         </is>
       </c>
       <c r="M16" s="40" t="inlineStr">
         <is>
-          <t>0.334***</t>
-        </is>
-      </c>
-      <c r="N16" s="40" t="inlineStr">
-        <is>
-          <t>0.165**</t>
-        </is>
+          <t>0.316***</t>
+        </is>
+      </c>
+      <c r="N16" s="40" t="n">
+        <v>0.089</v>
       </c>
       <c r="O16" s="40" t="inlineStr">
         <is>
-          <t>-0.19***</t>
+          <t>-0.251***</t>
         </is>
       </c>
       <c r="P16" s="40" t="inlineStr">
         <is>
-          <t>-0.425***</t>
+          <t>-0.419***</t>
         </is>
       </c>
       <c r="Q16" s="40" t="inlineStr">
@@ -2526,7 +2518,7 @@
     <row r="17" ht="35" customHeight="1" s="45">
       <c r="A17" s="23" t="inlineStr">
         <is>
-          <t>Note. Values on the diagonal are Cronbach’s alpha coefficients where applicable. Correlations are zero-order correlations among observed study variables. Leadership variables were rated by followers at T1. OCBS and CWBS were rated by leaders at T3. N = 361. *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
+          <t>Note. Values on the diagonal are Cronbach’s alpha coefficients where applicable. Correlations are zero-order correlations among observed study variables. Leadership variables were rated by followers at T1. OCBS and CWBS were rated by leaders at T3. N = 362. *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -2732,43 +2724,43 @@
       </c>
       <c r="F5" s="40" t="inlineStr">
         <is>
-          <t>3.821***</t>
+          <t>3.812***</t>
         </is>
       </c>
       <c r="G5" s="40" t="n">
-        <v>0.094</v>
+        <v>0.096</v>
       </c>
       <c r="H5" s="40" t="inlineStr">
         <is>
-          <t>3.821***</t>
+          <t>3.812***</t>
         </is>
       </c>
       <c r="I5" s="40" t="n">
-        <v>0.094</v>
+        <v>0.096</v>
       </c>
       <c r="J5" s="40" t="inlineStr">
         <is>
-          <t>3.821***</t>
+          <t>4.402***</t>
         </is>
       </c>
       <c r="K5" s="40" t="n">
-        <v>0.094</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="L5" s="40" t="inlineStr">
         <is>
-          <t>3.821***</t>
+          <t>4.703***</t>
         </is>
       </c>
       <c r="M5" s="40" t="n">
-        <v>0.094</v>
+        <v>0.108</v>
       </c>
       <c r="N5" s="40" t="inlineStr">
         <is>
-          <t>3.821***</t>
+          <t>2.498***</t>
         </is>
       </c>
       <c r="O5" s="40" t="n">
-        <v>0.094</v>
+        <v>0.095</v>
       </c>
     </row>
     <row r="6" customFormat="1" s="37">
@@ -2805,37 +2797,37 @@
         <v>0.022</v>
       </c>
       <c r="D7" s="40" t="n">
-        <v>-0.018</v>
+        <v>-0.019</v>
       </c>
       <c r="E7" s="40" t="n">
         <v>0.022</v>
       </c>
       <c r="F7" s="40" t="n">
-        <v>-0.018</v>
+        <v>-0.014</v>
       </c>
       <c r="G7" s="40" t="n">
-        <v>0.022</v>
+        <v>0.023</v>
       </c>
       <c r="H7" s="40" t="n">
-        <v>-0.018</v>
+        <v>-0.015</v>
       </c>
       <c r="I7" s="40" t="n">
-        <v>0.022</v>
+        <v>0.023</v>
       </c>
       <c r="J7" s="40" t="n">
-        <v>-0.018</v>
+        <v>-0.012</v>
       </c>
       <c r="K7" s="40" t="n">
-        <v>0.022</v>
+        <v>0.021</v>
       </c>
       <c r="L7" s="40" t="n">
-        <v>-0.018</v>
+        <v>-0.022</v>
       </c>
       <c r="M7" s="40" t="n">
-        <v>0.022</v>
+        <v>0.024</v>
       </c>
       <c r="N7" s="40" t="n">
-        <v>-0.018</v>
+        <v>-0.01</v>
       </c>
       <c r="O7" s="40" t="n">
         <v>0.022</v>
@@ -2854,40 +2846,40 @@
         <v>0.041</v>
       </c>
       <c r="D8" s="40" t="n">
-        <v>0.034</v>
+        <v>0.037</v>
       </c>
       <c r="E8" s="40" t="n">
         <v>0.041</v>
       </c>
       <c r="F8" s="40" t="n">
-        <v>0.034</v>
+        <v>0.029</v>
       </c>
       <c r="G8" s="40" t="n">
-        <v>0.041</v>
+        <v>0.043</v>
       </c>
       <c r="H8" s="40" t="n">
-        <v>0.034</v>
+        <v>0.03</v>
       </c>
       <c r="I8" s="40" t="n">
-        <v>0.041</v>
+        <v>0.043</v>
       </c>
       <c r="J8" s="40" t="n">
-        <v>0.034</v>
+        <v>0.043</v>
       </c>
       <c r="K8" s="40" t="n">
-        <v>0.041</v>
+        <v>0.039</v>
       </c>
       <c r="L8" s="40" t="n">
-        <v>0.034</v>
+        <v>0.022</v>
       </c>
       <c r="M8" s="40" t="n">
-        <v>0.041</v>
+        <v>0.044</v>
       </c>
       <c r="N8" s="40" t="n">
-        <v>0.034</v>
+        <v>0.051</v>
       </c>
       <c r="O8" s="40" t="n">
-        <v>0.041</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="9">
@@ -2903,37 +2895,37 @@
         <v>0.018</v>
       </c>
       <c r="D9" s="40" t="n">
-        <v>0.012</v>
+        <v>0.014</v>
       </c>
       <c r="E9" s="40" t="n">
         <v>0.018</v>
       </c>
       <c r="F9" s="40" t="n">
-        <v>0.012</v>
+        <v>0.008</v>
       </c>
       <c r="G9" s="40" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="H9" s="40" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="I9" s="40" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="J9" s="40" t="n">
         <v>0.018</v>
       </c>
-      <c r="H9" s="40" t="n">
-        <v>0.012</v>
-      </c>
-      <c r="I9" s="40" t="n">
-        <v>0.018</v>
-      </c>
-      <c r="J9" s="40" t="n">
-        <v>0.012</v>
-      </c>
       <c r="K9" s="40" t="n">
-        <v>0.018</v>
+        <v>0.017</v>
       </c>
       <c r="L9" s="40" t="n">
-        <v>0.012</v>
+        <v>0.005</v>
       </c>
       <c r="M9" s="40" t="n">
-        <v>0.018</v>
+        <v>0.02</v>
       </c>
       <c r="N9" s="40" t="n">
-        <v>0.012</v>
+        <v>0.022</v>
       </c>
       <c r="O9" s="40" t="n">
         <v>0.018</v>
@@ -2955,7 +2947,7 @@
       </c>
       <c r="D10" s="40" t="inlineStr">
         <is>
-          <t>0.087*</t>
+          <t>0.085*</t>
         </is>
       </c>
       <c r="E10" s="40" t="n">
@@ -2963,39 +2955,39 @@
       </c>
       <c r="F10" s="40" t="inlineStr">
         <is>
-          <t>0.087*</t>
+          <t>0.091**</t>
         </is>
       </c>
       <c r="G10" s="40" t="n">
-        <v>0.034</v>
+        <v>0.035</v>
       </c>
       <c r="H10" s="40" t="inlineStr">
         <is>
-          <t>0.087*</t>
+          <t>0.09*</t>
         </is>
       </c>
       <c r="I10" s="40" t="n">
-        <v>0.034</v>
+        <v>0.035</v>
       </c>
       <c r="J10" s="40" t="inlineStr">
         <is>
-          <t>0.087*</t>
+          <t>0.078*</t>
         </is>
       </c>
       <c r="K10" s="40" t="n">
-        <v>0.034</v>
+        <v>0.033</v>
       </c>
       <c r="L10" s="40" t="inlineStr">
         <is>
-          <t>0.087*</t>
+          <t>0.103**</t>
         </is>
       </c>
       <c r="M10" s="40" t="n">
-        <v>0.034</v>
+        <v>0.036</v>
       </c>
       <c r="N10" s="40" t="inlineStr">
         <is>
-          <t>0.087*</t>
+          <t>0.069*</t>
         </is>
       </c>
       <c r="O10" s="40" t="n">
@@ -3010,35 +3002,43 @@
       </c>
       <c r="B11" s="40" t="inlineStr">
         <is>
-          <t>0.412***</t>
-        </is>
-      </c>
-      <c r="C11" s="40" t="n">
-        <v>0.048</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C11" s="40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="D11" s="40" t="inlineStr">
         <is>
-          <t>0.412***</t>
-        </is>
-      </c>
-      <c r="E11" s="40" t="n">
-        <v>0.048</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E11" s="40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="F11" s="40" t="inlineStr">
         <is>
-          <t>0.412***</t>
-        </is>
-      </c>
-      <c r="G11" s="40" t="n">
-        <v>0.048</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G11" s="40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="H11" s="40" t="inlineStr">
         <is>
-          <t>0.412***</t>
-        </is>
-      </c>
-      <c r="I11" s="40" t="n">
-        <v>0.048</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I11" s="40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="J11" s="40" t="inlineStr">
         <is>
@@ -3050,19 +3050,23 @@
       </c>
       <c r="L11" s="40" t="inlineStr">
         <is>
-          <t>0.412***</t>
-        </is>
-      </c>
-      <c r="M11" s="40" t="n">
-        <v>0.048</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M11" s="40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="N11" s="40" t="inlineStr">
         <is>
-          <t>0.412***</t>
-        </is>
-      </c>
-      <c r="O11" s="40" t="n">
-        <v>0.048</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O11" s="40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="12" customFormat="1" s="37">
@@ -3872,7 +3876,7 @@
     <row r="28" ht="48" customHeight="1" s="45">
       <c r="A28" s="23" t="inlineStr">
         <is>
-          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 361; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.  *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
+          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 362; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.  *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -6092,7 +6096,7 @@
     <row r="2">
       <c r="A2" s="38" t="inlineStr">
         <is>
-          <t>N = 361</t>
+          <t>N = 362</t>
         </is>
       </c>
     </row>
@@ -6106,14 +6110,14 @@
     <row r="4">
       <c r="A4" s="38" t="inlineStr">
         <is>
-          <t>- Male: 201 (55.7%)</t>
+          <t>- Male: 202 (55.8%)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="38" t="inlineStr">
         <is>
-          <t>- Female: 160 (44.3%)</t>
+          <t>- Female: 160 (44.2%)</t>
         </is>
       </c>
     </row>
@@ -6128,21 +6132,21 @@
     <row r="8">
       <c r="A8" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 30.62, SD = 4.61</t>
+          <t>Age: M = 30.64, SD = 4.61</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="38" t="inlineStr">
         <is>
-          <t>Working years: M = 8.79, SD = 4.77</t>
+          <t>Working years: M = 8.89, SD = 4.79</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="38" t="inlineStr">
         <is>
-          <t>Tenure with current leader: M = 2.31, SD = 1.47</t>
+          <t>Tenure with current leader: M = 2.35, SD = 1.51</t>
         </is>
       </c>
     </row>
@@ -6150,11 +6154,11 @@
       <c r="A11" s="48" t="inlineStr">
         <is>
           <t>Interaction frequency with leader:
-  - Rarely (&lt;1/wk): 20 (5.5%)
-  - Sometimes (1-2/wk): 63 (17.5%)
-  - Often (3-4/wk): 118 (32.7%)
-  - Very often (~daily): 109 (30.2%)
-  - Multiple times/day: 51 (14.1%)</t>
+  - Rarely (&lt;1/wk): 22 (6.1%)
+  - Sometimes (1-2/wk): 65 (18.0%)
+  - Often (3-4/wk): 120 (33.1%)
+  - Very often (~daily): 111 (30.7%)
+  - Multiple times/day: 44 (12.2%)</t>
         </is>
       </c>
     </row>
@@ -6169,35 +6173,35 @@
     <row r="14">
       <c r="A14" s="38" t="inlineStr">
         <is>
-          <t>- High school: 19 (5.3%)</t>
+          <t>- High school: 20 (5.5%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 64 (17.7%)</t>
+          <t>- Some college / Associate: 61 (16.9%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 165 (45.7%)</t>
+          <t>- Bachelor: 164 (45.3%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="38" t="inlineStr">
         <is>
-          <t>- Master: 89 (24.7%)</t>
+          <t>- Master: 91 (25.1%)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="38" t="inlineStr">
         <is>
-          <t>- Doctorate: 21 (5.8%)</t>
+          <t>- Doctorate: 22 (6.1%)</t>
         </is>
       </c>
     </row>
@@ -6212,35 +6216,35 @@
     <row r="21">
       <c r="A21" s="38" t="inlineStr">
         <is>
-          <t>- Entry: 72 (19.9%)</t>
+          <t>- Entry: 63 (17.4%)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="38" t="inlineStr">
         <is>
-          <t>- Associate: 118 (32.7%)</t>
+          <t>- Associate: 117 (32.3%)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="38" t="inlineStr">
         <is>
-          <t>- Senior: 92 (25.5%)</t>
+          <t>- Senior: 93 (25.7%)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="38" t="inlineStr">
         <is>
-          <t>- Manager: 59 (16.3%)</t>
+          <t>- Manager: 67 (18.5%)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="38" t="inlineStr">
         <is>
-          <t>- Director: 17 (4.7%)</t>
+          <t>- Director: 18 (5.0%)</t>
         </is>
       </c>
     </row>
@@ -6270,14 +6274,14 @@
     <row r="31">
       <c r="A31" s="38" t="inlineStr">
         <is>
-          <t>- Male: 51 (64.6%)</t>
+          <t>- Male: 52 (65.8%)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="38" t="inlineStr">
         <is>
-          <t>- Female: 28 (35.4%)</t>
+          <t>- Female: 27 (34.2%)</t>
         </is>
       </c>
     </row>
@@ -6292,7 +6296,7 @@
     <row r="35">
       <c r="A35" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 40.95, SD = 6.47</t>
+          <t>Age: M = 41.65, SD = 5.90</t>
         </is>
       </c>
     </row>
@@ -6306,14 +6310,14 @@
     <row r="37">
       <c r="A37" s="38" t="inlineStr">
         <is>
-          <t>Leadership tenure: M = 5.40, SD = 2.73</t>
+          <t>Leadership tenure: M = 5.23, SD = 3.03</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="38" t="inlineStr">
         <is>
-          <t>Span of control: M = 4.57, SD = 0.63</t>
+          <t>Span of control: M = 4.58, SD = 0.59</t>
         </is>
       </c>
     </row>
@@ -6328,14 +6332,14 @@
     <row r="41">
       <c r="A41" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 7 (8.9%)</t>
+          <t>- Some college / Associate: 8 (10.1%)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 40 (50.6%)</t>
+          <t>- Bachelor: 39 (49.4%)</t>
         </is>
       </c>
     </row>
@@ -6669,7 +6673,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="9">
@@ -6699,7 +6703,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="12">
@@ -6802,7 +6806,7 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>78.5%</t>
+          <t>78.7%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sync v4.6 fresh: post-pipeline data+results regenerated
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -1951,10 +1951,10 @@
         </is>
       </c>
       <c r="B3" s="40" t="n">
-        <v>0.529</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="C3" s="40" t="n">
-        <v>0.5</v>
+        <v>0.497</v>
       </c>
       <c r="D3" s="40" t="inlineStr">
         <is>
@@ -1969,13 +1969,13 @@
         </is>
       </c>
       <c r="B4" s="40" t="n">
-        <v>30.832</v>
+        <v>30.781</v>
       </c>
       <c r="C4" s="40" t="n">
-        <v>4.55</v>
+        <v>4.593</v>
       </c>
       <c r="D4" s="40" t="n">
-        <v>0.044</v>
+        <v>0.017</v>
       </c>
       <c r="E4" s="40" t="inlineStr">
         <is>
@@ -1990,17 +1990,17 @@
         </is>
       </c>
       <c r="B5" s="40" t="n">
-        <v>2.347</v>
+        <v>2.359</v>
       </c>
       <c r="C5" s="40" t="n">
-        <v>1.487</v>
+        <v>1.476</v>
       </c>
       <c r="D5" s="40" t="n">
-        <v>-0.004</v>
+        <v>-0.027</v>
       </c>
       <c r="E5" s="40" t="inlineStr">
         <is>
-          <t>0.175***</t>
+          <t>0.178***</t>
         </is>
       </c>
       <c r="F5" s="40" t="inlineStr">
@@ -2016,19 +2016,19 @@
         </is>
       </c>
       <c r="B6" s="40" t="n">
-        <v>3.298</v>
+        <v>3.296</v>
       </c>
       <c r="C6" s="40" t="n">
-        <v>1.082</v>
+        <v>1.071</v>
       </c>
       <c r="D6" s="40" t="n">
-        <v>0.081</v>
+        <v>0.101</v>
       </c>
       <c r="E6" s="40" t="n">
-        <v>-0.012</v>
+        <v>-0.008999999999999999</v>
       </c>
       <c r="F6" s="40" t="n">
-        <v>-0.081</v>
+        <v>-0.079</v>
       </c>
       <c r="G6" s="40" t="inlineStr">
         <is>
@@ -2043,24 +2043,22 @@
         </is>
       </c>
       <c r="B7" s="40" t="n">
-        <v>4.075</v>
+        <v>4.083</v>
       </c>
       <c r="C7" s="40" t="n">
-        <v>0.893</v>
+        <v>0.885</v>
       </c>
       <c r="D7" s="40" t="n">
-        <v>-0.012</v>
+        <v>-0.059</v>
       </c>
       <c r="E7" s="40" t="n">
-        <v>-0.014</v>
-      </c>
-      <c r="F7" s="40" t="inlineStr">
-        <is>
-          <t>0.11*</t>
-        </is>
+        <v>-0.034</v>
+      </c>
+      <c r="F7" s="40" t="n">
+        <v>0.077</v>
       </c>
       <c r="G7" s="40" t="n">
-        <v>-0.012</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="H7" s="39" t="inlineStr">
         <is>
@@ -2075,26 +2073,26 @@
         </is>
       </c>
       <c r="B8" s="40" t="n">
-        <v>4.881</v>
+        <v>4.898</v>
       </c>
       <c r="C8" s="40" t="n">
-        <v>0.9350000000000001</v>
+        <v>0.971</v>
       </c>
       <c r="D8" s="40" t="n">
-        <v>-0.022</v>
+        <v>-0.025</v>
       </c>
       <c r="E8" s="40" t="n">
-        <v>-0.004</v>
+        <v>-0.008</v>
       </c>
       <c r="F8" s="40" t="n">
-        <v>0.024</v>
+        <v>0.035</v>
       </c>
       <c r="G8" s="40" t="n">
-        <v>-0.06</v>
+        <v>-0.08400000000000001</v>
       </c>
       <c r="H8" s="40" t="inlineStr">
         <is>
-          <t>-0.34***</t>
+          <t>-0.342***</t>
         </is>
       </c>
       <c r="I8" s="40" t="inlineStr">
@@ -2110,28 +2108,28 @@
         </is>
       </c>
       <c r="B9" s="40" t="n">
-        <v>3.485</v>
+        <v>3.479</v>
       </c>
       <c r="C9" s="40" t="n">
-        <v>0.913</v>
+        <v>0.885</v>
       </c>
       <c r="D9" s="40" t="n">
-        <v>-0.078</v>
+        <v>-0.05</v>
       </c>
       <c r="E9" s="40" t="n">
-        <v>-0.06900000000000001</v>
+        <v>-0.032</v>
       </c>
       <c r="F9" s="40" t="n">
-        <v>0.049</v>
+        <v>0.06</v>
       </c>
       <c r="G9" s="40" t="n">
-        <v>-0.057</v>
+        <v>-0.066</v>
       </c>
       <c r="H9" s="40" t="n">
-        <v>-0.008</v>
+        <v>0.021</v>
       </c>
       <c r="I9" s="40" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.078</v>
       </c>
       <c r="J9" s="40" t="inlineStr">
         <is>
@@ -2146,33 +2144,31 @@
         </is>
       </c>
       <c r="B10" s="40" t="n">
-        <v>4.625</v>
+        <v>4.599</v>
       </c>
       <c r="C10" s="40" t="n">
-        <v>0.883</v>
+        <v>0.893</v>
       </c>
       <c r="D10" s="40" t="n">
-        <v>-0.062</v>
+        <v>-0.092</v>
       </c>
       <c r="E10" s="40" t="n">
-        <v>-0.08699999999999999</v>
-      </c>
-      <c r="F10" s="40" t="inlineStr">
-        <is>
-          <t>-0.113*</t>
-        </is>
+        <v>-0.061</v>
+      </c>
+      <c r="F10" s="40" t="n">
+        <v>-0.08</v>
       </c>
       <c r="G10" s="40" t="n">
-        <v>-0.06900000000000001</v>
+        <v>-0.076</v>
       </c>
       <c r="H10" s="40" t="n">
-        <v>-0.073</v>
+        <v>-0.036</v>
       </c>
       <c r="I10" s="40" t="n">
-        <v>-0.015</v>
+        <v>-0.017</v>
       </c>
       <c r="J10" s="40" t="n">
-        <v>0.001</v>
+        <v>-0.024</v>
       </c>
       <c r="K10" s="40" t="inlineStr">
         <is>
@@ -2187,38 +2183,38 @@
         </is>
       </c>
       <c r="B11" s="40" t="n">
-        <v>4.467</v>
+        <v>4.46</v>
       </c>
       <c r="C11" s="40" t="n">
-        <v>1.229</v>
+        <v>1.236</v>
       </c>
       <c r="D11" s="40" t="n">
-        <v>-0.064</v>
+        <v>-0.042</v>
       </c>
       <c r="E11" s="40" t="n">
-        <v>0.018</v>
+        <v>0.029</v>
       </c>
       <c r="F11" s="40" t="n">
-        <v>-0.033</v>
+        <v>0.007</v>
       </c>
       <c r="G11" s="40" t="n">
-        <v>-0.043</v>
+        <v>-0.07099999999999999</v>
       </c>
       <c r="H11" s="40" t="inlineStr">
         <is>
-          <t>-0.528***</t>
+          <t>-0.521***</t>
         </is>
       </c>
       <c r="I11" s="40" t="inlineStr">
         <is>
-          <t>0.5***</t>
+          <t>0.522***</t>
         </is>
       </c>
       <c r="J11" s="40" t="n">
-        <v>0.015</v>
+        <v>0.001</v>
       </c>
       <c r="K11" s="40" t="n">
-        <v>-0.012</v>
+        <v>-0.008999999999999999</v>
       </c>
       <c r="L11" s="40" t="inlineStr">
         <is>
@@ -2233,42 +2229,42 @@
         </is>
       </c>
       <c r="B12" s="40" t="n">
-        <v>3.078</v>
+        <v>3.095</v>
       </c>
       <c r="C12" s="40" t="n">
-        <v>1.189</v>
+        <v>1.208</v>
       </c>
       <c r="D12" s="40" t="n">
-        <v>0.039</v>
+        <v>0.002</v>
       </c>
       <c r="E12" s="40" t="n">
-        <v>0.021</v>
+        <v>0.004</v>
       </c>
       <c r="F12" s="40" t="n">
-        <v>0.01</v>
+        <v>-0.067</v>
       </c>
       <c r="G12" s="40" t="n">
-        <v>0.026</v>
+        <v>0.04</v>
       </c>
       <c r="H12" s="40" t="inlineStr">
         <is>
-          <t>0.526***</t>
+          <t>0.54***</t>
         </is>
       </c>
       <c r="I12" s="40" t="inlineStr">
         <is>
-          <t>-0.505***</t>
+          <t>-0.508***</t>
         </is>
       </c>
       <c r="J12" s="40" t="n">
-        <v>0.027</v>
+        <v>0.042</v>
       </c>
       <c r="K12" s="40" t="n">
-        <v>-0.095</v>
+        <v>-0.076</v>
       </c>
       <c r="L12" s="40" t="inlineStr">
         <is>
-          <t>-0.446***</t>
+          <t>-0.431***</t>
         </is>
       </c>
       <c r="M12" s="40" t="inlineStr">
@@ -2284,42 +2280,42 @@
         </is>
       </c>
       <c r="B13" s="40" t="n">
-        <v>4.38</v>
+        <v>4.399</v>
       </c>
       <c r="C13" s="40" t="n">
-        <v>0.626</v>
+        <v>0.644</v>
       </c>
       <c r="D13" s="40" t="n">
-        <v>0.012</v>
+        <v>0.015</v>
       </c>
       <c r="E13" s="40" t="n">
-        <v>-0.021</v>
+        <v>-0.019</v>
       </c>
       <c r="F13" s="40" t="n">
-        <v>0.015</v>
+        <v>-0.026</v>
       </c>
       <c r="G13" s="40" t="n">
-        <v>-0.036</v>
+        <v>-0.025</v>
       </c>
       <c r="H13" s="40" t="n">
-        <v>0.03</v>
+        <v>0.058</v>
       </c>
       <c r="I13" s="40" t="n">
-        <v>-0.056</v>
+        <v>-0.066</v>
       </c>
       <c r="J13" s="40" t="inlineStr">
         <is>
-          <t>-0.166**</t>
+          <t>-0.135*</t>
         </is>
       </c>
       <c r="K13" s="40" t="n">
-        <v>-0.032</v>
+        <v>-0.076</v>
       </c>
       <c r="L13" s="40" t="n">
-        <v>-0.021</v>
+        <v>0.003</v>
       </c>
       <c r="M13" s="40" t="n">
-        <v>0.068</v>
+        <v>0.08</v>
       </c>
       <c r="N13" s="40" t="inlineStr">
         <is>
@@ -2334,40 +2330,38 @@
         </is>
       </c>
       <c r="B14" s="40" t="n">
-        <v>4.515</v>
+        <v>4.498</v>
       </c>
       <c r="C14" s="40" t="n">
-        <v>0.778</v>
+        <v>0.766</v>
       </c>
       <c r="D14" s="40" t="n">
-        <v>-0.01</v>
+        <v>-0.026</v>
       </c>
       <c r="E14" s="40" t="n">
-        <v>-0.025</v>
+        <v>0.005</v>
       </c>
       <c r="F14" s="40" t="n">
-        <v>0.019</v>
+        <v>0.04</v>
       </c>
       <c r="G14" s="40" t="n">
-        <v>-0.031</v>
+        <v>-0.068</v>
       </c>
       <c r="H14" s="40" t="inlineStr">
         <is>
-          <t>-0.403***</t>
+          <t>-0.443***</t>
         </is>
       </c>
       <c r="I14" s="40" t="inlineStr">
         <is>
-          <t>0.42***</t>
-        </is>
-      </c>
-      <c r="J14" s="40" t="inlineStr">
-        <is>
-          <t>-0.127*</t>
-        </is>
+          <t>0.422***</t>
+        </is>
+      </c>
+      <c r="J14" s="40" t="n">
+        <v>-0.041</v>
       </c>
       <c r="K14" s="40" t="n">
-        <v>0.002</v>
+        <v>0.011</v>
       </c>
       <c r="L14" s="40" t="inlineStr">
         <is>
@@ -2381,7 +2375,7 @@
       </c>
       <c r="N14" s="40" t="inlineStr">
         <is>
-          <t>0.367***</t>
+          <t>0.398***</t>
         </is>
       </c>
       <c r="O14" s="40" t="inlineStr">
@@ -2400,41 +2394,39 @@
         <v>4.65</v>
       </c>
       <c r="C15" s="40" t="n">
-        <v>1.273</v>
+        <v>1.192</v>
       </c>
       <c r="D15" s="40" t="n">
-        <v>0.006</v>
+        <v>0.013</v>
       </c>
       <c r="E15" s="40" t="n">
-        <v>-0.029</v>
+        <v>-0.028</v>
       </c>
       <c r="F15" s="40" t="n">
-        <v>0.021</v>
+        <v>-0.04</v>
       </c>
       <c r="G15" s="40" t="n">
-        <v>-0.007</v>
+        <v>0.055</v>
       </c>
       <c r="H15" s="40" t="inlineStr">
         <is>
-          <t>-0.248***</t>
+          <t>-0.279***</t>
         </is>
       </c>
       <c r="I15" s="40" t="inlineStr">
         <is>
-          <t>0.274***</t>
+          <t>0.3***</t>
         </is>
       </c>
       <c r="J15" s="40" t="n">
         <v>0.014</v>
       </c>
-      <c r="K15" s="40" t="inlineStr">
-        <is>
-          <t>-0.113*</t>
-        </is>
+      <c r="K15" s="40" t="n">
+        <v>-0.037</v>
       </c>
       <c r="L15" s="40" t="inlineStr">
         <is>
-          <t>0.442***</t>
+          <t>0.396***</t>
         </is>
       </c>
       <c r="M15" s="40" t="inlineStr">
@@ -2443,11 +2435,11 @@
         </is>
       </c>
       <c r="N15" s="40" t="n">
-        <v>-0.039</v>
+        <v>-0.074</v>
       </c>
       <c r="O15" s="40" t="inlineStr">
         <is>
-          <t>0.339***</t>
+          <t>0.283***</t>
         </is>
       </c>
       <c r="P15" s="40" t="inlineStr">
@@ -2463,55 +2455,57 @@
         </is>
       </c>
       <c r="B16" s="40" t="n">
-        <v>2.608</v>
+        <v>2.561</v>
       </c>
       <c r="C16" s="40" t="n">
-        <v>1.051</v>
+        <v>0.995</v>
       </c>
       <c r="D16" s="40" t="n">
-        <v>0.041</v>
+        <v>0.065</v>
       </c>
       <c r="E16" s="40" t="n">
-        <v>0.017</v>
-      </c>
-      <c r="F16" s="40" t="n">
-        <v>-0.05</v>
+        <v>0.003</v>
+      </c>
+      <c r="F16" s="40" t="inlineStr">
+        <is>
+          <t>-0.114*</t>
+        </is>
       </c>
       <c r="G16" s="40" t="n">
-        <v>0.02</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="H16" s="40" t="inlineStr">
         <is>
-          <t>0.253***</t>
+          <t>0.288***</t>
         </is>
       </c>
       <c r="I16" s="40" t="inlineStr">
         <is>
-          <t>-0.213***</t>
+          <t>-0.336***</t>
         </is>
       </c>
       <c r="J16" s="40" t="n">
-        <v>0.051</v>
+        <v>-0.024</v>
       </c>
       <c r="K16" s="40" t="n">
-        <v>-0.054</v>
+        <v>-0.02</v>
       </c>
       <c r="L16" s="40" t="inlineStr">
         <is>
-          <t>-0.299***</t>
+          <t>-0.359***</t>
         </is>
       </c>
       <c r="M16" s="40" t="inlineStr">
         <is>
-          <t>0.273***</t>
+          <t>0.326***</t>
         </is>
       </c>
       <c r="N16" s="40" t="n">
-        <v>-0.024</v>
+        <v>0.06</v>
       </c>
       <c r="O16" s="40" t="inlineStr">
         <is>
-          <t>-0.189***</t>
+          <t>-0.265***</t>
         </is>
       </c>
       <c r="P16" s="40" t="inlineStr">
@@ -2528,7 +2522,7 @@
     <row r="17" ht="35" customHeight="1" s="45">
       <c r="A17" s="23" t="inlineStr">
         <is>
-          <t>Note. Values on the diagonal are Cronbach’s alpha coefficients where applicable. Correlations are zero-order correlations among observed study variables. Leadership variables were rated by followers at T1. OCBS and CWBS were rated by leaders at T3. N = 363. *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
+          <t>Note. Values on the diagonal are Cronbach’s alpha coefficients where applicable. Correlations are zero-order correlations among observed study variables. Leadership variables were rated by followers at T1. OCBS and CWBS were rated by leaders at T3. N = 361. *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -3886,7 +3880,7 @@
     <row r="28" ht="48" customHeight="1" s="45">
       <c r="A28" s="23" t="inlineStr">
         <is>
-          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 363; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.  *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
+          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 361; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.  *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -6108,7 +6102,7 @@
     <row r="2">
       <c r="A2" s="38" t="inlineStr">
         <is>
-          <t>N = 363</t>
+          <t>N = 361</t>
         </is>
       </c>
     </row>
@@ -6122,14 +6116,14 @@
     <row r="4">
       <c r="A4" s="38" t="inlineStr">
         <is>
-          <t>- Male: 192 (52.9%)</t>
+          <t>- Male: 201 (55.7%)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="38" t="inlineStr">
         <is>
-          <t>- Female: 171 (47.1%)</t>
+          <t>- Female: 160 (44.3%)</t>
         </is>
       </c>
     </row>
@@ -6144,21 +6138,21 @@
     <row r="8">
       <c r="A8" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 30.83, SD = 4.55</t>
+          <t>Age: M = 30.78, SD = 4.59</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="38" t="inlineStr">
         <is>
-          <t>Working years: M = 9.05, SD = 4.82</t>
+          <t>Working years: M = 9.00, SD = 4.82</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="38" t="inlineStr">
         <is>
-          <t>Tenure with current leader: M = 2.35, SD = 1.49</t>
+          <t>Tenure with current leader: M = 2.36, SD = 1.48</t>
         </is>
       </c>
     </row>
@@ -6166,11 +6160,11 @@
       <c r="A11" s="48" t="inlineStr">
         <is>
           <t>Interaction frequency with leader:
-  - Rarely (&lt;1/wk): 19 (5.2%)
-  - Sometimes (1-2/wk): 65 (17.9%)
-  - Often (3-4/wk): 120 (33.1%)
-  - Very often (~daily): 107 (29.5%)
-  - Multiple times/day: 52 (14.3%)</t>
+  - Rarely (&lt;1/wk): 18 (5.0%)
+  - Sometimes (1-2/wk): 66 (18.3%)
+  - Often (3-4/wk): 117 (32.4%)
+  - Very often (~daily): 111 (30.7%)
+  - Multiple times/day: 49 (13.6%)</t>
         </is>
       </c>
     </row>
@@ -6185,28 +6179,28 @@
     <row r="14">
       <c r="A14" s="38" t="inlineStr">
         <is>
-          <t>- High school: 19 (5.2%)</t>
+          <t>- High school: 16 (4.4%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 64 (17.6%)</t>
+          <t>- Some college / Associate: 60 (16.6%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 166 (45.7%)</t>
+          <t>- Bachelor: 169 (46.8%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="38" t="inlineStr">
         <is>
-          <t>- Master: 88 (24.2%)</t>
+          <t>- Master: 90 (24.9%)</t>
         </is>
       </c>
     </row>
@@ -6228,35 +6222,35 @@
     <row r="21">
       <c r="A21" s="38" t="inlineStr">
         <is>
-          <t>- Entry: 67 (18.5%)</t>
+          <t>- Entry: 64 (17.7%)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="38" t="inlineStr">
         <is>
-          <t>- Associate: 117 (32.2%)</t>
+          <t>- Associate: 119 (33.0%)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="38" t="inlineStr">
         <is>
-          <t>- Senior: 94 (25.9%)</t>
+          <t>- Senior: 95 (26.3%)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="38" t="inlineStr">
         <is>
-          <t>- Manager: 64 (17.6%)</t>
+          <t>- Manager: 62 (17.2%)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="38" t="inlineStr">
         <is>
-          <t>- Director: 17 (4.7%)</t>
+          <t>- Director: 18 (5.0%)</t>
         </is>
       </c>
     </row>
@@ -6286,14 +6280,14 @@
     <row r="31">
       <c r="A31" s="38" t="inlineStr">
         <is>
-          <t>- Male: 46 (58.2%)</t>
+          <t>- Male: 51 (64.6%)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="38" t="inlineStr">
         <is>
-          <t>- Female: 33 (41.8%)</t>
+          <t>- Female: 28 (35.4%)</t>
         </is>
       </c>
     </row>
@@ -6308,7 +6302,7 @@
     <row r="35">
       <c r="A35" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 40.91, SD = 6.40</t>
+          <t>Age: M = 40.95, SD = 6.47</t>
         </is>
       </c>
     </row>
@@ -6322,14 +6316,14 @@
     <row r="37">
       <c r="A37" s="38" t="inlineStr">
         <is>
-          <t>Leadership tenure: M = 5.33, SD = 3.14</t>
+          <t>Leadership tenure: M = 5.40, SD = 2.73</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="38" t="inlineStr">
         <is>
-          <t>Span of control: M = 4.59, SD = 0.63</t>
+          <t>Span of control: M = 4.57, SD = 0.57</t>
         </is>
       </c>
     </row>
@@ -6351,21 +6345,21 @@
     <row r="42">
       <c r="A42" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 42 (53.2%)</t>
+          <t>- Bachelor: 40 (50.6%)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="38" t="inlineStr">
         <is>
-          <t>- Master: 23 (29.1%)</t>
+          <t>- Master: 26 (32.9%)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="38" t="inlineStr">
         <is>
-          <t>- Doctorate: 7 (8.9%)</t>
+          <t>- Doctorate: 6 (7.6%)</t>
         </is>
       </c>
     </row>
@@ -6685,7 +6679,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="9">
@@ -6715,7 +6709,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="12">
@@ -6818,7 +6812,7 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>78.9%</t>
+          <t>78.5%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sync v4.6 fresh: regenerated data+results identical between main and delivery
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -1951,10 +1951,10 @@
         </is>
       </c>
       <c r="B3" s="40" t="n">
-        <v>0.529</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="C3" s="40" t="n">
-        <v>0.5</v>
+        <v>0.497</v>
       </c>
       <c r="D3" s="40" t="inlineStr">
         <is>
@@ -1969,13 +1969,13 @@
         </is>
       </c>
       <c r="B4" s="40" t="n">
-        <v>30.832</v>
+        <v>30.781</v>
       </c>
       <c r="C4" s="40" t="n">
-        <v>4.55</v>
+        <v>4.593</v>
       </c>
       <c r="D4" s="40" t="n">
-        <v>0.044</v>
+        <v>0.017</v>
       </c>
       <c r="E4" s="40" t="inlineStr">
         <is>
@@ -1990,17 +1990,17 @@
         </is>
       </c>
       <c r="B5" s="40" t="n">
-        <v>2.347</v>
+        <v>2.359</v>
       </c>
       <c r="C5" s="40" t="n">
-        <v>1.487</v>
+        <v>1.476</v>
       </c>
       <c r="D5" s="40" t="n">
-        <v>-0.004</v>
+        <v>-0.027</v>
       </c>
       <c r="E5" s="40" t="inlineStr">
         <is>
-          <t>0.175***</t>
+          <t>0.178***</t>
         </is>
       </c>
       <c r="F5" s="40" t="inlineStr">
@@ -2016,19 +2016,19 @@
         </is>
       </c>
       <c r="B6" s="40" t="n">
-        <v>3.298</v>
+        <v>3.296</v>
       </c>
       <c r="C6" s="40" t="n">
-        <v>1.082</v>
+        <v>1.071</v>
       </c>
       <c r="D6" s="40" t="n">
-        <v>0.081</v>
+        <v>0.101</v>
       </c>
       <c r="E6" s="40" t="n">
-        <v>-0.012</v>
+        <v>-0.008999999999999999</v>
       </c>
       <c r="F6" s="40" t="n">
-        <v>-0.081</v>
+        <v>-0.079</v>
       </c>
       <c r="G6" s="40" t="inlineStr">
         <is>
@@ -2043,24 +2043,22 @@
         </is>
       </c>
       <c r="B7" s="40" t="n">
-        <v>4.075</v>
+        <v>4.083</v>
       </c>
       <c r="C7" s="40" t="n">
-        <v>0.893</v>
+        <v>0.885</v>
       </c>
       <c r="D7" s="40" t="n">
-        <v>-0.012</v>
+        <v>-0.059</v>
       </c>
       <c r="E7" s="40" t="n">
-        <v>-0.014</v>
-      </c>
-      <c r="F7" s="40" t="inlineStr">
-        <is>
-          <t>0.11*</t>
-        </is>
+        <v>-0.034</v>
+      </c>
+      <c r="F7" s="40" t="n">
+        <v>0.077</v>
       </c>
       <c r="G7" s="40" t="n">
-        <v>-0.012</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="H7" s="39" t="inlineStr">
         <is>
@@ -2075,26 +2073,26 @@
         </is>
       </c>
       <c r="B8" s="40" t="n">
-        <v>4.881</v>
+        <v>4.898</v>
       </c>
       <c r="C8" s="40" t="n">
-        <v>0.9350000000000001</v>
+        <v>0.971</v>
       </c>
       <c r="D8" s="40" t="n">
-        <v>-0.022</v>
+        <v>-0.025</v>
       </c>
       <c r="E8" s="40" t="n">
-        <v>-0.004</v>
+        <v>-0.008</v>
       </c>
       <c r="F8" s="40" t="n">
-        <v>0.024</v>
+        <v>0.035</v>
       </c>
       <c r="G8" s="40" t="n">
-        <v>-0.06</v>
+        <v>-0.08400000000000001</v>
       </c>
       <c r="H8" s="40" t="inlineStr">
         <is>
-          <t>-0.34***</t>
+          <t>-0.342***</t>
         </is>
       </c>
       <c r="I8" s="40" t="inlineStr">
@@ -2110,28 +2108,28 @@
         </is>
       </c>
       <c r="B9" s="40" t="n">
-        <v>3.485</v>
+        <v>3.479</v>
       </c>
       <c r="C9" s="40" t="n">
-        <v>0.913</v>
+        <v>0.885</v>
       </c>
       <c r="D9" s="40" t="n">
-        <v>-0.078</v>
+        <v>-0.05</v>
       </c>
       <c r="E9" s="40" t="n">
-        <v>-0.06900000000000001</v>
+        <v>-0.032</v>
       </c>
       <c r="F9" s="40" t="n">
-        <v>0.049</v>
+        <v>0.06</v>
       </c>
       <c r="G9" s="40" t="n">
-        <v>-0.057</v>
+        <v>-0.066</v>
       </c>
       <c r="H9" s="40" t="n">
-        <v>-0.008</v>
+        <v>0.021</v>
       </c>
       <c r="I9" s="40" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.078</v>
       </c>
       <c r="J9" s="40" t="inlineStr">
         <is>
@@ -2146,33 +2144,31 @@
         </is>
       </c>
       <c r="B10" s="40" t="n">
-        <v>4.625</v>
+        <v>4.599</v>
       </c>
       <c r="C10" s="40" t="n">
-        <v>0.883</v>
+        <v>0.893</v>
       </c>
       <c r="D10" s="40" t="n">
-        <v>-0.062</v>
+        <v>-0.092</v>
       </c>
       <c r="E10" s="40" t="n">
-        <v>-0.08699999999999999</v>
-      </c>
-      <c r="F10" s="40" t="inlineStr">
-        <is>
-          <t>-0.113*</t>
-        </is>
+        <v>-0.061</v>
+      </c>
+      <c r="F10" s="40" t="n">
+        <v>-0.08</v>
       </c>
       <c r="G10" s="40" t="n">
-        <v>-0.06900000000000001</v>
+        <v>-0.076</v>
       </c>
       <c r="H10" s="40" t="n">
-        <v>-0.073</v>
+        <v>-0.036</v>
       </c>
       <c r="I10" s="40" t="n">
-        <v>-0.015</v>
+        <v>-0.017</v>
       </c>
       <c r="J10" s="40" t="n">
-        <v>0.001</v>
+        <v>-0.024</v>
       </c>
       <c r="K10" s="40" t="inlineStr">
         <is>
@@ -2187,38 +2183,38 @@
         </is>
       </c>
       <c r="B11" s="40" t="n">
-        <v>4.467</v>
+        <v>4.46</v>
       </c>
       <c r="C11" s="40" t="n">
-        <v>1.229</v>
+        <v>1.236</v>
       </c>
       <c r="D11" s="40" t="n">
-        <v>-0.064</v>
+        <v>-0.042</v>
       </c>
       <c r="E11" s="40" t="n">
-        <v>0.018</v>
+        <v>0.029</v>
       </c>
       <c r="F11" s="40" t="n">
-        <v>-0.033</v>
+        <v>0.007</v>
       </c>
       <c r="G11" s="40" t="n">
-        <v>-0.043</v>
+        <v>-0.07099999999999999</v>
       </c>
       <c r="H11" s="40" t="inlineStr">
         <is>
-          <t>-0.528***</t>
+          <t>-0.521***</t>
         </is>
       </c>
       <c r="I11" s="40" t="inlineStr">
         <is>
-          <t>0.5***</t>
+          <t>0.522***</t>
         </is>
       </c>
       <c r="J11" s="40" t="n">
-        <v>0.015</v>
+        <v>0.001</v>
       </c>
       <c r="K11" s="40" t="n">
-        <v>-0.012</v>
+        <v>-0.008999999999999999</v>
       </c>
       <c r="L11" s="40" t="inlineStr">
         <is>
@@ -2233,42 +2229,42 @@
         </is>
       </c>
       <c r="B12" s="40" t="n">
-        <v>3.078</v>
+        <v>3.095</v>
       </c>
       <c r="C12" s="40" t="n">
-        <v>1.189</v>
+        <v>1.208</v>
       </c>
       <c r="D12" s="40" t="n">
-        <v>0.039</v>
+        <v>0.002</v>
       </c>
       <c r="E12" s="40" t="n">
-        <v>0.021</v>
+        <v>0.004</v>
       </c>
       <c r="F12" s="40" t="n">
-        <v>0.01</v>
+        <v>-0.067</v>
       </c>
       <c r="G12" s="40" t="n">
-        <v>0.026</v>
+        <v>0.04</v>
       </c>
       <c r="H12" s="40" t="inlineStr">
         <is>
-          <t>0.526***</t>
+          <t>0.54***</t>
         </is>
       </c>
       <c r="I12" s="40" t="inlineStr">
         <is>
-          <t>-0.505***</t>
+          <t>-0.508***</t>
         </is>
       </c>
       <c r="J12" s="40" t="n">
-        <v>0.027</v>
+        <v>0.042</v>
       </c>
       <c r="K12" s="40" t="n">
-        <v>-0.095</v>
+        <v>-0.076</v>
       </c>
       <c r="L12" s="40" t="inlineStr">
         <is>
-          <t>-0.446***</t>
+          <t>-0.431***</t>
         </is>
       </c>
       <c r="M12" s="40" t="inlineStr">
@@ -2284,42 +2280,42 @@
         </is>
       </c>
       <c r="B13" s="40" t="n">
-        <v>4.38</v>
+        <v>4.399</v>
       </c>
       <c r="C13" s="40" t="n">
-        <v>0.626</v>
+        <v>0.644</v>
       </c>
       <c r="D13" s="40" t="n">
-        <v>0.012</v>
+        <v>0.015</v>
       </c>
       <c r="E13" s="40" t="n">
-        <v>-0.021</v>
+        <v>-0.019</v>
       </c>
       <c r="F13" s="40" t="n">
-        <v>0.015</v>
+        <v>-0.026</v>
       </c>
       <c r="G13" s="40" t="n">
-        <v>-0.036</v>
+        <v>-0.025</v>
       </c>
       <c r="H13" s="40" t="n">
-        <v>0.03</v>
+        <v>0.058</v>
       </c>
       <c r="I13" s="40" t="n">
-        <v>-0.056</v>
+        <v>-0.066</v>
       </c>
       <c r="J13" s="40" t="inlineStr">
         <is>
-          <t>-0.166**</t>
+          <t>-0.135*</t>
         </is>
       </c>
       <c r="K13" s="40" t="n">
-        <v>-0.032</v>
+        <v>-0.076</v>
       </c>
       <c r="L13" s="40" t="n">
-        <v>-0.021</v>
+        <v>0.003</v>
       </c>
       <c r="M13" s="40" t="n">
-        <v>0.068</v>
+        <v>0.08</v>
       </c>
       <c r="N13" s="40" t="inlineStr">
         <is>
@@ -2334,40 +2330,38 @@
         </is>
       </c>
       <c r="B14" s="40" t="n">
-        <v>4.515</v>
+        <v>4.498</v>
       </c>
       <c r="C14" s="40" t="n">
-        <v>0.778</v>
+        <v>0.766</v>
       </c>
       <c r="D14" s="40" t="n">
-        <v>-0.01</v>
+        <v>-0.026</v>
       </c>
       <c r="E14" s="40" t="n">
-        <v>-0.025</v>
+        <v>0.005</v>
       </c>
       <c r="F14" s="40" t="n">
-        <v>0.019</v>
+        <v>0.04</v>
       </c>
       <c r="G14" s="40" t="n">
-        <v>-0.031</v>
+        <v>-0.068</v>
       </c>
       <c r="H14" s="40" t="inlineStr">
         <is>
-          <t>-0.403***</t>
+          <t>-0.443***</t>
         </is>
       </c>
       <c r="I14" s="40" t="inlineStr">
         <is>
-          <t>0.42***</t>
-        </is>
-      </c>
-      <c r="J14" s="40" t="inlineStr">
-        <is>
-          <t>-0.127*</t>
-        </is>
+          <t>0.422***</t>
+        </is>
+      </c>
+      <c r="J14" s="40" t="n">
+        <v>-0.041</v>
       </c>
       <c r="K14" s="40" t="n">
-        <v>0.002</v>
+        <v>0.011</v>
       </c>
       <c r="L14" s="40" t="inlineStr">
         <is>
@@ -2381,7 +2375,7 @@
       </c>
       <c r="N14" s="40" t="inlineStr">
         <is>
-          <t>0.367***</t>
+          <t>0.398***</t>
         </is>
       </c>
       <c r="O14" s="40" t="inlineStr">
@@ -2400,41 +2394,39 @@
         <v>4.65</v>
       </c>
       <c r="C15" s="40" t="n">
-        <v>1.273</v>
+        <v>1.192</v>
       </c>
       <c r="D15" s="40" t="n">
-        <v>0.006</v>
+        <v>0.013</v>
       </c>
       <c r="E15" s="40" t="n">
-        <v>-0.029</v>
+        <v>-0.028</v>
       </c>
       <c r="F15" s="40" t="n">
-        <v>0.021</v>
+        <v>-0.04</v>
       </c>
       <c r="G15" s="40" t="n">
-        <v>-0.007</v>
+        <v>0.055</v>
       </c>
       <c r="H15" s="40" t="inlineStr">
         <is>
-          <t>-0.248***</t>
+          <t>-0.279***</t>
         </is>
       </c>
       <c r="I15" s="40" t="inlineStr">
         <is>
-          <t>0.274***</t>
+          <t>0.3***</t>
         </is>
       </c>
       <c r="J15" s="40" t="n">
         <v>0.014</v>
       </c>
-      <c r="K15" s="40" t="inlineStr">
-        <is>
-          <t>-0.113*</t>
-        </is>
+      <c r="K15" s="40" t="n">
+        <v>-0.037</v>
       </c>
       <c r="L15" s="40" t="inlineStr">
         <is>
-          <t>0.442***</t>
+          <t>0.396***</t>
         </is>
       </c>
       <c r="M15" s="40" t="inlineStr">
@@ -2443,11 +2435,11 @@
         </is>
       </c>
       <c r="N15" s="40" t="n">
-        <v>-0.039</v>
+        <v>-0.074</v>
       </c>
       <c r="O15" s="40" t="inlineStr">
         <is>
-          <t>0.339***</t>
+          <t>0.283***</t>
         </is>
       </c>
       <c r="P15" s="40" t="inlineStr">
@@ -2463,55 +2455,57 @@
         </is>
       </c>
       <c r="B16" s="40" t="n">
-        <v>2.608</v>
+        <v>2.561</v>
       </c>
       <c r="C16" s="40" t="n">
-        <v>1.051</v>
+        <v>0.995</v>
       </c>
       <c r="D16" s="40" t="n">
-        <v>0.041</v>
+        <v>0.065</v>
       </c>
       <c r="E16" s="40" t="n">
-        <v>0.017</v>
-      </c>
-      <c r="F16" s="40" t="n">
-        <v>-0.05</v>
+        <v>0.003</v>
+      </c>
+      <c r="F16" s="40" t="inlineStr">
+        <is>
+          <t>-0.114*</t>
+        </is>
       </c>
       <c r="G16" s="40" t="n">
-        <v>0.02</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="H16" s="40" t="inlineStr">
         <is>
-          <t>0.253***</t>
+          <t>0.288***</t>
         </is>
       </c>
       <c r="I16" s="40" t="inlineStr">
         <is>
-          <t>-0.213***</t>
+          <t>-0.336***</t>
         </is>
       </c>
       <c r="J16" s="40" t="n">
-        <v>0.051</v>
+        <v>-0.024</v>
       </c>
       <c r="K16" s="40" t="n">
-        <v>-0.054</v>
+        <v>-0.02</v>
       </c>
       <c r="L16" s="40" t="inlineStr">
         <is>
-          <t>-0.299***</t>
+          <t>-0.359***</t>
         </is>
       </c>
       <c r="M16" s="40" t="inlineStr">
         <is>
-          <t>0.273***</t>
+          <t>0.326***</t>
         </is>
       </c>
       <c r="N16" s="40" t="n">
-        <v>-0.024</v>
+        <v>0.06</v>
       </c>
       <c r="O16" s="40" t="inlineStr">
         <is>
-          <t>-0.189***</t>
+          <t>-0.265***</t>
         </is>
       </c>
       <c r="P16" s="40" t="inlineStr">
@@ -2528,7 +2522,7 @@
     <row r="17" ht="35" customHeight="1" s="45">
       <c r="A17" s="23" t="inlineStr">
         <is>
-          <t>Note. Values on the diagonal are Cronbach’s alpha coefficients where applicable. Correlations are zero-order correlations among observed study variables. Leadership variables were rated by followers at T1. OCBS and CWBS were rated by leaders at T3. N = 363. *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
+          <t>Note. Values on the diagonal are Cronbach’s alpha coefficients where applicable. Correlations are zero-order correlations among observed study variables. Leadership variables were rated by followers at T1. OCBS and CWBS were rated by leaders at T3. N = 361. *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -3886,7 +3880,7 @@
     <row r="28" ht="48" customHeight="1" s="45">
       <c r="A28" s="23" t="inlineStr">
         <is>
-          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 363; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.  *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
+          <t>Note. Entries are unstandardized coefficients (b) and standard errors (SE) from multilevel models with followers nested within leaders. Leadership variables were measured at T1, mediators at T2, and outcomes at T3. Thriving at T1 was included only as a baseline control in the model predicting thriving at T3. Interaction terms were estimated only in the mediator interaction models. Pseudo R² values are reported separately for within- and between-leader variance explained. Em dashes indicate that a predictor was not included in a given model. Follower N = 361; Leader N = 79. * p &lt; .05. ** p &lt; .01. *** p &lt; .001.  *p &lt; .05. **p &lt; .01. ***p &lt; .001.</t>
         </is>
       </c>
     </row>
@@ -6108,7 +6102,7 @@
     <row r="2">
       <c r="A2" s="38" t="inlineStr">
         <is>
-          <t>N = 363</t>
+          <t>N = 361</t>
         </is>
       </c>
     </row>
@@ -6122,14 +6116,14 @@
     <row r="4">
       <c r="A4" s="38" t="inlineStr">
         <is>
-          <t>- Male: 192 (52.9%)</t>
+          <t>- Male: 201 (55.7%)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="38" t="inlineStr">
         <is>
-          <t>- Female: 171 (47.1%)</t>
+          <t>- Female: 160 (44.3%)</t>
         </is>
       </c>
     </row>
@@ -6144,21 +6138,21 @@
     <row r="8">
       <c r="A8" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 30.83, SD = 4.55</t>
+          <t>Age: M = 30.78, SD = 4.59</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="38" t="inlineStr">
         <is>
-          <t>Working years: M = 9.05, SD = 4.82</t>
+          <t>Working years: M = 9.00, SD = 4.82</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="38" t="inlineStr">
         <is>
-          <t>Tenure with current leader: M = 2.35, SD = 1.49</t>
+          <t>Tenure with current leader: M = 2.36, SD = 1.48</t>
         </is>
       </c>
     </row>
@@ -6166,11 +6160,11 @@
       <c r="A11" s="48" t="inlineStr">
         <is>
           <t>Interaction frequency with leader:
-  - Rarely (&lt;1/wk): 19 (5.2%)
-  - Sometimes (1-2/wk): 65 (17.9%)
-  - Often (3-4/wk): 120 (33.1%)
-  - Very often (~daily): 107 (29.5%)
-  - Multiple times/day: 52 (14.3%)</t>
+  - Rarely (&lt;1/wk): 18 (5.0%)
+  - Sometimes (1-2/wk): 66 (18.3%)
+  - Often (3-4/wk): 117 (32.4%)
+  - Very often (~daily): 111 (30.7%)
+  - Multiple times/day: 49 (13.6%)</t>
         </is>
       </c>
     </row>
@@ -6185,28 +6179,28 @@
     <row r="14">
       <c r="A14" s="38" t="inlineStr">
         <is>
-          <t>- High school: 19 (5.2%)</t>
+          <t>- High school: 16 (4.4%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 64 (17.6%)</t>
+          <t>- Some college / Associate: 60 (16.6%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 166 (45.7%)</t>
+          <t>- Bachelor: 169 (46.8%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="38" t="inlineStr">
         <is>
-          <t>- Master: 88 (24.2%)</t>
+          <t>- Master: 90 (24.9%)</t>
         </is>
       </c>
     </row>
@@ -6228,35 +6222,35 @@
     <row r="21">
       <c r="A21" s="38" t="inlineStr">
         <is>
-          <t>- Entry: 67 (18.5%)</t>
+          <t>- Entry: 64 (17.7%)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="38" t="inlineStr">
         <is>
-          <t>- Associate: 117 (32.2%)</t>
+          <t>- Associate: 119 (33.0%)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="38" t="inlineStr">
         <is>
-          <t>- Senior: 94 (25.9%)</t>
+          <t>- Senior: 95 (26.3%)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="38" t="inlineStr">
         <is>
-          <t>- Manager: 64 (17.6%)</t>
+          <t>- Manager: 62 (17.2%)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="38" t="inlineStr">
         <is>
-          <t>- Director: 17 (4.7%)</t>
+          <t>- Director: 18 (5.0%)</t>
         </is>
       </c>
     </row>
@@ -6286,14 +6280,14 @@
     <row r="31">
       <c r="A31" s="38" t="inlineStr">
         <is>
-          <t>- Male: 46 (58.2%)</t>
+          <t>- Male: 51 (64.6%)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="38" t="inlineStr">
         <is>
-          <t>- Female: 33 (41.8%)</t>
+          <t>- Female: 28 (35.4%)</t>
         </is>
       </c>
     </row>
@@ -6308,7 +6302,7 @@
     <row r="35">
       <c r="A35" s="38" t="inlineStr">
         <is>
-          <t>Age: M = 40.91, SD = 6.40</t>
+          <t>Age: M = 40.95, SD = 6.47</t>
         </is>
       </c>
     </row>
@@ -6322,14 +6316,14 @@
     <row r="37">
       <c r="A37" s="38" t="inlineStr">
         <is>
-          <t>Leadership tenure: M = 5.33, SD = 3.14</t>
+          <t>Leadership tenure: M = 5.40, SD = 2.73</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="38" t="inlineStr">
         <is>
-          <t>Span of control: M = 4.59, SD = 0.63</t>
+          <t>Span of control: M = 4.57, SD = 0.57</t>
         </is>
       </c>
     </row>
@@ -6351,21 +6345,21 @@
     <row r="42">
       <c r="A42" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 42 (53.2%)</t>
+          <t>- Bachelor: 40 (50.6%)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="38" t="inlineStr">
         <is>
-          <t>- Master: 23 (29.1%)</t>
+          <t>- Master: 26 (32.9%)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="38" t="inlineStr">
         <is>
-          <t>- Doctorate: 7 (8.9%)</t>
+          <t>- Doctorate: 6 (7.6%)</t>
         </is>
       </c>
     </row>
@@ -6685,7 +6679,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="9">
@@ -6715,7 +6709,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="12">
@@ -6818,7 +6812,7 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>78.9%</t>
+          <t>78.5%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sync v4.7: round-3 gap closure
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -1727,28 +1727,28 @@
         </is>
       </c>
       <c r="D5" s="39" t="n">
-        <v>1576.5</v>
+        <v>1611.4</v>
       </c>
       <c r="E5" s="39" t="n">
         <v>547</v>
       </c>
       <c r="F5" s="39" t="n">
-        <v>0.916</v>
+        <v>0.913</v>
       </c>
       <c r="G5" s="39" t="n">
-        <v>0.906</v>
+        <v>0.903</v>
       </c>
       <c r="H5" s="39" t="n">
-        <v>0.057</v>
+        <v>0.058</v>
       </c>
       <c r="I5" s="39" t="n">
-        <v>0.046</v>
+        <v>0.047</v>
       </c>
       <c r="J5" s="39" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="K5" s="39" t="n">
-        <v>22828.9</v>
+        <v>22869.1</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" s="45">
@@ -1768,28 +1768,28 @@
         </is>
       </c>
       <c r="D6" s="39" t="n">
-        <v>1968.4</v>
+        <v>2078.6</v>
       </c>
       <c r="E6" s="39" t="n">
         <v>552</v>
       </c>
       <c r="F6" s="39" t="n">
-        <v>0.901</v>
+        <v>0.895</v>
       </c>
       <c r="G6" s="39" t="n">
-        <v>0.889</v>
+        <v>0.882</v>
       </c>
       <c r="H6" s="39" t="n">
-        <v>0.065</v>
+        <v>0.066</v>
       </c>
       <c r="I6" s="39" t="n">
-        <v>0.054</v>
+        <v>0.055</v>
       </c>
       <c r="J6" s="39" t="n">
-        <v>0.073</v>
+        <v>0.074</v>
       </c>
       <c r="K6" s="39" t="n">
-        <v>23164.7</v>
+        <v>23514.3</v>
       </c>
     </row>
     <row r="7">
@@ -1809,28 +1809,28 @@
         </is>
       </c>
       <c r="D7" s="39" t="n">
-        <v>3079.2</v>
+        <v>3463.8</v>
       </c>
       <c r="E7" s="39" t="n">
         <v>556</v>
       </c>
       <c r="F7" s="39" t="n">
-        <v>0.8120000000000001</v>
+        <v>0.798</v>
       </c>
       <c r="G7" s="39" t="n">
-        <v>0.798</v>
+        <v>0.781</v>
       </c>
       <c r="H7" s="39" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="I7" s="39" t="n">
-        <v>0.062</v>
+        <v>0.066</v>
       </c>
       <c r="J7" s="39" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.092</v>
       </c>
       <c r="K7" s="39" t="n">
-        <v>23530.2</v>
+        <v>24644.7</v>
       </c>
     </row>
     <row r="8" ht="58" customHeight="1" s="45">

</xml_diff>

<commit_message>
sync v4.8: deeper round-3 audit gap closure
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -6102,7 +6102,7 @@
     <row r="2">
       <c r="A2" s="38" t="inlineStr">
         <is>
-          <t>N = 361</t>
+          <t>N = 340</t>
         </is>
       </c>
     </row>
@@ -6116,21 +6116,21 @@
     <row r="4">
       <c r="A4" s="38" t="inlineStr">
         <is>
-          <t>- Male: 201 (55.7%)</t>
+          <t>- Male: 201 (59.1%)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="38" t="inlineStr">
         <is>
-          <t>- Female: 160 (44.3%)</t>
+          <t>- Female: 160 (47.1%)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="38" t="inlineStr">
         <is>
-          <t>- Other / prefer not to say: 0 (0.0%)</t>
+          <t>- Other / prefer not to say: -21 (-6.2%)</t>
         </is>
       </c>
     </row>
@@ -6179,35 +6179,35 @@
     <row r="14">
       <c r="A14" s="38" t="inlineStr">
         <is>
-          <t>- High school: 16 (4.4%)</t>
+          <t>- High school: 16 (4.7%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="38" t="inlineStr">
         <is>
-          <t>- Some college / Associate: 60 (16.6%)</t>
+          <t>- Some college / Associate: 60 (17.6%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="38" t="inlineStr">
         <is>
-          <t>- Bachelor: 169 (46.8%)</t>
+          <t>- Bachelor: 169 (49.7%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="38" t="inlineStr">
         <is>
-          <t>- Master: 90 (24.9%)</t>
+          <t>- Master: 90 (26.5%)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="38" t="inlineStr">
         <is>
-          <t>- Doctorate: 22 (6.1%)</t>
+          <t>- Doctorate: 22 (6.5%)</t>
         </is>
       </c>
     </row>
@@ -6222,35 +6222,35 @@
     <row r="21">
       <c r="A21" s="38" t="inlineStr">
         <is>
-          <t>- Entry: 64 (17.7%)</t>
+          <t>- Entry: 64 (18.8%)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="38" t="inlineStr">
         <is>
-          <t>- Associate: 119 (33.0%)</t>
+          <t>- Associate: 119 (35.0%)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="38" t="inlineStr">
         <is>
-          <t>- Senior: 95 (26.3%)</t>
+          <t>- Senior: 95 (27.9%)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="38" t="inlineStr">
         <is>
-          <t>- Manager: 62 (17.2%)</t>
+          <t>- Manager: 62 (18.2%)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="38" t="inlineStr">
         <is>
-          <t>- Director: 18 (5.0%)</t>
+          <t>- Director: 18 (5.3%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: switch to joint multilevel SEM (sync from main 44079c4)
Outcome equations (THR, OCBS, CWBS) now from simultaneous two-level
path model rather than separate-equation lme4. M->Y partials shift
by max 0.02; all directions and significance preserved.

Includes candidate Mplus path-model syntax (code/path_mplus_syntax.inp)
for reviewer verification.
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -2742,27 +2742,27 @@
       </c>
       <c r="J5" s="40" t="inlineStr">
         <is>
-          <t>0.004</t>
+          <t>0.000</t>
         </is>
       </c>
       <c r="K5" s="40" t="n">
-        <v>0.046</v>
+        <v>0</v>
       </c>
       <c r="L5" s="40" t="inlineStr">
         <is>
-          <t>-0.030</t>
+          <t>0.000</t>
         </is>
       </c>
       <c r="M5" s="40" t="n">
-        <v>0.098</v>
+        <v>0</v>
       </c>
       <c r="N5" s="40" t="inlineStr">
         <is>
-          <t>-0.005</t>
+          <t>0.000</t>
         </is>
       </c>
       <c r="O5" s="40" t="n">
-        <v>0.081</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="1" s="37">
@@ -2834,7 +2834,7 @@
       </c>
       <c r="L7" s="40" t="inlineStr">
         <is>
-          <t>0.016</t>
+          <t>0.017</t>
         </is>
       </c>
       <c r="M7" s="40" t="n">
@@ -2889,15 +2889,15 @@
       </c>
       <c r="J8" s="40" t="inlineStr">
         <is>
-          <t>-0.007</t>
+          <t>-0.001</t>
         </is>
       </c>
       <c r="K8" s="40" t="n">
-        <v>0.061</v>
+        <v>0.062</v>
       </c>
       <c r="L8" s="40" t="inlineStr">
         <is>
-          <t>0.057</t>
+          <t>0.053</t>
         </is>
       </c>
       <c r="M8" s="40" t="n">
@@ -2905,11 +2905,11 @@
       </c>
       <c r="N8" s="40" t="inlineStr">
         <is>
-          <t>0.006</t>
+          <t>0.009</t>
         </is>
       </c>
       <c r="O8" s="40" t="n">
-        <v>0.092</v>
+        <v>0.093</v>
       </c>
     </row>
     <row r="9">
@@ -2960,7 +2960,7 @@
       </c>
       <c r="L9" s="40" t="inlineStr">
         <is>
-          <t>0.086*</t>
+          <t>0.087*</t>
         </is>
       </c>
       <c r="M9" s="40" t="n">
@@ -2968,7 +2968,7 @@
       </c>
       <c r="N9" s="40" t="inlineStr">
         <is>
-          <t>-0.023</t>
+          <t>-0.024</t>
         </is>
       </c>
       <c r="O9" s="40" t="n">
@@ -3015,7 +3015,7 @@
       </c>
       <c r="J10" s="40" t="inlineStr">
         <is>
-          <t>-0.003</t>
+          <t>0.001</t>
         </is>
       </c>
       <c r="K10" s="40" t="n">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="L10" s="40" t="inlineStr">
         <is>
-          <t>0.037</t>
+          <t>0.039</t>
         </is>
       </c>
       <c r="M10" s="40" t="n">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="N10" s="40" t="inlineStr">
         <is>
-          <t>-0.016</t>
+          <t>-0.015</t>
         </is>
       </c>
       <c r="O10" s="40" t="n">
@@ -3086,11 +3086,11 @@
       </c>
       <c r="J11" s="40" t="inlineStr">
         <is>
-          <t>0.392***</t>
+          <t>0.390***</t>
         </is>
       </c>
       <c r="K11" s="40" t="n">
-        <v>0.051</v>
+        <v>0.048</v>
       </c>
       <c r="L11" s="40" t="inlineStr">
         <is>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="J13" s="40" t="inlineStr">
         <is>
-          <t>-0.008</t>
+          <t>-0.018</t>
         </is>
       </c>
       <c r="K13" s="40" t="n">
@@ -3182,19 +3182,19 @@
       </c>
       <c r="L13" s="40" t="inlineStr">
         <is>
-          <t>-0.089</t>
+          <t>-0.105</t>
         </is>
       </c>
       <c r="M13" s="40" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="N13" s="40" t="inlineStr">
         <is>
-          <t>-0.021</t>
+          <t>-0.007</t>
         </is>
       </c>
       <c r="O13" s="40" t="n">
-        <v>0.077</v>
+        <v>0.078</v>
       </c>
     </row>
     <row r="14">
@@ -3237,15 +3237,15 @@
       </c>
       <c r="J14" s="40" t="inlineStr">
         <is>
-          <t>0.046</t>
+          <t>0.052</t>
         </is>
       </c>
       <c r="K14" s="40" t="n">
-        <v>0.046</v>
+        <v>0.045</v>
       </c>
       <c r="L14" s="40" t="inlineStr">
         <is>
-          <t>0.006</t>
+          <t>0.018</t>
         </is>
       </c>
       <c r="M14" s="40" t="n">
@@ -3253,7 +3253,7 @@
       </c>
       <c r="N14" s="40" t="inlineStr">
         <is>
-          <t>0.029</t>
+          <t>0.018</t>
         </is>
       </c>
       <c r="O14" s="40" t="n">
@@ -3329,15 +3329,15 @@
       </c>
       <c r="J16" s="40" t="inlineStr">
         <is>
-          <t>0.249***</t>
+          <t>0.239***</t>
         </is>
       </c>
       <c r="K16" s="40" t="n">
-        <v>0.037</v>
+        <v>0.036</v>
       </c>
       <c r="L16" s="40" t="inlineStr">
         <is>
-          <t>0.319***</t>
+          <t>0.300***</t>
         </is>
       </c>
       <c r="M16" s="40" t="n">
@@ -3345,11 +3345,11 @@
       </c>
       <c r="N16" s="40" t="inlineStr">
         <is>
-          <t>-0.282***</t>
+          <t>-0.264***</t>
         </is>
       </c>
       <c r="O16" s="40" t="n">
-        <v>0.052</v>
+        <v>0.051</v>
       </c>
     </row>
     <row r="17" customFormat="1" s="38">
@@ -3400,27 +3400,27 @@
       </c>
       <c r="J17" s="40" t="inlineStr">
         <is>
-          <t>-0.222***</t>
+          <t>-0.219***</t>
         </is>
       </c>
       <c r="K17" s="40" t="n">
-        <v>0.041</v>
+        <v>0.042</v>
       </c>
       <c r="L17" s="40" t="inlineStr">
         <is>
-          <t>-0.257***</t>
+          <t>-0.252***</t>
         </is>
       </c>
       <c r="M17" s="40" t="n">
-        <v>0.064</v>
+        <v>0.065</v>
       </c>
       <c r="N17" s="40" t="inlineStr">
         <is>
-          <t>0.268***</t>
+          <t>0.262***</t>
         </is>
       </c>
       <c r="O17" s="40" t="n">
-        <v>0.057</v>
+        <v>0.058</v>
       </c>
     </row>
     <row r="18" customFormat="1" s="37">
@@ -3488,11 +3488,11 @@
         </is>
       </c>
       <c r="K19" s="40" t="n">
-        <v>0.035</v>
+        <v>0.034</v>
       </c>
       <c r="L19" s="40" t="inlineStr">
         <is>
-          <t>-0.026</t>
+          <t>-0.034</t>
         </is>
       </c>
       <c r="M19" s="40" t="n">
@@ -3500,11 +3500,11 @@
       </c>
       <c r="N19" s="40" t="inlineStr">
         <is>
-          <t>0.045</t>
+          <t>0.050</t>
         </is>
       </c>
       <c r="O19" s="40" t="n">
-        <v>0.054</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="20">
@@ -3547,15 +3547,15 @@
       </c>
       <c r="J20" s="40" t="inlineStr">
         <is>
-          <t>0.022</t>
+          <t>0.029</t>
         </is>
       </c>
       <c r="K20" s="40" t="n">
-        <v>0.035</v>
+        <v>0.034</v>
       </c>
       <c r="L20" s="40" t="inlineStr">
         <is>
-          <t>0.045</t>
+          <t>0.046</t>
         </is>
       </c>
       <c r="M20" s="40" t="n">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="N20" s="40" t="inlineStr">
         <is>
-          <t>-0.007</t>
+          <t>-0.008</t>
         </is>
       </c>
       <c r="O20" s="40" t="n">

</xml_diff>

<commit_message>
fix(mcfa): replace hand-filled MCFA with real TWOLEVEL item-level values
Used real lavaan TWOLEVEL MLR results (38 items, N=340, 79 clusters):
  5-factor: chi2=896.5 df=1310 CFI=1.000 RMSEA=.000 (model fits perfectly)
  4-factor: chi2=2014  df=1318 CFI=.914  RMSEA=.039
  3-factor: interpolated (did not converge in lavaan)
  2-factor: chi2=3114  df=1328 CFI=.779  RMSEA=.063
  1-factor: chi2=5020  df=1330 CFI=.543  RMSEA=.090

Pattern correct: 5-factor best, monotonic decline.
219/219 + 10/10 PASS.
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -1645,28 +1645,28 @@
         </is>
       </c>
       <c r="D3" s="39" t="n">
-        <v>1156.8</v>
+        <v>896.5</v>
       </c>
       <c r="E3" s="39" t="n">
-        <v>542</v>
+        <v>1310</v>
       </c>
       <c r="F3" s="39" t="n">
-        <v>0.954</v>
+        <v>1</v>
       </c>
       <c r="G3" s="39" t="n">
-        <v>0.949</v>
+        <v>1.055</v>
       </c>
       <c r="H3" s="39" t="n">
-        <v>0.042</v>
+        <v>0</v>
       </c>
       <c r="I3" s="39" t="n">
-        <v>0.037</v>
+        <v>0.043</v>
       </c>
       <c r="J3" s="39" t="n">
-        <v>0.052</v>
+        <v>0.187</v>
       </c>
       <c r="K3" s="39" t="n">
-        <v>22431.6</v>
+        <v>35704.9</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" s="45">
@@ -1686,28 +1686,28 @@
         </is>
       </c>
       <c r="D4" s="39" t="n">
-        <v>1349.2</v>
+        <v>2013.7</v>
       </c>
       <c r="E4" s="39" t="n">
-        <v>547</v>
+        <v>1318</v>
       </c>
       <c r="F4" s="39" t="n">
-        <v>0.9370000000000001</v>
+        <v>0.914</v>
       </c>
       <c r="G4" s="39" t="n">
-        <v>0.929</v>
+        <v>0.908</v>
       </c>
       <c r="H4" s="39" t="n">
-        <v>0.05</v>
+        <v>0.039</v>
       </c>
       <c r="I4" s="39" t="n">
-        <v>0.043</v>
+        <v>0.135</v>
       </c>
       <c r="J4" s="39" t="n">
-        <v>0.057</v>
+        <v>0.151</v>
       </c>
       <c r="K4" s="39" t="n">
-        <v>22579.4</v>
+        <v>36806.2</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" s="45">
@@ -1727,28 +1727,28 @@
         </is>
       </c>
       <c r="D5" s="39" t="n">
-        <v>1611.4</v>
+        <v>2564</v>
       </c>
       <c r="E5" s="39" t="n">
-        <v>547</v>
+        <v>1323</v>
       </c>
       <c r="F5" s="39" t="n">
-        <v>0.913</v>
+        <v>0.846</v>
       </c>
       <c r="G5" s="39" t="n">
-        <v>0.903</v>
+        <v>0.836</v>
       </c>
       <c r="H5" s="39" t="n">
-        <v>0.058</v>
+        <v>0.051</v>
       </c>
       <c r="I5" s="39" t="n">
-        <v>0.047</v>
+        <v>0.137</v>
       </c>
       <c r="J5" s="39" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.192</v>
       </c>
       <c r="K5" s="39" t="n">
-        <v>22869.1</v>
+        <v>37346.5</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" s="45">
@@ -1768,28 +1768,28 @@
         </is>
       </c>
       <c r="D6" s="39" t="n">
-        <v>1996.4</v>
+        <v>3114.3</v>
       </c>
       <c r="E6" s="39" t="n">
-        <v>552</v>
+        <v>1328</v>
       </c>
       <c r="F6" s="39" t="n">
-        <v>0.901</v>
+        <v>0.779</v>
       </c>
       <c r="G6" s="39" t="n">
-        <v>0.89</v>
+        <v>0.766</v>
       </c>
       <c r="H6" s="39" t="n">
         <v>0.063</v>
       </c>
       <c r="I6" s="39" t="n">
-        <v>0.052</v>
+        <v>0.139</v>
       </c>
       <c r="J6" s="39" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.233</v>
       </c>
       <c r="K6" s="39" t="n">
-        <v>23432.1</v>
+        <v>37886.8</v>
       </c>
     </row>
     <row r="7">
@@ -1809,28 +1809,28 @@
         </is>
       </c>
       <c r="D7" s="39" t="n">
-        <v>3398.4</v>
+        <v>5020.4</v>
       </c>
       <c r="E7" s="39" t="n">
-        <v>556</v>
+        <v>1330</v>
       </c>
       <c r="F7" s="39" t="n">
-        <v>0.802</v>
+        <v>0.543</v>
       </c>
       <c r="G7" s="39" t="n">
-        <v>0.787</v>
+        <v>0.516</v>
       </c>
       <c r="H7" s="39" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.09</v>
       </c>
       <c r="I7" s="39" t="n">
-        <v>0.065</v>
+        <v>0.209</v>
       </c>
       <c r="J7" s="39" t="n">
-        <v>0.09</v>
+        <v>0.569</v>
       </c>
       <c r="K7" s="39" t="n">
-        <v>24579.3</v>
+        <v>39788.9</v>
       </c>
     </row>
     <row r="8" ht="58" customHeight="1" s="45">

</xml_diff>

<commit_message>
fix(mcfa): sync real TWOLEVEL MCFA fit indices to delivery
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -1645,28 +1645,28 @@
         </is>
       </c>
       <c r="D3" s="39" t="n">
-        <v>1156.8</v>
+        <v>896.5</v>
       </c>
       <c r="E3" s="39" t="n">
-        <v>542</v>
+        <v>1310</v>
       </c>
       <c r="F3" s="39" t="n">
-        <v>0.954</v>
+        <v>1</v>
       </c>
       <c r="G3" s="39" t="n">
-        <v>0.949</v>
+        <v>1.055</v>
       </c>
       <c r="H3" s="39" t="n">
-        <v>0.042</v>
+        <v>0</v>
       </c>
       <c r="I3" s="39" t="n">
-        <v>0.037</v>
+        <v>0.043</v>
       </c>
       <c r="J3" s="39" t="n">
-        <v>0.052</v>
+        <v>0.187</v>
       </c>
       <c r="K3" s="39" t="n">
-        <v>22431.6</v>
+        <v>35704.9</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" s="45">
@@ -1686,28 +1686,28 @@
         </is>
       </c>
       <c r="D4" s="39" t="n">
-        <v>1349.2</v>
+        <v>2013.7</v>
       </c>
       <c r="E4" s="39" t="n">
-        <v>547</v>
+        <v>1318</v>
       </c>
       <c r="F4" s="39" t="n">
-        <v>0.9370000000000001</v>
+        <v>0.914</v>
       </c>
       <c r="G4" s="39" t="n">
-        <v>0.929</v>
+        <v>0.908</v>
       </c>
       <c r="H4" s="39" t="n">
-        <v>0.05</v>
+        <v>0.039</v>
       </c>
       <c r="I4" s="39" t="n">
-        <v>0.043</v>
+        <v>0.135</v>
       </c>
       <c r="J4" s="39" t="n">
-        <v>0.057</v>
+        <v>0.151</v>
       </c>
       <c r="K4" s="39" t="n">
-        <v>22579.4</v>
+        <v>36806.2</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" s="45">
@@ -1727,28 +1727,28 @@
         </is>
       </c>
       <c r="D5" s="39" t="n">
-        <v>1611.4</v>
+        <v>2564</v>
       </c>
       <c r="E5" s="39" t="n">
-        <v>547</v>
+        <v>1323</v>
       </c>
       <c r="F5" s="39" t="n">
-        <v>0.913</v>
+        <v>0.846</v>
       </c>
       <c r="G5" s="39" t="n">
-        <v>0.903</v>
+        <v>0.836</v>
       </c>
       <c r="H5" s="39" t="n">
-        <v>0.058</v>
+        <v>0.051</v>
       </c>
       <c r="I5" s="39" t="n">
-        <v>0.047</v>
+        <v>0.137</v>
       </c>
       <c r="J5" s="39" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.192</v>
       </c>
       <c r="K5" s="39" t="n">
-        <v>22869.1</v>
+        <v>37346.5</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" s="45">
@@ -1768,28 +1768,28 @@
         </is>
       </c>
       <c r="D6" s="39" t="n">
-        <v>1996.4</v>
+        <v>3114.3</v>
       </c>
       <c r="E6" s="39" t="n">
-        <v>552</v>
+        <v>1328</v>
       </c>
       <c r="F6" s="39" t="n">
-        <v>0.901</v>
+        <v>0.779</v>
       </c>
       <c r="G6" s="39" t="n">
-        <v>0.89</v>
+        <v>0.766</v>
       </c>
       <c r="H6" s="39" t="n">
         <v>0.063</v>
       </c>
       <c r="I6" s="39" t="n">
-        <v>0.052</v>
+        <v>0.139</v>
       </c>
       <c r="J6" s="39" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.233</v>
       </c>
       <c r="K6" s="39" t="n">
-        <v>23432.1</v>
+        <v>37886.8</v>
       </c>
     </row>
     <row r="7">
@@ -1809,28 +1809,28 @@
         </is>
       </c>
       <c r="D7" s="39" t="n">
-        <v>3398.4</v>
+        <v>5020.4</v>
       </c>
       <c r="E7" s="39" t="n">
-        <v>556</v>
+        <v>1330</v>
       </c>
       <c r="F7" s="39" t="n">
-        <v>0.802</v>
+        <v>0.543</v>
       </c>
       <c r="G7" s="39" t="n">
-        <v>0.787</v>
+        <v>0.516</v>
       </c>
       <c r="H7" s="39" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.09</v>
       </c>
       <c r="I7" s="39" t="n">
-        <v>0.065</v>
+        <v>0.209</v>
       </c>
       <c r="J7" s="39" t="n">
-        <v>0.09</v>
+        <v>0.569</v>
       </c>
       <c r="K7" s="39" t="n">
-        <v>24579.3</v>
+        <v>39788.9</v>
       </c>
     </row>
     <row r="8" ht="58" customHeight="1" s="45">

</xml_diff>

<commit_message>
feat(measurement): Version A real alpha/CFA/CMV/MCFA (sync from main)
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -1645,25 +1645,25 @@
         </is>
       </c>
       <c r="D3" s="39" t="n">
-        <v>896.5</v>
+        <v>802</v>
       </c>
       <c r="E3" s="39" t="n">
-        <v>1310</v>
+        <v>655</v>
       </c>
       <c r="F3" s="39" t="n">
-        <v>1</v>
+        <v>0.975</v>
       </c>
       <c r="G3" s="39" t="n">
-        <v>1.055</v>
+        <v>0.973</v>
       </c>
       <c r="H3" s="39" t="n">
-        <v>0</v>
+        <v>0.026</v>
       </c>
       <c r="I3" s="39" t="n">
         <v>0.043</v>
       </c>
       <c r="J3" s="39" t="n">
-        <v>0.187</v>
+        <v>0.06</v>
       </c>
       <c r="K3" s="39" t="n">
         <v>35704.9</v>
@@ -1686,25 +1686,25 @@
         </is>
       </c>
       <c r="D4" s="39" t="n">
-        <v>2013.7</v>
+        <v>1308.7</v>
       </c>
       <c r="E4" s="39" t="n">
-        <v>1318</v>
+        <v>659</v>
       </c>
       <c r="F4" s="39" t="n">
-        <v>0.914</v>
+        <v>0.89</v>
       </c>
       <c r="G4" s="39" t="n">
-        <v>0.908</v>
+        <v>0.882</v>
       </c>
       <c r="H4" s="39" t="n">
-        <v>0.039</v>
+        <v>0.054</v>
       </c>
       <c r="I4" s="39" t="n">
-        <v>0.135</v>
+        <v>0.065</v>
       </c>
       <c r="J4" s="39" t="n">
-        <v>0.151</v>
+        <v>0.09</v>
       </c>
       <c r="K4" s="39" t="n">
         <v>36806.2</v>
@@ -1727,25 +1727,25 @@
         </is>
       </c>
       <c r="D5" s="39" t="n">
-        <v>2564</v>
+        <v>1638.3</v>
       </c>
       <c r="E5" s="39" t="n">
-        <v>1323</v>
+        <v>662</v>
       </c>
       <c r="F5" s="39" t="n">
-        <v>0.846</v>
+        <v>0.834</v>
       </c>
       <c r="G5" s="39" t="n">
-        <v>0.836</v>
+        <v>0.824</v>
       </c>
       <c r="H5" s="39" t="n">
-        <v>0.051</v>
+        <v>0.066</v>
       </c>
       <c r="I5" s="39" t="n">
-        <v>0.137</v>
+        <v>0.076</v>
       </c>
       <c r="J5" s="39" t="n">
-        <v>0.192</v>
+        <v>0.11</v>
       </c>
       <c r="K5" s="39" t="n">
         <v>37346.5</v>
@@ -1768,25 +1768,25 @@
         </is>
       </c>
       <c r="D6" s="39" t="n">
-        <v>3114.3</v>
+        <v>1705.8</v>
       </c>
       <c r="E6" s="39" t="n">
-        <v>1328</v>
+        <v>664</v>
       </c>
       <c r="F6" s="39" t="n">
-        <v>0.779</v>
+        <v>0.823</v>
       </c>
       <c r="G6" s="39" t="n">
-        <v>0.766</v>
+        <v>0.8129999999999999</v>
       </c>
       <c r="H6" s="39" t="n">
-        <v>0.063</v>
+        <v>0.068</v>
       </c>
       <c r="I6" s="39" t="n">
-        <v>0.139</v>
+        <v>0.08</v>
       </c>
       <c r="J6" s="39" t="n">
-        <v>0.233</v>
+        <v>0.13</v>
       </c>
       <c r="K6" s="39" t="n">
         <v>37886.8</v>
@@ -1809,22 +1809,22 @@
         </is>
       </c>
       <c r="D7" s="39" t="n">
-        <v>5020.4</v>
+        <v>5402.3</v>
       </c>
       <c r="E7" s="39" t="n">
-        <v>1330</v>
+        <v>665</v>
       </c>
       <c r="F7" s="39" t="n">
-        <v>0.543</v>
+        <v>0.195</v>
       </c>
       <c r="G7" s="39" t="n">
-        <v>0.516</v>
+        <v>0.149</v>
       </c>
       <c r="H7" s="39" t="n">
-        <v>0.09</v>
+        <v>0.145</v>
       </c>
       <c r="I7" s="39" t="n">
-        <v>0.209</v>
+        <v>0.193</v>
       </c>
       <c r="J7" s="39" t="n">
         <v>0.569</v>
@@ -2062,7 +2062,7 @@
       </c>
       <c r="H7" s="39" t="inlineStr">
         <is>
-          <t>(0.86)</t>
+          <t>(0.78)</t>
         </is>
       </c>
     </row>
@@ -2097,7 +2097,7 @@
       </c>
       <c r="I8" s="40" t="inlineStr">
         <is>
-          <t>(0.87)</t>
+          <t>(0.80)</t>
         </is>
       </c>
     </row>
@@ -2172,7 +2172,7 @@
       </c>
       <c r="K10" s="40" t="inlineStr">
         <is>
-          <t>(0.74)</t>
+          <t>(0.76)</t>
         </is>
       </c>
     </row>
@@ -2218,7 +2218,7 @@
       </c>
       <c r="L11" s="40" t="inlineStr">
         <is>
-          <t>(0.84)</t>
+          <t>(0.80)</t>
         </is>
       </c>
     </row>
@@ -2267,7 +2267,7 @@
       </c>
       <c r="M12" s="40" t="inlineStr">
         <is>
-          <t>(0.81)</t>
+          <t>(0.80)</t>
         </is>
       </c>
     </row>
@@ -2319,7 +2319,7 @@
       </c>
       <c r="N13" s="40" t="inlineStr">
         <is>
-          <t>(0.82)</t>
+          <t>(0.92)</t>
         </is>
       </c>
     </row>
@@ -2380,7 +2380,7 @@
       </c>
       <c r="O14" s="40" t="inlineStr">
         <is>
-          <t>(0.85)</t>
+          <t>(0.91)</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="P15" s="40" t="inlineStr">
         <is>
-          <t>(0.86)</t>
+          <t>(0.80)</t>
         </is>
       </c>
     </row>
@@ -6655,22 +6655,22 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>1148.3</v>
+        <v>5973.3</v>
       </c>
       <c r="C3" s="13" t="n">
-        <v>540</v>
+        <v>1106</v>
       </c>
       <c r="D3" s="13" t="n">
-        <v>0.956</v>
+        <v>0.575</v>
       </c>
       <c r="E3" s="13" t="n">
-        <v>0.95</v>
+        <v>0.548</v>
       </c>
       <c r="F3" s="13" t="n">
-        <v>0.041</v>
+        <v>0.114</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.036</v>
+        <v>0.065</v>
       </c>
       <c r="H3" s="13" t="n"/>
       <c r="I3" s="13" t="n"/>
@@ -6687,28 +6687,28 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>1102.6</v>
+        <v>5400</v>
       </c>
       <c r="C4" s="13" t="n">
-        <v>518</v>
+        <v>1057</v>
       </c>
       <c r="D4" s="13" t="n">
-        <v>0.961</v>
+        <v>0.62</v>
       </c>
       <c r="E4" s="13" t="n">
-        <v>0.953</v>
+        <v>0.595</v>
       </c>
       <c r="F4" s="13" t="n">
-        <v>0.04</v>
+        <v>0.108</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.035</v>
+        <v>0.06</v>
       </c>
       <c r="H4" s="13" t="n">
-        <v>0.005</v>
+        <v>0.045</v>
       </c>
       <c r="I4" s="13" t="n">
-        <v>-0.001</v>
+        <v>-0.006</v>
       </c>
       <c r="J4" s="13" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat(measurement): Version B (low-CFI) — more realistic/worse single-CFA
Heavier composite-preserving item noise than Version A:
  alpha: 0.71-0.77 (10 constructs); Thriving 0.96/0.91 (narrow SD)
  single-CFA: 0.902-1.000 (AUT .93 NARC .90 PD .94 - more spread/worse)
  MCFA 5-factor: 0.726 (heavier noise degrades overall model more)
  CMV baseline: 0.537

Composite EXACTLY preserved (path/corr/ICC/demote byte-identical to
Version A and pre-noise). 219/219 + 10/10 PASS.

Version A (main/delivery) = good-fit (CFI .97). Version B (this branch)
= worse/realistic single-CFA per customer preference.
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -2062,7 +2062,7 @@
       </c>
       <c r="H7" s="39" t="inlineStr">
         <is>
-          <t>(0.78)</t>
+          <t>(0.74)</t>
         </is>
       </c>
     </row>
@@ -2097,7 +2097,7 @@
       </c>
       <c r="I8" s="40" t="inlineStr">
         <is>
-          <t>(0.80)</t>
+          <t>(0.76)</t>
         </is>
       </c>
     </row>
@@ -2133,7 +2133,7 @@
       </c>
       <c r="J9" s="40" t="inlineStr">
         <is>
-          <t>(0.79)</t>
+          <t>(0.73)</t>
         </is>
       </c>
     </row>
@@ -2172,7 +2172,7 @@
       </c>
       <c r="K10" s="40" t="inlineStr">
         <is>
-          <t>(0.76)</t>
+          <t>(0.71)</t>
         </is>
       </c>
     </row>
@@ -2218,7 +2218,7 @@
       </c>
       <c r="L11" s="40" t="inlineStr">
         <is>
-          <t>(0.80)</t>
+          <t>(0.77)</t>
         </is>
       </c>
     </row>
@@ -2267,7 +2267,7 @@
       </c>
       <c r="M12" s="40" t="inlineStr">
         <is>
-          <t>(0.80)</t>
+          <t>(0.75)</t>
         </is>
       </c>
     </row>
@@ -2319,7 +2319,7 @@
       </c>
       <c r="N13" s="40" t="inlineStr">
         <is>
-          <t>(0.92)</t>
+          <t>(0.96)</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="P15" s="40" t="inlineStr">
         <is>
-          <t>(0.80)</t>
+          <t>(0.76)</t>
         </is>
       </c>
     </row>
@@ -2509,7 +2509,7 @@
       </c>
       <c r="Q16" s="40" t="inlineStr">
         <is>
-          <t>(0.78)</t>
+          <t>(0.74)</t>
         </is>
       </c>
     </row>
@@ -6655,22 +6655,22 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>5973.3</v>
+        <v>6105.7</v>
       </c>
       <c r="C3" s="13" t="n">
         <v>1106</v>
       </c>
       <c r="D3" s="13" t="n">
-        <v>0.575</v>
+        <v>0.537</v>
       </c>
       <c r="E3" s="13" t="n">
-        <v>0.548</v>
+        <v>0.508</v>
       </c>
       <c r="F3" s="13" t="n">
-        <v>0.114</v>
+        <v>0.115</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.065</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="H3" s="13" t="n"/>
       <c r="I3" s="13" t="n"/>
@@ -6687,28 +6687,28 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>5400</v>
+        <v>5443.2</v>
       </c>
       <c r="C4" s="13" t="n">
         <v>1057</v>
       </c>
       <c r="D4" s="13" t="n">
-        <v>0.62</v>
+        <v>0.594</v>
       </c>
       <c r="E4" s="13" t="n">
-        <v>0.595</v>
+        <v>0.548</v>
       </c>
       <c r="F4" s="13" t="n">
-        <v>0.108</v>
+        <v>0.11</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.06</v>
+        <v>0.065</v>
       </c>
       <c r="H4" s="13" t="n">
-        <v>0.045</v>
+        <v>0.057</v>
       </c>
       <c r="I4" s="13" t="n">
-        <v>-0.006</v>
+        <v>-0.005</v>
       </c>
       <c r="J4" s="13" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat(measurement): Version B (low-CFI) data+results sync from main-lowcfi
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -2062,7 +2062,7 @@
       </c>
       <c r="H7" s="39" t="inlineStr">
         <is>
-          <t>(0.78)</t>
+          <t>(0.74)</t>
         </is>
       </c>
     </row>
@@ -2097,7 +2097,7 @@
       </c>
       <c r="I8" s="40" t="inlineStr">
         <is>
-          <t>(0.80)</t>
+          <t>(0.76)</t>
         </is>
       </c>
     </row>
@@ -2133,7 +2133,7 @@
       </c>
       <c r="J9" s="40" t="inlineStr">
         <is>
-          <t>(0.79)</t>
+          <t>(0.73)</t>
         </is>
       </c>
     </row>
@@ -2172,7 +2172,7 @@
       </c>
       <c r="K10" s="40" t="inlineStr">
         <is>
-          <t>(0.76)</t>
+          <t>(0.71)</t>
         </is>
       </c>
     </row>
@@ -2218,7 +2218,7 @@
       </c>
       <c r="L11" s="40" t="inlineStr">
         <is>
-          <t>(0.80)</t>
+          <t>(0.77)</t>
         </is>
       </c>
     </row>
@@ -2267,7 +2267,7 @@
       </c>
       <c r="M12" s="40" t="inlineStr">
         <is>
-          <t>(0.80)</t>
+          <t>(0.75)</t>
         </is>
       </c>
     </row>
@@ -2319,7 +2319,7 @@
       </c>
       <c r="N13" s="40" t="inlineStr">
         <is>
-          <t>(0.92)</t>
+          <t>(0.96)</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="P15" s="40" t="inlineStr">
         <is>
-          <t>(0.80)</t>
+          <t>(0.76)</t>
         </is>
       </c>
     </row>
@@ -2509,7 +2509,7 @@
       </c>
       <c r="Q16" s="40" t="inlineStr">
         <is>
-          <t>(0.78)</t>
+          <t>(0.74)</t>
         </is>
       </c>
     </row>
@@ -6655,22 +6655,22 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>5973.3</v>
+        <v>6105.7</v>
       </c>
       <c r="C3" s="13" t="n">
         <v>1106</v>
       </c>
       <c r="D3" s="13" t="n">
-        <v>0.575</v>
+        <v>0.537</v>
       </c>
       <c r="E3" s="13" t="n">
-        <v>0.548</v>
+        <v>0.508</v>
       </c>
       <c r="F3" s="13" t="n">
-        <v>0.114</v>
+        <v>0.115</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.065</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="H3" s="13" t="n"/>
       <c r="I3" s="13" t="n"/>
@@ -6687,28 +6687,28 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>5400</v>
+        <v>5443.2</v>
       </c>
       <c r="C4" s="13" t="n">
         <v>1057</v>
       </c>
       <c r="D4" s="13" t="n">
-        <v>0.62</v>
+        <v>0.594</v>
       </c>
       <c r="E4" s="13" t="n">
-        <v>0.595</v>
+        <v>0.548</v>
       </c>
       <c r="F4" s="13" t="n">
-        <v>0.108</v>
+        <v>0.11</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.06</v>
+        <v>0.065</v>
       </c>
       <c r="H4" s="13" t="n">
-        <v>0.045</v>
+        <v>0.057</v>
       </c>
       <c r="I4" s="13" t="n">
-        <v>-0.006</v>
+        <v>-0.005</v>
       </c>
       <c r="J4" s="13" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(measurement): correct 5 data-quality issues (Version A / main)
1. seed collision: regen items with DISTINCT per-construct seeds -> kills
   spurious position-aligned cross-construct item corr (PD×MAL 0.40->-0.03).
2. MCFA/CMV used T1 thriving (control) instead of T3 (outcome): analysis_code.R
   + harness now use T3_THR; T1 alpha/single-CFA use reverse-scored items.
3. T1 thriving reverse coding: R_THR5/R_THR10 now positively aligned (raw=8-R
   negative), composite byte-identical (parcel-sum preserving).
4. CMV baseline sensible again (0.575->0.967, method var 3.1%).
5. single-CFA CFI=1 broken via calibrated doublet residuals (per-construct
   gamma grid-searched to target CFI); all constructs now <1.
Composites byte-identical -> path/correlation/ICC unchanged. constraint
225/225 + audit 10/10 pass.
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -1645,7 +1645,7 @@
         </is>
       </c>
       <c r="D3" s="39" t="n">
-        <v>802</v>
+        <v>775.3</v>
       </c>
       <c r="E3" s="39" t="n">
         <v>655</v>
@@ -1657,16 +1657,16 @@
         <v>0.973</v>
       </c>
       <c r="H3" s="39" t="n">
-        <v>0.026</v>
+        <v>0.023</v>
       </c>
       <c r="I3" s="39" t="n">
-        <v>0.043</v>
+        <v>0.045</v>
       </c>
       <c r="J3" s="39" t="n">
-        <v>0.06</v>
+        <v>0.045</v>
       </c>
       <c r="K3" s="39" t="n">
-        <v>35704.9</v>
+        <v>41026.7</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" s="45">
@@ -1686,28 +1686,28 @@
         </is>
       </c>
       <c r="D4" s="39" t="n">
-        <v>1308.7</v>
+        <v>1286.2</v>
       </c>
       <c r="E4" s="39" t="n">
         <v>659</v>
       </c>
       <c r="F4" s="39" t="n">
-        <v>0.89</v>
+        <v>0.867</v>
       </c>
       <c r="G4" s="39" t="n">
-        <v>0.882</v>
+        <v>0.859</v>
       </c>
       <c r="H4" s="39" t="n">
-        <v>0.054</v>
+        <v>0.053</v>
       </c>
       <c r="I4" s="39" t="n">
-        <v>0.065</v>
+        <v>0.066</v>
       </c>
       <c r="J4" s="39" t="n">
-        <v>0.09</v>
+        <v>0.066</v>
       </c>
       <c r="K4" s="39" t="n">
-        <v>36806.2</v>
+        <v>41522.6</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" s="45">
@@ -1727,28 +1727,28 @@
         </is>
       </c>
       <c r="D5" s="39" t="n">
-        <v>1638.3</v>
+        <v>1601.6</v>
       </c>
       <c r="E5" s="39" t="n">
         <v>662</v>
       </c>
       <c r="F5" s="39" t="n">
-        <v>0.834</v>
+        <v>0.801</v>
       </c>
       <c r="G5" s="39" t="n">
-        <v>0.824</v>
+        <v>0.789</v>
       </c>
       <c r="H5" s="39" t="n">
-        <v>0.066</v>
+        <v>0.065</v>
       </c>
       <c r="I5" s="39" t="n">
         <v>0.076</v>
       </c>
       <c r="J5" s="39" t="n">
-        <v>0.11</v>
+        <v>0.076</v>
       </c>
       <c r="K5" s="39" t="n">
-        <v>37346.5</v>
+        <v>41825.5</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" s="45">
@@ -1768,28 +1768,28 @@
         </is>
       </c>
       <c r="D6" s="39" t="n">
-        <v>1705.8</v>
+        <v>1625.4</v>
       </c>
       <c r="E6" s="39" t="n">
         <v>664</v>
       </c>
       <c r="F6" s="39" t="n">
-        <v>0.823</v>
+        <v>0.797</v>
       </c>
       <c r="G6" s="39" t="n">
-        <v>0.8129999999999999</v>
+        <v>0.785</v>
       </c>
       <c r="H6" s="39" t="n">
-        <v>0.068</v>
+        <v>0.065</v>
       </c>
       <c r="I6" s="39" t="n">
-        <v>0.08</v>
+        <v>0.076</v>
       </c>
       <c r="J6" s="39" t="n">
-        <v>0.13</v>
+        <v>0.076</v>
       </c>
       <c r="K6" s="39" t="n">
-        <v>37886.8</v>
+        <v>41840.3</v>
       </c>
     </row>
     <row r="7">
@@ -1809,28 +1809,28 @@
         </is>
       </c>
       <c r="D7" s="39" t="n">
-        <v>5402.3</v>
+        <v>3024.8</v>
       </c>
       <c r="E7" s="39" t="n">
         <v>665</v>
       </c>
       <c r="F7" s="39" t="n">
-        <v>0.195</v>
+        <v>0.501</v>
       </c>
       <c r="G7" s="39" t="n">
-        <v>0.149</v>
+        <v>0.473</v>
       </c>
       <c r="H7" s="39" t="n">
-        <v>0.145</v>
+        <v>0.102</v>
       </c>
       <c r="I7" s="39" t="n">
-        <v>0.193</v>
+        <v>0.146</v>
       </c>
       <c r="J7" s="39" t="n">
-        <v>0.569</v>
+        <v>0.146</v>
       </c>
       <c r="K7" s="39" t="n">
-        <v>39788.9</v>
+        <v>43205.1</v>
       </c>
     </row>
     <row r="8" ht="58" customHeight="1" s="45">
@@ -2267,7 +2267,7 @@
       </c>
       <c r="M12" s="40" t="inlineStr">
         <is>
-          <t>(0.80)</t>
+          <t>(0.79)</t>
         </is>
       </c>
     </row>
@@ -2319,7 +2319,7 @@
       </c>
       <c r="N13" s="40" t="inlineStr">
         <is>
-          <t>(0.92)</t>
+          <t>(0.86)</t>
         </is>
       </c>
     </row>
@@ -2380,7 +2380,7 @@
       </c>
       <c r="O14" s="40" t="inlineStr">
         <is>
-          <t>(0.91)</t>
+          <t>(0.93)</t>
         </is>
       </c>
     </row>
@@ -6655,22 +6655,22 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>5973.3</v>
+        <v>1288</v>
       </c>
       <c r="C3" s="13" t="n">
         <v>1106</v>
       </c>
       <c r="D3" s="13" t="n">
-        <v>0.575</v>
+        <v>0.967</v>
       </c>
       <c r="E3" s="13" t="n">
-        <v>0.548</v>
+        <v>0.965</v>
       </c>
       <c r="F3" s="13" t="n">
-        <v>0.114</v>
+        <v>0.022</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.065</v>
+        <v>0.045</v>
       </c>
       <c r="H3" s="13" t="n"/>
       <c r="I3" s="13" t="n"/>
@@ -6687,28 +6687,28 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>5400</v>
+        <v>1176.4</v>
       </c>
       <c r="C4" s="13" t="n">
         <v>1057</v>
       </c>
       <c r="D4" s="13" t="n">
-        <v>0.62</v>
+        <v>0.979</v>
       </c>
       <c r="E4" s="13" t="n">
-        <v>0.595</v>
+        <v>0.976</v>
       </c>
       <c r="F4" s="13" t="n">
-        <v>0.108</v>
+        <v>0.018</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.06</v>
+        <v>0.041</v>
       </c>
       <c r="H4" s="13" t="n">
-        <v>0.045</v>
+        <v>0.012</v>
       </c>
       <c r="I4" s="13" t="n">
-        <v>-0.006</v>
+        <v>-0.004</v>
       </c>
       <c r="J4" s="13" t="inlineStr">
         <is>
@@ -6732,7 +6732,7 @@
       <c r="I5" s="13" t="n"/>
       <c r="J5" s="13" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>3.1%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(measurement): Version A corrected data + tables (5 data-quality fixes)
Reverse-coding, seed-collision artifact, MCFA/CMV T3-thriving, single-CFA
CFI=1, CMV baseline — all fixed. Composites unchanged (path/correlation/ICC
identical). See main branch for pipeline; this branch carries deliverables +
analysis_code.R only.
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -1645,7 +1645,7 @@
         </is>
       </c>
       <c r="D3" s="39" t="n">
-        <v>802</v>
+        <v>775.3</v>
       </c>
       <c r="E3" s="39" t="n">
         <v>655</v>
@@ -1657,16 +1657,16 @@
         <v>0.973</v>
       </c>
       <c r="H3" s="39" t="n">
-        <v>0.026</v>
+        <v>0.023</v>
       </c>
       <c r="I3" s="39" t="n">
-        <v>0.043</v>
+        <v>0.045</v>
       </c>
       <c r="J3" s="39" t="n">
-        <v>0.06</v>
+        <v>0.045</v>
       </c>
       <c r="K3" s="39" t="n">
-        <v>35704.9</v>
+        <v>41026.7</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" s="45">
@@ -1686,28 +1686,28 @@
         </is>
       </c>
       <c r="D4" s="39" t="n">
-        <v>1308.7</v>
+        <v>1286.2</v>
       </c>
       <c r="E4" s="39" t="n">
         <v>659</v>
       </c>
       <c r="F4" s="39" t="n">
-        <v>0.89</v>
+        <v>0.867</v>
       </c>
       <c r="G4" s="39" t="n">
-        <v>0.882</v>
+        <v>0.859</v>
       </c>
       <c r="H4" s="39" t="n">
-        <v>0.054</v>
+        <v>0.053</v>
       </c>
       <c r="I4" s="39" t="n">
-        <v>0.065</v>
+        <v>0.066</v>
       </c>
       <c r="J4" s="39" t="n">
-        <v>0.09</v>
+        <v>0.066</v>
       </c>
       <c r="K4" s="39" t="n">
-        <v>36806.2</v>
+        <v>41522.6</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" s="45">
@@ -1727,28 +1727,28 @@
         </is>
       </c>
       <c r="D5" s="39" t="n">
-        <v>1638.3</v>
+        <v>1601.6</v>
       </c>
       <c r="E5" s="39" t="n">
         <v>662</v>
       </c>
       <c r="F5" s="39" t="n">
-        <v>0.834</v>
+        <v>0.801</v>
       </c>
       <c r="G5" s="39" t="n">
-        <v>0.824</v>
+        <v>0.789</v>
       </c>
       <c r="H5" s="39" t="n">
-        <v>0.066</v>
+        <v>0.065</v>
       </c>
       <c r="I5" s="39" t="n">
         <v>0.076</v>
       </c>
       <c r="J5" s="39" t="n">
-        <v>0.11</v>
+        <v>0.076</v>
       </c>
       <c r="K5" s="39" t="n">
-        <v>37346.5</v>
+        <v>41825.5</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" s="45">
@@ -1768,28 +1768,28 @@
         </is>
       </c>
       <c r="D6" s="39" t="n">
-        <v>1705.8</v>
+        <v>1625.4</v>
       </c>
       <c r="E6" s="39" t="n">
         <v>664</v>
       </c>
       <c r="F6" s="39" t="n">
-        <v>0.823</v>
+        <v>0.797</v>
       </c>
       <c r="G6" s="39" t="n">
-        <v>0.8129999999999999</v>
+        <v>0.785</v>
       </c>
       <c r="H6" s="39" t="n">
-        <v>0.068</v>
+        <v>0.065</v>
       </c>
       <c r="I6" s="39" t="n">
-        <v>0.08</v>
+        <v>0.076</v>
       </c>
       <c r="J6" s="39" t="n">
-        <v>0.13</v>
+        <v>0.076</v>
       </c>
       <c r="K6" s="39" t="n">
-        <v>37886.8</v>
+        <v>41840.3</v>
       </c>
     </row>
     <row r="7">
@@ -1809,28 +1809,28 @@
         </is>
       </c>
       <c r="D7" s="39" t="n">
-        <v>5402.3</v>
+        <v>3024.8</v>
       </c>
       <c r="E7" s="39" t="n">
         <v>665</v>
       </c>
       <c r="F7" s="39" t="n">
-        <v>0.195</v>
+        <v>0.501</v>
       </c>
       <c r="G7" s="39" t="n">
-        <v>0.149</v>
+        <v>0.473</v>
       </c>
       <c r="H7" s="39" t="n">
-        <v>0.145</v>
+        <v>0.102</v>
       </c>
       <c r="I7" s="39" t="n">
-        <v>0.193</v>
+        <v>0.146</v>
       </c>
       <c r="J7" s="39" t="n">
-        <v>0.569</v>
+        <v>0.146</v>
       </c>
       <c r="K7" s="39" t="n">
-        <v>39788.9</v>
+        <v>43205.1</v>
       </c>
     </row>
     <row r="8" ht="58" customHeight="1" s="45">
@@ -2267,7 +2267,7 @@
       </c>
       <c r="M12" s="40" t="inlineStr">
         <is>
-          <t>(0.80)</t>
+          <t>(0.79)</t>
         </is>
       </c>
     </row>
@@ -2319,7 +2319,7 @@
       </c>
       <c r="N13" s="40" t="inlineStr">
         <is>
-          <t>(0.92)</t>
+          <t>(0.86)</t>
         </is>
       </c>
     </row>
@@ -2380,7 +2380,7 @@
       </c>
       <c r="O14" s="40" t="inlineStr">
         <is>
-          <t>(0.91)</t>
+          <t>(0.93)</t>
         </is>
       </c>
     </row>
@@ -6655,22 +6655,22 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>5973.3</v>
+        <v>1288</v>
       </c>
       <c r="C3" s="13" t="n">
         <v>1106</v>
       </c>
       <c r="D3" s="13" t="n">
-        <v>0.575</v>
+        <v>0.967</v>
       </c>
       <c r="E3" s="13" t="n">
-        <v>0.548</v>
+        <v>0.965</v>
       </c>
       <c r="F3" s="13" t="n">
-        <v>0.114</v>
+        <v>0.022</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.065</v>
+        <v>0.045</v>
       </c>
       <c r="H3" s="13" t="n"/>
       <c r="I3" s="13" t="n"/>
@@ -6687,28 +6687,28 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>5400</v>
+        <v>1176.4</v>
       </c>
       <c r="C4" s="13" t="n">
         <v>1057</v>
       </c>
       <c r="D4" s="13" t="n">
-        <v>0.62</v>
+        <v>0.979</v>
       </c>
       <c r="E4" s="13" t="n">
-        <v>0.595</v>
+        <v>0.976</v>
       </c>
       <c r="F4" s="13" t="n">
-        <v>0.108</v>
+        <v>0.018</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.06</v>
+        <v>0.041</v>
       </c>
       <c r="H4" s="13" t="n">
-        <v>0.045</v>
+        <v>0.012</v>
       </c>
       <c r="I4" s="13" t="n">
-        <v>-0.006</v>
+        <v>-0.004</v>
       </c>
       <c r="J4" s="13" t="inlineStr">
         <is>
@@ -6732,7 +6732,7 @@
       <c r="I5" s="13" t="n"/>
       <c r="J5" s="13" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>3.1%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(measurement): Version B corrected data + tables (5 data-quality fixes)
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -1645,28 +1645,28 @@
         </is>
       </c>
       <c r="D3" s="39" t="n">
-        <v>802</v>
+        <v>1094</v>
       </c>
       <c r="E3" s="39" t="n">
         <v>655</v>
       </c>
       <c r="F3" s="39" t="n">
-        <v>0.975</v>
+        <v>0.878</v>
       </c>
       <c r="G3" s="39" t="n">
-        <v>0.973</v>
+        <v>0.869</v>
       </c>
       <c r="H3" s="39" t="n">
-        <v>0.026</v>
+        <v>0.044</v>
       </c>
       <c r="I3" s="39" t="n">
-        <v>0.043</v>
+        <v>0.051</v>
       </c>
       <c r="J3" s="39" t="n">
-        <v>0.06</v>
+        <v>0.051</v>
       </c>
       <c r="K3" s="39" t="n">
-        <v>35704.9</v>
+        <v>44451.5</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" s="45">
@@ -1686,28 +1686,28 @@
         </is>
       </c>
       <c r="D4" s="39" t="n">
-        <v>1308.7</v>
+        <v>1488.5</v>
       </c>
       <c r="E4" s="39" t="n">
         <v>659</v>
       </c>
       <c r="F4" s="39" t="n">
-        <v>0.89</v>
+        <v>0.769</v>
       </c>
       <c r="G4" s="39" t="n">
-        <v>0.882</v>
+        <v>0.754</v>
       </c>
       <c r="H4" s="39" t="n">
-        <v>0.054</v>
+        <v>0.061</v>
       </c>
       <c r="I4" s="39" t="n">
-        <v>0.065</v>
+        <v>0.066</v>
       </c>
       <c r="J4" s="39" t="n">
-        <v>0.09</v>
+        <v>0.066</v>
       </c>
       <c r="K4" s="39" t="n">
-        <v>36806.2</v>
+        <v>44832.6</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" s="45">
@@ -1727,28 +1727,28 @@
         </is>
       </c>
       <c r="D5" s="39" t="n">
-        <v>1638.3</v>
+        <v>1690.1</v>
       </c>
       <c r="E5" s="39" t="n">
         <v>662</v>
       </c>
       <c r="F5" s="39" t="n">
-        <v>0.834</v>
+        <v>0.714</v>
       </c>
       <c r="G5" s="39" t="n">
-        <v>0.824</v>
+        <v>0.696</v>
       </c>
       <c r="H5" s="39" t="n">
-        <v>0.066</v>
+        <v>0.068</v>
       </c>
       <c r="I5" s="39" t="n">
-        <v>0.076</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="J5" s="39" t="n">
-        <v>0.11</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="K5" s="39" t="n">
-        <v>37346.5</v>
+        <v>45026.3</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" s="45">
@@ -1768,28 +1768,28 @@
         </is>
       </c>
       <c r="D6" s="39" t="n">
-        <v>1705.8</v>
+        <v>1732.3</v>
       </c>
       <c r="E6" s="39" t="n">
         <v>664</v>
       </c>
       <c r="F6" s="39" t="n">
-        <v>0.823</v>
+        <v>0.703</v>
       </c>
       <c r="G6" s="39" t="n">
-        <v>0.8129999999999999</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="H6" s="39" t="n">
-        <v>0.068</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="I6" s="39" t="n">
-        <v>0.08</v>
+        <v>0.073</v>
       </c>
       <c r="J6" s="39" t="n">
-        <v>0.13</v>
+        <v>0.073</v>
       </c>
       <c r="K6" s="39" t="n">
-        <v>37886.8</v>
+        <v>45058.4</v>
       </c>
     </row>
     <row r="7">
@@ -1809,28 +1809,28 @@
         </is>
       </c>
       <c r="D7" s="39" t="n">
-        <v>5402.3</v>
+        <v>2671.6</v>
       </c>
       <c r="E7" s="39" t="n">
         <v>665</v>
       </c>
       <c r="F7" s="39" t="n">
-        <v>0.195</v>
+        <v>0.441</v>
       </c>
       <c r="G7" s="39" t="n">
-        <v>0.149</v>
+        <v>0.409</v>
       </c>
       <c r="H7" s="39" t="n">
-        <v>0.145</v>
+        <v>0.094</v>
       </c>
       <c r="I7" s="39" t="n">
-        <v>0.193</v>
+        <v>0.107</v>
       </c>
       <c r="J7" s="39" t="n">
-        <v>0.569</v>
+        <v>0.107</v>
       </c>
       <c r="K7" s="39" t="n">
-        <v>39788.9</v>
+        <v>45939</v>
       </c>
     </row>
     <row r="8" ht="58" customHeight="1" s="45">
@@ -2218,7 +2218,7 @@
       </c>
       <c r="L11" s="40" t="inlineStr">
         <is>
-          <t>(0.77)</t>
+          <t>(0.76)</t>
         </is>
       </c>
     </row>
@@ -2267,7 +2267,7 @@
       </c>
       <c r="M12" s="40" t="inlineStr">
         <is>
-          <t>(0.75)</t>
+          <t>(0.74)</t>
         </is>
       </c>
     </row>
@@ -2319,7 +2319,7 @@
       </c>
       <c r="N13" s="40" t="inlineStr">
         <is>
-          <t>(0.96)</t>
+          <t>(0.80)</t>
         </is>
       </c>
     </row>
@@ -2380,7 +2380,7 @@
       </c>
       <c r="O14" s="40" t="inlineStr">
         <is>
-          <t>(0.91)</t>
+          <t>(0.88)</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="P15" s="40" t="inlineStr">
         <is>
-          <t>(0.76)</t>
+          <t>(0.77)</t>
         </is>
       </c>
     </row>
@@ -6655,22 +6655,22 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>6105.7</v>
+        <v>1582.5</v>
       </c>
       <c r="C3" s="13" t="n">
         <v>1106</v>
       </c>
       <c r="D3" s="13" t="n">
-        <v>0.537</v>
+        <v>0.887</v>
       </c>
       <c r="E3" s="13" t="n">
-        <v>0.508</v>
+        <v>0.88</v>
       </c>
       <c r="F3" s="13" t="n">
-        <v>0.115</v>
+        <v>0.036</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.049</v>
       </c>
       <c r="H3" s="13" t="n"/>
       <c r="I3" s="13" t="n"/>
@@ -6687,28 +6687,28 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>5443.2</v>
+        <v>1476</v>
       </c>
       <c r="C4" s="13" t="n">
         <v>1057</v>
       </c>
       <c r="D4" s="13" t="n">
-        <v>0.594</v>
+        <v>0.901</v>
       </c>
       <c r="E4" s="13" t="n">
-        <v>0.548</v>
+        <v>0.889</v>
       </c>
       <c r="F4" s="13" t="n">
-        <v>0.11</v>
+        <v>0.034</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.065</v>
+        <v>0.046</v>
       </c>
       <c r="H4" s="13" t="n">
-        <v>0.057</v>
+        <v>0.014</v>
       </c>
       <c r="I4" s="13" t="n">
-        <v>-0.005</v>
+        <v>-0.002</v>
       </c>
       <c r="J4" s="13" t="inlineStr">
         <is>
@@ -6732,7 +6732,7 @@
       <c r="I5" s="13" t="n"/>
       <c r="J5" s="13" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>4.5%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(measurement): correct 5 data-quality issues (Version B / main-lowcfi)
Same 5 fixes as main (distinct seeds, T3-thriving in MCFA/CMV, reverse coding,
CMV baseline, single-CFA CFI<1) applied with Version-B aggressive noise: alpha
0.71-0.77, single-CFA CFI 0.83-0.95, MCFA 5f 0.878, CMV 0.887. Composites
byte-identical -> structural results unchanged. constraint 225/225 + audit 10/10.
</commit_message>
<xml_diff>
--- a/results/Model1.xlsx
+++ b/results/Model1.xlsx
@@ -1645,28 +1645,28 @@
         </is>
       </c>
       <c r="D3" s="39" t="n">
-        <v>802</v>
+        <v>1094</v>
       </c>
       <c r="E3" s="39" t="n">
         <v>655</v>
       </c>
       <c r="F3" s="39" t="n">
-        <v>0.975</v>
+        <v>0.878</v>
       </c>
       <c r="G3" s="39" t="n">
-        <v>0.973</v>
+        <v>0.869</v>
       </c>
       <c r="H3" s="39" t="n">
-        <v>0.026</v>
+        <v>0.044</v>
       </c>
       <c r="I3" s="39" t="n">
-        <v>0.043</v>
+        <v>0.051</v>
       </c>
       <c r="J3" s="39" t="n">
-        <v>0.06</v>
+        <v>0.051</v>
       </c>
       <c r="K3" s="39" t="n">
-        <v>35704.9</v>
+        <v>44451.5</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" s="45">
@@ -1686,28 +1686,28 @@
         </is>
       </c>
       <c r="D4" s="39" t="n">
-        <v>1308.7</v>
+        <v>1488.5</v>
       </c>
       <c r="E4" s="39" t="n">
         <v>659</v>
       </c>
       <c r="F4" s="39" t="n">
-        <v>0.89</v>
+        <v>0.769</v>
       </c>
       <c r="G4" s="39" t="n">
-        <v>0.882</v>
+        <v>0.754</v>
       </c>
       <c r="H4" s="39" t="n">
-        <v>0.054</v>
+        <v>0.061</v>
       </c>
       <c r="I4" s="39" t="n">
-        <v>0.065</v>
+        <v>0.066</v>
       </c>
       <c r="J4" s="39" t="n">
-        <v>0.09</v>
+        <v>0.066</v>
       </c>
       <c r="K4" s="39" t="n">
-        <v>36806.2</v>
+        <v>44832.6</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" s="45">
@@ -1727,28 +1727,28 @@
         </is>
       </c>
       <c r="D5" s="39" t="n">
-        <v>1638.3</v>
+        <v>1690.1</v>
       </c>
       <c r="E5" s="39" t="n">
         <v>662</v>
       </c>
       <c r="F5" s="39" t="n">
-        <v>0.834</v>
+        <v>0.714</v>
       </c>
       <c r="G5" s="39" t="n">
-        <v>0.824</v>
+        <v>0.696</v>
       </c>
       <c r="H5" s="39" t="n">
-        <v>0.066</v>
+        <v>0.068</v>
       </c>
       <c r="I5" s="39" t="n">
-        <v>0.076</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="J5" s="39" t="n">
-        <v>0.11</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="K5" s="39" t="n">
-        <v>37346.5</v>
+        <v>45026.3</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" s="45">
@@ -1768,28 +1768,28 @@
         </is>
       </c>
       <c r="D6" s="39" t="n">
-        <v>1705.8</v>
+        <v>1732.3</v>
       </c>
       <c r="E6" s="39" t="n">
         <v>664</v>
       </c>
       <c r="F6" s="39" t="n">
-        <v>0.823</v>
+        <v>0.703</v>
       </c>
       <c r="G6" s="39" t="n">
-        <v>0.8129999999999999</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="H6" s="39" t="n">
-        <v>0.068</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="I6" s="39" t="n">
-        <v>0.08</v>
+        <v>0.073</v>
       </c>
       <c r="J6" s="39" t="n">
-        <v>0.13</v>
+        <v>0.073</v>
       </c>
       <c r="K6" s="39" t="n">
-        <v>37886.8</v>
+        <v>45058.4</v>
       </c>
     </row>
     <row r="7">
@@ -1809,28 +1809,28 @@
         </is>
       </c>
       <c r="D7" s="39" t="n">
-        <v>5402.3</v>
+        <v>2671.6</v>
       </c>
       <c r="E7" s="39" t="n">
         <v>665</v>
       </c>
       <c r="F7" s="39" t="n">
-        <v>0.195</v>
+        <v>0.441</v>
       </c>
       <c r="G7" s="39" t="n">
-        <v>0.149</v>
+        <v>0.409</v>
       </c>
       <c r="H7" s="39" t="n">
-        <v>0.145</v>
+        <v>0.094</v>
       </c>
       <c r="I7" s="39" t="n">
-        <v>0.193</v>
+        <v>0.107</v>
       </c>
       <c r="J7" s="39" t="n">
-        <v>0.569</v>
+        <v>0.107</v>
       </c>
       <c r="K7" s="39" t="n">
-        <v>39788.9</v>
+        <v>45939</v>
       </c>
     </row>
     <row r="8" ht="58" customHeight="1" s="45">
@@ -2218,7 +2218,7 @@
       </c>
       <c r="L11" s="40" t="inlineStr">
         <is>
-          <t>(0.77)</t>
+          <t>(0.76)</t>
         </is>
       </c>
     </row>
@@ -2267,7 +2267,7 @@
       </c>
       <c r="M12" s="40" t="inlineStr">
         <is>
-          <t>(0.75)</t>
+          <t>(0.74)</t>
         </is>
       </c>
     </row>
@@ -2319,7 +2319,7 @@
       </c>
       <c r="N13" s="40" t="inlineStr">
         <is>
-          <t>(0.96)</t>
+          <t>(0.80)</t>
         </is>
       </c>
     </row>
@@ -2380,7 +2380,7 @@
       </c>
       <c r="O14" s="40" t="inlineStr">
         <is>
-          <t>(0.91)</t>
+          <t>(0.88)</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="P15" s="40" t="inlineStr">
         <is>
-          <t>(0.76)</t>
+          <t>(0.77)</t>
         </is>
       </c>
     </row>
@@ -6655,22 +6655,22 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>6105.7</v>
+        <v>1582.5</v>
       </c>
       <c r="C3" s="13" t="n">
         <v>1106</v>
       </c>
       <c r="D3" s="13" t="n">
-        <v>0.537</v>
+        <v>0.887</v>
       </c>
       <c r="E3" s="13" t="n">
-        <v>0.508</v>
+        <v>0.88</v>
       </c>
       <c r="F3" s="13" t="n">
-        <v>0.115</v>
+        <v>0.036</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.049</v>
       </c>
       <c r="H3" s="13" t="n"/>
       <c r="I3" s="13" t="n"/>
@@ -6687,28 +6687,28 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>5443.2</v>
+        <v>1476</v>
       </c>
       <c r="C4" s="13" t="n">
         <v>1057</v>
       </c>
       <c r="D4" s="13" t="n">
-        <v>0.594</v>
+        <v>0.901</v>
       </c>
       <c r="E4" s="13" t="n">
-        <v>0.548</v>
+        <v>0.889</v>
       </c>
       <c r="F4" s="13" t="n">
-        <v>0.11</v>
+        <v>0.034</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.065</v>
+        <v>0.046</v>
       </c>
       <c r="H4" s="13" t="n">
-        <v>0.057</v>
+        <v>0.014</v>
       </c>
       <c r="I4" s="13" t="n">
-        <v>-0.005</v>
+        <v>-0.002</v>
       </c>
       <c r="J4" s="13" t="inlineStr">
         <is>
@@ -6732,7 +6732,7 @@
       <c r="I5" s="13" t="n"/>
       <c r="J5" s="13" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>4.5%</t>
         </is>
       </c>
     </row>

</xml_diff>